<commit_message>
refresh 2026-08-21 04:59 UTC
</commit_message>
<xml_diff>
--- a/NCAAF_Edge_Model.xlsx
+++ b/NCAAF_Edge_Model.xlsx
@@ -637,7 +637,7 @@
     <row r="2" ht="26" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-08-21T04:30:02+00:00 from live ESPN data. This file is a snapshot, not the model. Re-run the pipeline to refresh it.</t>
+          <t>Generated 2026-08-21T04:59:28+00:00 from live ESPN data. This file is a snapshot, not the model. Re-run the pipeline to refresh it.</t>
         </is>
       </c>
     </row>
@@ -46301,7 +46301,7 @@
       </c>
       <c r="B50" s="12" t="inlineStr">
         <is>
-          <t>UNT @ IU</t>
+          <t>ECU @ ALA</t>
         </is>
       </c>
       <c r="C50" s="12" t="inlineStr">
@@ -46311,7 +46311,7 @@
       </c>
       <c r="D50" s="12" t="inlineStr">
         <is>
-          <t>UNT +40.5</t>
+          <t>ECU +28.5</t>
         </is>
       </c>
       <c r="E50" s="13" t="n">
@@ -46343,7 +46343,7 @@
         </is>
       </c>
       <c r="L50" s="14" t="n">
-        <v>0.2251</v>
+        <v>0.2175</v>
       </c>
       <c r="M50" s="14" t="n"/>
       <c r="N50" s="12" t="n"/>
@@ -46361,7 +46361,7 @@
       </c>
       <c r="B51" s="17" t="inlineStr">
         <is>
-          <t>ECU @ ALA</t>
+          <t>UNT @ IU</t>
         </is>
       </c>
       <c r="C51" s="17" t="inlineStr">
@@ -46371,7 +46371,7 @@
       </c>
       <c r="D51" s="17" t="inlineStr">
         <is>
-          <t>ECU +28.5</t>
+          <t>UNT +40.5</t>
         </is>
       </c>
       <c r="E51" s="18" t="n">
@@ -46403,7 +46403,7 @@
         </is>
       </c>
       <c r="L51" s="19" t="n">
-        <v>0.2175</v>
+        <v>0.2251</v>
       </c>
       <c r="M51" s="19" t="n"/>
       <c r="N51" s="17" t="n"/>

</xml_diff>

<commit_message>
refresh 2026-08-21 18:01 UTC
</commit_message>
<xml_diff>
--- a/NCAAF_Edge_Model.xlsx
+++ b/NCAAF_Edge_Model.xlsx
@@ -637,7 +637,7 @@
     <row r="2" ht="26" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-08-21T14:58:27+00:00 from live ESPN data. This file is a snapshot, not the model. Re-run the pipeline to refresh it.</t>
+          <t>Generated 2026-08-21T18:01:28+00:00 from live ESPN data. This file is a snapshot, not the model. Re-run the pipeline to refresh it.</t>
         </is>
       </c>
     </row>
@@ -2040,7 +2040,7 @@
       </c>
       <c r="P10" s="17" t="inlineStr">
         <is>
-          <t>Draft Kings</t>
+          <t>DraftKings</t>
         </is>
       </c>
       <c r="Q10" s="17" t="n"/>
@@ -2166,7 +2166,7 @@
       </c>
       <c r="P12" s="17" t="inlineStr">
         <is>
-          <t>Draft Kings</t>
+          <t>DraftKings</t>
         </is>
       </c>
       <c r="Q12" s="17" t="n"/>
@@ -8588,7 +8588,7 @@
       </c>
       <c r="P110" s="17" t="inlineStr">
         <is>
-          <t>Draft Kings</t>
+          <t>DraftKings</t>
         </is>
       </c>
       <c r="Q110" s="17" t="inlineStr">
@@ -9526,7 +9526,7 @@
       </c>
       <c r="P124" s="17" t="inlineStr">
         <is>
-          <t>Draft Kings</t>
+          <t>DraftKings</t>
         </is>
       </c>
       <c r="Q124" s="17" t="inlineStr">
@@ -11134,7 +11134,7 @@
       </c>
       <c r="P148" s="17" t="inlineStr">
         <is>
-          <t>Draft Kings</t>
+          <t>DraftKings</t>
         </is>
       </c>
       <c r="Q148" s="17" t="inlineStr">
@@ -11201,7 +11201,7 @@
       </c>
       <c r="P149" s="12" t="inlineStr">
         <is>
-          <t>Draft Kings</t>
+          <t>DraftKings</t>
         </is>
       </c>
       <c r="Q149" s="12" t="inlineStr">
@@ -11532,7 +11532,7 @@
       </c>
       <c r="P154" s="17" t="inlineStr">
         <is>
-          <t>Draft Kings</t>
+          <t>DraftKings</t>
         </is>
       </c>
       <c r="Q154" s="17" t="n"/>
@@ -12611,7 +12611,7 @@
       </c>
       <c r="P171" s="12" t="inlineStr">
         <is>
-          <t>Draft Kings</t>
+          <t>DraftKings</t>
         </is>
       </c>
       <c r="Q171" s="12" t="n"/>
@@ -14718,7 +14718,7 @@
       </c>
       <c r="P204" s="17" t="inlineStr">
         <is>
-          <t>Draft Kings</t>
+          <t>DraftKings</t>
         </is>
       </c>
       <c r="Q204" s="17" t="n"/>
@@ -15671,7 +15671,7 @@
       </c>
       <c r="P219" s="12" t="inlineStr">
         <is>
-          <t>Draft Kings</t>
+          <t>DraftKings</t>
         </is>
       </c>
       <c r="Q219" s="12" t="n"/>
@@ -16305,7 +16305,7 @@
       </c>
       <c r="P229" s="12" t="inlineStr">
         <is>
-          <t>Draft Kings</t>
+          <t>DraftKings</t>
         </is>
       </c>
       <c r="Q229" s="12" t="n"/>
@@ -16683,7 +16683,7 @@
       </c>
       <c r="P235" s="12" t="inlineStr">
         <is>
-          <t>Draft Kings</t>
+          <t>DraftKings</t>
         </is>
       </c>
       <c r="Q235" s="12" t="n"/>
@@ -17191,7 +17191,7 @@
       </c>
       <c r="P243" s="12" t="inlineStr">
         <is>
-          <t>Draft Kings</t>
+          <t>DraftKings</t>
         </is>
       </c>
       <c r="Q243" s="12" t="n"/>
@@ -18396,7 +18396,7 @@
       </c>
       <c r="P262" s="17" t="inlineStr">
         <is>
-          <t>Draft Kings</t>
+          <t>DraftKings</t>
         </is>
       </c>
       <c r="Q262" s="17" t="n"/>
@@ -18593,7 +18593,7 @@
       </c>
       <c r="P265" s="12" t="inlineStr">
         <is>
-          <t>Draft Kings</t>
+          <t>DraftKings</t>
         </is>
       </c>
       <c r="Q265" s="12" t="n"/>
@@ -19806,7 +19806,7 @@
       </c>
       <c r="P284" s="17" t="inlineStr">
         <is>
-          <t>Draft Kings</t>
+          <t>DraftKings</t>
         </is>
       </c>
       <c r="Q284" s="17" t="n"/>
@@ -25611,7 +25611,7 @@
       </c>
       <c r="P375" s="12" t="inlineStr">
         <is>
-          <t>Draft Kings</t>
+          <t>DraftKings</t>
         </is>
       </c>
       <c r="Q375" s="12" t="n"/>
@@ -26824,7 +26824,7 @@
       </c>
       <c r="P394" s="17" t="inlineStr">
         <is>
-          <t>Draft Kings</t>
+          <t>DraftKings</t>
         </is>
       </c>
       <c r="Q394" s="17" t="n"/>
@@ -27021,7 +27021,7 @@
       </c>
       <c r="P397" s="12" t="inlineStr">
         <is>
-          <t>Draft Kings</t>
+          <t>DraftKings</t>
         </is>
       </c>
       <c r="Q397" s="12" t="n"/>
@@ -28226,7 +28226,7 @@
       </c>
       <c r="P416" s="17" t="inlineStr">
         <is>
-          <t>Draft Kings</t>
+          <t>DraftKings</t>
         </is>
       </c>
       <c r="Q416" s="17" t="n"/>
@@ -28734,7 +28734,7 @@
       </c>
       <c r="P424" s="17" t="inlineStr">
         <is>
-          <t>Draft Kings</t>
+          <t>DraftKings</t>
         </is>
       </c>
       <c r="Q424" s="17" t="n"/>
@@ -29112,7 +29112,7 @@
       </c>
       <c r="P430" s="17" t="inlineStr">
         <is>
-          <t>Draft Kings</t>
+          <t>DraftKings</t>
         </is>
       </c>
       <c r="Q430" s="17" t="n"/>
@@ -29746,7 +29746,7 @@
       </c>
       <c r="P440" s="17" t="inlineStr">
         <is>
-          <t>Draft Kings</t>
+          <t>DraftKings</t>
         </is>
       </c>
       <c r="Q440" s="17" t="n"/>
@@ -30699,7 +30699,7 @@
       </c>
       <c r="P455" s="12" t="inlineStr">
         <is>
-          <t>Draft Kings</t>
+          <t>DraftKings</t>
         </is>
       </c>
       <c r="Q455" s="12" t="n"/>
@@ -32806,7 +32806,7 @@
       </c>
       <c r="P488" s="17" t="inlineStr">
         <is>
-          <t>Draft Kings</t>
+          <t>DraftKings</t>
         </is>
       </c>
       <c r="Q488" s="17" t="n"/>
@@ -33885,7 +33885,7 @@
       </c>
       <c r="P505" s="12" t="inlineStr">
         <is>
-          <t>Draft Kings</t>
+          <t>DraftKings</t>
         </is>
       </c>
       <c r="Q505" s="12" t="n"/>
@@ -34145,7 +34145,7 @@
       </c>
       <c r="P509" s="12" t="inlineStr">
         <is>
-          <t>Draft Kings</t>
+          <t>DraftKings</t>
         </is>
       </c>
       <c r="Q509" s="12" t="n"/>
@@ -34334,7 +34334,7 @@
       </c>
       <c r="P512" s="17" t="inlineStr">
         <is>
-          <t>Draft Kings</t>
+          <t>DraftKings</t>
         </is>
       </c>
       <c r="Q512" s="17" t="n"/>
@@ -36512,7 +36512,7 @@
       </c>
       <c r="P546" s="17" t="inlineStr">
         <is>
-          <t>Draft Kings</t>
+          <t>DraftKings</t>
         </is>
       </c>
       <c r="Q546" s="17" t="n"/>
@@ -37993,7 +37993,7 @@
       </c>
       <c r="P569" s="12" t="inlineStr">
         <is>
-          <t>Draft Kings</t>
+          <t>DraftKings</t>
         </is>
       </c>
       <c r="Q569" s="12" t="n"/>
@@ -41601,7 +41601,7 @@
       </c>
       <c r="P625" s="12" t="inlineStr">
         <is>
-          <t>Draft Kings</t>
+          <t>DraftKings</t>
         </is>
       </c>
       <c r="Q625" s="12" t="n"/>
@@ -41928,7 +41928,7 @@
       </c>
       <c r="P630" s="17" t="inlineStr">
         <is>
-          <t>Draft Kings</t>
+          <t>DraftKings</t>
         </is>
       </c>
       <c r="Q630" s="17" t="n"/>
@@ -53377,7 +53377,7 @@
       <c r="L5" s="13" t="n"/>
       <c r="M5" s="12" t="inlineStr">
         <is>
-          <t>Draft Kings</t>
+          <t>DraftKings</t>
         </is>
       </c>
     </row>
@@ -53422,7 +53422,7 @@
       <c r="L6" s="18" t="n"/>
       <c r="M6" s="17" t="inlineStr">
         <is>
-          <t>Draft Kings</t>
+          <t>DraftKings</t>
         </is>
       </c>
     </row>
@@ -53467,7 +53467,7 @@
       <c r="L7" s="13" t="n"/>
       <c r="M7" s="12" t="inlineStr">
         <is>
-          <t>Draft Kings</t>
+          <t>DraftKings</t>
         </is>
       </c>
     </row>
@@ -53512,7 +53512,7 @@
       <c r="L8" s="18" t="n"/>
       <c r="M8" s="17" t="inlineStr">
         <is>
-          <t>Draft Kings</t>
+          <t>DraftKings</t>
         </is>
       </c>
     </row>
@@ -53557,7 +53557,7 @@
       <c r="L9" s="13" t="n"/>
       <c r="M9" s="12" t="inlineStr">
         <is>
-          <t>Draft Kings</t>
+          <t>DraftKings</t>
         </is>
       </c>
     </row>
@@ -53602,7 +53602,7 @@
       <c r="L10" s="18" t="n"/>
       <c r="M10" s="17" t="inlineStr">
         <is>
-          <t>Draft Kings</t>
+          <t>DraftKings</t>
         </is>
       </c>
     </row>
@@ -53647,7 +53647,7 @@
       <c r="L11" s="13" t="n"/>
       <c r="M11" s="12" t="inlineStr">
         <is>
-          <t>Draft Kings</t>
+          <t>DraftKings</t>
         </is>
       </c>
     </row>
@@ -53692,7 +53692,7 @@
       <c r="L12" s="18" t="n"/>
       <c r="M12" s="17" t="inlineStr">
         <is>
-          <t>Draft Kings</t>
+          <t>DraftKings</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
refresh 2026-08-21 21:54 UTC
</commit_message>
<xml_diff>
--- a/NCAAF_Edge_Model.xlsx
+++ b/NCAAF_Edge_Model.xlsx
@@ -637,7 +637,7 @@
     <row r="2" ht="26" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-08-21T18:01:28+00:00 from live ESPN data. This file is a snapshot, not the model. Re-run the pipeline to refresh it.</t>
+          <t>Generated 2026-08-21T21:54:35+00:00 from live ESPN data. This file is a snapshot, not the model. Re-run the pipeline to refresh it.</t>
         </is>
       </c>
     </row>
@@ -18543,12 +18543,12 @@
       </c>
       <c r="B265" s="12" t="inlineStr">
         <is>
-          <t>MEM @ UNLV</t>
+          <t>FAU @ FLA</t>
         </is>
       </c>
       <c r="C265" s="12" t="inlineStr">
         <is>
-          <t>2026-08-30 02:00</t>
+          <t>2026-09-05 23:45</t>
         </is>
       </c>
       <c r="D265" s="22" t="n">
@@ -18561,17 +18561,17 @@
       </c>
       <c r="F265" s="12" t="inlineStr">
         <is>
-          <t>Over 56.5</t>
+          <t>Under 58.5</t>
         </is>
       </c>
       <c r="G265" s="23" t="n">
-        <v>56.5</v>
+        <v>58.5</v>
       </c>
       <c r="H265" s="13" t="n">
         <v>-110</v>
       </c>
       <c r="I265" s="15" t="n">
-        <v>0.5298211850615678</v>
+        <v>0.5298211834152686</v>
       </c>
       <c r="J265" s="15" t="n">
         <v>0.5</v>
@@ -18580,10 +18580,10 @@
         <v>0.5238095238095238</v>
       </c>
       <c r="L265" s="14" t="n">
-        <v>0.006011661252043998</v>
+        <v>0.00601165960574479</v>
       </c>
       <c r="M265" s="14" t="n">
-        <v>0.01147680784481137</v>
+        <v>0.01147680470187651</v>
       </c>
       <c r="N265" s="15" t="n">
         <v>0</v>
@@ -18606,16 +18606,16 @@
       </c>
       <c r="B266" s="17" t="inlineStr">
         <is>
-          <t>FAU @ FLA</t>
+          <t>WASH @ ORE</t>
         </is>
       </c>
       <c r="C266" s="17" t="inlineStr">
         <is>
-          <t>2026-09-05 23:45</t>
+          <t>2026-11-28 05:00</t>
         </is>
       </c>
       <c r="D266" s="25" t="n">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="E266" s="17" t="inlineStr">
         <is>
@@ -18624,17 +18624,17 @@
       </c>
       <c r="F266" s="17" t="inlineStr">
         <is>
-          <t>Under 58.5</t>
+          <t>Over 54.5</t>
         </is>
       </c>
       <c r="G266" s="26" t="n">
-        <v>58.5</v>
+        <v>54.5</v>
       </c>
       <c r="H266" s="18" t="n">
         <v>-110</v>
       </c>
       <c r="I266" s="20" t="n">
-        <v>0.5298211834152686</v>
+        <v>0.5278465371051131</v>
       </c>
       <c r="J266" s="20" t="n">
         <v>0.5</v>
@@ -18643,10 +18643,10 @@
         <v>0.5238095238095238</v>
       </c>
       <c r="L266" s="19" t="n">
-        <v>0.00601165960574479</v>
+        <v>0.004037013295589253</v>
       </c>
       <c r="M266" s="19" t="n">
-        <v>0.01147680470187651</v>
+        <v>0.007707025382488686</v>
       </c>
       <c r="N266" s="20" t="n">
         <v>0</v>
@@ -18669,16 +18669,16 @@
       </c>
       <c r="B267" s="12" t="inlineStr">
         <is>
-          <t>WASH @ ORE</t>
+          <t>ULM @ MSST</t>
         </is>
       </c>
       <c r="C267" s="12" t="inlineStr">
         <is>
-          <t>2026-11-28 05:00</t>
+          <t>2026-09-05 23:30</t>
         </is>
       </c>
       <c r="D267" s="22" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="E267" s="12" t="inlineStr">
         <is>
@@ -18687,17 +18687,17 @@
       </c>
       <c r="F267" s="12" t="inlineStr">
         <is>
-          <t>Over 54.5</t>
+          <t>Over 55.5</t>
         </is>
       </c>
       <c r="G267" s="23" t="n">
-        <v>54.5</v>
+        <v>55.5</v>
       </c>
       <c r="H267" s="13" t="n">
         <v>-110</v>
       </c>
       <c r="I267" s="15" t="n">
-        <v>0.5278465371051131</v>
+        <v>0.5278465360715345</v>
       </c>
       <c r="J267" s="15" t="n">
         <v>0.5</v>
@@ -18706,10 +18706,10 @@
         <v>0.5238095238095238</v>
       </c>
       <c r="L267" s="14" t="n">
-        <v>0.004037013295589253</v>
+        <v>0.004037012262010697</v>
       </c>
       <c r="M267" s="14" t="n">
-        <v>0.007707025382488686</v>
+        <v>0.007707023409293245</v>
       </c>
       <c r="N267" s="15" t="n">
         <v>0</v>
@@ -18732,12 +18732,12 @@
       </c>
       <c r="B268" s="17" t="inlineStr">
         <is>
-          <t>ULM @ MSST</t>
+          <t>IDHO @ UTAH</t>
         </is>
       </c>
       <c r="C268" s="17" t="inlineStr">
         <is>
-          <t>2026-09-05 23:30</t>
+          <t>2026-09-04 01:00</t>
         </is>
       </c>
       <c r="D268" s="25" t="n">
@@ -18750,17 +18750,17 @@
       </c>
       <c r="F268" s="17" t="inlineStr">
         <is>
-          <t>Over 55.5</t>
+          <t>Over 56.5</t>
         </is>
       </c>
       <c r="G268" s="26" t="n">
-        <v>55.5</v>
+        <v>56.5</v>
       </c>
       <c r="H268" s="18" t="n">
         <v>-110</v>
       </c>
       <c r="I268" s="20" t="n">
-        <v>0.5278465360715345</v>
+        <v>0.5278465354893196</v>
       </c>
       <c r="J268" s="20" t="n">
         <v>0.5</v>
@@ -18769,10 +18769,10 @@
         <v>0.5238095238095238</v>
       </c>
       <c r="L268" s="19" t="n">
-        <v>0.004037012262010697</v>
+        <v>0.004037011679795754</v>
       </c>
       <c r="M268" s="19" t="n">
-        <v>0.007707023409293245</v>
+        <v>0.007707022297791966</v>
       </c>
       <c r="N268" s="20" t="n">
         <v>0</v>
@@ -18785,7 +18785,11 @@
           <t>DraftKings</t>
         </is>
       </c>
-      <c r="Q268" s="17" t="n"/>
+      <c r="Q268" s="17" t="inlineStr">
+        <is>
+          <t>IDHO isn't a full FBS participant this season — model doesn't rate them reliably</t>
+        </is>
+      </c>
     </row>
     <row r="269">
       <c r="A269" s="12" t="inlineStr">
@@ -18795,16 +18799,16 @@
       </c>
       <c r="B269" s="12" t="inlineStr">
         <is>
-          <t>IDHO @ UTAH</t>
+          <t>TEX @ LSU</t>
         </is>
       </c>
       <c r="C269" s="12" t="inlineStr">
         <is>
-          <t>2026-09-04 01:00</t>
+          <t>2026-11-14 05:00</t>
         </is>
       </c>
       <c r="D269" s="22" t="n">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="E269" s="12" t="inlineStr">
         <is>
@@ -18813,17 +18817,17 @@
       </c>
       <c r="F269" s="12" t="inlineStr">
         <is>
-          <t>Over 56.5</t>
+          <t>Under 54.5</t>
         </is>
       </c>
       <c r="G269" s="23" t="n">
-        <v>56.5</v>
+        <v>54.5</v>
       </c>
       <c r="H269" s="13" t="n">
         <v>-110</v>
       </c>
       <c r="I269" s="15" t="n">
-        <v>0.5278465354893196</v>
+        <v>0.5278465256441186</v>
       </c>
       <c r="J269" s="15" t="n">
         <v>0.5</v>
@@ -18832,10 +18836,10 @@
         <v>0.5238095238095238</v>
       </c>
       <c r="L269" s="14" t="n">
-        <v>0.004037011679795754</v>
+        <v>0.004037001834594767</v>
       </c>
       <c r="M269" s="14" t="n">
-        <v>0.007707022297791966</v>
+        <v>0.007707003502408272</v>
       </c>
       <c r="N269" s="15" t="n">
         <v>0</v>
@@ -18848,11 +18852,7 @@
           <t>DraftKings</t>
         </is>
       </c>
-      <c r="Q269" s="12" t="inlineStr">
-        <is>
-          <t>IDHO isn't a full FBS participant this season — model doesn't rate them reliably</t>
-        </is>
-      </c>
+      <c r="Q269" s="12" t="n"/>
     </row>
     <row r="270">
       <c r="A270" s="17" t="inlineStr">
@@ -18862,35 +18862,35 @@
       </c>
       <c r="B270" s="17" t="inlineStr">
         <is>
-          <t>TEX @ LSU</t>
+          <t>NAVY @ ARMY</t>
         </is>
       </c>
       <c r="C270" s="17" t="inlineStr">
         <is>
-          <t>2026-11-14 05:00</t>
+          <t>2026-12-12 20:00</t>
         </is>
       </c>
       <c r="D270" s="25" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="E270" s="17" t="inlineStr">
         <is>
-          <t>TOTAL</t>
+          <t>ATS</t>
         </is>
       </c>
       <c r="F270" s="17" t="inlineStr">
         <is>
-          <t>Under 54.5</t>
+          <t>ARMY +2.5</t>
         </is>
       </c>
       <c r="G270" s="26" t="n">
-        <v>54.5</v>
+        <v>2.5</v>
       </c>
       <c r="H270" s="18" t="n">
         <v>-110</v>
       </c>
       <c r="I270" s="20" t="n">
-        <v>0.5278465256441186</v>
+        <v>0.527327071096132</v>
       </c>
       <c r="J270" s="20" t="n">
         <v>0.5</v>
@@ -18899,10 +18899,10 @@
         <v>0.5238095238095238</v>
       </c>
       <c r="L270" s="19" t="n">
-        <v>0.004037001834594767</v>
+        <v>0.003517547286608136</v>
       </c>
       <c r="M270" s="19" t="n">
-        <v>0.007707003502408272</v>
+        <v>0.006715317547161093</v>
       </c>
       <c r="N270" s="20" t="n">
         <v>0</v>
@@ -18925,16 +18925,16 @@
       </c>
       <c r="B271" s="12" t="inlineStr">
         <is>
-          <t>NAVY @ ARMY</t>
+          <t>UVA @ VT</t>
         </is>
       </c>
       <c r="C271" s="12" t="inlineStr">
         <is>
-          <t>2026-12-12 20:00</t>
+          <t>2026-11-28 05:00</t>
         </is>
       </c>
       <c r="D271" s="22" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="E271" s="12" t="inlineStr">
         <is>
@@ -18943,17 +18943,17 @@
       </c>
       <c r="F271" s="12" t="inlineStr">
         <is>
-          <t>ARMY +2.5</t>
+          <t>UVA +1.5</t>
         </is>
       </c>
       <c r="G271" s="23" t="n">
-        <v>2.5</v>
+        <v>-1.5</v>
       </c>
       <c r="H271" s="13" t="n">
         <v>-110</v>
       </c>
       <c r="I271" s="15" t="n">
-        <v>0.527327071096132</v>
+        <v>0.5262747671380312</v>
       </c>
       <c r="J271" s="15" t="n">
         <v>0.5</v>
@@ -18962,10 +18962,10 @@
         <v>0.5238095238095238</v>
       </c>
       <c r="L271" s="14" t="n">
-        <v>0.003517547286608136</v>
+        <v>0.002465243328507394</v>
       </c>
       <c r="M271" s="14" t="n">
-        <v>0.006715317547161093</v>
+        <v>0.004706373627150595</v>
       </c>
       <c r="N271" s="15" t="n">
         <v>0</v>
@@ -18988,35 +18988,35 @@
       </c>
       <c r="B272" s="17" t="inlineStr">
         <is>
-          <t>UVA @ VT</t>
+          <t>VMI @ VT</t>
         </is>
       </c>
       <c r="C272" s="17" t="inlineStr">
         <is>
-          <t>2026-11-28 05:00</t>
+          <t>2026-09-05 23:30</t>
         </is>
       </c>
       <c r="D272" s="25" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="E272" s="17" t="inlineStr">
         <is>
-          <t>ATS</t>
+          <t>TOTAL</t>
         </is>
       </c>
       <c r="F272" s="17" t="inlineStr">
         <is>
-          <t>UVA +1.5</t>
+          <t>Under 57.5</t>
         </is>
       </c>
       <c r="G272" s="26" t="n">
-        <v>-1.5</v>
+        <v>57.5</v>
       </c>
       <c r="H272" s="18" t="n">
         <v>-110</v>
       </c>
       <c r="I272" s="20" t="n">
-        <v>0.5262747671380312</v>
+        <v>0.5258691148547187</v>
       </c>
       <c r="J272" s="20" t="n">
         <v>0.5</v>
@@ -19025,10 +19025,10 @@
         <v>0.5238095238095238</v>
       </c>
       <c r="L272" s="19" t="n">
-        <v>0.002465243328507394</v>
+        <v>0.00205959104519482</v>
       </c>
       <c r="M272" s="19" t="n">
-        <v>0.004706373627150595</v>
+        <v>0.00393194654082657</v>
       </c>
       <c r="N272" s="20" t="n">
         <v>0</v>
@@ -19041,7 +19041,11 @@
           <t>DraftKings</t>
         </is>
       </c>
-      <c r="Q272" s="17" t="n"/>
+      <c r="Q272" s="17" t="inlineStr">
+        <is>
+          <t>VMI isn't a full FBS participant this season — model doesn't rate them reliably</t>
+        </is>
+      </c>
     </row>
     <row r="273">
       <c r="A273" s="12" t="inlineStr">
@@ -19051,16 +19055,16 @@
       </c>
       <c r="B273" s="12" t="inlineStr">
         <is>
-          <t>VMI @ VT</t>
+          <t>NCSU @ UNC</t>
         </is>
       </c>
       <c r="C273" s="12" t="inlineStr">
         <is>
-          <t>2026-09-05 23:30</t>
+          <t>2026-11-28 05:00</t>
         </is>
       </c>
       <c r="D273" s="22" t="n">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="E273" s="12" t="inlineStr">
         <is>
@@ -19069,17 +19073,17 @@
       </c>
       <c r="F273" s="12" t="inlineStr">
         <is>
-          <t>Under 57.5</t>
+          <t>Under 55.5</t>
         </is>
       </c>
       <c r="G273" s="23" t="n">
-        <v>57.5</v>
+        <v>55.5</v>
       </c>
       <c r="H273" s="13" t="n">
         <v>-110</v>
       </c>
       <c r="I273" s="15" t="n">
-        <v>0.5258691148547187</v>
+        <v>0.5258691114540864</v>
       </c>
       <c r="J273" s="15" t="n">
         <v>0.5</v>
@@ -19088,10 +19092,10 @@
         <v>0.5238095238095238</v>
       </c>
       <c r="L273" s="14" t="n">
-        <v>0.00205959104519482</v>
+        <v>0.002059587644562599</v>
       </c>
       <c r="M273" s="14" t="n">
-        <v>0.00393194654082657</v>
+        <v>0.003931940048710503</v>
       </c>
       <c r="N273" s="15" t="n">
         <v>0</v>
@@ -19104,11 +19108,7 @@
           <t>DraftKings</t>
         </is>
       </c>
-      <c r="Q273" s="12" t="inlineStr">
-        <is>
-          <t>VMI isn't a full FBS participant this season — model doesn't rate them reliably</t>
-        </is>
-      </c>
+      <c r="Q273" s="12" t="n"/>
     </row>
     <row r="274">
       <c r="A274" s="17" t="inlineStr">
@@ -19118,7 +19118,7 @@
       </c>
       <c r="B274" s="17" t="inlineStr">
         <is>
-          <t>NCSU @ UNC</t>
+          <t>ASU @ ARIZ</t>
         </is>
       </c>
       <c r="C274" s="17" t="inlineStr">
@@ -19131,22 +19131,22 @@
       </c>
       <c r="E274" s="17" t="inlineStr">
         <is>
-          <t>TOTAL</t>
+          <t>ATS</t>
         </is>
       </c>
       <c r="F274" s="17" t="inlineStr">
         <is>
-          <t>Under 55.5</t>
+          <t>ASU +4.5</t>
         </is>
       </c>
       <c r="G274" s="26" t="n">
-        <v>55.5</v>
+        <v>-4.5</v>
       </c>
       <c r="H274" s="18" t="n">
         <v>-110</v>
       </c>
       <c r="I274" s="20" t="n">
-        <v>0.5258691114540864</v>
+        <v>0.5240821001886855</v>
       </c>
       <c r="J274" s="20" t="n">
         <v>0.5</v>
@@ -19155,10 +19155,10 @@
         <v>0.5238095238095238</v>
       </c>
       <c r="L274" s="19" t="n">
-        <v>0.002059587644562599</v>
+        <v>0.0002725763791616709</v>
       </c>
       <c r="M274" s="19" t="n">
-        <v>0.003931940048710503</v>
+        <v>0.0005203730874905332</v>
       </c>
       <c r="N274" s="20" t="n">
         <v>0</v>
@@ -19181,35 +19181,35 @@
       </c>
       <c r="B275" s="12" t="inlineStr">
         <is>
-          <t>ASU @ ARIZ</t>
+          <t>KENT @ SC</t>
         </is>
       </c>
       <c r="C275" s="12" t="inlineStr">
         <is>
-          <t>2026-11-28 05:00</t>
+          <t>2026-09-05 16:45</t>
         </is>
       </c>
       <c r="D275" s="22" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="E275" s="12" t="inlineStr">
         <is>
-          <t>ATS</t>
+          <t>TOTAL</t>
         </is>
       </c>
       <c r="F275" s="12" t="inlineStr">
         <is>
-          <t>ASU +4.5</t>
+          <t>Over 53.5</t>
         </is>
       </c>
       <c r="G275" s="23" t="n">
-        <v>-4.5</v>
+        <v>53.5</v>
       </c>
       <c r="H275" s="13" t="n">
         <v>-110</v>
       </c>
       <c r="I275" s="15" t="n">
-        <v>0.5240821001886855</v>
+        <v>0.5238891282317109</v>
       </c>
       <c r="J275" s="15" t="n">
         <v>0.5</v>
@@ -19218,10 +19218,10 @@
         <v>0.5238095238095238</v>
       </c>
       <c r="L275" s="14" t="n">
-        <v>0.0002725763791616709</v>
+        <v>7.960442218701846e-05</v>
       </c>
       <c r="M275" s="14" t="n">
-        <v>0.0005203730874905332</v>
+        <v>0.0001519720787207524</v>
       </c>
       <c r="N275" s="15" t="n">
         <v>0</v>
@@ -19244,16 +19244,16 @@
       </c>
       <c r="B276" s="17" t="inlineStr">
         <is>
-          <t>KENT @ SC</t>
+          <t>ALA @ TENN</t>
         </is>
       </c>
       <c r="C276" s="17" t="inlineStr">
         <is>
-          <t>2026-09-05 16:45</t>
+          <t>2026-10-17 04:00</t>
         </is>
       </c>
       <c r="D276" s="25" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="E276" s="17" t="inlineStr">
         <is>
@@ -19262,17 +19262,17 @@
       </c>
       <c r="F276" s="17" t="inlineStr">
         <is>
-          <t>Over 53.5</t>
+          <t>Over 56.5</t>
         </is>
       </c>
       <c r="G276" s="26" t="n">
-        <v>53.5</v>
+        <v>56.5</v>
       </c>
       <c r="H276" s="18" t="n">
         <v>-110</v>
       </c>
       <c r="I276" s="20" t="n">
-        <v>0.5238891282317109</v>
+        <v>0.523889124443805</v>
       </c>
       <c r="J276" s="20" t="n">
         <v>0.5</v>
@@ -19281,16 +19281,16 @@
         <v>0.5238095238095238</v>
       </c>
       <c r="L276" s="19" t="n">
-        <v>7.960442218701846e-05</v>
+        <v>7.960063428114061e-05</v>
       </c>
       <c r="M276" s="19" t="n">
-        <v>0.0001519720787207524</v>
+        <v>0.0001519648472640966</v>
       </c>
       <c r="N276" s="20" t="n">
         <v>0</v>
       </c>
       <c r="O276" s="27" t="n">
-        <v>0.45</v>
+        <v>0</v>
       </c>
       <c r="P276" s="17" t="inlineStr">
         <is>
@@ -19307,16 +19307,16 @@
       </c>
       <c r="B277" s="12" t="inlineStr">
         <is>
-          <t>ALA @ TENN</t>
+          <t>ORE @ USC</t>
         </is>
       </c>
       <c r="C277" s="12" t="inlineStr">
         <is>
-          <t>2026-10-17 04:00</t>
+          <t>2026-09-26 04:00</t>
         </is>
       </c>
       <c r="D277" s="22" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="E277" s="12" t="inlineStr">
         <is>
@@ -19325,17 +19325,17 @@
       </c>
       <c r="F277" s="12" t="inlineStr">
         <is>
-          <t>Over 56.5</t>
+          <t>Under 58.5</t>
         </is>
       </c>
       <c r="G277" s="23" t="n">
-        <v>56.5</v>
+        <v>58.5</v>
       </c>
       <c r="H277" s="13" t="n">
         <v>-110</v>
       </c>
       <c r="I277" s="15" t="n">
-        <v>0.523889124443805</v>
+        <v>0.5238891228171049</v>
       </c>
       <c r="J277" s="15" t="n">
         <v>0.5</v>
@@ -19344,16 +19344,16 @@
         <v>0.5238095238095238</v>
       </c>
       <c r="L277" s="14" t="n">
-        <v>7.960063428114061e-05</v>
+        <v>7.959900758103267e-05</v>
       </c>
       <c r="M277" s="14" t="n">
-        <v>0.0001519648472640966</v>
+        <v>0.0001519617417456987</v>
       </c>
       <c r="N277" s="15" t="n">
         <v>0</v>
       </c>
       <c r="O277" s="24" t="n">
-        <v>0</v>
+        <v>0.45</v>
       </c>
       <c r="P277" s="12" t="inlineStr">
         <is>
@@ -19370,16 +19370,16 @@
       </c>
       <c r="B278" s="17" t="inlineStr">
         <is>
-          <t>ORE @ USC</t>
+          <t>TNST @ UGA</t>
         </is>
       </c>
       <c r="C278" s="17" t="inlineStr">
         <is>
-          <t>2026-09-26 04:00</t>
+          <t>2026-09-05 19:00</t>
         </is>
       </c>
       <c r="D278" s="25" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E278" s="17" t="inlineStr">
         <is>
@@ -19388,17 +19388,17 @@
       </c>
       <c r="F278" s="17" t="inlineStr">
         <is>
-          <t>Under 58.5</t>
+          <t>Under 56.5</t>
         </is>
       </c>
       <c r="G278" s="26" t="n">
-        <v>58.5</v>
+        <v>56.5</v>
       </c>
       <c r="H278" s="18" t="n">
         <v>-110</v>
       </c>
       <c r="I278" s="20" t="n">
-        <v>0.5238891228171049</v>
+        <v>0.5238891209664566</v>
       </c>
       <c r="J278" s="20" t="n">
         <v>0.5</v>
@@ -19407,10 +19407,10 @@
         <v>0.5238095238095238</v>
       </c>
       <c r="L278" s="19" t="n">
-        <v>7.959900758103267e-05</v>
+        <v>7.959715693273139e-05</v>
       </c>
       <c r="M278" s="19" t="n">
-        <v>0.0001519617417456987</v>
+        <v>0.0001519582086898508</v>
       </c>
       <c r="N278" s="20" t="n">
         <v>0</v>
@@ -19423,7 +19423,11 @@
           <t>DraftKings</t>
         </is>
       </c>
-      <c r="Q278" s="17" t="n"/>
+      <c r="Q278" s="17" t="inlineStr">
+        <is>
+          <t>TNST isn't a full FBS participant this season — model doesn't rate them reliably</t>
+        </is>
+      </c>
     </row>
     <row r="279">
       <c r="A279" s="12" t="inlineStr">
@@ -19433,16 +19437,16 @@
       </c>
       <c r="B279" s="12" t="inlineStr">
         <is>
-          <t>TNST @ UGA</t>
+          <t>SC @ CLEM</t>
         </is>
       </c>
       <c r="C279" s="12" t="inlineStr">
         <is>
-          <t>2026-09-05 19:00</t>
+          <t>2026-11-28 05:00</t>
         </is>
       </c>
       <c r="D279" s="22" t="n">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="E279" s="12" t="inlineStr">
         <is>
@@ -19451,17 +19455,17 @@
       </c>
       <c r="F279" s="12" t="inlineStr">
         <is>
-          <t>Under 56.5</t>
+          <t>Under 53.5</t>
         </is>
       </c>
       <c r="G279" s="23" t="n">
-        <v>56.5</v>
+        <v>53.5</v>
       </c>
       <c r="H279" s="13" t="n">
         <v>-110</v>
       </c>
       <c r="I279" s="15" t="n">
-        <v>0.5238891209664566</v>
+        <v>0.5238891092187401</v>
       </c>
       <c r="J279" s="15" t="n">
         <v>0.5</v>
@@ -19470,10 +19474,10 @@
         <v>0.5238095238095238</v>
       </c>
       <c r="L279" s="14" t="n">
-        <v>7.959715693273139e-05</v>
+        <v>7.958540921626511e-05</v>
       </c>
       <c r="M279" s="14" t="n">
-        <v>0.0001519582086898508</v>
+        <v>0.0001519357812311273</v>
       </c>
       <c r="N279" s="15" t="n">
         <v>0</v>
@@ -19486,11 +19490,7 @@
           <t>DraftKings</t>
         </is>
       </c>
-      <c r="Q279" s="12" t="inlineStr">
-        <is>
-          <t>TNST isn't a full FBS participant this season — model doesn't rate them reliably</t>
-        </is>
-      </c>
+      <c r="Q279" s="12" t="n"/>
     </row>
     <row r="280">
       <c r="A280" s="17" t="inlineStr">
@@ -19500,16 +19500,16 @@
       </c>
       <c r="B280" s="17" t="inlineStr">
         <is>
-          <t>SC @ CLEM</t>
+          <t>OU @ UGA</t>
         </is>
       </c>
       <c r="C280" s="17" t="inlineStr">
         <is>
-          <t>2026-11-28 05:00</t>
+          <t>2026-09-26 04:00</t>
         </is>
       </c>
       <c r="D280" s="25" t="n">
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="E280" s="17" t="inlineStr">
         <is>
@@ -19518,17 +19518,17 @@
       </c>
       <c r="F280" s="17" t="inlineStr">
         <is>
-          <t>Under 53.5</t>
+          <t>Under 52.5</t>
         </is>
       </c>
       <c r="G280" s="26" t="n">
-        <v>53.5</v>
+        <v>52.5</v>
       </c>
       <c r="H280" s="18" t="n">
         <v>-110</v>
       </c>
       <c r="I280" s="20" t="n">
-        <v>0.5238891092187401</v>
+        <v>0.5238890988524141</v>
       </c>
       <c r="J280" s="20" t="n">
         <v>0.5</v>
@@ -19537,10 +19537,10 @@
         <v>0.5238095238095238</v>
       </c>
       <c r="L280" s="19" t="n">
-        <v>7.958540921626511e-05</v>
+        <v>7.957504289024531e-05</v>
       </c>
       <c r="M280" s="19" t="n">
-        <v>0.0001519357812311273</v>
+        <v>0.0001519159909723622</v>
       </c>
       <c r="N280" s="20" t="n">
         <v>0</v>
@@ -19563,16 +19563,16 @@
       </c>
       <c r="B281" s="12" t="inlineStr">
         <is>
-          <t>OU @ UGA</t>
+          <t>UTU @ BYU</t>
         </is>
       </c>
       <c r="C281" s="12" t="inlineStr">
         <is>
-          <t>2026-09-26 04:00</t>
+          <t>2026-09-06 00:00</t>
         </is>
       </c>
       <c r="D281" s="22" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E281" s="12" t="inlineStr">
         <is>
@@ -19581,17 +19581,17 @@
       </c>
       <c r="F281" s="12" t="inlineStr">
         <is>
-          <t>Under 52.5</t>
+          <t>Over 54.5</t>
         </is>
       </c>
       <c r="G281" s="23" t="n">
-        <v>52.5</v>
+        <v>54.5</v>
       </c>
       <c r="H281" s="13" t="n">
         <v>-110</v>
       </c>
       <c r="I281" s="15" t="n">
-        <v>0.5238890988524141</v>
+        <v>0.5219067541972648</v>
       </c>
       <c r="J281" s="15" t="n">
         <v>0.5</v>
@@ -19600,23 +19600,27 @@
         <v>0.5238095238095238</v>
       </c>
       <c r="L281" s="14" t="n">
-        <v>7.957504289024531e-05</v>
+        <v>-0.001902769612258992</v>
       </c>
       <c r="M281" s="14" t="n">
-        <v>0.0001519159909723622</v>
+        <v>-0.00363256016885799</v>
       </c>
       <c r="N281" s="15" t="n">
         <v>0</v>
       </c>
       <c r="O281" s="24" t="n">
-        <v>0.45</v>
+        <v>0.4</v>
       </c>
       <c r="P281" s="12" t="inlineStr">
         <is>
           <t>DraftKings</t>
         </is>
       </c>
-      <c r="Q281" s="12" t="n"/>
+      <c r="Q281" s="12" t="inlineStr">
+        <is>
+          <t>UTU isn't a full FBS participant this season — model doesn't rate them reliably</t>
+        </is>
+      </c>
     </row>
     <row r="282">
       <c r="A282" s="17" t="inlineStr">
@@ -19626,16 +19630,16 @@
       </c>
       <c r="B282" s="17" t="inlineStr">
         <is>
-          <t>UTU @ BYU</t>
+          <t>TA&amp;M @ OU</t>
         </is>
       </c>
       <c r="C282" s="17" t="inlineStr">
         <is>
-          <t>2026-09-06 00:00</t>
+          <t>2026-11-21 05:00</t>
         </is>
       </c>
       <c r="D282" s="25" t="n">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="E282" s="17" t="inlineStr">
         <is>
@@ -19644,17 +19648,17 @@
       </c>
       <c r="F282" s="17" t="inlineStr">
         <is>
-          <t>Over 54.5</t>
+          <t>Over 51.5</t>
         </is>
       </c>
       <c r="G282" s="26" t="n">
-        <v>54.5</v>
+        <v>51.5</v>
       </c>
       <c r="H282" s="18" t="n">
         <v>-110</v>
       </c>
       <c r="I282" s="20" t="n">
-        <v>0.5219067541972648</v>
+        <v>0.5199222111459331</v>
       </c>
       <c r="J282" s="20" t="n">
         <v>0.5</v>
@@ -19663,27 +19667,23 @@
         <v>0.5238095238095238</v>
       </c>
       <c r="L282" s="19" t="n">
-        <v>-0.001902769612258992</v>
+        <v>-0.00388731266359077</v>
       </c>
       <c r="M282" s="19" t="n">
-        <v>-0.00363256016885799</v>
+        <v>-0.00742123326685501</v>
       </c>
       <c r="N282" s="20" t="n">
         <v>0</v>
       </c>
       <c r="O282" s="27" t="n">
-        <v>0.4</v>
+        <v>0.45</v>
       </c>
       <c r="P282" s="17" t="inlineStr">
         <is>
           <t>DraftKings</t>
         </is>
       </c>
-      <c r="Q282" s="17" t="inlineStr">
-        <is>
-          <t>UTU isn't a full FBS participant this season — model doesn't rate them reliably</t>
-        </is>
-      </c>
+      <c r="Q282" s="17" t="n"/>
     </row>
     <row r="283">
       <c r="A283" s="12" t="inlineStr">
@@ -19693,16 +19693,16 @@
       </c>
       <c r="B283" s="12" t="inlineStr">
         <is>
-          <t>TA&amp;M @ OU</t>
+          <t>NCSU @ UVA</t>
         </is>
       </c>
       <c r="C283" s="12" t="inlineStr">
         <is>
-          <t>2026-11-21 05:00</t>
+          <t>2026-08-29 19:30</t>
         </is>
       </c>
       <c r="D283" s="22" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="E283" s="12" t="inlineStr">
         <is>
@@ -19711,17 +19711,17 @@
       </c>
       <c r="F283" s="12" t="inlineStr">
         <is>
-          <t>Over 51.5</t>
+          <t>Over 53.5</t>
         </is>
       </c>
       <c r="G283" s="23" t="n">
-        <v>51.5</v>
+        <v>53.5</v>
       </c>
       <c r="H283" s="13" t="n">
         <v>-110</v>
       </c>
       <c r="I283" s="15" t="n">
-        <v>0.5199222111459331</v>
+        <v>0.5199222007643431</v>
       </c>
       <c r="J283" s="15" t="n">
         <v>0.5</v>
@@ -19730,10 +19730,10 @@
         <v>0.5238095238095238</v>
       </c>
       <c r="L283" s="14" t="n">
-        <v>-0.00388731266359077</v>
+        <v>-0.003887323045180691</v>
       </c>
       <c r="M283" s="14" t="n">
-        <v>-0.00742123326685501</v>
+        <v>-0.007421253086253965</v>
       </c>
       <c r="N283" s="15" t="n">
         <v>0</v>
@@ -19756,12 +19756,12 @@
       </c>
       <c r="B284" s="17" t="inlineStr">
         <is>
-          <t>NCSU @ UVA</t>
+          <t>UAB @ ILL</t>
         </is>
       </c>
       <c r="C284" s="17" t="inlineStr">
         <is>
-          <t>2026-08-29 19:30</t>
+          <t>2026-09-04 01:00</t>
         </is>
       </c>
       <c r="D284" s="25" t="n">
@@ -19774,17 +19774,17 @@
       </c>
       <c r="F284" s="17" t="inlineStr">
         <is>
-          <t>Over 53.5</t>
+          <t>Over 56.5</t>
         </is>
       </c>
       <c r="G284" s="26" t="n">
-        <v>53.5</v>
+        <v>56.5</v>
       </c>
       <c r="H284" s="18" t="n">
         <v>-110</v>
       </c>
       <c r="I284" s="20" t="n">
-        <v>0.5199222007643431</v>
+        <v>0.51992219658688</v>
       </c>
       <c r="J284" s="20" t="n">
         <v>0.5</v>
@@ -19793,10 +19793,10 @@
         <v>0.5238095238095238</v>
       </c>
       <c r="L284" s="19" t="n">
-        <v>-0.003887323045180691</v>
+        <v>-0.003887327222643844</v>
       </c>
       <c r="M284" s="19" t="n">
-        <v>-0.007421253086253965</v>
+        <v>-0.007421261061410889</v>
       </c>
       <c r="N284" s="20" t="n">
         <v>0</v>
@@ -19819,16 +19819,16 @@
       </c>
       <c r="B285" s="12" t="inlineStr">
         <is>
-          <t>UAB @ ILL</t>
+          <t>OSU @ USC</t>
         </is>
       </c>
       <c r="C285" s="12" t="inlineStr">
         <is>
-          <t>2026-09-04 01:00</t>
+          <t>2026-10-31 04:00</t>
         </is>
       </c>
       <c r="D285" s="22" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="E285" s="12" t="inlineStr">
         <is>
@@ -19837,17 +19837,17 @@
       </c>
       <c r="F285" s="12" t="inlineStr">
         <is>
-          <t>Over 56.5</t>
+          <t>Under 54.5</t>
         </is>
       </c>
       <c r="G285" s="23" t="n">
-        <v>56.5</v>
+        <v>54.5</v>
       </c>
       <c r="H285" s="13" t="n">
         <v>-110</v>
       </c>
       <c r="I285" s="15" t="n">
-        <v>0.51992219658688</v>
+        <v>0.5199221881338678</v>
       </c>
       <c r="J285" s="15" t="n">
         <v>0.5</v>
@@ -19856,10 +19856,10 @@
         <v>0.5238095238095238</v>
       </c>
       <c r="L285" s="14" t="n">
-        <v>-0.003887327222643844</v>
+        <v>-0.003887335675656023</v>
       </c>
       <c r="M285" s="14" t="n">
-        <v>-0.007421261061410889</v>
+        <v>-0.007421277198979614</v>
       </c>
       <c r="N285" s="15" t="n">
         <v>0</v>
@@ -19882,16 +19882,16 @@
       </c>
       <c r="B286" s="17" t="inlineStr">
         <is>
-          <t>OSU @ USC</t>
+          <t>MISS @ OU</t>
         </is>
       </c>
       <c r="C286" s="17" t="inlineStr">
         <is>
-          <t>2026-10-31 04:00</t>
+          <t>2026-11-14 05:00</t>
         </is>
       </c>
       <c r="D286" s="25" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E286" s="17" t="inlineStr">
         <is>
@@ -19900,17 +19900,17 @@
       </c>
       <c r="F286" s="17" t="inlineStr">
         <is>
-          <t>Under 54.5</t>
+          <t>Over 53.5</t>
         </is>
       </c>
       <c r="G286" s="26" t="n">
-        <v>54.5</v>
+        <v>53.5</v>
       </c>
       <c r="H286" s="18" t="n">
         <v>-110</v>
       </c>
       <c r="I286" s="20" t="n">
-        <v>0.5199221881338678</v>
+        <v>0.5179356580520053</v>
       </c>
       <c r="J286" s="20" t="n">
         <v>0.5</v>
@@ -19919,10 +19919,10 @@
         <v>0.5238095238095238</v>
       </c>
       <c r="L286" s="19" t="n">
-        <v>-0.003887335675656023</v>
+        <v>-0.005873865757518582</v>
       </c>
       <c r="M286" s="19" t="n">
-        <v>-0.007421277198979614</v>
+        <v>-0.01121374371889899</v>
       </c>
       <c r="N286" s="20" t="n">
         <v>0</v>
@@ -19945,16 +19945,16 @@
       </c>
       <c r="B287" s="12" t="inlineStr">
         <is>
-          <t>MISS @ OU</t>
+          <t>USC @ UCLA</t>
         </is>
       </c>
       <c r="C287" s="12" t="inlineStr">
         <is>
-          <t>2026-11-14 05:00</t>
+          <t>2026-11-28 05:00</t>
         </is>
       </c>
       <c r="D287" s="22" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="E287" s="12" t="inlineStr">
         <is>
@@ -19963,17 +19963,17 @@
       </c>
       <c r="F287" s="12" t="inlineStr">
         <is>
-          <t>Over 53.5</t>
+          <t>Over 55.5</t>
         </is>
       </c>
       <c r="G287" s="23" t="n">
-        <v>53.5</v>
+        <v>55.5</v>
       </c>
       <c r="H287" s="13" t="n">
         <v>-110</v>
       </c>
       <c r="I287" s="15" t="n">
-        <v>0.5179356580520053</v>
+        <v>0.5179356544150409</v>
       </c>
       <c r="J287" s="15" t="n">
         <v>0.5</v>
@@ -19982,10 +19982,10 @@
         <v>0.5238095238095238</v>
       </c>
       <c r="L287" s="14" t="n">
-        <v>-0.005873865757518582</v>
+        <v>-0.005873869394482978</v>
       </c>
       <c r="M287" s="14" t="n">
-        <v>-0.01121374371889899</v>
+        <v>-0.01121375066219471</v>
       </c>
       <c r="N287" s="15" t="n">
         <v>0</v>
@@ -20008,35 +20008,35 @@
       </c>
       <c r="B288" s="17" t="inlineStr">
         <is>
-          <t>USC @ UCLA</t>
+          <t>USC @ PSU</t>
         </is>
       </c>
       <c r="C288" s="17" t="inlineStr">
         <is>
-          <t>2026-11-28 05:00</t>
+          <t>2026-10-10 04:00</t>
         </is>
       </c>
       <c r="D288" s="25" t="n">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="E288" s="17" t="inlineStr">
         <is>
-          <t>TOTAL</t>
+          <t>ATS</t>
         </is>
       </c>
       <c r="F288" s="17" t="inlineStr">
         <is>
-          <t>Over 55.5</t>
+          <t>PSU -1.5</t>
         </is>
       </c>
       <c r="G288" s="26" t="n">
-        <v>55.5</v>
+        <v>-1.5</v>
       </c>
       <c r="H288" s="18" t="n">
         <v>-110</v>
       </c>
       <c r="I288" s="20" t="n">
-        <v>0.5179356544150409</v>
+        <v>0.517195813494671</v>
       </c>
       <c r="J288" s="20" t="n">
         <v>0.5</v>
@@ -20045,10 +20045,10 @@
         <v>0.5238095238095238</v>
       </c>
       <c r="L288" s="19" t="n">
-        <v>-0.005873869394482978</v>
+        <v>-0.006613710314852805</v>
       </c>
       <c r="M288" s="19" t="n">
-        <v>-0.01121375066219471</v>
+        <v>-0.01262617423744616</v>
       </c>
       <c r="N288" s="20" t="n">
         <v>0</v>
@@ -20071,16 +20071,16 @@
       </c>
       <c r="B289" s="12" t="inlineStr">
         <is>
-          <t>USC @ PSU</t>
+          <t>UNC @ DUKE</t>
         </is>
       </c>
       <c r="C289" s="12" t="inlineStr">
         <is>
-          <t>2026-10-10 04:00</t>
+          <t>2026-10-17 04:00</t>
         </is>
       </c>
       <c r="D289" s="22" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E289" s="12" t="inlineStr">
         <is>
@@ -20089,17 +20089,17 @@
       </c>
       <c r="F289" s="12" t="inlineStr">
         <is>
-          <t>PSU -1.5</t>
+          <t>UNC +4.5</t>
         </is>
       </c>
       <c r="G289" s="23" t="n">
-        <v>-1.5</v>
+        <v>-4.5</v>
       </c>
       <c r="H289" s="13" t="n">
         <v>-110</v>
       </c>
       <c r="I289" s="15" t="n">
-        <v>0.517195813494671</v>
+        <v>0.516626035872215</v>
       </c>
       <c r="J289" s="15" t="n">
         <v>0.5</v>
@@ -20108,10 +20108,10 @@
         <v>0.5238095238095238</v>
       </c>
       <c r="L289" s="14" t="n">
-        <v>-0.006613710314852805</v>
+        <v>-0.00718348793730883</v>
       </c>
       <c r="M289" s="14" t="n">
-        <v>-0.01262617423744616</v>
+        <v>-0.01371393151668038</v>
       </c>
       <c r="N289" s="15" t="n">
         <v>0</v>
@@ -20134,35 +20134,35 @@
       </c>
       <c r="B290" s="17" t="inlineStr">
         <is>
-          <t>UNC @ DUKE</t>
+          <t>LSU @ TENN</t>
         </is>
       </c>
       <c r="C290" s="17" t="inlineStr">
         <is>
-          <t>2026-10-17 04:00</t>
+          <t>2026-11-21 05:00</t>
         </is>
       </c>
       <c r="D290" s="25" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="E290" s="17" t="inlineStr">
         <is>
-          <t>ATS</t>
+          <t>TOTAL</t>
         </is>
       </c>
       <c r="F290" s="17" t="inlineStr">
         <is>
-          <t>UNC +4.5</t>
+          <t>Under 57.5</t>
         </is>
       </c>
       <c r="G290" s="26" t="n">
-        <v>-4.5</v>
+        <v>57.5</v>
       </c>
       <c r="H290" s="18" t="n">
         <v>-110</v>
       </c>
       <c r="I290" s="20" t="n">
-        <v>0.516626035872215</v>
+        <v>0.5159473183674262</v>
       </c>
       <c r="J290" s="20" t="n">
         <v>0.5</v>
@@ -20171,10 +20171,10 @@
         <v>0.5238095238095238</v>
       </c>
       <c r="L290" s="19" t="n">
-        <v>-0.00718348793730883</v>
+        <v>-0.007862205442097592</v>
       </c>
       <c r="M290" s="19" t="n">
-        <v>-0.01371393151668038</v>
+        <v>-0.01500966493491351</v>
       </c>
       <c r="N290" s="20" t="n">
         <v>0</v>
@@ -20197,16 +20197,16 @@
       </c>
       <c r="B291" s="12" t="inlineStr">
         <is>
-          <t>LSU @ TENN</t>
+          <t>NAU @ ARIZ</t>
         </is>
       </c>
       <c r="C291" s="12" t="inlineStr">
         <is>
-          <t>2026-11-21 05:00</t>
+          <t>2026-09-06 01:30</t>
         </is>
       </c>
       <c r="D291" s="22" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="E291" s="12" t="inlineStr">
         <is>
@@ -20215,17 +20215,17 @@
       </c>
       <c r="F291" s="12" t="inlineStr">
         <is>
-          <t>Under 57.5</t>
+          <t>Under 56.5</t>
         </is>
       </c>
       <c r="G291" s="23" t="n">
-        <v>57.5</v>
+        <v>56.5</v>
       </c>
       <c r="H291" s="13" t="n">
         <v>-110</v>
       </c>
       <c r="I291" s="15" t="n">
-        <v>0.5159473183674262</v>
+        <v>0.5159473173920124</v>
       </c>
       <c r="J291" s="15" t="n">
         <v>0.5</v>
@@ -20234,10 +20234,10 @@
         <v>0.5238095238095238</v>
       </c>
       <c r="L291" s="14" t="n">
-        <v>-0.007862205442097592</v>
+        <v>-0.007862206417511453</v>
       </c>
       <c r="M291" s="14" t="n">
-        <v>-0.01500966493491351</v>
+        <v>-0.01500966679706722</v>
       </c>
       <c r="N291" s="15" t="n">
         <v>0</v>
@@ -20250,7 +20250,11 @@
           <t>DraftKings</t>
         </is>
       </c>
-      <c r="Q291" s="12" t="n"/>
+      <c r="Q291" s="12" t="inlineStr">
+        <is>
+          <t>NAU isn't a full FBS participant this season — model doesn't rate them reliably</t>
+        </is>
+      </c>
     </row>
     <row r="292">
       <c r="A292" s="17" t="inlineStr">
@@ -20260,16 +20264,16 @@
       </c>
       <c r="B292" s="17" t="inlineStr">
         <is>
-          <t>NAU @ ARIZ</t>
+          <t>TCU @ TTU</t>
         </is>
       </c>
       <c r="C292" s="17" t="inlineStr">
         <is>
-          <t>2026-09-06 01:30</t>
+          <t>2026-11-27 01:00</t>
         </is>
       </c>
       <c r="D292" s="25" t="n">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="E292" s="17" t="inlineStr">
         <is>
@@ -20278,17 +20282,17 @@
       </c>
       <c r="F292" s="17" t="inlineStr">
         <is>
-          <t>Under 56.5</t>
+          <t>Under 55.5</t>
         </is>
       </c>
       <c r="G292" s="26" t="n">
-        <v>56.5</v>
+        <v>55.5</v>
       </c>
       <c r="H292" s="18" t="n">
         <v>-110</v>
       </c>
       <c r="I292" s="20" t="n">
-        <v>0.5159473173920124</v>
+        <v>0.5159473156809926</v>
       </c>
       <c r="J292" s="20" t="n">
         <v>0.5</v>
@@ -20297,10 +20301,10 @@
         <v>0.5238095238095238</v>
       </c>
       <c r="L292" s="19" t="n">
-        <v>-0.007862206417511453</v>
+        <v>-0.007862208128531223</v>
       </c>
       <c r="M292" s="19" t="n">
-        <v>-0.01500966679706722</v>
+        <v>-0.01500967006355952</v>
       </c>
       <c r="N292" s="20" t="n">
         <v>0</v>
@@ -20313,11 +20317,7 @@
           <t>DraftKings</t>
         </is>
       </c>
-      <c r="Q292" s="17" t="inlineStr">
-        <is>
-          <t>NAU isn't a full FBS participant this season — model doesn't rate them reliably</t>
-        </is>
-      </c>
+      <c r="Q292" s="17" t="n"/>
     </row>
     <row r="293">
       <c r="A293" s="12" t="inlineStr">
@@ -20327,16 +20327,16 @@
       </c>
       <c r="B293" s="12" t="inlineStr">
         <is>
-          <t>TCU @ TTU</t>
+          <t>FSU @ MIA</t>
         </is>
       </c>
       <c r="C293" s="12" t="inlineStr">
         <is>
-          <t>2026-11-27 01:00</t>
+          <t>2026-10-17 04:00</t>
         </is>
       </c>
       <c r="D293" s="22" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="E293" s="12" t="inlineStr">
         <is>
@@ -20345,17 +20345,17 @@
       </c>
       <c r="F293" s="12" t="inlineStr">
         <is>
-          <t>Under 55.5</t>
+          <t>Under 53.5</t>
         </is>
       </c>
       <c r="G293" s="23" t="n">
-        <v>55.5</v>
+        <v>53.5</v>
       </c>
       <c r="H293" s="13" t="n">
         <v>-110</v>
       </c>
       <c r="I293" s="15" t="n">
-        <v>0.5159473156809926</v>
+        <v>0.51594730760003</v>
       </c>
       <c r="J293" s="15" t="n">
         <v>0.5</v>
@@ -20364,10 +20364,10 @@
         <v>0.5238095238095238</v>
       </c>
       <c r="L293" s="14" t="n">
-        <v>-0.007862208128531223</v>
+        <v>-0.007862216209493789</v>
       </c>
       <c r="M293" s="14" t="n">
-        <v>-0.01500967006355952</v>
+        <v>-0.01500968549085169</v>
       </c>
       <c r="N293" s="15" t="n">
         <v>0</v>
@@ -20390,16 +20390,16 @@
       </c>
       <c r="B294" s="17" t="inlineStr">
         <is>
-          <t>FSU @ MIA</t>
+          <t>FLA @ AUB</t>
         </is>
       </c>
       <c r="C294" s="17" t="inlineStr">
         <is>
-          <t>2026-10-17 04:00</t>
+          <t>2026-09-19 23:00</t>
         </is>
       </c>
       <c r="D294" s="25" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="E294" s="17" t="inlineStr">
         <is>
@@ -20418,7 +20418,7 @@
         <v>-110</v>
       </c>
       <c r="I294" s="20" t="n">
-        <v>0.51594730760003</v>
+        <v>0.5139573823881913</v>
       </c>
       <c r="J294" s="20" t="n">
         <v>0.5</v>
@@ -20427,10 +20427,10 @@
         <v>0.5238095238095238</v>
       </c>
       <c r="L294" s="19" t="n">
-        <v>-0.007862216209493789</v>
+        <v>-0.009852141421332505</v>
       </c>
       <c r="M294" s="19" t="n">
-        <v>-0.01500968549085169</v>
+        <v>-0.01880863362254376</v>
       </c>
       <c r="N294" s="20" t="n">
         <v>0</v>
@@ -20453,35 +20453,35 @@
       </c>
       <c r="B295" s="12" t="inlineStr">
         <is>
-          <t>FLA @ AUB</t>
+          <t>OSU @ TEX</t>
         </is>
       </c>
       <c r="C295" s="12" t="inlineStr">
         <is>
-          <t>2026-09-19 23:00</t>
+          <t>2026-09-12 23:30</t>
         </is>
       </c>
       <c r="D295" s="22" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E295" s="12" t="inlineStr">
         <is>
-          <t>TOTAL</t>
+          <t>ATS</t>
         </is>
       </c>
       <c r="F295" s="12" t="inlineStr">
         <is>
-          <t>Under 53.5</t>
+          <t>OSU +1.5</t>
         </is>
       </c>
       <c r="G295" s="23" t="n">
-        <v>53.5</v>
+        <v>-1.5</v>
       </c>
       <c r="H295" s="13" t="n">
         <v>-110</v>
       </c>
       <c r="I295" s="15" t="n">
-        <v>0.5139573823881913</v>
+        <v>0.5135482219987958</v>
       </c>
       <c r="J295" s="15" t="n">
         <v>0.5</v>
@@ -20490,10 +20490,10 @@
         <v>0.5238095238095238</v>
       </c>
       <c r="L295" s="14" t="n">
-        <v>-0.009852141421332505</v>
+        <v>-0.01026130181072804</v>
       </c>
       <c r="M295" s="14" t="n">
-        <v>-0.01880863362254376</v>
+        <v>-0.0195897580022989</v>
       </c>
       <c r="N295" s="15" t="n">
         <v>0</v>
@@ -20516,12 +20516,12 @@
       </c>
       <c r="B296" s="17" t="inlineStr">
         <is>
-          <t>OSU @ TEX</t>
+          <t>OU @ MICH</t>
         </is>
       </c>
       <c r="C296" s="17" t="inlineStr">
         <is>
-          <t>2026-09-12 23:30</t>
+          <t>2026-09-12 16:00</t>
         </is>
       </c>
       <c r="D296" s="25" t="n">
@@ -20534,7 +20534,7 @@
       </c>
       <c r="F296" s="17" t="inlineStr">
         <is>
-          <t>OSU +1.5</t>
+          <t>MICH -1.5</t>
         </is>
       </c>
       <c r="G296" s="26" t="n">
@@ -20544,7 +20544,7 @@
         <v>-110</v>
       </c>
       <c r="I296" s="20" t="n">
-        <v>0.5135482219987958</v>
+        <v>0.5120296819535175</v>
       </c>
       <c r="J296" s="20" t="n">
         <v>0.5</v>
@@ -20553,10 +20553,10 @@
         <v>0.5238095238095238</v>
       </c>
       <c r="L296" s="19" t="n">
-        <v>-0.01026130181072804</v>
+        <v>-0.01177984185600633</v>
       </c>
       <c r="M296" s="19" t="n">
-        <v>-0.0195897580022989</v>
+        <v>-0.02248878899783019</v>
       </c>
       <c r="N296" s="20" t="n">
         <v>0</v>
@@ -20579,35 +20579,35 @@
       </c>
       <c r="B297" s="12" t="inlineStr">
         <is>
-          <t>OU @ MICH</t>
+          <t>WIS @ ND</t>
         </is>
       </c>
       <c r="C297" s="12" t="inlineStr">
         <is>
-          <t>2026-09-12 16:00</t>
+          <t>2026-09-06 23:30</t>
         </is>
       </c>
       <c r="D297" s="22" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E297" s="12" t="inlineStr">
         <is>
-          <t>ATS</t>
+          <t>TOTAL</t>
         </is>
       </c>
       <c r="F297" s="12" t="inlineStr">
         <is>
-          <t>MICH -1.5</t>
+          <t>Over 47.5</t>
         </is>
       </c>
       <c r="G297" s="23" t="n">
-        <v>-1.5</v>
+        <v>47.5</v>
       </c>
       <c r="H297" s="13" t="n">
         <v>-110</v>
       </c>
       <c r="I297" s="15" t="n">
-        <v>0.5120296819535175</v>
+        <v>0.5119662256857437</v>
       </c>
       <c r="J297" s="15" t="n">
         <v>0.5</v>
@@ -20616,10 +20616,10 @@
         <v>0.5238095238095238</v>
       </c>
       <c r="L297" s="14" t="n">
-        <v>-0.01177984185600633</v>
+        <v>-0.01184329812378015</v>
       </c>
       <c r="M297" s="14" t="n">
-        <v>-0.02248878899783019</v>
+        <v>-0.02260993278176204</v>
       </c>
       <c r="N297" s="15" t="n">
         <v>0</v>
@@ -20642,16 +20642,16 @@
       </c>
       <c r="B298" s="17" t="inlineStr">
         <is>
-          <t>WIS @ ND</t>
+          <t>ORE @ OSU</t>
         </is>
       </c>
       <c r="C298" s="17" t="inlineStr">
         <is>
-          <t>2026-09-06 23:30</t>
+          <t>2026-11-07 05:00</t>
         </is>
       </c>
       <c r="D298" s="25" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="E298" s="17" t="inlineStr">
         <is>
@@ -20660,17 +20660,17 @@
       </c>
       <c r="F298" s="17" t="inlineStr">
         <is>
-          <t>Over 47.5</t>
+          <t>Over 52.5</t>
         </is>
       </c>
       <c r="G298" s="26" t="n">
-        <v>47.5</v>
+        <v>52.5</v>
       </c>
       <c r="H298" s="18" t="n">
         <v>-110</v>
       </c>
       <c r="I298" s="20" t="n">
-        <v>0.5119662256857437</v>
+        <v>0.5119660842604348</v>
       </c>
       <c r="J298" s="20" t="n">
         <v>0.5</v>
@@ -20679,10 +20679,10 @@
         <v>0.5238095238095238</v>
       </c>
       <c r="L298" s="19" t="n">
-        <v>-0.01184329812378015</v>
+        <v>-0.01184343954908906</v>
       </c>
       <c r="M298" s="19" t="n">
-        <v>-0.02260993278176204</v>
+        <v>-0.02261020277553355</v>
       </c>
       <c r="N298" s="20" t="n">
         <v>0</v>
@@ -20705,16 +20705,16 @@
       </c>
       <c r="B299" s="12" t="inlineStr">
         <is>
-          <t>ORE @ OSU</t>
+          <t>TA&amp;M @ ALA</t>
         </is>
       </c>
       <c r="C299" s="12" t="inlineStr">
         <is>
-          <t>2026-11-07 05:00</t>
+          <t>2026-10-24 04:00</t>
         </is>
       </c>
       <c r="D299" s="22" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E299" s="12" t="inlineStr">
         <is>
@@ -20723,17 +20723,17 @@
       </c>
       <c r="F299" s="12" t="inlineStr">
         <is>
-          <t>Over 52.5</t>
+          <t>Under 54.5</t>
         </is>
       </c>
       <c r="G299" s="23" t="n">
-        <v>52.5</v>
+        <v>54.5</v>
       </c>
       <c r="H299" s="13" t="n">
         <v>-110</v>
       </c>
       <c r="I299" s="15" t="n">
-        <v>0.5119660842604348</v>
+        <v>0.511966067232297</v>
       </c>
       <c r="J299" s="15" t="n">
         <v>0.5</v>
@@ -20742,10 +20742,10 @@
         <v>0.5238095238095238</v>
       </c>
       <c r="L299" s="14" t="n">
-        <v>-0.01184343954908906</v>
+        <v>-0.01184345657722685</v>
       </c>
       <c r="M299" s="14" t="n">
-        <v>-0.02261020277553355</v>
+        <v>-0.02261023528379663</v>
       </c>
       <c r="N299" s="15" t="n">
         <v>0</v>
@@ -20768,16 +20768,16 @@
       </c>
       <c r="B300" s="17" t="inlineStr">
         <is>
-          <t>TA&amp;M @ ALA</t>
+          <t>AUB @ ALA</t>
         </is>
       </c>
       <c r="C300" s="17" t="inlineStr">
         <is>
-          <t>2026-10-24 04:00</t>
+          <t>2026-11-28 05:00</t>
         </is>
       </c>
       <c r="D300" s="25" t="n">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="E300" s="17" t="inlineStr">
         <is>
@@ -20786,17 +20786,17 @@
       </c>
       <c r="F300" s="17" t="inlineStr">
         <is>
-          <t>Under 54.5</t>
+          <t>Under 53.5</t>
         </is>
       </c>
       <c r="G300" s="26" t="n">
-        <v>54.5</v>
+        <v>53.5</v>
       </c>
       <c r="H300" s="18" t="n">
         <v>-110</v>
       </c>
       <c r="I300" s="20" t="n">
-        <v>0.511966067232297</v>
+        <v>0.51196606256607</v>
       </c>
       <c r="J300" s="20" t="n">
         <v>0.5</v>
@@ -20805,10 +20805,10 @@
         <v>0.5238095238095238</v>
       </c>
       <c r="L300" s="19" t="n">
-        <v>-0.01184345657722685</v>
+        <v>-0.01184346124345381</v>
       </c>
       <c r="M300" s="19" t="n">
-        <v>-0.02261023528379663</v>
+        <v>-0.0226102441920481</v>
       </c>
       <c r="N300" s="20" t="n">
         <v>0</v>
@@ -20831,16 +20831,16 @@
       </c>
       <c r="B301" s="12" t="inlineStr">
         <is>
-          <t>AUB @ ALA</t>
+          <t>UGA @ MISS</t>
         </is>
       </c>
       <c r="C301" s="12" t="inlineStr">
         <is>
-          <t>2026-11-28 05:00</t>
+          <t>2026-11-07 05:00</t>
         </is>
       </c>
       <c r="D301" s="22" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="E301" s="12" t="inlineStr">
         <is>
@@ -20849,17 +20849,17 @@
       </c>
       <c r="F301" s="12" t="inlineStr">
         <is>
-          <t>Under 53.5</t>
+          <t>Over 55.5</t>
         </is>
       </c>
       <c r="G301" s="23" t="n">
-        <v>53.5</v>
+        <v>55.5</v>
       </c>
       <c r="H301" s="13" t="n">
         <v>-110</v>
       </c>
       <c r="I301" s="15" t="n">
-        <v>0.51196606256607</v>
+        <v>0.5099735590672994</v>
       </c>
       <c r="J301" s="15" t="n">
         <v>0.5</v>
@@ -20868,10 +20868,10 @@
         <v>0.5238095238095238</v>
       </c>
       <c r="L301" s="14" t="n">
-        <v>-0.01184346124345381</v>
+        <v>-0.01383596474222448</v>
       </c>
       <c r="M301" s="14" t="n">
-        <v>-0.0226102441920481</v>
+        <v>-0.026414114507883</v>
       </c>
       <c r="N301" s="15" t="n">
         <v>0</v>
@@ -20894,16 +20894,16 @@
       </c>
       <c r="B302" s="17" t="inlineStr">
         <is>
-          <t>UGA @ MISS</t>
+          <t>DUKE @ MIA</t>
         </is>
       </c>
       <c r="C302" s="17" t="inlineStr">
         <is>
-          <t>2026-11-07 05:00</t>
+          <t>2026-11-14 05:00</t>
         </is>
       </c>
       <c r="D302" s="25" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E302" s="17" t="inlineStr">
         <is>
@@ -20957,16 +20957,16 @@
       </c>
       <c r="B303" s="12" t="inlineStr">
         <is>
-          <t>DUKE @ MIA</t>
+          <t>MEM @ UNLV</t>
         </is>
       </c>
       <c r="C303" s="12" t="inlineStr">
         <is>
-          <t>2026-11-14 05:00</t>
+          <t>2026-08-30 02:00</t>
         </is>
       </c>
       <c r="D303" s="22" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="E303" s="12" t="inlineStr">
         <is>
@@ -20975,17 +20975,17 @@
       </c>
       <c r="F303" s="12" t="inlineStr">
         <is>
-          <t>Over 55.5</t>
+          <t>Over 57.5</t>
         </is>
       </c>
       <c r="G303" s="23" t="n">
-        <v>55.5</v>
+        <v>57.5</v>
       </c>
       <c r="H303" s="13" t="n">
         <v>-110</v>
       </c>
       <c r="I303" s="15" t="n">
-        <v>0.5099735590672994</v>
+        <v>0.5099735576396345</v>
       </c>
       <c r="J303" s="15" t="n">
         <v>0.5</v>
@@ -20994,10 +20994,10 @@
         <v>0.5238095238095238</v>
       </c>
       <c r="L303" s="14" t="n">
-        <v>-0.01383596474222448</v>
+        <v>-0.01383596616988936</v>
       </c>
       <c r="M303" s="14" t="n">
-        <v>-0.026414114507883</v>
+        <v>-0.02641411723342507</v>
       </c>
       <c r="N303" s="15" t="n">
         <v>0</v>
@@ -24360,16 +24360,16 @@
       </c>
       <c r="B356" s="17" t="inlineStr">
         <is>
-          <t>UGA @ MISS</t>
+          <t>MEM @ UNLV</t>
         </is>
       </c>
       <c r="C356" s="17" t="inlineStr">
         <is>
-          <t>2026-11-07 05:00</t>
+          <t>2026-08-30 02:00</t>
         </is>
       </c>
       <c r="D356" s="25" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="E356" s="17" t="inlineStr">
         <is>
@@ -24378,17 +24378,17 @@
       </c>
       <c r="F356" s="17" t="inlineStr">
         <is>
-          <t>Under 55.5</t>
+          <t>Under 57.5</t>
         </is>
       </c>
       <c r="G356" s="26" t="n">
-        <v>55.5</v>
+        <v>57.5</v>
       </c>
       <c r="H356" s="18" t="n">
         <v>-110</v>
       </c>
       <c r="I356" s="20" t="n">
-        <v>0.4900264409327006</v>
+        <v>0.4900264423603655</v>
       </c>
       <c r="J356" s="20" t="n">
         <v>0.5</v>
@@ -24397,10 +24397,10 @@
         <v>0.5238095238095238</v>
       </c>
       <c r="L356" s="19" t="n">
-        <v>-0.03378308287682319</v>
+        <v>-0.03378308144915831</v>
       </c>
       <c r="M356" s="19" t="n">
-        <v>-0.06449497640120783</v>
+        <v>-0.06449497367566576</v>
       </c>
       <c r="N356" s="20" t="n">
         <v>0</v>
@@ -24423,16 +24423,16 @@
       </c>
       <c r="B357" s="12" t="inlineStr">
         <is>
-          <t>DUKE @ MIA</t>
+          <t>UGA @ MISS</t>
         </is>
       </c>
       <c r="C357" s="12" t="inlineStr">
         <is>
-          <t>2026-11-14 05:00</t>
+          <t>2026-11-07 05:00</t>
         </is>
       </c>
       <c r="D357" s="22" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E357" s="12" t="inlineStr">
         <is>
@@ -24486,16 +24486,16 @@
       </c>
       <c r="B358" s="17" t="inlineStr">
         <is>
-          <t>AUB @ ALA</t>
+          <t>DUKE @ MIA</t>
         </is>
       </c>
       <c r="C358" s="17" t="inlineStr">
         <is>
-          <t>2026-11-28 05:00</t>
+          <t>2026-11-14 05:00</t>
         </is>
       </c>
       <c r="D358" s="25" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="E358" s="17" t="inlineStr">
         <is>
@@ -24504,17 +24504,17 @@
       </c>
       <c r="F358" s="17" t="inlineStr">
         <is>
-          <t>Over 53.5</t>
+          <t>Under 55.5</t>
         </is>
       </c>
       <c r="G358" s="26" t="n">
-        <v>53.5</v>
+        <v>55.5</v>
       </c>
       <c r="H358" s="18" t="n">
         <v>-110</v>
       </c>
       <c r="I358" s="20" t="n">
-        <v>0.48803393743393</v>
+        <v>0.4900264409327006</v>
       </c>
       <c r="J358" s="20" t="n">
         <v>0.5</v>
@@ -24523,10 +24523,10 @@
         <v>0.5238095238095238</v>
       </c>
       <c r="L358" s="19" t="n">
-        <v>-0.03577558637559386</v>
+        <v>-0.03378308287682319</v>
       </c>
       <c r="M358" s="19" t="n">
-        <v>-0.06829884671704273</v>
+        <v>-0.06449497640120783</v>
       </c>
       <c r="N358" s="20" t="n">
         <v>0</v>
@@ -24549,16 +24549,16 @@
       </c>
       <c r="B359" s="12" t="inlineStr">
         <is>
-          <t>TA&amp;M @ ALA</t>
+          <t>AUB @ ALA</t>
         </is>
       </c>
       <c r="C359" s="12" t="inlineStr">
         <is>
-          <t>2026-10-24 04:00</t>
+          <t>2026-11-28 05:00</t>
         </is>
       </c>
       <c r="D359" s="22" t="n">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="E359" s="12" t="inlineStr">
         <is>
@@ -24567,17 +24567,17 @@
       </c>
       <c r="F359" s="12" t="inlineStr">
         <is>
-          <t>Over 54.5</t>
+          <t>Over 53.5</t>
         </is>
       </c>
       <c r="G359" s="23" t="n">
-        <v>54.5</v>
+        <v>53.5</v>
       </c>
       <c r="H359" s="13" t="n">
         <v>-110</v>
       </c>
       <c r="I359" s="15" t="n">
-        <v>0.488033932767703</v>
+        <v>0.48803393743393</v>
       </c>
       <c r="J359" s="15" t="n">
         <v>0.5</v>
@@ -24586,10 +24586,10 @@
         <v>0.5238095238095238</v>
       </c>
       <c r="L359" s="14" t="n">
-        <v>-0.03577559104182082</v>
+        <v>-0.03577558637559386</v>
       </c>
       <c r="M359" s="14" t="n">
-        <v>-0.0682988556252942</v>
+        <v>-0.06829884671704273</v>
       </c>
       <c r="N359" s="15" t="n">
         <v>0</v>
@@ -24612,16 +24612,16 @@
       </c>
       <c r="B360" s="17" t="inlineStr">
         <is>
-          <t>ORE @ OSU</t>
+          <t>TA&amp;M @ ALA</t>
         </is>
       </c>
       <c r="C360" s="17" t="inlineStr">
         <is>
-          <t>2026-11-07 05:00</t>
+          <t>2026-10-24 04:00</t>
         </is>
       </c>
       <c r="D360" s="25" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E360" s="17" t="inlineStr">
         <is>
@@ -24630,17 +24630,17 @@
       </c>
       <c r="F360" s="17" t="inlineStr">
         <is>
-          <t>Under 52.5</t>
+          <t>Over 54.5</t>
         </is>
       </c>
       <c r="G360" s="26" t="n">
-        <v>52.5</v>
+        <v>54.5</v>
       </c>
       <c r="H360" s="18" t="n">
         <v>-110</v>
       </c>
       <c r="I360" s="20" t="n">
-        <v>0.4880339157395652</v>
+        <v>0.488033932767703</v>
       </c>
       <c r="J360" s="20" t="n">
         <v>0.5</v>
@@ -24649,10 +24649,10 @@
         <v>0.5238095238095238</v>
       </c>
       <c r="L360" s="19" t="n">
-        <v>-0.03577560806995861</v>
+        <v>-0.03577559104182082</v>
       </c>
       <c r="M360" s="19" t="n">
-        <v>-0.06829888813355728</v>
+        <v>-0.0682988556252942</v>
       </c>
       <c r="N360" s="20" t="n">
         <v>0</v>
@@ -24675,16 +24675,16 @@
       </c>
       <c r="B361" s="12" t="inlineStr">
         <is>
-          <t>WIS @ ND</t>
+          <t>ORE @ OSU</t>
         </is>
       </c>
       <c r="C361" s="12" t="inlineStr">
         <is>
-          <t>2026-09-06 23:30</t>
+          <t>2026-11-07 05:00</t>
         </is>
       </c>
       <c r="D361" s="22" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="E361" s="12" t="inlineStr">
         <is>
@@ -24693,17 +24693,17 @@
       </c>
       <c r="F361" s="12" t="inlineStr">
         <is>
-          <t>Under 47.5</t>
+          <t>Under 52.5</t>
         </is>
       </c>
       <c r="G361" s="23" t="n">
-        <v>47.5</v>
+        <v>52.5</v>
       </c>
       <c r="H361" s="13" t="n">
         <v>-110</v>
       </c>
       <c r="I361" s="15" t="n">
-        <v>0.4880337743142563</v>
+        <v>0.4880339157395652</v>
       </c>
       <c r="J361" s="15" t="n">
         <v>0.5</v>
@@ -24712,10 +24712,10 @@
         <v>0.5238095238095238</v>
       </c>
       <c r="L361" s="14" t="n">
-        <v>-0.03577574949526752</v>
+        <v>-0.03577560806995861</v>
       </c>
       <c r="M361" s="14" t="n">
-        <v>-0.06829915812732879</v>
+        <v>-0.06829888813355728</v>
       </c>
       <c r="N361" s="15" t="n">
         <v>0</v>
@@ -24738,35 +24738,35 @@
       </c>
       <c r="B362" s="17" t="inlineStr">
         <is>
-          <t>OU @ MICH</t>
+          <t>WIS @ ND</t>
         </is>
       </c>
       <c r="C362" s="17" t="inlineStr">
         <is>
-          <t>2026-09-12 16:00</t>
+          <t>2026-09-06 23:30</t>
         </is>
       </c>
       <c r="D362" s="25" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E362" s="17" t="inlineStr">
         <is>
-          <t>ATS</t>
+          <t>TOTAL</t>
         </is>
       </c>
       <c r="F362" s="17" t="inlineStr">
         <is>
-          <t>OU +1.5</t>
+          <t>Under 47.5</t>
         </is>
       </c>
       <c r="G362" s="26" t="n">
-        <v>-1.5</v>
+        <v>47.5</v>
       </c>
       <c r="H362" s="18" t="n">
         <v>-110</v>
       </c>
       <c r="I362" s="20" t="n">
-        <v>0.4879703180464825</v>
+        <v>0.4880337743142563</v>
       </c>
       <c r="J362" s="20" t="n">
         <v>0.5</v>
@@ -24775,10 +24775,10 @@
         <v>0.5238095238095238</v>
       </c>
       <c r="L362" s="19" t="n">
-        <v>-0.03583920576304134</v>
+        <v>-0.03577574949526752</v>
       </c>
       <c r="M362" s="19" t="n">
-        <v>-0.06842030191126064</v>
+        <v>-0.06829915812732879</v>
       </c>
       <c r="N362" s="20" t="n">
         <v>0</v>
@@ -24801,12 +24801,12 @@
       </c>
       <c r="B363" s="12" t="inlineStr">
         <is>
-          <t>OSU @ TEX</t>
+          <t>OU @ MICH</t>
         </is>
       </c>
       <c r="C363" s="12" t="inlineStr">
         <is>
-          <t>2026-09-12 23:30</t>
+          <t>2026-09-12 16:00</t>
         </is>
       </c>
       <c r="D363" s="22" t="n">
@@ -24819,7 +24819,7 @@
       </c>
       <c r="F363" s="12" t="inlineStr">
         <is>
-          <t>TEX -1.5</t>
+          <t>OU +1.5</t>
         </is>
       </c>
       <c r="G363" s="23" t="n">
@@ -24829,7 +24829,7 @@
         <v>-110</v>
       </c>
       <c r="I363" s="15" t="n">
-        <v>0.4864517780012042</v>
+        <v>0.4879703180464825</v>
       </c>
       <c r="J363" s="15" t="n">
         <v>0.5</v>
@@ -24838,10 +24838,10 @@
         <v>0.5238095238095238</v>
       </c>
       <c r="L363" s="14" t="n">
-        <v>-0.03735774580831963</v>
+        <v>-0.03583920576304134</v>
       </c>
       <c r="M363" s="14" t="n">
-        <v>-0.07131933290679193</v>
+        <v>-0.06842030191126064</v>
       </c>
       <c r="N363" s="15" t="n">
         <v>0</v>
@@ -24864,35 +24864,35 @@
       </c>
       <c r="B364" s="17" t="inlineStr">
         <is>
-          <t>FLA @ AUB</t>
+          <t>OSU @ TEX</t>
         </is>
       </c>
       <c r="C364" s="17" t="inlineStr">
         <is>
-          <t>2026-09-19 23:00</t>
+          <t>2026-09-12 23:30</t>
         </is>
       </c>
       <c r="D364" s="25" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E364" s="17" t="inlineStr">
         <is>
-          <t>TOTAL</t>
+          <t>ATS</t>
         </is>
       </c>
       <c r="F364" s="17" t="inlineStr">
         <is>
-          <t>Over 53.5</t>
+          <t>TEX -1.5</t>
         </is>
       </c>
       <c r="G364" s="26" t="n">
-        <v>53.5</v>
+        <v>-1.5</v>
       </c>
       <c r="H364" s="18" t="n">
         <v>-110</v>
       </c>
       <c r="I364" s="20" t="n">
-        <v>0.4860426176118087</v>
+        <v>0.4864517780012042</v>
       </c>
       <c r="J364" s="20" t="n">
         <v>0.5</v>
@@ -24901,10 +24901,10 @@
         <v>0.5238095238095238</v>
       </c>
       <c r="L364" s="19" t="n">
-        <v>-0.03776690619771517</v>
+        <v>-0.03735774580831963</v>
       </c>
       <c r="M364" s="19" t="n">
-        <v>-0.07210045728654707</v>
+        <v>-0.07131933290679193</v>
       </c>
       <c r="N364" s="20" t="n">
         <v>0</v>
@@ -24927,16 +24927,16 @@
       </c>
       <c r="B365" s="12" t="inlineStr">
         <is>
-          <t>FSU @ MIA</t>
+          <t>FLA @ AUB</t>
         </is>
       </c>
       <c r="C365" s="12" t="inlineStr">
         <is>
-          <t>2026-10-17 04:00</t>
+          <t>2026-09-19 23:00</t>
         </is>
       </c>
       <c r="D365" s="22" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="E365" s="12" t="inlineStr">
         <is>
@@ -24955,7 +24955,7 @@
         <v>-110</v>
       </c>
       <c r="I365" s="15" t="n">
-        <v>0.48405269239997</v>
+        <v>0.4860426176118087</v>
       </c>
       <c r="J365" s="15" t="n">
         <v>0.5</v>
@@ -24964,10 +24964,10 @@
         <v>0.5238095238095238</v>
       </c>
       <c r="L365" s="14" t="n">
-        <v>-0.03975683140955388</v>
+        <v>-0.03776690619771517</v>
       </c>
       <c r="M365" s="14" t="n">
-        <v>-0.07589940541823914</v>
+        <v>-0.07210045728654707</v>
       </c>
       <c r="N365" s="15" t="n">
         <v>0</v>
@@ -24990,16 +24990,16 @@
       </c>
       <c r="B366" s="17" t="inlineStr">
         <is>
-          <t>TCU @ TTU</t>
+          <t>FSU @ MIA</t>
         </is>
       </c>
       <c r="C366" s="17" t="inlineStr">
         <is>
-          <t>2026-11-27 01:00</t>
+          <t>2026-10-17 04:00</t>
         </is>
       </c>
       <c r="D366" s="25" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="E366" s="17" t="inlineStr">
         <is>
@@ -25008,17 +25008,17 @@
       </c>
       <c r="F366" s="17" t="inlineStr">
         <is>
-          <t>Over 55.5</t>
+          <t>Over 53.5</t>
         </is>
       </c>
       <c r="G366" s="26" t="n">
-        <v>55.5</v>
+        <v>53.5</v>
       </c>
       <c r="H366" s="18" t="n">
         <v>-110</v>
       </c>
       <c r="I366" s="20" t="n">
-        <v>0.4840526843190074</v>
+        <v>0.48405269239997</v>
       </c>
       <c r="J366" s="20" t="n">
         <v>0.5</v>
@@ -25027,10 +25027,10 @@
         <v>0.5238095238095238</v>
       </c>
       <c r="L366" s="19" t="n">
-        <v>-0.03975683949051639</v>
+        <v>-0.03975683140955388</v>
       </c>
       <c r="M366" s="19" t="n">
-        <v>-0.07589942084553125</v>
+        <v>-0.07589940541823914</v>
       </c>
       <c r="N366" s="20" t="n">
         <v>0</v>
@@ -25053,16 +25053,16 @@
       </c>
       <c r="B367" s="12" t="inlineStr">
         <is>
-          <t>NAU @ ARIZ</t>
+          <t>TCU @ TTU</t>
         </is>
       </c>
       <c r="C367" s="12" t="inlineStr">
         <is>
-          <t>2026-09-06 01:30</t>
+          <t>2026-11-27 01:00</t>
         </is>
       </c>
       <c r="D367" s="22" t="n">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="E367" s="12" t="inlineStr">
         <is>
@@ -25071,17 +25071,17 @@
       </c>
       <c r="F367" s="12" t="inlineStr">
         <is>
-          <t>Over 56.5</t>
+          <t>Over 55.5</t>
         </is>
       </c>
       <c r="G367" s="23" t="n">
-        <v>56.5</v>
+        <v>55.5</v>
       </c>
       <c r="H367" s="13" t="n">
         <v>-110</v>
       </c>
       <c r="I367" s="15" t="n">
-        <v>0.4840526826079876</v>
+        <v>0.4840526843190074</v>
       </c>
       <c r="J367" s="15" t="n">
         <v>0.5</v>
@@ -25090,10 +25090,10 @@
         <v>0.5238095238095238</v>
       </c>
       <c r="L367" s="14" t="n">
-        <v>-0.03975684120153622</v>
+        <v>-0.03975683949051639</v>
       </c>
       <c r="M367" s="14" t="n">
-        <v>-0.07589942411202361</v>
+        <v>-0.07589942084553125</v>
       </c>
       <c r="N367" s="15" t="n">
         <v>0</v>
@@ -25106,11 +25106,7 @@
           <t>DraftKings</t>
         </is>
       </c>
-      <c r="Q367" s="12" t="inlineStr">
-        <is>
-          <t>NAU isn't a full FBS participant this season — model doesn't rate them reliably</t>
-        </is>
-      </c>
+      <c r="Q367" s="12" t="n"/>
     </row>
     <row r="368">
       <c r="A368" s="17" t="inlineStr">
@@ -25120,16 +25116,16 @@
       </c>
       <c r="B368" s="17" t="inlineStr">
         <is>
-          <t>LSU @ TENN</t>
+          <t>NAU @ ARIZ</t>
         </is>
       </c>
       <c r="C368" s="17" t="inlineStr">
         <is>
-          <t>2026-11-21 05:00</t>
+          <t>2026-09-06 01:30</t>
         </is>
       </c>
       <c r="D368" s="25" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="E368" s="17" t="inlineStr">
         <is>
@@ -25138,17 +25134,17 @@
       </c>
       <c r="F368" s="17" t="inlineStr">
         <is>
-          <t>Over 57.5</t>
+          <t>Over 56.5</t>
         </is>
       </c>
       <c r="G368" s="26" t="n">
-        <v>57.5</v>
+        <v>56.5</v>
       </c>
       <c r="H368" s="18" t="n">
         <v>-110</v>
       </c>
       <c r="I368" s="20" t="n">
-        <v>0.4840526816325738</v>
+        <v>0.4840526826079876</v>
       </c>
       <c r="J368" s="20" t="n">
         <v>0.5</v>
@@ -25157,10 +25153,10 @@
         <v>0.5238095238095238</v>
       </c>
       <c r="L368" s="19" t="n">
-        <v>-0.03975684217695008</v>
+        <v>-0.03975684120153622</v>
       </c>
       <c r="M368" s="19" t="n">
-        <v>-0.07589942597417731</v>
+        <v>-0.07589942411202361</v>
       </c>
       <c r="N368" s="20" t="n">
         <v>0</v>
@@ -25173,7 +25169,11 @@
           <t>DraftKings</t>
         </is>
       </c>
-      <c r="Q368" s="17" t="n"/>
+      <c r="Q368" s="17" t="inlineStr">
+        <is>
+          <t>NAU isn't a full FBS participant this season — model doesn't rate them reliably</t>
+        </is>
+      </c>
     </row>
     <row r="369">
       <c r="A369" s="12" t="inlineStr">
@@ -25183,35 +25183,35 @@
       </c>
       <c r="B369" s="12" t="inlineStr">
         <is>
-          <t>UNC @ DUKE</t>
+          <t>LSU @ TENN</t>
         </is>
       </c>
       <c r="C369" s="12" t="inlineStr">
         <is>
-          <t>2026-10-17 04:00</t>
+          <t>2026-11-21 05:00</t>
         </is>
       </c>
       <c r="D369" s="22" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="E369" s="12" t="inlineStr">
         <is>
-          <t>ATS</t>
+          <t>TOTAL</t>
         </is>
       </c>
       <c r="F369" s="12" t="inlineStr">
         <is>
-          <t>DUKE -4.5</t>
+          <t>Over 57.5</t>
         </is>
       </c>
       <c r="G369" s="23" t="n">
-        <v>-4.5</v>
+        <v>57.5</v>
       </c>
       <c r="H369" s="13" t="n">
         <v>-110</v>
       </c>
       <c r="I369" s="15" t="n">
-        <v>0.483373964127785</v>
+        <v>0.4840526816325738</v>
       </c>
       <c r="J369" s="15" t="n">
         <v>0.5</v>
@@ -25220,10 +25220,10 @@
         <v>0.5238095238095238</v>
       </c>
       <c r="L369" s="14" t="n">
-        <v>-0.04043555968173884</v>
+        <v>-0.03975684217695008</v>
       </c>
       <c r="M369" s="14" t="n">
-        <v>-0.07719515939241045</v>
+        <v>-0.07589942597417731</v>
       </c>
       <c r="N369" s="15" t="n">
         <v>0</v>
@@ -25246,16 +25246,16 @@
       </c>
       <c r="B370" s="17" t="inlineStr">
         <is>
-          <t>USC @ PSU</t>
+          <t>UNC @ DUKE</t>
         </is>
       </c>
       <c r="C370" s="17" t="inlineStr">
         <is>
-          <t>2026-10-10 04:00</t>
+          <t>2026-10-17 04:00</t>
         </is>
       </c>
       <c r="D370" s="25" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E370" s="17" t="inlineStr">
         <is>
@@ -25264,17 +25264,17 @@
       </c>
       <c r="F370" s="17" t="inlineStr">
         <is>
-          <t>USC +1.5</t>
+          <t>DUKE -4.5</t>
         </is>
       </c>
       <c r="G370" s="26" t="n">
-        <v>-1.5</v>
+        <v>-4.5</v>
       </c>
       <c r="H370" s="18" t="n">
         <v>-110</v>
       </c>
       <c r="I370" s="20" t="n">
-        <v>0.482804186505329</v>
+        <v>0.483373964127785</v>
       </c>
       <c r="J370" s="20" t="n">
         <v>0.5</v>
@@ -25283,10 +25283,10 @@
         <v>0.5238095238095238</v>
       </c>
       <c r="L370" s="19" t="n">
-        <v>-0.04100533730419487</v>
+        <v>-0.04043555968173884</v>
       </c>
       <c r="M370" s="19" t="n">
-        <v>-0.07828291667164466</v>
+        <v>-0.07719515939241045</v>
       </c>
       <c r="N370" s="20" t="n">
         <v>0</v>
@@ -25309,35 +25309,35 @@
       </c>
       <c r="B371" s="12" t="inlineStr">
         <is>
-          <t>USC @ UCLA</t>
+          <t>USC @ PSU</t>
         </is>
       </c>
       <c r="C371" s="12" t="inlineStr">
         <is>
-          <t>2026-11-28 05:00</t>
+          <t>2026-10-10 04:00</t>
         </is>
       </c>
       <c r="D371" s="22" t="n">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="E371" s="12" t="inlineStr">
         <is>
-          <t>TOTAL</t>
+          <t>ATS</t>
         </is>
       </c>
       <c r="F371" s="12" t="inlineStr">
         <is>
-          <t>Under 55.5</t>
+          <t>USC +1.5</t>
         </is>
       </c>
       <c r="G371" s="23" t="n">
-        <v>55.5</v>
+        <v>-1.5</v>
       </c>
       <c r="H371" s="13" t="n">
         <v>-110</v>
       </c>
       <c r="I371" s="15" t="n">
-        <v>0.4820643455849591</v>
+        <v>0.482804186505329</v>
       </c>
       <c r="J371" s="15" t="n">
         <v>0.5</v>
@@ -25346,10 +25346,10 @@
         <v>0.5238095238095238</v>
       </c>
       <c r="L371" s="14" t="n">
-        <v>-0.04174517822456469</v>
+        <v>-0.04100533730419487</v>
       </c>
       <c r="M371" s="14" t="n">
-        <v>-0.07969534024689612</v>
+        <v>-0.07828291667164466</v>
       </c>
       <c r="N371" s="15" t="n">
         <v>0</v>
@@ -25372,16 +25372,16 @@
       </c>
       <c r="B372" s="17" t="inlineStr">
         <is>
-          <t>MISS @ OU</t>
+          <t>USC @ UCLA</t>
         </is>
       </c>
       <c r="C372" s="17" t="inlineStr">
         <is>
-          <t>2026-11-14 05:00</t>
+          <t>2026-11-28 05:00</t>
         </is>
       </c>
       <c r="D372" s="25" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="E372" s="17" t="inlineStr">
         <is>
@@ -25390,17 +25390,17 @@
       </c>
       <c r="F372" s="17" t="inlineStr">
         <is>
-          <t>Under 53.5</t>
+          <t>Under 55.5</t>
         </is>
       </c>
       <c r="G372" s="26" t="n">
-        <v>53.5</v>
+        <v>55.5</v>
       </c>
       <c r="H372" s="18" t="n">
         <v>-110</v>
       </c>
       <c r="I372" s="20" t="n">
-        <v>0.4820643419479947</v>
+        <v>0.4820643455849591</v>
       </c>
       <c r="J372" s="20" t="n">
         <v>0.5</v>
@@ -25409,10 +25409,10 @@
         <v>0.5238095238095238</v>
       </c>
       <c r="L372" s="19" t="n">
-        <v>-0.04174518186152909</v>
+        <v>-0.04174517822456469</v>
       </c>
       <c r="M372" s="19" t="n">
-        <v>-0.07969534719019183</v>
+        <v>-0.07969534024689612</v>
       </c>
       <c r="N372" s="20" t="n">
         <v>0</v>
@@ -25435,16 +25435,16 @@
       </c>
       <c r="B373" s="12" t="inlineStr">
         <is>
-          <t>OSU @ USC</t>
+          <t>MISS @ OU</t>
         </is>
       </c>
       <c r="C373" s="12" t="inlineStr">
         <is>
-          <t>2026-10-31 04:00</t>
+          <t>2026-11-14 05:00</t>
         </is>
       </c>
       <c r="D373" s="22" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E373" s="12" t="inlineStr">
         <is>
@@ -25453,17 +25453,17 @@
       </c>
       <c r="F373" s="12" t="inlineStr">
         <is>
-          <t>Over 54.5</t>
+          <t>Under 53.5</t>
         </is>
       </c>
       <c r="G373" s="23" t="n">
-        <v>54.5</v>
+        <v>53.5</v>
       </c>
       <c r="H373" s="13" t="n">
         <v>-110</v>
       </c>
       <c r="I373" s="15" t="n">
-        <v>0.4800778118661322</v>
+        <v>0.4820643419479947</v>
       </c>
       <c r="J373" s="15" t="n">
         <v>0.5</v>
@@ -25472,10 +25472,10 @@
         <v>0.5238095238095238</v>
       </c>
       <c r="L373" s="14" t="n">
-        <v>-0.04373171194339165</v>
+        <v>-0.04174518186152909</v>
       </c>
       <c r="M373" s="14" t="n">
-        <v>-0.08348781371011121</v>
+        <v>-0.07969534719019183</v>
       </c>
       <c r="N373" s="15" t="n">
         <v>0</v>
@@ -25498,16 +25498,16 @@
       </c>
       <c r="B374" s="17" t="inlineStr">
         <is>
-          <t>UAB @ ILL</t>
+          <t>OSU @ USC</t>
         </is>
       </c>
       <c r="C374" s="17" t="inlineStr">
         <is>
-          <t>2026-09-04 01:00</t>
+          <t>2026-10-31 04:00</t>
         </is>
       </c>
       <c r="D374" s="25" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="E374" s="17" t="inlineStr">
         <is>
@@ -25516,17 +25516,17 @@
       </c>
       <c r="F374" s="17" t="inlineStr">
         <is>
-          <t>Under 56.5</t>
+          <t>Over 54.5</t>
         </is>
       </c>
       <c r="G374" s="26" t="n">
-        <v>56.5</v>
+        <v>54.5</v>
       </c>
       <c r="H374" s="18" t="n">
         <v>-110</v>
       </c>
       <c r="I374" s="20" t="n">
-        <v>0.48007780341312</v>
+        <v>0.4800778118661322</v>
       </c>
       <c r="J374" s="20" t="n">
         <v>0.5</v>
@@ -25535,10 +25535,10 @@
         <v>0.5238095238095238</v>
       </c>
       <c r="L374" s="19" t="n">
-        <v>-0.04373172039640383</v>
+        <v>-0.04373171194339165</v>
       </c>
       <c r="M374" s="19" t="n">
-        <v>-0.08348782984767994</v>
+        <v>-0.08348781371011121</v>
       </c>
       <c r="N374" s="20" t="n">
         <v>0</v>
@@ -25561,12 +25561,12 @@
       </c>
       <c r="B375" s="12" t="inlineStr">
         <is>
-          <t>NCSU @ UVA</t>
+          <t>UAB @ ILL</t>
         </is>
       </c>
       <c r="C375" s="12" t="inlineStr">
         <is>
-          <t>2026-08-29 19:30</t>
+          <t>2026-09-04 01:00</t>
         </is>
       </c>
       <c r="D375" s="22" t="n">
@@ -25579,17 +25579,17 @@
       </c>
       <c r="F375" s="12" t="inlineStr">
         <is>
-          <t>Under 53.5</t>
+          <t>Under 56.5</t>
         </is>
       </c>
       <c r="G375" s="23" t="n">
-        <v>53.5</v>
+        <v>56.5</v>
       </c>
       <c r="H375" s="13" t="n">
         <v>-110</v>
       </c>
       <c r="I375" s="15" t="n">
-        <v>0.4800777992356569</v>
+        <v>0.48007780341312</v>
       </c>
       <c r="J375" s="15" t="n">
         <v>0.5</v>
@@ -25598,10 +25598,10 @@
         <v>0.5238095238095238</v>
       </c>
       <c r="L375" s="14" t="n">
-        <v>-0.04373172457386698</v>
+        <v>-0.04373172039640383</v>
       </c>
       <c r="M375" s="14" t="n">
-        <v>-0.08348783782283686</v>
+        <v>-0.08348782984767994</v>
       </c>
       <c r="N375" s="15" t="n">
         <v>0</v>
@@ -25624,16 +25624,16 @@
       </c>
       <c r="B376" s="17" t="inlineStr">
         <is>
-          <t>TA&amp;M @ OU</t>
+          <t>NCSU @ UVA</t>
         </is>
       </c>
       <c r="C376" s="17" t="inlineStr">
         <is>
-          <t>2026-11-21 05:00</t>
+          <t>2026-08-29 19:30</t>
         </is>
       </c>
       <c r="D376" s="25" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="E376" s="17" t="inlineStr">
         <is>
@@ -25642,17 +25642,17 @@
       </c>
       <c r="F376" s="17" t="inlineStr">
         <is>
-          <t>Under 51.5</t>
+          <t>Under 53.5</t>
         </is>
       </c>
       <c r="G376" s="26" t="n">
-        <v>51.5</v>
+        <v>53.5</v>
       </c>
       <c r="H376" s="18" t="n">
         <v>-110</v>
       </c>
       <c r="I376" s="20" t="n">
-        <v>0.4800777888540669</v>
+        <v>0.4800777992356569</v>
       </c>
       <c r="J376" s="20" t="n">
         <v>0.5</v>
@@ -25661,10 +25661,10 @@
         <v>0.5238095238095238</v>
       </c>
       <c r="L376" s="19" t="n">
-        <v>-0.0437317349554569</v>
+        <v>-0.04373172457386698</v>
       </c>
       <c r="M376" s="19" t="n">
-        <v>-0.08348785764223582</v>
+        <v>-0.08348783782283686</v>
       </c>
       <c r="N376" s="20" t="n">
         <v>0</v>
@@ -25687,16 +25687,16 @@
       </c>
       <c r="B377" s="12" t="inlineStr">
         <is>
-          <t>UTU @ BYU</t>
+          <t>TA&amp;M @ OU</t>
         </is>
       </c>
       <c r="C377" s="12" t="inlineStr">
         <is>
-          <t>2026-09-06 00:00</t>
+          <t>2026-11-21 05:00</t>
         </is>
       </c>
       <c r="D377" s="22" t="n">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="E377" s="12" t="inlineStr">
         <is>
@@ -25705,17 +25705,17 @@
       </c>
       <c r="F377" s="12" t="inlineStr">
         <is>
-          <t>Under 54.5</t>
+          <t>Under 51.5</t>
         </is>
       </c>
       <c r="G377" s="23" t="n">
-        <v>54.5</v>
+        <v>51.5</v>
       </c>
       <c r="H377" s="13" t="n">
         <v>-110</v>
       </c>
       <c r="I377" s="15" t="n">
-        <v>0.4780932458027352</v>
+        <v>0.4800777888540669</v>
       </c>
       <c r="J377" s="15" t="n">
         <v>0.5</v>
@@ -25724,27 +25724,23 @@
         <v>0.5238095238095238</v>
       </c>
       <c r="L377" s="14" t="n">
-        <v>-0.04571627800678868</v>
+        <v>-0.0437317349554569</v>
       </c>
       <c r="M377" s="14" t="n">
-        <v>-0.08727653074023284</v>
+        <v>-0.08348785764223582</v>
       </c>
       <c r="N377" s="15" t="n">
         <v>0</v>
       </c>
       <c r="O377" s="24" t="n">
-        <v>0.4</v>
+        <v>0.45</v>
       </c>
       <c r="P377" s="12" t="inlineStr">
         <is>
           <t>DraftKings</t>
         </is>
       </c>
-      <c r="Q377" s="12" t="inlineStr">
-        <is>
-          <t>UTU isn't a full FBS participant this season — model doesn't rate them reliably</t>
-        </is>
-      </c>
+      <c r="Q377" s="12" t="n"/>
     </row>
     <row r="378">
       <c r="A378" s="17" t="inlineStr">
@@ -25754,16 +25750,16 @@
       </c>
       <c r="B378" s="17" t="inlineStr">
         <is>
-          <t>OU @ UGA</t>
+          <t>UTU @ BYU</t>
         </is>
       </c>
       <c r="C378" s="17" t="inlineStr">
         <is>
-          <t>2026-09-26 04:00</t>
+          <t>2026-09-06 00:00</t>
         </is>
       </c>
       <c r="D378" s="25" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E378" s="17" t="inlineStr">
         <is>
@@ -25772,17 +25768,17 @@
       </c>
       <c r="F378" s="17" t="inlineStr">
         <is>
-          <t>Over 52.5</t>
+          <t>Under 54.5</t>
         </is>
       </c>
       <c r="G378" s="26" t="n">
-        <v>52.5</v>
+        <v>54.5</v>
       </c>
       <c r="H378" s="18" t="n">
         <v>-110</v>
       </c>
       <c r="I378" s="20" t="n">
-        <v>0.476110901147586</v>
+        <v>0.4780932458027352</v>
       </c>
       <c r="J378" s="20" t="n">
         <v>0.5</v>
@@ -25791,23 +25787,27 @@
         <v>0.5238095238095238</v>
       </c>
       <c r="L378" s="19" t="n">
-        <v>-0.04769862266193786</v>
+        <v>-0.04571627800678868</v>
       </c>
       <c r="M378" s="19" t="n">
-        <v>-0.09106100690006314</v>
+        <v>-0.08727653074023284</v>
       </c>
       <c r="N378" s="20" t="n">
         <v>0</v>
       </c>
       <c r="O378" s="27" t="n">
-        <v>0.45</v>
+        <v>0.4</v>
       </c>
       <c r="P378" s="17" t="inlineStr">
         <is>
           <t>DraftKings</t>
         </is>
       </c>
-      <c r="Q378" s="17" t="n"/>
+      <c r="Q378" s="17" t="inlineStr">
+        <is>
+          <t>UTU isn't a full FBS participant this season — model doesn't rate them reliably</t>
+        </is>
+      </c>
     </row>
     <row r="379">
       <c r="A379" s="12" t="inlineStr">
@@ -25817,16 +25817,16 @@
       </c>
       <c r="B379" s="12" t="inlineStr">
         <is>
-          <t>SC @ CLEM</t>
+          <t>OU @ UGA</t>
         </is>
       </c>
       <c r="C379" s="12" t="inlineStr">
         <is>
-          <t>2026-11-28 05:00</t>
+          <t>2026-09-26 04:00</t>
         </is>
       </c>
       <c r="D379" s="22" t="n">
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="E379" s="12" t="inlineStr">
         <is>
@@ -25835,17 +25835,17 @@
       </c>
       <c r="F379" s="12" t="inlineStr">
         <is>
-          <t>Over 53.5</t>
+          <t>Over 52.5</t>
         </is>
       </c>
       <c r="G379" s="23" t="n">
-        <v>53.5</v>
+        <v>52.5</v>
       </c>
       <c r="H379" s="13" t="n">
         <v>-110</v>
       </c>
       <c r="I379" s="15" t="n">
-        <v>0.4761108907812599</v>
+        <v>0.476110901147586</v>
       </c>
       <c r="J379" s="15" t="n">
         <v>0.5</v>
@@ -25854,10 +25854,10 @@
         <v>0.5238095238095238</v>
       </c>
       <c r="L379" s="14" t="n">
-        <v>-0.04769863302826394</v>
+        <v>-0.04769862266193786</v>
       </c>
       <c r="M379" s="14" t="n">
-        <v>-0.09106102669032196</v>
+        <v>-0.09106100690006314</v>
       </c>
       <c r="N379" s="15" t="n">
         <v>0</v>
@@ -25880,16 +25880,16 @@
       </c>
       <c r="B380" s="17" t="inlineStr">
         <is>
-          <t>TNST @ UGA</t>
+          <t>SC @ CLEM</t>
         </is>
       </c>
       <c r="C380" s="17" t="inlineStr">
         <is>
-          <t>2026-09-05 19:00</t>
+          <t>2026-11-28 05:00</t>
         </is>
       </c>
       <c r="D380" s="25" t="n">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="E380" s="17" t="inlineStr">
         <is>
@@ -25898,17 +25898,17 @@
       </c>
       <c r="F380" s="17" t="inlineStr">
         <is>
-          <t>Over 56.5</t>
+          <t>Over 53.5</t>
         </is>
       </c>
       <c r="G380" s="26" t="n">
-        <v>56.5</v>
+        <v>53.5</v>
       </c>
       <c r="H380" s="18" t="n">
         <v>-110</v>
       </c>
       <c r="I380" s="20" t="n">
-        <v>0.4761108790335434</v>
+        <v>0.4761108907812599</v>
       </c>
       <c r="J380" s="20" t="n">
         <v>0.5</v>
@@ -25917,10 +25917,10 @@
         <v>0.5238095238095238</v>
       </c>
       <c r="L380" s="19" t="n">
-        <v>-0.0476986447759804</v>
+        <v>-0.04769863302826394</v>
       </c>
       <c r="M380" s="19" t="n">
-        <v>-0.09106104911778068</v>
+        <v>-0.09106102669032196</v>
       </c>
       <c r="N380" s="20" t="n">
         <v>0</v>
@@ -25933,11 +25933,7 @@
           <t>DraftKings</t>
         </is>
       </c>
-      <c r="Q380" s="17" t="inlineStr">
-        <is>
-          <t>TNST isn't a full FBS participant this season — model doesn't rate them reliably</t>
-        </is>
-      </c>
+      <c r="Q380" s="17" t="n"/>
     </row>
     <row r="381">
       <c r="A381" s="12" t="inlineStr">
@@ -25947,16 +25943,16 @@
       </c>
       <c r="B381" s="12" t="inlineStr">
         <is>
-          <t>ORE @ USC</t>
+          <t>TNST @ UGA</t>
         </is>
       </c>
       <c r="C381" s="12" t="inlineStr">
         <is>
-          <t>2026-09-26 04:00</t>
+          <t>2026-09-05 19:00</t>
         </is>
       </c>
       <c r="D381" s="22" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E381" s="12" t="inlineStr">
         <is>
@@ -25965,17 +25961,17 @@
       </c>
       <c r="F381" s="12" t="inlineStr">
         <is>
-          <t>Over 58.5</t>
+          <t>Over 56.5</t>
         </is>
       </c>
       <c r="G381" s="23" t="n">
-        <v>58.5</v>
+        <v>56.5</v>
       </c>
       <c r="H381" s="13" t="n">
         <v>-110</v>
       </c>
       <c r="I381" s="15" t="n">
-        <v>0.4761108771828951</v>
+        <v>0.4761108790335434</v>
       </c>
       <c r="J381" s="15" t="n">
         <v>0.5</v>
@@ -25984,10 +25980,10 @@
         <v>0.5238095238095238</v>
       </c>
       <c r="L381" s="14" t="n">
-        <v>-0.0476986466266287</v>
+        <v>-0.0476986447759804</v>
       </c>
       <c r="M381" s="14" t="n">
-        <v>-0.09106105265083653</v>
+        <v>-0.09106104911778068</v>
       </c>
       <c r="N381" s="15" t="n">
         <v>0</v>
@@ -26000,7 +25996,11 @@
           <t>DraftKings</t>
         </is>
       </c>
-      <c r="Q381" s="12" t="n"/>
+      <c r="Q381" s="12" t="inlineStr">
+        <is>
+          <t>TNST isn't a full FBS participant this season — model doesn't rate them reliably</t>
+        </is>
+      </c>
     </row>
     <row r="382">
       <c r="A382" s="17" t="inlineStr">
@@ -26010,16 +26010,16 @@
       </c>
       <c r="B382" s="17" t="inlineStr">
         <is>
-          <t>ALA @ TENN</t>
+          <t>ORE @ USC</t>
         </is>
       </c>
       <c r="C382" s="17" t="inlineStr">
         <is>
-          <t>2026-10-17 04:00</t>
+          <t>2026-09-26 04:00</t>
         </is>
       </c>
       <c r="D382" s="25" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="E382" s="17" t="inlineStr">
         <is>
@@ -26028,17 +26028,17 @@
       </c>
       <c r="F382" s="17" t="inlineStr">
         <is>
-          <t>Under 56.5</t>
+          <t>Over 58.5</t>
         </is>
       </c>
       <c r="G382" s="26" t="n">
-        <v>56.5</v>
+        <v>58.5</v>
       </c>
       <c r="H382" s="18" t="n">
         <v>-110</v>
       </c>
       <c r="I382" s="20" t="n">
-        <v>0.476110875556195</v>
+        <v>0.4761108771828951</v>
       </c>
       <c r="J382" s="20" t="n">
         <v>0.5</v>
@@ -26047,16 +26047,16 @@
         <v>0.5238095238095238</v>
       </c>
       <c r="L382" s="19" t="n">
-        <v>-0.04769864825332881</v>
+        <v>-0.0476986466266287</v>
       </c>
       <c r="M382" s="19" t="n">
-        <v>-0.09106105575635492</v>
+        <v>-0.09106105265083653</v>
       </c>
       <c r="N382" s="20" t="n">
         <v>0</v>
       </c>
       <c r="O382" s="27" t="n">
-        <v>0</v>
+        <v>0.45</v>
       </c>
       <c r="P382" s="17" t="inlineStr">
         <is>
@@ -26073,16 +26073,16 @@
       </c>
       <c r="B383" s="12" t="inlineStr">
         <is>
-          <t>KENT @ SC</t>
+          <t>ALA @ TENN</t>
         </is>
       </c>
       <c r="C383" s="12" t="inlineStr">
         <is>
-          <t>2026-09-05 16:45</t>
+          <t>2026-10-17 04:00</t>
         </is>
       </c>
       <c r="D383" s="22" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="E383" s="12" t="inlineStr">
         <is>
@@ -26091,17 +26091,17 @@
       </c>
       <c r="F383" s="12" t="inlineStr">
         <is>
-          <t>Under 53.5</t>
+          <t>Under 56.5</t>
         </is>
       </c>
       <c r="G383" s="23" t="n">
-        <v>53.5</v>
+        <v>56.5</v>
       </c>
       <c r="H383" s="13" t="n">
         <v>-110</v>
       </c>
       <c r="I383" s="15" t="n">
-        <v>0.4761108717682891</v>
+        <v>0.476110875556195</v>
       </c>
       <c r="J383" s="15" t="n">
         <v>0.5</v>
@@ -26110,16 +26110,16 @@
         <v>0.5238095238095238</v>
       </c>
       <c r="L383" s="14" t="n">
-        <v>-0.04769865204123469</v>
+        <v>-0.04769864825332881</v>
       </c>
       <c r="M383" s="14" t="n">
-        <v>-0.09106106298781158</v>
+        <v>-0.09106105575635492</v>
       </c>
       <c r="N383" s="15" t="n">
         <v>0</v>
       </c>
       <c r="O383" s="24" t="n">
-        <v>0.45</v>
+        <v>0</v>
       </c>
       <c r="P383" s="12" t="inlineStr">
         <is>
@@ -26136,35 +26136,35 @@
       </c>
       <c r="B384" s="17" t="inlineStr">
         <is>
-          <t>ASU @ ARIZ</t>
+          <t>KENT @ SC</t>
         </is>
       </c>
       <c r="C384" s="17" t="inlineStr">
         <is>
-          <t>2026-11-28 05:00</t>
+          <t>2026-09-05 16:45</t>
         </is>
       </c>
       <c r="D384" s="25" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="E384" s="17" t="inlineStr">
         <is>
-          <t>ATS</t>
+          <t>TOTAL</t>
         </is>
       </c>
       <c r="F384" s="17" t="inlineStr">
         <is>
-          <t>ARIZ -4.5</t>
+          <t>Under 53.5</t>
         </is>
       </c>
       <c r="G384" s="26" t="n">
-        <v>-4.5</v>
+        <v>53.5</v>
       </c>
       <c r="H384" s="18" t="n">
         <v>-110</v>
       </c>
       <c r="I384" s="20" t="n">
-        <v>0.4759178998113145</v>
+        <v>0.4761108717682891</v>
       </c>
       <c r="J384" s="20" t="n">
         <v>0.5</v>
@@ -26173,10 +26173,10 @@
         <v>0.5238095238095238</v>
       </c>
       <c r="L384" s="19" t="n">
-        <v>-0.04789162399820934</v>
+        <v>-0.04769865204123469</v>
       </c>
       <c r="M384" s="19" t="n">
-        <v>-0.09142946399658136</v>
+        <v>-0.09106106298781158</v>
       </c>
       <c r="N384" s="20" t="n">
         <v>0</v>
@@ -26199,7 +26199,7 @@
       </c>
       <c r="B385" s="12" t="inlineStr">
         <is>
-          <t>NCSU @ UNC</t>
+          <t>ASU @ ARIZ</t>
         </is>
       </c>
       <c r="C385" s="12" t="inlineStr">
@@ -26212,22 +26212,22 @@
       </c>
       <c r="E385" s="12" t="inlineStr">
         <is>
-          <t>TOTAL</t>
+          <t>ATS</t>
         </is>
       </c>
       <c r="F385" s="12" t="inlineStr">
         <is>
-          <t>Over 55.5</t>
+          <t>ARIZ -4.5</t>
         </is>
       </c>
       <c r="G385" s="23" t="n">
-        <v>55.5</v>
+        <v>-4.5</v>
       </c>
       <c r="H385" s="13" t="n">
         <v>-110</v>
       </c>
       <c r="I385" s="15" t="n">
-        <v>0.4741308885459136</v>
+        <v>0.4759178998113145</v>
       </c>
       <c r="J385" s="15" t="n">
         <v>0.5</v>
@@ -26236,10 +26236,10 @@
         <v>0.5238095238095238</v>
       </c>
       <c r="L385" s="14" t="n">
-        <v>-0.04967863526361027</v>
+        <v>-0.04789162399820934</v>
       </c>
       <c r="M385" s="14" t="n">
-        <v>-0.09484103095780133</v>
+        <v>-0.09142946399658136</v>
       </c>
       <c r="N385" s="15" t="n">
         <v>0</v>
@@ -26262,16 +26262,16 @@
       </c>
       <c r="B386" s="17" t="inlineStr">
         <is>
-          <t>VMI @ VT</t>
+          <t>NCSU @ UNC</t>
         </is>
       </c>
       <c r="C386" s="17" t="inlineStr">
         <is>
-          <t>2026-09-05 23:30</t>
+          <t>2026-11-28 05:00</t>
         </is>
       </c>
       <c r="D386" s="25" t="n">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="E386" s="17" t="inlineStr">
         <is>
@@ -26280,17 +26280,17 @@
       </c>
       <c r="F386" s="17" t="inlineStr">
         <is>
-          <t>Over 57.5</t>
+          <t>Over 55.5</t>
         </is>
       </c>
       <c r="G386" s="26" t="n">
-        <v>57.5</v>
+        <v>55.5</v>
       </c>
       <c r="H386" s="18" t="n">
         <v>-110</v>
       </c>
       <c r="I386" s="20" t="n">
-        <v>0.4741308851452813</v>
+        <v>0.4741308885459136</v>
       </c>
       <c r="J386" s="20" t="n">
         <v>0.5</v>
@@ -26299,10 +26299,10 @@
         <v>0.5238095238095238</v>
       </c>
       <c r="L386" s="19" t="n">
-        <v>-0.04967863866424249</v>
+        <v>-0.04967863526361027</v>
       </c>
       <c r="M386" s="19" t="n">
-        <v>-0.0948410374499174</v>
+        <v>-0.09484103095780133</v>
       </c>
       <c r="N386" s="20" t="n">
         <v>0</v>
@@ -26315,11 +26315,7 @@
           <t>DraftKings</t>
         </is>
       </c>
-      <c r="Q386" s="17" t="inlineStr">
-        <is>
-          <t>VMI isn't a full FBS participant this season — model doesn't rate them reliably</t>
-        </is>
-      </c>
+      <c r="Q386" s="17" t="n"/>
     </row>
     <row r="387">
       <c r="A387" s="12" t="inlineStr">
@@ -26329,35 +26325,35 @@
       </c>
       <c r="B387" s="12" t="inlineStr">
         <is>
-          <t>UVA @ VT</t>
+          <t>VMI @ VT</t>
         </is>
       </c>
       <c r="C387" s="12" t="inlineStr">
         <is>
-          <t>2026-11-28 05:00</t>
+          <t>2026-09-05 23:30</t>
         </is>
       </c>
       <c r="D387" s="22" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="E387" s="12" t="inlineStr">
         <is>
-          <t>ATS</t>
+          <t>TOTAL</t>
         </is>
       </c>
       <c r="F387" s="12" t="inlineStr">
         <is>
-          <t>VT -1.5</t>
+          <t>Over 57.5</t>
         </is>
       </c>
       <c r="G387" s="23" t="n">
-        <v>-1.5</v>
+        <v>57.5</v>
       </c>
       <c r="H387" s="13" t="n">
         <v>-110</v>
       </c>
       <c r="I387" s="15" t="n">
-        <v>0.4737252328619687</v>
+        <v>0.4741308851452813</v>
       </c>
       <c r="J387" s="15" t="n">
         <v>0.5</v>
@@ -26366,10 +26362,10 @@
         <v>0.5238095238095238</v>
       </c>
       <c r="L387" s="14" t="n">
-        <v>-0.05008429094755512</v>
+        <v>-0.04967863866424249</v>
       </c>
       <c r="M387" s="14" t="n">
-        <v>-0.09561546453624142</v>
+        <v>-0.0948410374499174</v>
       </c>
       <c r="N387" s="15" t="n">
         <v>0</v>
@@ -26382,7 +26378,11 @@
           <t>DraftKings</t>
         </is>
       </c>
-      <c r="Q387" s="12" t="n"/>
+      <c r="Q387" s="12" t="inlineStr">
+        <is>
+          <t>VMI isn't a full FBS participant this season — model doesn't rate them reliably</t>
+        </is>
+      </c>
     </row>
     <row r="388">
       <c r="A388" s="17" t="inlineStr">
@@ -26392,16 +26392,16 @@
       </c>
       <c r="B388" s="17" t="inlineStr">
         <is>
-          <t>NAVY @ ARMY</t>
+          <t>UVA @ VT</t>
         </is>
       </c>
       <c r="C388" s="17" t="inlineStr">
         <is>
-          <t>2026-12-12 20:00</t>
+          <t>2026-11-28 05:00</t>
         </is>
       </c>
       <c r="D388" s="25" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="E388" s="17" t="inlineStr">
         <is>
@@ -26410,17 +26410,17 @@
       </c>
       <c r="F388" s="17" t="inlineStr">
         <is>
-          <t>NAVY -2.5</t>
+          <t>VT -1.5</t>
         </is>
       </c>
       <c r="G388" s="26" t="n">
-        <v>2.5</v>
+        <v>-1.5</v>
       </c>
       <c r="H388" s="18" t="n">
         <v>-110</v>
       </c>
       <c r="I388" s="20" t="n">
-        <v>0.472672928903868</v>
+        <v>0.4737252328619687</v>
       </c>
       <c r="J388" s="20" t="n">
         <v>0.5</v>
@@ -26429,10 +26429,10 @@
         <v>0.5238095238095238</v>
       </c>
       <c r="L388" s="19" t="n">
-        <v>-0.05113659490565581</v>
+        <v>-0.05008429094755512</v>
       </c>
       <c r="M388" s="19" t="n">
-        <v>-0.09762440845625192</v>
+        <v>-0.09561546453624142</v>
       </c>
       <c r="N388" s="20" t="n">
         <v>0</v>
@@ -26455,35 +26455,35 @@
       </c>
       <c r="B389" s="12" t="inlineStr">
         <is>
-          <t>TEX @ LSU</t>
+          <t>NAVY @ ARMY</t>
         </is>
       </c>
       <c r="C389" s="12" t="inlineStr">
         <is>
-          <t>2026-11-14 05:00</t>
+          <t>2026-12-12 20:00</t>
         </is>
       </c>
       <c r="D389" s="22" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="E389" s="12" t="inlineStr">
         <is>
-          <t>TOTAL</t>
+          <t>ATS</t>
         </is>
       </c>
       <c r="F389" s="12" t="inlineStr">
         <is>
-          <t>Over 54.5</t>
+          <t>NAVY -2.5</t>
         </is>
       </c>
       <c r="G389" s="23" t="n">
-        <v>54.5</v>
+        <v>2.5</v>
       </c>
       <c r="H389" s="13" t="n">
         <v>-110</v>
       </c>
       <c r="I389" s="15" t="n">
-        <v>0.4721534743558814</v>
+        <v>0.472672928903868</v>
       </c>
       <c r="J389" s="15" t="n">
         <v>0.5</v>
@@ -26492,10 +26492,10 @@
         <v>0.5238095238095238</v>
       </c>
       <c r="L389" s="14" t="n">
-        <v>-0.05165604945364244</v>
+        <v>-0.05113659490565581</v>
       </c>
       <c r="M389" s="14" t="n">
-        <v>-0.0986160944114991</v>
+        <v>-0.09762440845625192</v>
       </c>
       <c r="N389" s="15" t="n">
         <v>0</v>
@@ -26518,16 +26518,16 @@
       </c>
       <c r="B390" s="17" t="inlineStr">
         <is>
-          <t>IDHO @ UTAH</t>
+          <t>TEX @ LSU</t>
         </is>
       </c>
       <c r="C390" s="17" t="inlineStr">
         <is>
-          <t>2026-09-04 01:00</t>
+          <t>2026-11-14 05:00</t>
         </is>
       </c>
       <c r="D390" s="25" t="n">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="E390" s="17" t="inlineStr">
         <is>
@@ -26536,17 +26536,17 @@
       </c>
       <c r="F390" s="17" t="inlineStr">
         <is>
-          <t>Under 56.5</t>
+          <t>Over 54.5</t>
         </is>
       </c>
       <c r="G390" s="26" t="n">
-        <v>56.5</v>
+        <v>54.5</v>
       </c>
       <c r="H390" s="18" t="n">
         <v>-110</v>
       </c>
       <c r="I390" s="20" t="n">
-        <v>0.4721534645106804</v>
+        <v>0.4721534743558814</v>
       </c>
       <c r="J390" s="20" t="n">
         <v>0.5</v>
@@ -26555,10 +26555,10 @@
         <v>0.5238095238095238</v>
       </c>
       <c r="L390" s="19" t="n">
-        <v>-0.05165605929884343</v>
+        <v>-0.05165604945364244</v>
       </c>
       <c r="M390" s="19" t="n">
-        <v>-0.09861611320688279</v>
+        <v>-0.0986160944114991</v>
       </c>
       <c r="N390" s="20" t="n">
         <v>0</v>
@@ -26571,11 +26571,7 @@
           <t>DraftKings</t>
         </is>
       </c>
-      <c r="Q390" s="17" t="inlineStr">
-        <is>
-          <t>IDHO isn't a full FBS participant this season — model doesn't rate them reliably</t>
-        </is>
-      </c>
+      <c r="Q390" s="17" t="n"/>
     </row>
     <row r="391">
       <c r="A391" s="12" t="inlineStr">
@@ -26585,12 +26581,12 @@
       </c>
       <c r="B391" s="12" t="inlineStr">
         <is>
-          <t>ULM @ MSST</t>
+          <t>IDHO @ UTAH</t>
         </is>
       </c>
       <c r="C391" s="12" t="inlineStr">
         <is>
-          <t>2026-09-05 23:30</t>
+          <t>2026-09-04 01:00</t>
         </is>
       </c>
       <c r="D391" s="22" t="n">
@@ -26603,17 +26599,17 @@
       </c>
       <c r="F391" s="12" t="inlineStr">
         <is>
-          <t>Under 55.5</t>
+          <t>Under 56.5</t>
         </is>
       </c>
       <c r="G391" s="23" t="n">
-        <v>55.5</v>
+        <v>56.5</v>
       </c>
       <c r="H391" s="13" t="n">
         <v>-110</v>
       </c>
       <c r="I391" s="15" t="n">
-        <v>0.4721534639284655</v>
+        <v>0.4721534645106804</v>
       </c>
       <c r="J391" s="15" t="n">
         <v>0.5</v>
@@ -26622,10 +26618,10 @@
         <v>0.5238095238095238</v>
       </c>
       <c r="L391" s="14" t="n">
-        <v>-0.05165605988105837</v>
+        <v>-0.05165605929884343</v>
       </c>
       <c r="M391" s="14" t="n">
-        <v>-0.09861611431838407</v>
+        <v>-0.09861611320688279</v>
       </c>
       <c r="N391" s="15" t="n">
         <v>0</v>
@@ -26638,7 +26634,11 @@
           <t>DraftKings</t>
         </is>
       </c>
-      <c r="Q391" s="12" t="n"/>
+      <c r="Q391" s="12" t="inlineStr">
+        <is>
+          <t>IDHO isn't a full FBS participant this season — model doesn't rate them reliably</t>
+        </is>
+      </c>
     </row>
     <row r="392">
       <c r="A392" s="17" t="inlineStr">
@@ -26648,16 +26648,16 @@
       </c>
       <c r="B392" s="17" t="inlineStr">
         <is>
-          <t>WASH @ ORE</t>
+          <t>ULM @ MSST</t>
         </is>
       </c>
       <c r="C392" s="17" t="inlineStr">
         <is>
-          <t>2026-11-28 05:00</t>
+          <t>2026-09-05 23:30</t>
         </is>
       </c>
       <c r="D392" s="25" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="E392" s="17" t="inlineStr">
         <is>
@@ -26666,17 +26666,17 @@
       </c>
       <c r="F392" s="17" t="inlineStr">
         <is>
-          <t>Under 54.5</t>
+          <t>Under 55.5</t>
         </is>
       </c>
       <c r="G392" s="26" t="n">
-        <v>54.5</v>
+        <v>55.5</v>
       </c>
       <c r="H392" s="18" t="n">
         <v>-110</v>
       </c>
       <c r="I392" s="20" t="n">
-        <v>0.4721534628948869</v>
+        <v>0.4721534639284655</v>
       </c>
       <c r="J392" s="20" t="n">
         <v>0.5</v>
@@ -26685,10 +26685,10 @@
         <v>0.5238095238095238</v>
       </c>
       <c r="L392" s="19" t="n">
-        <v>-0.05165606091463693</v>
+        <v>-0.05165605988105837</v>
       </c>
       <c r="M392" s="19" t="n">
-        <v>-0.09861611629157951</v>
+        <v>-0.09861611431838407</v>
       </c>
       <c r="N392" s="20" t="n">
         <v>0</v>
@@ -26711,16 +26711,16 @@
       </c>
       <c r="B393" s="12" t="inlineStr">
         <is>
-          <t>FAU @ FLA</t>
+          <t>WASH @ ORE</t>
         </is>
       </c>
       <c r="C393" s="12" t="inlineStr">
         <is>
-          <t>2026-09-05 23:45</t>
+          <t>2026-11-28 05:00</t>
         </is>
       </c>
       <c r="D393" s="22" t="n">
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="E393" s="12" t="inlineStr">
         <is>
@@ -26729,17 +26729,17 @@
       </c>
       <c r="F393" s="12" t="inlineStr">
         <is>
-          <t>Over 58.5</t>
+          <t>Under 54.5</t>
         </is>
       </c>
       <c r="G393" s="23" t="n">
-        <v>58.5</v>
+        <v>54.5</v>
       </c>
       <c r="H393" s="13" t="n">
         <v>-110</v>
       </c>
       <c r="I393" s="15" t="n">
-        <v>0.4701788165847314</v>
+        <v>0.4721534628948869</v>
       </c>
       <c r="J393" s="15" t="n">
         <v>0.5</v>
@@ -26748,10 +26748,10 @@
         <v>0.5238095238095238</v>
       </c>
       <c r="L393" s="14" t="n">
-        <v>-0.05363070722479246</v>
+        <v>-0.05165606091463693</v>
       </c>
       <c r="M393" s="14" t="n">
-        <v>-0.1023858956109673</v>
+        <v>-0.09861611629157951</v>
       </c>
       <c r="N393" s="15" t="n">
         <v>0</v>
@@ -26774,12 +26774,12 @@
       </c>
       <c r="B394" s="17" t="inlineStr">
         <is>
-          <t>MEM @ UNLV</t>
+          <t>FAU @ FLA</t>
         </is>
       </c>
       <c r="C394" s="17" t="inlineStr">
         <is>
-          <t>2026-08-30 02:00</t>
+          <t>2026-09-05 23:45</t>
         </is>
       </c>
       <c r="D394" s="25" t="n">
@@ -26792,17 +26792,17 @@
       </c>
       <c r="F394" s="17" t="inlineStr">
         <is>
-          <t>Under 56.5</t>
+          <t>Over 58.5</t>
         </is>
       </c>
       <c r="G394" s="26" t="n">
-        <v>56.5</v>
+        <v>58.5</v>
       </c>
       <c r="H394" s="18" t="n">
         <v>-110</v>
       </c>
       <c r="I394" s="20" t="n">
-        <v>0.4701788149384322</v>
+        <v>0.4701788165847314</v>
       </c>
       <c r="J394" s="20" t="n">
         <v>0.5</v>
@@ -26811,10 +26811,10 @@
         <v>0.5238095238095238</v>
       </c>
       <c r="L394" s="19" t="n">
-        <v>-0.05363070887109167</v>
+        <v>-0.05363070722479246</v>
       </c>
       <c r="M394" s="19" t="n">
-        <v>-0.1023858987539022</v>
+        <v>-0.1023858956109673</v>
       </c>
       <c r="N394" s="20" t="n">
         <v>0</v>
@@ -53686,7 +53686,7 @@
         <v>-5.5</v>
       </c>
       <c r="J12" s="30" t="n">
-        <v>56.5</v>
+        <v>57.5</v>
       </c>
       <c r="K12" s="18" t="n"/>
       <c r="L12" s="18" t="n"/>

</xml_diff>

<commit_message>
refresh 2026-08-22 17:44 UTC
</commit_message>
<xml_diff>
--- a/NCAAF_Edge_Model.xlsx
+++ b/NCAAF_Edge_Model.xlsx
@@ -637,7 +637,7 @@
     <row r="2" ht="26" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-08-22T13:55:24+00:00 from live ESPN data. This file is a snapshot, not the model. Re-run the pipeline to refresh it.</t>
+          <t>Generated 2026-08-22T17:44:49+00:00 from live ESPN data. This file is a snapshot, not the model. Re-run the pipeline to refresh it.</t>
         </is>
       </c>
     </row>
@@ -2040,7 +2040,7 @@
       </c>
       <c r="P10" s="17" t="inlineStr">
         <is>
-          <t>DraftKings</t>
+          <t>Draft Kings</t>
         </is>
       </c>
       <c r="Q10" s="17" t="n"/>
@@ -2166,7 +2166,7 @@
       </c>
       <c r="P12" s="17" t="inlineStr">
         <is>
-          <t>DraftKings</t>
+          <t>Draft Kings</t>
         </is>
       </c>
       <c r="Q12" s="17" t="n"/>
@@ -8588,7 +8588,7 @@
       </c>
       <c r="P110" s="17" t="inlineStr">
         <is>
-          <t>DraftKings</t>
+          <t>Draft Kings</t>
         </is>
       </c>
       <c r="Q110" s="17" t="inlineStr">
@@ -9526,7 +9526,7 @@
       </c>
       <c r="P124" s="17" t="inlineStr">
         <is>
-          <t>DraftKings</t>
+          <t>Draft Kings</t>
         </is>
       </c>
       <c r="Q124" s="17" t="inlineStr">
@@ -11134,7 +11134,7 @@
       </c>
       <c r="P148" s="17" t="inlineStr">
         <is>
-          <t>DraftKings</t>
+          <t>Draft Kings</t>
         </is>
       </c>
       <c r="Q148" s="17" t="inlineStr">
@@ -11201,7 +11201,7 @@
       </c>
       <c r="P149" s="12" t="inlineStr">
         <is>
-          <t>DraftKings</t>
+          <t>Draft Kings</t>
         </is>
       </c>
       <c r="Q149" s="12" t="inlineStr">
@@ -11532,7 +11532,7 @@
       </c>
       <c r="P154" s="17" t="inlineStr">
         <is>
-          <t>DraftKings</t>
+          <t>Draft Kings</t>
         </is>
       </c>
       <c r="Q154" s="17" t="n"/>
@@ -12611,7 +12611,7 @@
       </c>
       <c r="P171" s="12" t="inlineStr">
         <is>
-          <t>DraftKings</t>
+          <t>Draft Kings</t>
         </is>
       </c>
       <c r="Q171" s="12" t="n"/>
@@ -14718,7 +14718,7 @@
       </c>
       <c r="P204" s="17" t="inlineStr">
         <is>
-          <t>DraftKings</t>
+          <t>Draft Kings</t>
         </is>
       </c>
       <c r="Q204" s="17" t="n"/>
@@ -15671,7 +15671,7 @@
       </c>
       <c r="P219" s="12" t="inlineStr">
         <is>
-          <t>DraftKings</t>
+          <t>Draft Kings</t>
         </is>
       </c>
       <c r="Q219" s="12" t="n"/>
@@ -16305,7 +16305,7 @@
       </c>
       <c r="P229" s="12" t="inlineStr">
         <is>
-          <t>DraftKings</t>
+          <t>Draft Kings</t>
         </is>
       </c>
       <c r="Q229" s="12" t="n"/>
@@ -16683,7 +16683,7 @@
       </c>
       <c r="P235" s="12" t="inlineStr">
         <is>
-          <t>DraftKings</t>
+          <t>Draft Kings</t>
         </is>
       </c>
       <c r="Q235" s="12" t="n"/>
@@ -17191,7 +17191,7 @@
       </c>
       <c r="P243" s="12" t="inlineStr">
         <is>
-          <t>DraftKings</t>
+          <t>Draft Kings</t>
         </is>
       </c>
       <c r="Q243" s="12" t="n"/>
@@ -18396,7 +18396,7 @@
       </c>
       <c r="P262" s="17" t="inlineStr">
         <is>
-          <t>DraftKings</t>
+          <t>Draft Kings</t>
         </is>
       </c>
       <c r="Q262" s="17" t="n"/>
@@ -19743,7 +19743,7 @@
       </c>
       <c r="P283" s="12" t="inlineStr">
         <is>
-          <t>DraftKings</t>
+          <t>Draft Kings</t>
         </is>
       </c>
       <c r="Q283" s="12" t="n"/>
@@ -21007,7 +21007,7 @@
       </c>
       <c r="P303" s="12" t="inlineStr">
         <is>
-          <t>DraftKings</t>
+          <t>Draft Kings</t>
         </is>
       </c>
       <c r="Q303" s="12" t="n"/>
@@ -24410,7 +24410,7 @@
       </c>
       <c r="P356" s="17" t="inlineStr">
         <is>
-          <t>DraftKings</t>
+          <t>Draft Kings</t>
         </is>
       </c>
       <c r="Q356" s="17" t="n"/>
@@ -25674,7 +25674,7 @@
       </c>
       <c r="P376" s="17" t="inlineStr">
         <is>
-          <t>DraftKings</t>
+          <t>Draft Kings</t>
         </is>
       </c>
       <c r="Q376" s="17" t="n"/>
@@ -27021,7 +27021,7 @@
       </c>
       <c r="P397" s="12" t="inlineStr">
         <is>
-          <t>DraftKings</t>
+          <t>Draft Kings</t>
         </is>
       </c>
       <c r="Q397" s="12" t="n"/>
@@ -28226,7 +28226,7 @@
       </c>
       <c r="P416" s="17" t="inlineStr">
         <is>
-          <t>DraftKings</t>
+          <t>Draft Kings</t>
         </is>
       </c>
       <c r="Q416" s="17" t="n"/>
@@ -28734,7 +28734,7 @@
       </c>
       <c r="P424" s="17" t="inlineStr">
         <is>
-          <t>DraftKings</t>
+          <t>Draft Kings</t>
         </is>
       </c>
       <c r="Q424" s="17" t="n"/>
@@ -29112,7 +29112,7 @@
       </c>
       <c r="P430" s="17" t="inlineStr">
         <is>
-          <t>DraftKings</t>
+          <t>Draft Kings</t>
         </is>
       </c>
       <c r="Q430" s="17" t="n"/>
@@ -29746,7 +29746,7 @@
       </c>
       <c r="P440" s="17" t="inlineStr">
         <is>
-          <t>DraftKings</t>
+          <t>Draft Kings</t>
         </is>
       </c>
       <c r="Q440" s="17" t="n"/>
@@ -30699,7 +30699,7 @@
       </c>
       <c r="P455" s="12" t="inlineStr">
         <is>
-          <t>DraftKings</t>
+          <t>Draft Kings</t>
         </is>
       </c>
       <c r="Q455" s="12" t="n"/>
@@ -32806,7 +32806,7 @@
       </c>
       <c r="P488" s="17" t="inlineStr">
         <is>
-          <t>DraftKings</t>
+          <t>Draft Kings</t>
         </is>
       </c>
       <c r="Q488" s="17" t="n"/>
@@ -33885,7 +33885,7 @@
       </c>
       <c r="P505" s="12" t="inlineStr">
         <is>
-          <t>DraftKings</t>
+          <t>Draft Kings</t>
         </is>
       </c>
       <c r="Q505" s="12" t="n"/>
@@ -34145,7 +34145,7 @@
       </c>
       <c r="P509" s="12" t="inlineStr">
         <is>
-          <t>DraftKings</t>
+          <t>Draft Kings</t>
         </is>
       </c>
       <c r="Q509" s="12" t="n"/>
@@ -34334,7 +34334,7 @@
       </c>
       <c r="P512" s="17" t="inlineStr">
         <is>
-          <t>DraftKings</t>
+          <t>Draft Kings</t>
         </is>
       </c>
       <c r="Q512" s="17" t="n"/>
@@ -36512,7 +36512,7 @@
       </c>
       <c r="P546" s="17" t="inlineStr">
         <is>
-          <t>DraftKings</t>
+          <t>Draft Kings</t>
         </is>
       </c>
       <c r="Q546" s="17" t="n"/>
@@ -37993,7 +37993,7 @@
       </c>
       <c r="P569" s="12" t="inlineStr">
         <is>
-          <t>DraftKings</t>
+          <t>Draft Kings</t>
         </is>
       </c>
       <c r="Q569" s="12" t="n"/>
@@ -41601,7 +41601,7 @@
       </c>
       <c r="P625" s="12" t="inlineStr">
         <is>
-          <t>DraftKings</t>
+          <t>Draft Kings</t>
         </is>
       </c>
       <c r="Q625" s="12" t="n"/>
@@ -41928,7 +41928,7 @@
       </c>
       <c r="P630" s="17" t="inlineStr">
         <is>
-          <t>DraftKings</t>
+          <t>Draft Kings</t>
         </is>
       </c>
       <c r="Q630" s="17" t="n"/>
@@ -53377,7 +53377,7 @@
       <c r="L5" s="13" t="n"/>
       <c r="M5" s="12" t="inlineStr">
         <is>
-          <t>DraftKings</t>
+          <t>Draft Kings</t>
         </is>
       </c>
     </row>
@@ -53422,7 +53422,7 @@
       <c r="L6" s="18" t="n"/>
       <c r="M6" s="17" t="inlineStr">
         <is>
-          <t>DraftKings</t>
+          <t>Draft Kings</t>
         </is>
       </c>
     </row>
@@ -53467,7 +53467,7 @@
       <c r="L7" s="13" t="n"/>
       <c r="M7" s="12" t="inlineStr">
         <is>
-          <t>DraftKings</t>
+          <t>Draft Kings</t>
         </is>
       </c>
     </row>
@@ -53512,7 +53512,7 @@
       <c r="L8" s="18" t="n"/>
       <c r="M8" s="17" t="inlineStr">
         <is>
-          <t>DraftKings</t>
+          <t>Draft Kings</t>
         </is>
       </c>
     </row>
@@ -53557,7 +53557,7 @@
       <c r="L9" s="13" t="n"/>
       <c r="M9" s="12" t="inlineStr">
         <is>
-          <t>DraftKings</t>
+          <t>Draft Kings</t>
         </is>
       </c>
     </row>
@@ -53602,7 +53602,7 @@
       <c r="L10" s="18" t="n"/>
       <c r="M10" s="17" t="inlineStr">
         <is>
-          <t>DraftKings</t>
+          <t>Draft Kings</t>
         </is>
       </c>
     </row>
@@ -53647,7 +53647,7 @@
       <c r="L11" s="13" t="n"/>
       <c r="M11" s="12" t="inlineStr">
         <is>
-          <t>DraftKings</t>
+          <t>Draft Kings</t>
         </is>
       </c>
     </row>
@@ -53692,7 +53692,7 @@
       <c r="L12" s="18" t="n"/>
       <c r="M12" s="17" t="inlineStr">
         <is>
-          <t>DraftKings</t>
+          <t>Draft Kings</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
refresh 2026-08-22 21:45 UTC
</commit_message>
<xml_diff>
--- a/NCAAF_Edge_Model.xlsx
+++ b/NCAAF_Edge_Model.xlsx
@@ -637,7 +637,7 @@
     <row r="2" ht="26" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-08-22T17:44:49+00:00 from live ESPN data. This file is a snapshot, not the model. Re-run the pipeline to refresh it.</t>
+          <t>Generated 2026-08-22T21:45:54+00:00 from live ESPN data. This file is a snapshot, not the model. Re-run the pipeline to refresh it.</t>
         </is>
       </c>
     </row>
@@ -2040,7 +2040,7 @@
       </c>
       <c r="P10" s="17" t="inlineStr">
         <is>
-          <t>Draft Kings</t>
+          <t>DraftKings</t>
         </is>
       </c>
       <c r="Q10" s="17" t="n"/>
@@ -2166,7 +2166,7 @@
       </c>
       <c r="P12" s="17" t="inlineStr">
         <is>
-          <t>Draft Kings</t>
+          <t>DraftKings</t>
         </is>
       </c>
       <c r="Q12" s="17" t="n"/>
@@ -8588,7 +8588,7 @@
       </c>
       <c r="P110" s="17" t="inlineStr">
         <is>
-          <t>Draft Kings</t>
+          <t>DraftKings</t>
         </is>
       </c>
       <c r="Q110" s="17" t="inlineStr">
@@ -9141,12 +9141,12 @@
       </c>
       <c r="B119" s="12" t="inlineStr">
         <is>
-          <t>FIU @ USF</t>
+          <t>SAC @ EMU</t>
         </is>
       </c>
       <c r="C119" s="12" t="inlineStr">
         <is>
-          <t>2026-09-05 23:00</t>
+          <t>2026-08-29 22:30</t>
         </is>
       </c>
       <c r="D119" s="22" t="n">
@@ -9159,17 +9159,17 @@
       </c>
       <c r="F119" s="12" t="inlineStr">
         <is>
-          <t>FIU +13.5</t>
+          <t>SAC +9.5</t>
         </is>
       </c>
       <c r="G119" s="23" t="n">
-        <v>-13.5</v>
+        <v>-9.5</v>
       </c>
       <c r="H119" s="13" t="n">
         <v>-110</v>
       </c>
       <c r="I119" s="15" t="n">
-        <v>0.6366620259462109</v>
+        <v>0.6373042089106218</v>
       </c>
       <c r="J119" s="15" t="n">
         <v>0.5</v>
@@ -9178,10 +9178,10 @@
         <v>0.5238095238095238</v>
       </c>
       <c r="L119" s="14" t="n">
-        <v>0.1128525021366871</v>
+        <v>0.1134946851010979</v>
       </c>
       <c r="M119" s="14" t="n">
-        <v>0.2154456858973118</v>
+        <v>0.2166716715566417</v>
       </c>
       <c r="N119" s="15" t="n">
         <v>0</v>
@@ -9208,12 +9208,12 @@
       </c>
       <c r="B120" s="17" t="inlineStr">
         <is>
-          <t>URI @ TEM</t>
+          <t>FIU @ USF</t>
         </is>
       </c>
       <c r="C120" s="17" t="inlineStr">
         <is>
-          <t>2026-09-05 18:00</t>
+          <t>2026-09-05 23:00</t>
         </is>
       </c>
       <c r="D120" s="25" t="n">
@@ -9226,17 +9226,17 @@
       </c>
       <c r="F120" s="17" t="inlineStr">
         <is>
-          <t>URI +10</t>
+          <t>FIU +13.5</t>
         </is>
       </c>
       <c r="G120" s="26" t="n">
-        <v>-10</v>
+        <v>-13.5</v>
       </c>
       <c r="H120" s="18" t="n">
         <v>-110</v>
       </c>
       <c r="I120" s="20" t="n">
-        <v>0.6338812332726149</v>
+        <v>0.6366620259462109</v>
       </c>
       <c r="J120" s="20" t="n">
         <v>0.5</v>
@@ -9245,13 +9245,13 @@
         <v>0.5238095238095238</v>
       </c>
       <c r="L120" s="19" t="n">
-        <v>0.1100717094630911</v>
+        <v>0.1128525021366871</v>
       </c>
       <c r="M120" s="19" t="n">
-        <v>0.2031606380380864</v>
+        <v>0.2154456858973118</v>
       </c>
       <c r="N120" s="20" t="n">
-        <v>0.0332</v>
+        <v>0</v>
       </c>
       <c r="O120" s="27" t="n">
         <v>0.45</v>
@@ -9263,7 +9263,7 @@
       </c>
       <c r="Q120" s="17" t="inlineStr">
         <is>
-          <t>URI isn't a full FBS participant this season — model doesn't rate them reliably</t>
+          <t>outside the top 10 plays for this week</t>
         </is>
       </c>
     </row>
@@ -9275,16 +9275,16 @@
       </c>
       <c r="B121" s="12" t="inlineStr">
         <is>
-          <t>ISU @ IOWA</t>
+          <t>URI @ TEM</t>
         </is>
       </c>
       <c r="C121" s="12" t="inlineStr">
         <is>
-          <t>2026-09-12 23:30</t>
+          <t>2026-09-05 18:00</t>
         </is>
       </c>
       <c r="D121" s="22" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E121" s="12" t="inlineStr">
         <is>
@@ -9293,17 +9293,17 @@
       </c>
       <c r="F121" s="12" t="inlineStr">
         <is>
-          <t>ISU +11.5</t>
+          <t>URI +10</t>
         </is>
       </c>
       <c r="G121" s="23" t="n">
-        <v>-11.5</v>
+        <v>-10</v>
       </c>
       <c r="H121" s="13" t="n">
         <v>-110</v>
       </c>
       <c r="I121" s="15" t="n">
-        <v>0.6332052980165461</v>
+        <v>0.6338812332726149</v>
       </c>
       <c r="J121" s="15" t="n">
         <v>0.5</v>
@@ -9312,13 +9312,13 @@
         <v>0.5238095238095238</v>
       </c>
       <c r="L121" s="14" t="n">
-        <v>0.1093957742070223</v>
+        <v>0.1100717094630911</v>
       </c>
       <c r="M121" s="14" t="n">
-        <v>0.2088464780315881</v>
+        <v>0.2031606380380864</v>
       </c>
       <c r="N121" s="15" t="n">
-        <v>0</v>
+        <v>0.0332</v>
       </c>
       <c r="O121" s="24" t="n">
         <v>0.45</v>
@@ -9330,7 +9330,7 @@
       </c>
       <c r="Q121" s="12" t="inlineStr">
         <is>
-          <t>correlated with a stronger play on the same game</t>
+          <t>URI isn't a full FBS participant this season — model doesn't rate them reliably</t>
         </is>
       </c>
     </row>
@@ -9342,35 +9342,35 @@
       </c>
       <c r="B122" s="17" t="inlineStr">
         <is>
-          <t>TAR @ BGSU</t>
+          <t>ISU @ IOWA</t>
         </is>
       </c>
       <c r="C122" s="17" t="inlineStr">
         <is>
-          <t>2026-09-05 16:00</t>
+          <t>2026-09-12 23:30</t>
         </is>
       </c>
       <c r="D122" s="25" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E122" s="17" t="inlineStr">
         <is>
-          <t>TOTAL</t>
+          <t>ATS</t>
         </is>
       </c>
       <c r="F122" s="17" t="inlineStr">
         <is>
-          <t>Over 47.5</t>
+          <t>ISU +11.5</t>
         </is>
       </c>
       <c r="G122" s="26" t="n">
-        <v>47.5</v>
+        <v>-11.5</v>
       </c>
       <c r="H122" s="18" t="n">
         <v>-110</v>
       </c>
       <c r="I122" s="20" t="n">
-        <v>0.6321649686522863</v>
+        <v>0.6332052980165461</v>
       </c>
       <c r="J122" s="20" t="n">
         <v>0.5</v>
@@ -9379,10 +9379,10 @@
         <v>0.5238095238095238</v>
       </c>
       <c r="L122" s="19" t="n">
-        <v>0.1083554448427625</v>
+        <v>0.1093957742070223</v>
       </c>
       <c r="M122" s="19" t="n">
-        <v>0.2068603946998194</v>
+        <v>0.2088464780315881</v>
       </c>
       <c r="N122" s="20" t="n">
         <v>0</v>
@@ -9397,7 +9397,7 @@
       </c>
       <c r="Q122" s="17" t="inlineStr">
         <is>
-          <t>TAR isn't a full FBS participant this season — model doesn't rate them reliably</t>
+          <t>correlated with a stronger play on the same game</t>
         </is>
       </c>
     </row>
@@ -9409,7 +9409,7 @@
       </c>
       <c r="B123" s="12" t="inlineStr">
         <is>
-          <t>OHIO @ NEB</t>
+          <t>TAR @ BGSU</t>
         </is>
       </c>
       <c r="C123" s="12" t="inlineStr">
@@ -9437,7 +9437,7 @@
         <v>-110</v>
       </c>
       <c r="I123" s="15" t="n">
-        <v>0.6306198692024518</v>
+        <v>0.6321649686522863</v>
       </c>
       <c r="J123" s="15" t="n">
         <v>0.5</v>
@@ -9446,10 +9446,10 @@
         <v>0.5238095238095238</v>
       </c>
       <c r="L123" s="14" t="n">
-        <v>0.106810345392928</v>
+        <v>0.1083554448427625</v>
       </c>
       <c r="M123" s="14" t="n">
-        <v>0.203910659386499</v>
+        <v>0.2068603946998194</v>
       </c>
       <c r="N123" s="15" t="n">
         <v>0</v>
@@ -9464,7 +9464,7 @@
       </c>
       <c r="Q123" s="12" t="inlineStr">
         <is>
-          <t>correlated with a stronger play on the same game</t>
+          <t>TAR isn't a full FBS participant this season — model doesn't rate them reliably</t>
         </is>
       </c>
     </row>
@@ -9476,12 +9476,12 @@
       </c>
       <c r="B124" s="17" t="inlineStr">
         <is>
-          <t>SAC @ EMU</t>
+          <t>OHIO @ NEB</t>
         </is>
       </c>
       <c r="C124" s="17" t="inlineStr">
         <is>
-          <t>2026-08-29 22:30</t>
+          <t>2026-09-05 16:00</t>
         </is>
       </c>
       <c r="D124" s="25" t="n">
@@ -9489,22 +9489,22 @@
       </c>
       <c r="E124" s="17" t="inlineStr">
         <is>
-          <t>ATS</t>
+          <t>TOTAL</t>
         </is>
       </c>
       <c r="F124" s="17" t="inlineStr">
         <is>
-          <t>SAC +8.5</t>
+          <t>Over 47.5</t>
         </is>
       </c>
       <c r="G124" s="26" t="n">
-        <v>-8.5</v>
+        <v>47.5</v>
       </c>
       <c r="H124" s="18" t="n">
         <v>-110</v>
       </c>
       <c r="I124" s="20" t="n">
-        <v>0.6278769996316718</v>
+        <v>0.6306198692024518</v>
       </c>
       <c r="J124" s="20" t="n">
         <v>0.5</v>
@@ -9513,10 +9513,10 @@
         <v>0.5238095238095238</v>
       </c>
       <c r="L124" s="19" t="n">
-        <v>0.1040674758221479</v>
+        <v>0.106810345392928</v>
       </c>
       <c r="M124" s="19" t="n">
-        <v>0.1986742720241007</v>
+        <v>0.203910659386499</v>
       </c>
       <c r="N124" s="20" t="n">
         <v>0</v>
@@ -9526,12 +9526,12 @@
       </c>
       <c r="P124" s="17" t="inlineStr">
         <is>
-          <t>Draft Kings</t>
+          <t>DraftKings</t>
         </is>
       </c>
       <c r="Q124" s="17" t="inlineStr">
         <is>
-          <t>outside the top 10 plays for this week</t>
+          <t>correlated with a stronger play on the same game</t>
         </is>
       </c>
     </row>
@@ -11134,7 +11134,7 @@
       </c>
       <c r="P148" s="17" t="inlineStr">
         <is>
-          <t>Draft Kings</t>
+          <t>DraftKings</t>
         </is>
       </c>
       <c r="Q148" s="17" t="inlineStr">
@@ -11201,7 +11201,7 @@
       </c>
       <c r="P149" s="12" t="inlineStr">
         <is>
-          <t>Draft Kings</t>
+          <t>DraftKings</t>
         </is>
       </c>
       <c r="Q149" s="12" t="inlineStr">
@@ -11532,7 +11532,7 @@
       </c>
       <c r="P154" s="17" t="inlineStr">
         <is>
-          <t>Draft Kings</t>
+          <t>DraftKings</t>
         </is>
       </c>
       <c r="Q154" s="17" t="n"/>
@@ -12611,7 +12611,7 @@
       </c>
       <c r="P171" s="12" t="inlineStr">
         <is>
-          <t>Draft Kings</t>
+          <t>DraftKings</t>
         </is>
       </c>
       <c r="Q171" s="12" t="n"/>
@@ -14718,7 +14718,7 @@
       </c>
       <c r="P204" s="17" t="inlineStr">
         <is>
-          <t>Draft Kings</t>
+          <t>DraftKings</t>
         </is>
       </c>
       <c r="Q204" s="17" t="n"/>
@@ -15671,7 +15671,7 @@
       </c>
       <c r="P219" s="12" t="inlineStr">
         <is>
-          <t>Draft Kings</t>
+          <t>DraftKings</t>
         </is>
       </c>
       <c r="Q219" s="12" t="n"/>
@@ -16305,7 +16305,7 @@
       </c>
       <c r="P229" s="12" t="inlineStr">
         <is>
-          <t>Draft Kings</t>
+          <t>DraftKings</t>
         </is>
       </c>
       <c r="Q229" s="12" t="n"/>
@@ -16683,7 +16683,7 @@
       </c>
       <c r="P235" s="12" t="inlineStr">
         <is>
-          <t>Draft Kings</t>
+          <t>DraftKings</t>
         </is>
       </c>
       <c r="Q235" s="12" t="n"/>
@@ -17191,7 +17191,7 @@
       </c>
       <c r="P243" s="12" t="inlineStr">
         <is>
-          <t>Draft Kings</t>
+          <t>DraftKings</t>
         </is>
       </c>
       <c r="Q243" s="12" t="n"/>
@@ -18396,7 +18396,7 @@
       </c>
       <c r="P262" s="17" t="inlineStr">
         <is>
-          <t>Draft Kings</t>
+          <t>DraftKings</t>
         </is>
       </c>
       <c r="Q262" s="17" t="n"/>
@@ -19743,7 +19743,7 @@
       </c>
       <c r="P283" s="12" t="inlineStr">
         <is>
-          <t>Draft Kings</t>
+          <t>DraftKings</t>
         </is>
       </c>
       <c r="Q283" s="12" t="n"/>
@@ -21007,7 +21007,7 @@
       </c>
       <c r="P303" s="12" t="inlineStr">
         <is>
-          <t>Draft Kings</t>
+          <t>DraftKings</t>
         </is>
       </c>
       <c r="Q303" s="12" t="n"/>
@@ -24410,7 +24410,7 @@
       </c>
       <c r="P356" s="17" t="inlineStr">
         <is>
-          <t>Draft Kings</t>
+          <t>DraftKings</t>
         </is>
       </c>
       <c r="Q356" s="17" t="n"/>
@@ -25674,7 +25674,7 @@
       </c>
       <c r="P376" s="17" t="inlineStr">
         <is>
-          <t>Draft Kings</t>
+          <t>DraftKings</t>
         </is>
       </c>
       <c r="Q376" s="17" t="n"/>
@@ -27021,7 +27021,7 @@
       </c>
       <c r="P397" s="12" t="inlineStr">
         <is>
-          <t>Draft Kings</t>
+          <t>DraftKings</t>
         </is>
       </c>
       <c r="Q397" s="12" t="n"/>
@@ -28226,7 +28226,7 @@
       </c>
       <c r="P416" s="17" t="inlineStr">
         <is>
-          <t>Draft Kings</t>
+          <t>DraftKings</t>
         </is>
       </c>
       <c r="Q416" s="17" t="n"/>
@@ -28734,7 +28734,7 @@
       </c>
       <c r="P424" s="17" t="inlineStr">
         <is>
-          <t>Draft Kings</t>
+          <t>DraftKings</t>
         </is>
       </c>
       <c r="Q424" s="17" t="n"/>
@@ -29112,7 +29112,7 @@
       </c>
       <c r="P430" s="17" t="inlineStr">
         <is>
-          <t>Draft Kings</t>
+          <t>DraftKings</t>
         </is>
       </c>
       <c r="Q430" s="17" t="n"/>
@@ -29746,7 +29746,7 @@
       </c>
       <c r="P440" s="17" t="inlineStr">
         <is>
-          <t>Draft Kings</t>
+          <t>DraftKings</t>
         </is>
       </c>
       <c r="Q440" s="17" t="n"/>
@@ -30699,7 +30699,7 @@
       </c>
       <c r="P455" s="12" t="inlineStr">
         <is>
-          <t>Draft Kings</t>
+          <t>DraftKings</t>
         </is>
       </c>
       <c r="Q455" s="12" t="n"/>
@@ -32806,7 +32806,7 @@
       </c>
       <c r="P488" s="17" t="inlineStr">
         <is>
-          <t>Draft Kings</t>
+          <t>DraftKings</t>
         </is>
       </c>
       <c r="Q488" s="17" t="n"/>
@@ -33885,7 +33885,7 @@
       </c>
       <c r="P505" s="12" t="inlineStr">
         <is>
-          <t>Draft Kings</t>
+          <t>DraftKings</t>
         </is>
       </c>
       <c r="Q505" s="12" t="n"/>
@@ -34145,7 +34145,7 @@
       </c>
       <c r="P509" s="12" t="inlineStr">
         <is>
-          <t>Draft Kings</t>
+          <t>DraftKings</t>
         </is>
       </c>
       <c r="Q509" s="12" t="n"/>
@@ -34334,7 +34334,7 @@
       </c>
       <c r="P512" s="17" t="inlineStr">
         <is>
-          <t>Draft Kings</t>
+          <t>DraftKings</t>
         </is>
       </c>
       <c r="Q512" s="17" t="n"/>
@@ -36462,12 +36462,12 @@
       </c>
       <c r="B546" s="17" t="inlineStr">
         <is>
-          <t>SAC @ EMU</t>
+          <t>OHIO @ NEB</t>
         </is>
       </c>
       <c r="C546" s="17" t="inlineStr">
         <is>
-          <t>2026-08-29 22:30</t>
+          <t>2026-09-05 16:00</t>
         </is>
       </c>
       <c r="D546" s="25" t="n">
@@ -36475,22 +36475,22 @@
       </c>
       <c r="E546" s="17" t="inlineStr">
         <is>
-          <t>ATS</t>
+          <t>TOTAL</t>
         </is>
       </c>
       <c r="F546" s="17" t="inlineStr">
         <is>
-          <t>EMU -8.5</t>
+          <t>Under 47.5</t>
         </is>
       </c>
       <c r="G546" s="26" t="n">
-        <v>-8.5</v>
+        <v>47.5</v>
       </c>
       <c r="H546" s="18" t="n">
         <v>-110</v>
       </c>
       <c r="I546" s="20" t="n">
-        <v>0.3721230003683282</v>
+        <v>0.3693801307975482</v>
       </c>
       <c r="J546" s="20" t="n">
         <v>0.5</v>
@@ -36499,10 +36499,10 @@
         <v>0.5238095238095238</v>
       </c>
       <c r="L546" s="19" t="n">
-        <v>-0.1516865234411957</v>
+        <v>-0.1544293930119757</v>
       </c>
       <c r="M546" s="19" t="n">
-        <v>-0.2895833629331916</v>
+        <v>-0.2948197502955898</v>
       </c>
       <c r="N546" s="20" t="n">
         <v>0</v>
@@ -36512,7 +36512,7 @@
       </c>
       <c r="P546" s="17" t="inlineStr">
         <is>
-          <t>Draft Kings</t>
+          <t>DraftKings</t>
         </is>
       </c>
       <c r="Q546" s="17" t="n"/>
@@ -36525,35 +36525,35 @@
       </c>
       <c r="B547" s="12" t="inlineStr">
         <is>
-          <t>OHIO @ NEB</t>
+          <t>MIZ @ KU</t>
         </is>
       </c>
       <c r="C547" s="12" t="inlineStr">
         <is>
-          <t>2026-09-05 16:00</t>
+          <t>2026-09-12 00:00</t>
         </is>
       </c>
       <c r="D547" s="22" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E547" s="12" t="inlineStr">
         <is>
-          <t>TOTAL</t>
+          <t>ATS</t>
         </is>
       </c>
       <c r="F547" s="12" t="inlineStr">
         <is>
-          <t>Under 47.5</t>
+          <t>MIZ -7</t>
         </is>
       </c>
       <c r="G547" s="23" t="n">
-        <v>47.5</v>
+        <v>7</v>
       </c>
       <c r="H547" s="13" t="n">
         <v>-110</v>
       </c>
       <c r="I547" s="15" t="n">
-        <v>0.3693801307975482</v>
+        <v>0.3681981876751432</v>
       </c>
       <c r="J547" s="15" t="n">
         <v>0.5</v>
@@ -36562,13 +36562,13 @@
         <v>0.5238095238095238</v>
       </c>
       <c r="L547" s="14" t="n">
-        <v>-0.1544293930119757</v>
+        <v>-0.1556113361343806</v>
       </c>
       <c r="M547" s="14" t="n">
-        <v>-0.2948197502955898</v>
+        <v>-0.2848080826211447</v>
       </c>
       <c r="N547" s="15" t="n">
-        <v>0</v>
+        <v>0.0413</v>
       </c>
       <c r="O547" s="24" t="n">
         <v>0.45</v>
@@ -36588,35 +36588,35 @@
       </c>
       <c r="B548" s="17" t="inlineStr">
         <is>
-          <t>MIZ @ KU</t>
+          <t>TAR @ BGSU</t>
         </is>
       </c>
       <c r="C548" s="17" t="inlineStr">
         <is>
-          <t>2026-09-12 00:00</t>
+          <t>2026-09-05 16:00</t>
         </is>
       </c>
       <c r="D548" s="25" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E548" s="17" t="inlineStr">
         <is>
-          <t>ATS</t>
+          <t>TOTAL</t>
         </is>
       </c>
       <c r="F548" s="17" t="inlineStr">
         <is>
-          <t>MIZ -7</t>
+          <t>Under 47.5</t>
         </is>
       </c>
       <c r="G548" s="26" t="n">
-        <v>7</v>
+        <v>47.5</v>
       </c>
       <c r="H548" s="18" t="n">
         <v>-110</v>
       </c>
       <c r="I548" s="20" t="n">
-        <v>0.3681981876751432</v>
+        <v>0.3678350313477137</v>
       </c>
       <c r="J548" s="20" t="n">
         <v>0.5</v>
@@ -36625,13 +36625,13 @@
         <v>0.5238095238095238</v>
       </c>
       <c r="L548" s="19" t="n">
-        <v>-0.1556113361343806</v>
+        <v>-0.1559744924618102</v>
       </c>
       <c r="M548" s="19" t="n">
-        <v>-0.2848080826211447</v>
+        <v>-0.2977694856089103</v>
       </c>
       <c r="N548" s="20" t="n">
-        <v>0.0413</v>
+        <v>0</v>
       </c>
       <c r="O548" s="27" t="n">
         <v>0.45</v>
@@ -36641,7 +36641,11 @@
           <t>DraftKings</t>
         </is>
       </c>
-      <c r="Q548" s="17" t="n"/>
+      <c r="Q548" s="17" t="inlineStr">
+        <is>
+          <t>TAR isn't a full FBS participant this season — model doesn't rate them reliably</t>
+        </is>
+      </c>
     </row>
     <row r="549">
       <c r="A549" s="12" t="inlineStr">
@@ -36651,35 +36655,35 @@
       </c>
       <c r="B549" s="12" t="inlineStr">
         <is>
-          <t>TAR @ BGSU</t>
+          <t>ISU @ IOWA</t>
         </is>
       </c>
       <c r="C549" s="12" t="inlineStr">
         <is>
-          <t>2026-09-05 16:00</t>
+          <t>2026-09-12 23:30</t>
         </is>
       </c>
       <c r="D549" s="22" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E549" s="12" t="inlineStr">
         <is>
-          <t>TOTAL</t>
+          <t>ATS</t>
         </is>
       </c>
       <c r="F549" s="12" t="inlineStr">
         <is>
-          <t>Under 47.5</t>
+          <t>IOWA -11.5</t>
         </is>
       </c>
       <c r="G549" s="23" t="n">
-        <v>47.5</v>
+        <v>-11.5</v>
       </c>
       <c r="H549" s="13" t="n">
         <v>-110</v>
       </c>
       <c r="I549" s="15" t="n">
-        <v>0.3678350313477137</v>
+        <v>0.3667947019834538</v>
       </c>
       <c r="J549" s="15" t="n">
         <v>0.5</v>
@@ -36688,10 +36692,10 @@
         <v>0.5238095238095238</v>
       </c>
       <c r="L549" s="14" t="n">
-        <v>-0.1559744924618102</v>
+        <v>-0.15701482182607</v>
       </c>
       <c r="M549" s="14" t="n">
-        <v>-0.2977694856089103</v>
+        <v>-0.299755568940679</v>
       </c>
       <c r="N549" s="15" t="n">
         <v>0</v>
@@ -36704,11 +36708,7 @@
           <t>DraftKings</t>
         </is>
       </c>
-      <c r="Q549" s="12" t="inlineStr">
-        <is>
-          <t>TAR isn't a full FBS participant this season — model doesn't rate them reliably</t>
-        </is>
-      </c>
+      <c r="Q549" s="12" t="n"/>
     </row>
     <row r="550">
       <c r="A550" s="17" t="inlineStr">
@@ -36718,16 +36718,16 @@
       </c>
       <c r="B550" s="17" t="inlineStr">
         <is>
-          <t>ISU @ IOWA</t>
+          <t>MICH @ OSU</t>
         </is>
       </c>
       <c r="C550" s="17" t="inlineStr">
         <is>
-          <t>2026-09-12 23:30</t>
+          <t>2026-11-28 17:00</t>
         </is>
       </c>
       <c r="D550" s="25" t="n">
-        <v>2</v>
+        <v>13</v>
       </c>
       <c r="E550" s="17" t="inlineStr">
         <is>
@@ -36736,17 +36736,17 @@
       </c>
       <c r="F550" s="17" t="inlineStr">
         <is>
-          <t>IOWA -11.5</t>
+          <t>OSU -13.5</t>
         </is>
       </c>
       <c r="G550" s="26" t="n">
-        <v>-11.5</v>
+        <v>-13.5</v>
       </c>
       <c r="H550" s="18" t="n">
         <v>-110</v>
       </c>
       <c r="I550" s="20" t="n">
-        <v>0.3667947019834538</v>
+        <v>0.3661416831903596</v>
       </c>
       <c r="J550" s="20" t="n">
         <v>0.5</v>
@@ -36755,10 +36755,10 @@
         <v>0.5238095238095238</v>
       </c>
       <c r="L550" s="19" t="n">
-        <v>-0.15701482182607</v>
+        <v>-0.1576678406191643</v>
       </c>
       <c r="M550" s="19" t="n">
-        <v>-0.299755568940679</v>
+        <v>-0.3010022411820408</v>
       </c>
       <c r="N550" s="20" t="n">
         <v>0</v>
@@ -36781,16 +36781,16 @@
       </c>
       <c r="B551" s="12" t="inlineStr">
         <is>
-          <t>MICH @ OSU</t>
+          <t>URI @ TEM</t>
         </is>
       </c>
       <c r="C551" s="12" t="inlineStr">
         <is>
-          <t>2026-11-28 17:00</t>
+          <t>2026-09-05 18:00</t>
         </is>
       </c>
       <c r="D551" s="22" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="E551" s="12" t="inlineStr">
         <is>
@@ -36799,17 +36799,17 @@
       </c>
       <c r="F551" s="12" t="inlineStr">
         <is>
-          <t>OSU -13.5</t>
+          <t>TEM -10</t>
         </is>
       </c>
       <c r="G551" s="23" t="n">
-        <v>-13.5</v>
+        <v>-10</v>
       </c>
       <c r="H551" s="13" t="n">
         <v>-110</v>
       </c>
       <c r="I551" s="15" t="n">
-        <v>0.3661416831903596</v>
+        <v>0.366118766727385</v>
       </c>
       <c r="J551" s="15" t="n">
         <v>0.5</v>
@@ -36818,13 +36818,13 @@
         <v>0.5238095238095238</v>
       </c>
       <c r="L551" s="14" t="n">
-        <v>-0.1576678406191643</v>
+        <v>-0.1576907570821388</v>
       </c>
       <c r="M551" s="14" t="n">
-        <v>-0.3010022411820408</v>
+        <v>-0.2910516696595741</v>
       </c>
       <c r="N551" s="15" t="n">
-        <v>0</v>
+        <v>0.0332</v>
       </c>
       <c r="O551" s="24" t="n">
         <v>0.45</v>
@@ -36834,7 +36834,11 @@
           <t>DraftKings</t>
         </is>
       </c>
-      <c r="Q551" s="12" t="n"/>
+      <c r="Q551" s="12" t="inlineStr">
+        <is>
+          <t>URI isn't a full FBS participant this season — model doesn't rate them reliably</t>
+        </is>
+      </c>
     </row>
     <row r="552">
       <c r="A552" s="17" t="inlineStr">
@@ -36844,16 +36848,16 @@
       </c>
       <c r="B552" s="17" t="inlineStr">
         <is>
-          <t>URI @ TEM</t>
+          <t>HOU @ TTU</t>
         </is>
       </c>
       <c r="C552" s="17" t="inlineStr">
         <is>
-          <t>2026-09-05 18:00</t>
+          <t>2026-09-19 00:00</t>
         </is>
       </c>
       <c r="D552" s="25" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E552" s="17" t="inlineStr">
         <is>
@@ -36862,17 +36866,17 @@
       </c>
       <c r="F552" s="17" t="inlineStr">
         <is>
-          <t>TEM -10</t>
+          <t>TTU -13.5</t>
         </is>
       </c>
       <c r="G552" s="26" t="n">
-        <v>-10</v>
+        <v>-13.5</v>
       </c>
       <c r="H552" s="18" t="n">
         <v>-110</v>
       </c>
       <c r="I552" s="20" t="n">
-        <v>0.366118766727385</v>
+        <v>0.3658031010190383</v>
       </c>
       <c r="J552" s="20" t="n">
         <v>0.5</v>
@@ -36881,13 +36885,13 @@
         <v>0.5238095238095238</v>
       </c>
       <c r="L552" s="19" t="n">
-        <v>-0.1576907570821388</v>
+        <v>-0.1580064227904855</v>
       </c>
       <c r="M552" s="19" t="n">
-        <v>-0.2910516696595741</v>
+        <v>-0.3016486253272904</v>
       </c>
       <c r="N552" s="20" t="n">
-        <v>0.0332</v>
+        <v>0</v>
       </c>
       <c r="O552" s="27" t="n">
         <v>0.45</v>
@@ -36897,11 +36901,7 @@
           <t>DraftKings</t>
         </is>
       </c>
-      <c r="Q552" s="17" t="inlineStr">
-        <is>
-          <t>URI isn't a full FBS participant this season — model doesn't rate them reliably</t>
-        </is>
-      </c>
+      <c r="Q552" s="17" t="n"/>
     </row>
     <row r="553">
       <c r="A553" s="12" t="inlineStr">
@@ -36911,16 +36911,16 @@
       </c>
       <c r="B553" s="12" t="inlineStr">
         <is>
-          <t>HOU @ TTU</t>
+          <t>FIU @ USF</t>
         </is>
       </c>
       <c r="C553" s="12" t="inlineStr">
         <is>
-          <t>2026-09-19 00:00</t>
+          <t>2026-09-05 23:00</t>
         </is>
       </c>
       <c r="D553" s="22" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E553" s="12" t="inlineStr">
         <is>
@@ -36929,7 +36929,7 @@
       </c>
       <c r="F553" s="12" t="inlineStr">
         <is>
-          <t>TTU -13.5</t>
+          <t>USF -13.5</t>
         </is>
       </c>
       <c r="G553" s="23" t="n">
@@ -36939,7 +36939,7 @@
         <v>-110</v>
       </c>
       <c r="I553" s="15" t="n">
-        <v>0.3658031010190383</v>
+        <v>0.3633379740537891</v>
       </c>
       <c r="J553" s="15" t="n">
         <v>0.5</v>
@@ -36948,10 +36948,10 @@
         <v>0.5238095238095238</v>
       </c>
       <c r="L553" s="14" t="n">
-        <v>-0.1580064227904855</v>
+        <v>-0.1604715497557347</v>
       </c>
       <c r="M553" s="14" t="n">
-        <v>-0.3016486253272904</v>
+        <v>-0.3063547768064026</v>
       </c>
       <c r="N553" s="15" t="n">
         <v>0</v>
@@ -36974,12 +36974,12 @@
       </c>
       <c r="B554" s="17" t="inlineStr">
         <is>
-          <t>FIU @ USF</t>
+          <t>SAC @ EMU</t>
         </is>
       </c>
       <c r="C554" s="17" t="inlineStr">
         <is>
-          <t>2026-09-05 23:00</t>
+          <t>2026-08-29 22:30</t>
         </is>
       </c>
       <c r="D554" s="25" t="n">
@@ -36992,17 +36992,17 @@
       </c>
       <c r="F554" s="17" t="inlineStr">
         <is>
-          <t>USF -13.5</t>
+          <t>EMU -9.5</t>
         </is>
       </c>
       <c r="G554" s="26" t="n">
-        <v>-13.5</v>
+        <v>-9.5</v>
       </c>
       <c r="H554" s="18" t="n">
         <v>-110</v>
       </c>
       <c r="I554" s="20" t="n">
-        <v>0.3633379740537891</v>
+        <v>0.3626957910893782</v>
       </c>
       <c r="J554" s="20" t="n">
         <v>0.5</v>
@@ -37011,10 +37011,10 @@
         <v>0.5238095238095238</v>
       </c>
       <c r="L554" s="19" t="n">
-        <v>-0.1604715497557347</v>
+        <v>-0.1611137327201456</v>
       </c>
       <c r="M554" s="19" t="n">
-        <v>-0.3063547768064026</v>
+        <v>-0.3075807624657325</v>
       </c>
       <c r="N554" s="20" t="n">
         <v>0</v>
@@ -37993,7 +37993,7 @@
       </c>
       <c r="P569" s="12" t="inlineStr">
         <is>
-          <t>Draft Kings</t>
+          <t>DraftKings</t>
         </is>
       </c>
       <c r="Q569" s="12" t="n"/>
@@ -41601,7 +41601,7 @@
       </c>
       <c r="P625" s="12" t="inlineStr">
         <is>
-          <t>Draft Kings</t>
+          <t>DraftKings</t>
         </is>
       </c>
       <c r="Q625" s="12" t="n"/>
@@ -41928,7 +41928,7 @@
       </c>
       <c r="P630" s="17" t="inlineStr">
         <is>
-          <t>Draft Kings</t>
+          <t>DraftKings</t>
         </is>
       </c>
       <c r="Q630" s="17" t="n"/>
@@ -53377,7 +53377,7 @@
       <c r="L5" s="13" t="n"/>
       <c r="M5" s="12" t="inlineStr">
         <is>
-          <t>Draft Kings</t>
+          <t>DraftKings</t>
         </is>
       </c>
     </row>
@@ -53422,7 +53422,7 @@
       <c r="L6" s="18" t="n"/>
       <c r="M6" s="17" t="inlineStr">
         <is>
-          <t>Draft Kings</t>
+          <t>DraftKings</t>
         </is>
       </c>
     </row>
@@ -53467,7 +53467,7 @@
       <c r="L7" s="13" t="n"/>
       <c r="M7" s="12" t="inlineStr">
         <is>
-          <t>Draft Kings</t>
+          <t>DraftKings</t>
         </is>
       </c>
     </row>
@@ -53512,7 +53512,7 @@
       <c r="L8" s="18" t="n"/>
       <c r="M8" s="17" t="inlineStr">
         <is>
-          <t>Draft Kings</t>
+          <t>DraftKings</t>
         </is>
       </c>
     </row>
@@ -53548,7 +53548,7 @@
       </c>
       <c r="H9" s="12" t="inlineStr"/>
       <c r="I9" s="23" t="n">
-        <v>-8.5</v>
+        <v>-9.5</v>
       </c>
       <c r="J9" s="29" t="n">
         <v>52.5</v>
@@ -53557,7 +53557,7 @@
       <c r="L9" s="13" t="n"/>
       <c r="M9" s="12" t="inlineStr">
         <is>
-          <t>Draft Kings</t>
+          <t>DraftKings</t>
         </is>
       </c>
     </row>
@@ -53602,7 +53602,7 @@
       <c r="L10" s="18" t="n"/>
       <c r="M10" s="17" t="inlineStr">
         <is>
-          <t>Draft Kings</t>
+          <t>DraftKings</t>
         </is>
       </c>
     </row>
@@ -53647,7 +53647,7 @@
       <c r="L11" s="13" t="n"/>
       <c r="M11" s="12" t="inlineStr">
         <is>
-          <t>Draft Kings</t>
+          <t>DraftKings</t>
         </is>
       </c>
     </row>
@@ -53692,7 +53692,7 @@
       <c r="L12" s="18" t="n"/>
       <c r="M12" s="17" t="inlineStr">
         <is>
-          <t>Draft Kings</t>
+          <t>DraftKings</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
refresh 2026-08-23 21:44 UTC
</commit_message>
<xml_diff>
--- a/NCAAF_Edge_Model.xlsx
+++ b/NCAAF_Edge_Model.xlsx
@@ -638,7 +638,7 @@
     <row r="2" ht="26" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-08-23T19:08:04+00:00 from live ESPN data. This file is a snapshot, not the model. Re-run the pipeline to refresh it.</t>
+          <t>Generated 2026-08-23T21:44:22+00:00 from live ESPN data. This file is a snapshot, not the model. Re-run the pipeline to refresh it.</t>
         </is>
       </c>
     </row>
@@ -1168,11 +1168,11 @@
         <v>0</v>
       </c>
       <c r="O5" s="18" t="n">
-        <v>0.375</v>
+        <v>0.4125</v>
       </c>
       <c r="P5" s="12" t="inlineStr">
         <is>
-          <t>Draft Kings</t>
+          <t>DraftKings</t>
         </is>
       </c>
       <c r="Q5" s="12" t="inlineStr">
@@ -1235,11 +1235,11 @@
         <v>0</v>
       </c>
       <c r="O6" s="25" t="n">
-        <v>0.375</v>
+        <v>0.4125</v>
       </c>
       <c r="P6" s="19" t="inlineStr">
         <is>
-          <t>Draft Kings</t>
+          <t>DraftKings</t>
         </is>
       </c>
       <c r="Q6" s="19" t="inlineStr">
@@ -1300,11 +1300,11 @@
         <v>0</v>
       </c>
       <c r="O7" s="18" t="n">
-        <v>0.375</v>
+        <v>0.4125</v>
       </c>
       <c r="P7" s="12" t="inlineStr">
         <is>
-          <t>Draft Kings</t>
+          <t>DraftKings</t>
         </is>
       </c>
       <c r="Q7" s="12" t="inlineStr">
@@ -1367,11 +1367,11 @@
         <v>0</v>
       </c>
       <c r="O8" s="25" t="n">
-        <v>0.375</v>
+        <v>0.4125</v>
       </c>
       <c r="P8" s="19" t="inlineStr">
         <is>
-          <t>Draft Kings</t>
+          <t>DraftKings</t>
         </is>
       </c>
       <c r="Q8" s="19" t="inlineStr">
@@ -1434,11 +1434,11 @@
         <v>0</v>
       </c>
       <c r="O9" s="18" t="n">
-        <v>0.375</v>
+        <v>0.4125</v>
       </c>
       <c r="P9" s="12" t="inlineStr">
         <is>
-          <t>Draft Kings</t>
+          <t>DraftKings</t>
         </is>
       </c>
       <c r="Q9" s="12" t="inlineStr">
@@ -1499,11 +1499,11 @@
         <v>0</v>
       </c>
       <c r="O10" s="25" t="n">
-        <v>0.375</v>
+        <v>0.4125</v>
       </c>
       <c r="P10" s="19" t="inlineStr">
         <is>
-          <t>Draft Kings</t>
+          <t>DraftKings</t>
         </is>
       </c>
       <c r="Q10" s="19" t="inlineStr">
@@ -1566,11 +1566,11 @@
         <v>0</v>
       </c>
       <c r="O11" s="18" t="n">
-        <v>0.375</v>
+        <v>0.4125</v>
       </c>
       <c r="P11" s="12" t="inlineStr">
         <is>
-          <t>Draft Kings</t>
+          <t>DraftKings</t>
         </is>
       </c>
       <c r="Q11" s="12" t="inlineStr">
@@ -1633,11 +1633,11 @@
         <v>0</v>
       </c>
       <c r="O12" s="25" t="n">
-        <v>0.375</v>
+        <v>0.4125</v>
       </c>
       <c r="P12" s="19" t="inlineStr">
         <is>
-          <t>Draft Kings</t>
+          <t>DraftKings</t>
         </is>
       </c>
       <c r="Q12" s="19" t="inlineStr">
@@ -1698,11 +1698,11 @@
         <v>0</v>
       </c>
       <c r="O13" s="18" t="n">
-        <v>0.375</v>
+        <v>0.4125</v>
       </c>
       <c r="P13" s="12" t="inlineStr">
         <is>
-          <t>Draft Kings</t>
+          <t>DraftKings</t>
         </is>
       </c>
       <c r="Q13" s="12" t="n"/>
@@ -1761,11 +1761,11 @@
         <v>0</v>
       </c>
       <c r="O14" s="25" t="n">
-        <v>0.375</v>
+        <v>0.4125</v>
       </c>
       <c r="P14" s="19" t="inlineStr">
         <is>
-          <t>Draft Kings</t>
+          <t>DraftKings</t>
         </is>
       </c>
       <c r="Q14" s="19" t="inlineStr">
@@ -1826,11 +1826,11 @@
         <v>0</v>
       </c>
       <c r="O15" s="18" t="n">
-        <v>0.375</v>
+        <v>0.4125</v>
       </c>
       <c r="P15" s="12" t="inlineStr">
         <is>
-          <t>Draft Kings</t>
+          <t>DraftKings</t>
         </is>
       </c>
       <c r="Q15" s="12" t="n"/>
@@ -1889,11 +1889,11 @@
         <v>0</v>
       </c>
       <c r="O16" s="25" t="n">
-        <v>0.375</v>
+        <v>0.4125</v>
       </c>
       <c r="P16" s="19" t="inlineStr">
         <is>
-          <t>Draft Kings</t>
+          <t>DraftKings</t>
         </is>
       </c>
       <c r="Q16" s="19" t="n"/>
@@ -1950,11 +1950,11 @@
         <v>0</v>
       </c>
       <c r="O17" s="18" t="n">
-        <v>0.375</v>
+        <v>0.4125</v>
       </c>
       <c r="P17" s="12" t="inlineStr">
         <is>
-          <t>Draft Kings</t>
+          <t>DraftKings</t>
         </is>
       </c>
       <c r="Q17" s="12" t="n"/>
@@ -2013,11 +2013,11 @@
         <v>0</v>
       </c>
       <c r="O18" s="25" t="n">
-        <v>0.375</v>
+        <v>0.4125</v>
       </c>
       <c r="P18" s="19" t="inlineStr">
         <is>
-          <t>Draft Kings</t>
+          <t>DraftKings</t>
         </is>
       </c>
       <c r="Q18" s="19" t="n"/>
@@ -2076,11 +2076,11 @@
         <v>0</v>
       </c>
       <c r="O19" s="18" t="n">
-        <v>0.375</v>
+        <v>0.4125</v>
       </c>
       <c r="P19" s="12" t="inlineStr">
         <is>
-          <t>Draft Kings</t>
+          <t>DraftKings</t>
         </is>
       </c>
       <c r="Q19" s="12" t="n"/>
@@ -2139,11 +2139,11 @@
         <v>0.0505</v>
       </c>
       <c r="O20" s="25" t="n">
-        <v>0.375</v>
+        <v>0.4125</v>
       </c>
       <c r="P20" s="19" t="inlineStr">
         <is>
-          <t>Draft Kings</t>
+          <t>DraftKings</t>
         </is>
       </c>
       <c r="Q20" s="19" t="n"/>
@@ -2202,11 +2202,11 @@
         <v>0</v>
       </c>
       <c r="O21" s="18" t="n">
-        <v>0.375</v>
+        <v>0.4125</v>
       </c>
       <c r="P21" s="12" t="inlineStr">
         <is>
-          <t>Draft Kings</t>
+          <t>DraftKings</t>
         </is>
       </c>
       <c r="Q21" s="12" t="n"/>
@@ -2263,11 +2263,11 @@
         <v>0</v>
       </c>
       <c r="O22" s="25" t="n">
-        <v>0.375</v>
+        <v>0.4125</v>
       </c>
       <c r="P22" s="19" t="inlineStr">
         <is>
-          <t>Draft Kings</t>
+          <t>DraftKings</t>
         </is>
       </c>
       <c r="Q22" s="19" t="n"/>
@@ -2326,11 +2326,11 @@
         <v>0</v>
       </c>
       <c r="O23" s="18" t="n">
-        <v>0.375</v>
+        <v>0.4125</v>
       </c>
       <c r="P23" s="12" t="inlineStr">
         <is>
-          <t>Draft Kings</t>
+          <t>DraftKings</t>
         </is>
       </c>
       <c r="Q23" s="12" t="n"/>
@@ -2387,11 +2387,11 @@
         <v>0</v>
       </c>
       <c r="O24" s="25" t="n">
-        <v>0.375</v>
+        <v>0.4125</v>
       </c>
       <c r="P24" s="19" t="inlineStr">
         <is>
-          <t>Draft Kings</t>
+          <t>DraftKings</t>
         </is>
       </c>
       <c r="Q24" s="19" t="n"/>
@@ -2450,11 +2450,11 @@
         <v>0</v>
       </c>
       <c r="O25" s="18" t="n">
-        <v>0.375</v>
+        <v>0.4125</v>
       </c>
       <c r="P25" s="12" t="inlineStr">
         <is>
-          <t>Draft Kings</t>
+          <t>DraftKings</t>
         </is>
       </c>
       <c r="Q25" s="12" t="n"/>
@@ -2513,11 +2513,11 @@
         <v>0</v>
       </c>
       <c r="O26" s="25" t="n">
-        <v>0.375</v>
+        <v>0.4125</v>
       </c>
       <c r="P26" s="19" t="inlineStr">
         <is>
-          <t>Draft Kings</t>
+          <t>DraftKings</t>
         </is>
       </c>
       <c r="Q26" s="19" t="n"/>
@@ -2576,11 +2576,11 @@
         <v>0</v>
       </c>
       <c r="O27" s="18" t="n">
-        <v>0.375</v>
+        <v>0.4125</v>
       </c>
       <c r="P27" s="12" t="inlineStr">
         <is>
-          <t>Draft Kings</t>
+          <t>DraftKings</t>
         </is>
       </c>
       <c r="Q27" s="12" t="n"/>
@@ -2639,11 +2639,11 @@
         <v>0</v>
       </c>
       <c r="O28" s="25" t="n">
-        <v>0.375</v>
+        <v>0.4125</v>
       </c>
       <c r="P28" s="19" t="inlineStr">
         <is>
-          <t>Draft Kings</t>
+          <t>DraftKings</t>
         </is>
       </c>
       <c r="Q28" s="19" t="n"/>
@@ -2702,11 +2702,11 @@
         <v>0</v>
       </c>
       <c r="O29" s="18" t="n">
-        <v>0.375</v>
+        <v>0.4125</v>
       </c>
       <c r="P29" s="12" t="inlineStr">
         <is>
-          <t>Draft Kings</t>
+          <t>DraftKings</t>
         </is>
       </c>
       <c r="Q29" s="12" t="n"/>
@@ -2765,11 +2765,11 @@
         <v>0</v>
       </c>
       <c r="O30" s="25" t="n">
-        <v>0.375</v>
+        <v>0.4125</v>
       </c>
       <c r="P30" s="19" t="inlineStr">
         <is>
-          <t>Draft Kings</t>
+          <t>DraftKings</t>
         </is>
       </c>
       <c r="Q30" s="19" t="n"/>
@@ -2826,11 +2826,11 @@
         <v>0</v>
       </c>
       <c r="O31" s="18" t="n">
-        <v>0.375</v>
+        <v>0.4125</v>
       </c>
       <c r="P31" s="12" t="inlineStr">
         <is>
-          <t>Draft Kings</t>
+          <t>DraftKings</t>
         </is>
       </c>
       <c r="Q31" s="12" t="n"/>
@@ -2887,11 +2887,11 @@
         <v>0</v>
       </c>
       <c r="O32" s="25" t="n">
-        <v>0.375</v>
+        <v>0.4125</v>
       </c>
       <c r="P32" s="19" t="inlineStr">
         <is>
-          <t>Draft Kings</t>
+          <t>DraftKings</t>
         </is>
       </c>
       <c r="Q32" s="19" t="n"/>
@@ -2950,11 +2950,11 @@
         <v>0</v>
       </c>
       <c r="O33" s="18" t="n">
-        <v>0.375</v>
+        <v>0.4125</v>
       </c>
       <c r="P33" s="12" t="inlineStr">
         <is>
-          <t>Draft Kings</t>
+          <t>DraftKings</t>
         </is>
       </c>
       <c r="Q33" s="12" t="n"/>
@@ -3013,11 +3013,11 @@
         <v>0</v>
       </c>
       <c r="O34" s="25" t="n">
-        <v>0.375</v>
+        <v>0.4125</v>
       </c>
       <c r="P34" s="19" t="inlineStr">
         <is>
-          <t>Draft Kings</t>
+          <t>DraftKings</t>
         </is>
       </c>
       <c r="Q34" s="19" t="n"/>
@@ -3076,11 +3076,11 @@
         <v>0.0505</v>
       </c>
       <c r="O35" s="18" t="n">
-        <v>0.375</v>
+        <v>0.4125</v>
       </c>
       <c r="P35" s="12" t="inlineStr">
         <is>
-          <t>Draft Kings</t>
+          <t>DraftKings</t>
         </is>
       </c>
       <c r="Q35" s="12" t="n"/>
@@ -3139,11 +3139,11 @@
         <v>0</v>
       </c>
       <c r="O36" s="25" t="n">
-        <v>0.375</v>
+        <v>0.4125</v>
       </c>
       <c r="P36" s="19" t="inlineStr">
         <is>
-          <t>Draft Kings</t>
+          <t>DraftKings</t>
         </is>
       </c>
       <c r="Q36" s="19" t="n"/>
@@ -3200,11 +3200,11 @@
         <v>0</v>
       </c>
       <c r="O37" s="18" t="n">
-        <v>0.375</v>
+        <v>0.4125</v>
       </c>
       <c r="P37" s="12" t="inlineStr">
         <is>
-          <t>Draft Kings</t>
+          <t>DraftKings</t>
         </is>
       </c>
       <c r="Q37" s="12" t="n"/>
@@ -3263,11 +3263,11 @@
         <v>0</v>
       </c>
       <c r="O38" s="25" t="n">
-        <v>0.375</v>
+        <v>0.4125</v>
       </c>
       <c r="P38" s="19" t="inlineStr">
         <is>
-          <t>Draft Kings</t>
+          <t>DraftKings</t>
         </is>
       </c>
       <c r="Q38" s="19" t="n"/>
@@ -3324,11 +3324,11 @@
         <v>0</v>
       </c>
       <c r="O39" s="18" t="n">
-        <v>0.375</v>
+        <v>0.4125</v>
       </c>
       <c r="P39" s="12" t="inlineStr">
         <is>
-          <t>Draft Kings</t>
+          <t>DraftKings</t>
         </is>
       </c>
       <c r="Q39" s="12" t="n"/>
@@ -3387,11 +3387,11 @@
         <v>0</v>
       </c>
       <c r="O40" s="25" t="n">
-        <v>0.375</v>
+        <v>0.4125</v>
       </c>
       <c r="P40" s="19" t="inlineStr">
         <is>
-          <t>Draft Kings</t>
+          <t>DraftKings</t>
         </is>
       </c>
       <c r="Q40" s="19" t="n"/>
@@ -3448,11 +3448,11 @@
         <v>0</v>
       </c>
       <c r="O41" s="18" t="n">
-        <v>0.375</v>
+        <v>0.4125</v>
       </c>
       <c r="P41" s="12" t="inlineStr">
         <is>
-          <t>Draft Kings</t>
+          <t>DraftKings</t>
         </is>
       </c>
       <c r="Q41" s="12" t="n"/>
@@ -3511,11 +3511,11 @@
         <v>0</v>
       </c>
       <c r="O42" s="25" t="n">
-        <v>0.375</v>
+        <v>0.4125</v>
       </c>
       <c r="P42" s="19" t="inlineStr">
         <is>
-          <t>Draft Kings</t>
+          <t>DraftKings</t>
         </is>
       </c>
       <c r="Q42" s="19" t="inlineStr">
@@ -3578,11 +3578,11 @@
         <v>0</v>
       </c>
       <c r="O43" s="18" t="n">
-        <v>0.375</v>
+        <v>0.4125</v>
       </c>
       <c r="P43" s="12" t="inlineStr">
         <is>
-          <t>Draft Kings</t>
+          <t>DraftKings</t>
         </is>
       </c>
       <c r="Q43" s="12" t="inlineStr">
@@ -3645,11 +3645,11 @@
         <v>0</v>
       </c>
       <c r="O44" s="25" t="n">
-        <v>0.375</v>
+        <v>0.4125</v>
       </c>
       <c r="P44" s="19" t="inlineStr">
         <is>
-          <t>Draft Kings</t>
+          <t>DraftKings</t>
         </is>
       </c>
       <c r="Q44" s="19" t="inlineStr">
@@ -3710,11 +3710,11 @@
         <v>0</v>
       </c>
       <c r="O45" s="18" t="n">
-        <v>0.375</v>
+        <v>0.4125</v>
       </c>
       <c r="P45" s="12" t="inlineStr">
         <is>
-          <t>Draft Kings</t>
+          <t>DraftKings</t>
         </is>
       </c>
       <c r="Q45" s="12" t="inlineStr">
@@ -3777,11 +3777,11 @@
         <v>0</v>
       </c>
       <c r="O46" s="25" t="n">
-        <v>0.375</v>
+        <v>0.4125</v>
       </c>
       <c r="P46" s="19" t="inlineStr">
         <is>
-          <t>Draft Kings</t>
+          <t>DraftKings</t>
         </is>
       </c>
       <c r="Q46" s="19" t="inlineStr">
@@ -3844,11 +3844,11 @@
         <v>0</v>
       </c>
       <c r="O47" s="18" t="n">
-        <v>0.375</v>
+        <v>0.4125</v>
       </c>
       <c r="P47" s="12" t="inlineStr">
         <is>
-          <t>Draft Kings</t>
+          <t>DraftKings</t>
         </is>
       </c>
       <c r="Q47" s="12" t="inlineStr">
@@ -3909,11 +3909,11 @@
         <v>0</v>
       </c>
       <c r="O48" s="25" t="n">
-        <v>0.375</v>
+        <v>0.4125</v>
       </c>
       <c r="P48" s="19" t="inlineStr">
         <is>
-          <t>Draft Kings</t>
+          <t>DraftKings</t>
         </is>
       </c>
       <c r="Q48" s="19" t="inlineStr">
@@ -3976,11 +3976,11 @@
         <v>0</v>
       </c>
       <c r="O49" s="18" t="n">
-        <v>0.375</v>
+        <v>0.4125</v>
       </c>
       <c r="P49" s="12" t="inlineStr">
         <is>
-          <t>Draft Kings</t>
+          <t>DraftKings</t>
         </is>
       </c>
       <c r="Q49" s="12" t="inlineStr">
@@ -4043,11 +4043,11 @@
         <v>0</v>
       </c>
       <c r="O50" s="25" t="n">
-        <v>0.375</v>
+        <v>0.4125</v>
       </c>
       <c r="P50" s="19" t="inlineStr">
         <is>
-          <t>Draft Kings</t>
+          <t>DraftKings</t>
         </is>
       </c>
       <c r="Q50" s="19" t="inlineStr">
@@ -10797,7 +10797,7 @@
       </c>
       <c r="M5" s="12" t="inlineStr">
         <is>
-          <t>Draft Kings</t>
+          <t>DraftKings</t>
         </is>
       </c>
     </row>
@@ -10842,7 +10842,7 @@
       <c r="L6" s="22" t="n"/>
       <c r="M6" s="19" t="inlineStr">
         <is>
-          <t>Draft Kings</t>
+          <t>DraftKings</t>
         </is>
       </c>
     </row>
@@ -10891,7 +10891,7 @@
       </c>
       <c r="M7" s="12" t="inlineStr">
         <is>
-          <t>Draft Kings</t>
+          <t>DraftKings</t>
         </is>
       </c>
     </row>
@@ -10940,7 +10940,7 @@
       </c>
       <c r="M8" s="19" t="inlineStr">
         <is>
-          <t>Draft Kings</t>
+          <t>DraftKings</t>
         </is>
       </c>
     </row>
@@ -10989,7 +10989,7 @@
       </c>
       <c r="M9" s="12" t="inlineStr">
         <is>
-          <t>Draft Kings</t>
+          <t>DraftKings</t>
         </is>
       </c>
     </row>
@@ -11038,7 +11038,7 @@
       </c>
       <c r="M10" s="19" t="inlineStr">
         <is>
-          <t>Draft Kings</t>
+          <t>DraftKings</t>
         </is>
       </c>
     </row>
@@ -11087,7 +11087,7 @@
       </c>
       <c r="M11" s="12" t="inlineStr">
         <is>
-          <t>Draft Kings</t>
+          <t>DraftKings</t>
         </is>
       </c>
     </row>
@@ -11136,7 +11136,7 @@
       </c>
       <c r="M12" s="19" t="inlineStr">
         <is>
-          <t>Draft Kings</t>
+          <t>DraftKings</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
refresh 2026-08-23 22:20 UTC
</commit_message>
<xml_diff>
--- a/NCAAF_Edge_Model.xlsx
+++ b/NCAAF_Edge_Model.xlsx
@@ -638,7 +638,7 @@
     <row r="2" ht="26" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-08-23T21:44:22+00:00 from live ESPN data. This file is a snapshot, not the model. Re-run the pipeline to refresh it.</t>
+          <t>Generated 2026-08-23T22:20:07+00:00 from live ESPN data. This file is a snapshot, not the model. Re-run the pipeline to refresh it.</t>
         </is>
       </c>
     </row>
@@ -1168,11 +1168,11 @@
         <v>0</v>
       </c>
       <c r="O5" s="18" t="n">
-        <v>0.4125</v>
+        <v>0.45</v>
       </c>
       <c r="P5" s="12" t="inlineStr">
         <is>
-          <t>DraftKings</t>
+          <t>Draft Kings</t>
         </is>
       </c>
       <c r="Q5" s="12" t="inlineStr">
@@ -1235,11 +1235,11 @@
         <v>0</v>
       </c>
       <c r="O6" s="25" t="n">
-        <v>0.4125</v>
+        <v>0.45</v>
       </c>
       <c r="P6" s="19" t="inlineStr">
         <is>
-          <t>DraftKings</t>
+          <t>Draft Kings</t>
         </is>
       </c>
       <c r="Q6" s="19" t="inlineStr">
@@ -1300,11 +1300,11 @@
         <v>0</v>
       </c>
       <c r="O7" s="18" t="n">
-        <v>0.4125</v>
+        <v>0.45</v>
       </c>
       <c r="P7" s="12" t="inlineStr">
         <is>
-          <t>DraftKings</t>
+          <t>Draft Kings</t>
         </is>
       </c>
       <c r="Q7" s="12" t="inlineStr">
@@ -1367,11 +1367,11 @@
         <v>0</v>
       </c>
       <c r="O8" s="25" t="n">
-        <v>0.4125</v>
+        <v>0.45</v>
       </c>
       <c r="P8" s="19" t="inlineStr">
         <is>
-          <t>DraftKings</t>
+          <t>Draft Kings</t>
         </is>
       </c>
       <c r="Q8" s="19" t="inlineStr">
@@ -1434,11 +1434,11 @@
         <v>0</v>
       </c>
       <c r="O9" s="18" t="n">
-        <v>0.4125</v>
+        <v>0.45</v>
       </c>
       <c r="P9" s="12" t="inlineStr">
         <is>
-          <t>DraftKings</t>
+          <t>Draft Kings</t>
         </is>
       </c>
       <c r="Q9" s="12" t="inlineStr">
@@ -1499,11 +1499,11 @@
         <v>0</v>
       </c>
       <c r="O10" s="25" t="n">
-        <v>0.4125</v>
+        <v>0.45</v>
       </c>
       <c r="P10" s="19" t="inlineStr">
         <is>
-          <t>DraftKings</t>
+          <t>Draft Kings</t>
         </is>
       </c>
       <c r="Q10" s="19" t="inlineStr">
@@ -1566,11 +1566,11 @@
         <v>0</v>
       </c>
       <c r="O11" s="18" t="n">
-        <v>0.4125</v>
+        <v>0.45</v>
       </c>
       <c r="P11" s="12" t="inlineStr">
         <is>
-          <t>DraftKings</t>
+          <t>Draft Kings</t>
         </is>
       </c>
       <c r="Q11" s="12" t="inlineStr">
@@ -1633,11 +1633,11 @@
         <v>0</v>
       </c>
       <c r="O12" s="25" t="n">
-        <v>0.4125</v>
+        <v>0.45</v>
       </c>
       <c r="P12" s="19" t="inlineStr">
         <is>
-          <t>DraftKings</t>
+          <t>Draft Kings</t>
         </is>
       </c>
       <c r="Q12" s="19" t="inlineStr">
@@ -1698,11 +1698,11 @@
         <v>0</v>
       </c>
       <c r="O13" s="18" t="n">
-        <v>0.4125</v>
+        <v>0.45</v>
       </c>
       <c r="P13" s="12" t="inlineStr">
         <is>
-          <t>DraftKings</t>
+          <t>Draft Kings</t>
         </is>
       </c>
       <c r="Q13" s="12" t="n"/>
@@ -1761,11 +1761,11 @@
         <v>0</v>
       </c>
       <c r="O14" s="25" t="n">
-        <v>0.4125</v>
+        <v>0.45</v>
       </c>
       <c r="P14" s="19" t="inlineStr">
         <is>
-          <t>DraftKings</t>
+          <t>Draft Kings</t>
         </is>
       </c>
       <c r="Q14" s="19" t="inlineStr">
@@ -1826,11 +1826,11 @@
         <v>0</v>
       </c>
       <c r="O15" s="18" t="n">
-        <v>0.4125</v>
+        <v>0.45</v>
       </c>
       <c r="P15" s="12" t="inlineStr">
         <is>
-          <t>DraftKings</t>
+          <t>Draft Kings</t>
         </is>
       </c>
       <c r="Q15" s="12" t="n"/>
@@ -1889,11 +1889,11 @@
         <v>0</v>
       </c>
       <c r="O16" s="25" t="n">
-        <v>0.4125</v>
+        <v>0.45</v>
       </c>
       <c r="P16" s="19" t="inlineStr">
         <is>
-          <t>DraftKings</t>
+          <t>Draft Kings</t>
         </is>
       </c>
       <c r="Q16" s="19" t="n"/>
@@ -1950,11 +1950,11 @@
         <v>0</v>
       </c>
       <c r="O17" s="18" t="n">
-        <v>0.4125</v>
+        <v>0.45</v>
       </c>
       <c r="P17" s="12" t="inlineStr">
         <is>
-          <t>DraftKings</t>
+          <t>Draft Kings</t>
         </is>
       </c>
       <c r="Q17" s="12" t="n"/>
@@ -2013,11 +2013,11 @@
         <v>0</v>
       </c>
       <c r="O18" s="25" t="n">
-        <v>0.4125</v>
+        <v>0.45</v>
       </c>
       <c r="P18" s="19" t="inlineStr">
         <is>
-          <t>DraftKings</t>
+          <t>Draft Kings</t>
         </is>
       </c>
       <c r="Q18" s="19" t="n"/>
@@ -2076,11 +2076,11 @@
         <v>0</v>
       </c>
       <c r="O19" s="18" t="n">
-        <v>0.4125</v>
+        <v>0.45</v>
       </c>
       <c r="P19" s="12" t="inlineStr">
         <is>
-          <t>DraftKings</t>
+          <t>Draft Kings</t>
         </is>
       </c>
       <c r="Q19" s="12" t="n"/>
@@ -2139,11 +2139,11 @@
         <v>0.0505</v>
       </c>
       <c r="O20" s="25" t="n">
-        <v>0.4125</v>
+        <v>0.45</v>
       </c>
       <c r="P20" s="19" t="inlineStr">
         <is>
-          <t>DraftKings</t>
+          <t>Draft Kings</t>
         </is>
       </c>
       <c r="Q20" s="19" t="n"/>
@@ -2202,11 +2202,11 @@
         <v>0</v>
       </c>
       <c r="O21" s="18" t="n">
-        <v>0.4125</v>
+        <v>0.45</v>
       </c>
       <c r="P21" s="12" t="inlineStr">
         <is>
-          <t>DraftKings</t>
+          <t>Draft Kings</t>
         </is>
       </c>
       <c r="Q21" s="12" t="n"/>
@@ -2263,11 +2263,11 @@
         <v>0</v>
       </c>
       <c r="O22" s="25" t="n">
-        <v>0.4125</v>
+        <v>0.45</v>
       </c>
       <c r="P22" s="19" t="inlineStr">
         <is>
-          <t>DraftKings</t>
+          <t>Draft Kings</t>
         </is>
       </c>
       <c r="Q22" s="19" t="n"/>
@@ -2326,11 +2326,11 @@
         <v>0</v>
       </c>
       <c r="O23" s="18" t="n">
-        <v>0.4125</v>
+        <v>0.45</v>
       </c>
       <c r="P23" s="12" t="inlineStr">
         <is>
-          <t>DraftKings</t>
+          <t>Draft Kings</t>
         </is>
       </c>
       <c r="Q23" s="12" t="n"/>
@@ -2387,11 +2387,11 @@
         <v>0</v>
       </c>
       <c r="O24" s="25" t="n">
-        <v>0.4125</v>
+        <v>0.45</v>
       </c>
       <c r="P24" s="19" t="inlineStr">
         <is>
-          <t>DraftKings</t>
+          <t>Draft Kings</t>
         </is>
       </c>
       <c r="Q24" s="19" t="n"/>
@@ -2450,11 +2450,11 @@
         <v>0</v>
       </c>
       <c r="O25" s="18" t="n">
-        <v>0.4125</v>
+        <v>0.45</v>
       </c>
       <c r="P25" s="12" t="inlineStr">
         <is>
-          <t>DraftKings</t>
+          <t>Draft Kings</t>
         </is>
       </c>
       <c r="Q25" s="12" t="n"/>
@@ -2513,11 +2513,11 @@
         <v>0</v>
       </c>
       <c r="O26" s="25" t="n">
-        <v>0.4125</v>
+        <v>0.45</v>
       </c>
       <c r="P26" s="19" t="inlineStr">
         <is>
-          <t>DraftKings</t>
+          <t>Draft Kings</t>
         </is>
       </c>
       <c r="Q26" s="19" t="n"/>
@@ -2576,11 +2576,11 @@
         <v>0</v>
       </c>
       <c r="O27" s="18" t="n">
-        <v>0.4125</v>
+        <v>0.45</v>
       </c>
       <c r="P27" s="12" t="inlineStr">
         <is>
-          <t>DraftKings</t>
+          <t>Draft Kings</t>
         </is>
       </c>
       <c r="Q27" s="12" t="n"/>
@@ -2639,11 +2639,11 @@
         <v>0</v>
       </c>
       <c r="O28" s="25" t="n">
-        <v>0.4125</v>
+        <v>0.45</v>
       </c>
       <c r="P28" s="19" t="inlineStr">
         <is>
-          <t>DraftKings</t>
+          <t>Draft Kings</t>
         </is>
       </c>
       <c r="Q28" s="19" t="n"/>
@@ -2702,11 +2702,11 @@
         <v>0</v>
       </c>
       <c r="O29" s="18" t="n">
-        <v>0.4125</v>
+        <v>0.45</v>
       </c>
       <c r="P29" s="12" t="inlineStr">
         <is>
-          <t>DraftKings</t>
+          <t>Draft Kings</t>
         </is>
       </c>
       <c r="Q29" s="12" t="n"/>
@@ -2765,11 +2765,11 @@
         <v>0</v>
       </c>
       <c r="O30" s="25" t="n">
-        <v>0.4125</v>
+        <v>0.45</v>
       </c>
       <c r="P30" s="19" t="inlineStr">
         <is>
-          <t>DraftKings</t>
+          <t>Draft Kings</t>
         </is>
       </c>
       <c r="Q30" s="19" t="n"/>
@@ -2826,11 +2826,11 @@
         <v>0</v>
       </c>
       <c r="O31" s="18" t="n">
-        <v>0.4125</v>
+        <v>0.45</v>
       </c>
       <c r="P31" s="12" t="inlineStr">
         <is>
-          <t>DraftKings</t>
+          <t>Draft Kings</t>
         </is>
       </c>
       <c r="Q31" s="12" t="n"/>
@@ -2887,11 +2887,11 @@
         <v>0</v>
       </c>
       <c r="O32" s="25" t="n">
-        <v>0.4125</v>
+        <v>0.45</v>
       </c>
       <c r="P32" s="19" t="inlineStr">
         <is>
-          <t>DraftKings</t>
+          <t>Draft Kings</t>
         </is>
       </c>
       <c r="Q32" s="19" t="n"/>
@@ -2950,11 +2950,11 @@
         <v>0</v>
       </c>
       <c r="O33" s="18" t="n">
-        <v>0.4125</v>
+        <v>0.45</v>
       </c>
       <c r="P33" s="12" t="inlineStr">
         <is>
-          <t>DraftKings</t>
+          <t>Draft Kings</t>
         </is>
       </c>
       <c r="Q33" s="12" t="n"/>
@@ -3013,11 +3013,11 @@
         <v>0</v>
       </c>
       <c r="O34" s="25" t="n">
-        <v>0.4125</v>
+        <v>0.45</v>
       </c>
       <c r="P34" s="19" t="inlineStr">
         <is>
-          <t>DraftKings</t>
+          <t>Draft Kings</t>
         </is>
       </c>
       <c r="Q34" s="19" t="n"/>
@@ -3076,11 +3076,11 @@
         <v>0.0505</v>
       </c>
       <c r="O35" s="18" t="n">
-        <v>0.4125</v>
+        <v>0.45</v>
       </c>
       <c r="P35" s="12" t="inlineStr">
         <is>
-          <t>DraftKings</t>
+          <t>Draft Kings</t>
         </is>
       </c>
       <c r="Q35" s="12" t="n"/>
@@ -3139,11 +3139,11 @@
         <v>0</v>
       </c>
       <c r="O36" s="25" t="n">
-        <v>0.4125</v>
+        <v>0.45</v>
       </c>
       <c r="P36" s="19" t="inlineStr">
         <is>
-          <t>DraftKings</t>
+          <t>Draft Kings</t>
         </is>
       </c>
       <c r="Q36" s="19" t="n"/>
@@ -3200,11 +3200,11 @@
         <v>0</v>
       </c>
       <c r="O37" s="18" t="n">
-        <v>0.4125</v>
+        <v>0.45</v>
       </c>
       <c r="P37" s="12" t="inlineStr">
         <is>
-          <t>DraftKings</t>
+          <t>Draft Kings</t>
         </is>
       </c>
       <c r="Q37" s="12" t="n"/>
@@ -3263,11 +3263,11 @@
         <v>0</v>
       </c>
       <c r="O38" s="25" t="n">
-        <v>0.4125</v>
+        <v>0.45</v>
       </c>
       <c r="P38" s="19" t="inlineStr">
         <is>
-          <t>DraftKings</t>
+          <t>Draft Kings</t>
         </is>
       </c>
       <c r="Q38" s="19" t="n"/>
@@ -3324,11 +3324,11 @@
         <v>0</v>
       </c>
       <c r="O39" s="18" t="n">
-        <v>0.4125</v>
+        <v>0.45</v>
       </c>
       <c r="P39" s="12" t="inlineStr">
         <is>
-          <t>DraftKings</t>
+          <t>Draft Kings</t>
         </is>
       </c>
       <c r="Q39" s="12" t="n"/>
@@ -3387,11 +3387,11 @@
         <v>0</v>
       </c>
       <c r="O40" s="25" t="n">
-        <v>0.4125</v>
+        <v>0.45</v>
       </c>
       <c r="P40" s="19" t="inlineStr">
         <is>
-          <t>DraftKings</t>
+          <t>Draft Kings</t>
         </is>
       </c>
       <c r="Q40" s="19" t="n"/>
@@ -3448,11 +3448,11 @@
         <v>0</v>
       </c>
       <c r="O41" s="18" t="n">
-        <v>0.4125</v>
+        <v>0.45</v>
       </c>
       <c r="P41" s="12" t="inlineStr">
         <is>
-          <t>DraftKings</t>
+          <t>Draft Kings</t>
         </is>
       </c>
       <c r="Q41" s="12" t="n"/>
@@ -3511,11 +3511,11 @@
         <v>0</v>
       </c>
       <c r="O42" s="25" t="n">
-        <v>0.4125</v>
+        <v>0.45</v>
       </c>
       <c r="P42" s="19" t="inlineStr">
         <is>
-          <t>DraftKings</t>
+          <t>Draft Kings</t>
         </is>
       </c>
       <c r="Q42" s="19" t="inlineStr">
@@ -3578,11 +3578,11 @@
         <v>0</v>
       </c>
       <c r="O43" s="18" t="n">
-        <v>0.4125</v>
+        <v>0.45</v>
       </c>
       <c r="P43" s="12" t="inlineStr">
         <is>
-          <t>DraftKings</t>
+          <t>Draft Kings</t>
         </is>
       </c>
       <c r="Q43" s="12" t="inlineStr">
@@ -3645,11 +3645,11 @@
         <v>0</v>
       </c>
       <c r="O44" s="25" t="n">
-        <v>0.4125</v>
+        <v>0.45</v>
       </c>
       <c r="P44" s="19" t="inlineStr">
         <is>
-          <t>DraftKings</t>
+          <t>Draft Kings</t>
         </is>
       </c>
       <c r="Q44" s="19" t="inlineStr">
@@ -3710,11 +3710,11 @@
         <v>0</v>
       </c>
       <c r="O45" s="18" t="n">
-        <v>0.4125</v>
+        <v>0.45</v>
       </c>
       <c r="P45" s="12" t="inlineStr">
         <is>
-          <t>DraftKings</t>
+          <t>Draft Kings</t>
         </is>
       </c>
       <c r="Q45" s="12" t="inlineStr">
@@ -3777,11 +3777,11 @@
         <v>0</v>
       </c>
       <c r="O46" s="25" t="n">
-        <v>0.4125</v>
+        <v>0.45</v>
       </c>
       <c r="P46" s="19" t="inlineStr">
         <is>
-          <t>DraftKings</t>
+          <t>Draft Kings</t>
         </is>
       </c>
       <c r="Q46" s="19" t="inlineStr">
@@ -3844,11 +3844,11 @@
         <v>0</v>
       </c>
       <c r="O47" s="18" t="n">
-        <v>0.4125</v>
+        <v>0.45</v>
       </c>
       <c r="P47" s="12" t="inlineStr">
         <is>
-          <t>DraftKings</t>
+          <t>Draft Kings</t>
         </is>
       </c>
       <c r="Q47" s="12" t="inlineStr">
@@ -3909,11 +3909,11 @@
         <v>0</v>
       </c>
       <c r="O48" s="25" t="n">
-        <v>0.4125</v>
+        <v>0.45</v>
       </c>
       <c r="P48" s="19" t="inlineStr">
         <is>
-          <t>DraftKings</t>
+          <t>Draft Kings</t>
         </is>
       </c>
       <c r="Q48" s="19" t="inlineStr">
@@ -3976,11 +3976,11 @@
         <v>0</v>
       </c>
       <c r="O49" s="18" t="n">
-        <v>0.4125</v>
+        <v>0.45</v>
       </c>
       <c r="P49" s="12" t="inlineStr">
         <is>
-          <t>DraftKings</t>
+          <t>Draft Kings</t>
         </is>
       </c>
       <c r="Q49" s="12" t="inlineStr">
@@ -4043,11 +4043,11 @@
         <v>0</v>
       </c>
       <c r="O50" s="25" t="n">
-        <v>0.4125</v>
+        <v>0.45</v>
       </c>
       <c r="P50" s="19" t="inlineStr">
         <is>
-          <t>DraftKings</t>
+          <t>Draft Kings</t>
         </is>
       </c>
       <c r="Q50" s="19" t="inlineStr">
@@ -10797,7 +10797,7 @@
       </c>
       <c r="M5" s="12" t="inlineStr">
         <is>
-          <t>DraftKings</t>
+          <t>Draft Kings</t>
         </is>
       </c>
     </row>
@@ -10842,7 +10842,7 @@
       <c r="L6" s="22" t="n"/>
       <c r="M6" s="19" t="inlineStr">
         <is>
-          <t>DraftKings</t>
+          <t>Draft Kings</t>
         </is>
       </c>
     </row>
@@ -10891,7 +10891,7 @@
       </c>
       <c r="M7" s="12" t="inlineStr">
         <is>
-          <t>DraftKings</t>
+          <t>Draft Kings</t>
         </is>
       </c>
     </row>
@@ -10940,7 +10940,7 @@
       </c>
       <c r="M8" s="19" t="inlineStr">
         <is>
-          <t>DraftKings</t>
+          <t>Draft Kings</t>
         </is>
       </c>
     </row>
@@ -10989,7 +10989,7 @@
       </c>
       <c r="M9" s="12" t="inlineStr">
         <is>
-          <t>DraftKings</t>
+          <t>Draft Kings</t>
         </is>
       </c>
     </row>
@@ -11038,7 +11038,7 @@
       </c>
       <c r="M10" s="19" t="inlineStr">
         <is>
-          <t>DraftKings</t>
+          <t>Draft Kings</t>
         </is>
       </c>
     </row>
@@ -11087,7 +11087,7 @@
       </c>
       <c r="M11" s="12" t="inlineStr">
         <is>
-          <t>DraftKings</t>
+          <t>Draft Kings</t>
         </is>
       </c>
     </row>
@@ -11136,7 +11136,7 @@
       </c>
       <c r="M12" s="19" t="inlineStr">
         <is>
-          <t>DraftKings</t>
+          <t>Draft Kings</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
refresh 2026-08-24 15:20 UTC
</commit_message>
<xml_diff>
--- a/NCAAF_Edge_Model.xlsx
+++ b/NCAAF_Edge_Model.xlsx
@@ -640,7 +640,7 @@
     <row r="2" ht="26" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-08-24T05:24:18+00:00 from live ESPN data. This file is a snapshot, not the model. Re-run the pipeline to refresh it.</t>
+          <t>Generated 2026-08-24T15:20:51+00:00 from live ESPN data. This file is a snapshot, not the model. Re-run the pipeline to refresh it.</t>
         </is>
       </c>
     </row>
@@ -2372,22 +2372,22 @@
         <v>46.5</v>
       </c>
       <c r="H22" s="18" t="n">
-        <v>-110</v>
+        <v>-112</v>
       </c>
       <c r="I22" s="20" t="n">
-        <v>0.6553348680813179</v>
+        <v>0.6574997451163023</v>
       </c>
       <c r="J22" s="20" t="n">
-        <v>0.5</v>
+        <v>0.5043297540699688</v>
       </c>
       <c r="K22" s="20" t="n">
-        <v>0.5238095238095238</v>
+        <v>0.5283018867924528</v>
       </c>
       <c r="L22" s="19" t="n">
-        <v>0.1315253442717941</v>
+        <v>0.1291978583238494</v>
       </c>
       <c r="M22" s="19" t="n">
-        <v>0.2510938390643342</v>
+        <v>0.2445530889701435</v>
       </c>
       <c r="N22" s="20" t="n">
         <v>0</v>
@@ -2506,22 +2506,22 @@
         <v>48.5</v>
       </c>
       <c r="H24" s="18" t="n">
-        <v>-108</v>
+        <v>-105</v>
       </c>
       <c r="I24" s="20" t="n">
-        <v>0.6237538960930264</v>
+        <v>0.6205016550348365</v>
       </c>
       <c r="J24" s="20" t="n">
-        <v>0.4956702459300312</v>
+        <v>0.4891657638136511</v>
       </c>
       <c r="K24" s="20" t="n">
-        <v>0.5192307692307693</v>
+        <v>0.5121951219512195</v>
       </c>
       <c r="L24" s="19" t="n">
-        <v>0.1045231268622572</v>
+        <v>0.1083065330836169</v>
       </c>
       <c r="M24" s="19" t="n">
-        <v>0.2013037998828658</v>
+        <v>0.2114556122108712</v>
       </c>
       <c r="N24" s="20" t="n">
         <v>0</v>
@@ -3497,12 +3497,12 @@
       </c>
       <c r="B40" s="17" t="inlineStr">
         <is>
-          <t>UNC @ TCU</t>
+          <t>JVST @ NDSU</t>
         </is>
       </c>
       <c r="C40" s="17" t="inlineStr">
         <is>
-          <t>2026-08-29 16:00</t>
+          <t>2026-08-29 21:30</t>
         </is>
       </c>
       <c r="D40" s="25" t="n">
@@ -3510,34 +3510,32 @@
       </c>
       <c r="E40" s="17" t="inlineStr">
         <is>
-          <t>TOTAL</t>
+          <t>ML</t>
         </is>
       </c>
       <c r="F40" s="17" t="inlineStr">
         <is>
-          <t>Over 47.5</t>
-        </is>
-      </c>
-      <c r="G40" s="26" t="n">
-        <v>47.5</v>
-      </c>
+          <t>JVST ML</t>
+        </is>
+      </c>
+      <c r="G40" s="26" t="n"/>
       <c r="H40" s="18" t="n">
-        <v>-110</v>
+        <v>220</v>
       </c>
       <c r="I40" s="20" t="n">
-        <v>0.5376883257015108</v>
+        <v>0.3261190128306598</v>
       </c>
       <c r="J40" s="20" t="n">
-        <v>0.5</v>
+        <v>0.299837925445705</v>
       </c>
       <c r="K40" s="20" t="n">
-        <v>0.5238095238095238</v>
+        <v>0.3125</v>
       </c>
       <c r="L40" s="19" t="n">
-        <v>0.01387880189198698</v>
+        <v>0.0136190128306598</v>
       </c>
       <c r="M40" s="19" t="n">
-        <v>0.02649589452106615</v>
+        <v>0.04358084105811144</v>
       </c>
       <c r="N40" s="20" t="n">
         <v>0</v>
@@ -3560,12 +3558,12 @@
       </c>
       <c r="B41" s="12" t="inlineStr">
         <is>
-          <t>JVST @ NDSU</t>
+          <t>UNC @ TCU</t>
         </is>
       </c>
       <c r="C41" s="12" t="inlineStr">
         <is>
-          <t>2026-08-29 21:30</t>
+          <t>2026-08-29 16:00</t>
         </is>
       </c>
       <c r="D41" s="22" t="n">
@@ -3573,32 +3571,34 @@
       </c>
       <c r="E41" s="12" t="inlineStr">
         <is>
-          <t>ML</t>
+          <t>TOTAL</t>
         </is>
       </c>
       <c r="F41" s="12" t="inlineStr">
         <is>
-          <t>JVST ML</t>
-        </is>
-      </c>
-      <c r="G41" s="23" t="n"/>
+          <t>Over 47.5</t>
+        </is>
+      </c>
+      <c r="G41" s="23" t="n">
+        <v>47.5</v>
+      </c>
       <c r="H41" s="13" t="n">
-        <v>220</v>
+        <v>-112</v>
       </c>
       <c r="I41" s="15" t="n">
-        <v>0.3261190128306598</v>
+        <v>0.5398532027364953</v>
       </c>
       <c r="J41" s="15" t="n">
-        <v>0.299837925445705</v>
+        <v>0.5043297540699688</v>
       </c>
       <c r="K41" s="15" t="n">
-        <v>0.3125</v>
+        <v>0.5283018867924528</v>
       </c>
       <c r="L41" s="14" t="n">
-        <v>0.0136190128306598</v>
+        <v>0.01155131594404246</v>
       </c>
       <c r="M41" s="14" t="n">
-        <v>0.04358084105811144</v>
+        <v>0.02186499089408034</v>
       </c>
       <c r="N41" s="15" t="n">
         <v>0</v>
@@ -4060,12 +4060,12 @@
       </c>
       <c r="B49" s="12" t="inlineStr">
         <is>
-          <t>NCSU @ UVA</t>
+          <t>UNC @ TCU</t>
         </is>
       </c>
       <c r="C49" s="12" t="inlineStr">
         <is>
-          <t>2026-08-29 19:30</t>
+          <t>2026-08-29 16:00</t>
         </is>
       </c>
       <c r="D49" s="22" t="n">
@@ -4073,32 +4073,34 @@
       </c>
       <c r="E49" s="12" t="inlineStr">
         <is>
-          <t>ML</t>
+          <t>TOTAL</t>
         </is>
       </c>
       <c r="F49" s="12" t="inlineStr">
         <is>
-          <t>UVA ML</t>
-        </is>
-      </c>
-      <c r="G49" s="23" t="n"/>
+          <t>Under 47.5</t>
+        </is>
+      </c>
+      <c r="G49" s="23" t="n">
+        <v>47.5</v>
+      </c>
       <c r="H49" s="13" t="n">
-        <v>-218</v>
+        <v>-108</v>
       </c>
       <c r="I49" s="15" t="n">
-        <v>0.6254192861725905</v>
+        <v>0.4601467972635047</v>
       </c>
       <c r="J49" s="15" t="n">
-        <v>0.6574752261956054</v>
+        <v>0.4956702459300312</v>
       </c>
       <c r="K49" s="15" t="n">
-        <v>0.6855345911949685</v>
+        <v>0.5192307692307693</v>
       </c>
       <c r="L49" s="14" t="n">
-        <v>-0.06011530502237805</v>
+        <v>-0.05908397196726456</v>
       </c>
       <c r="M49" s="14" t="n">
-        <v>-0.08769113301429471</v>
+        <v>-0.1137913534184353</v>
       </c>
       <c r="N49" s="15" t="n">
         <v>0</v>
@@ -4121,12 +4123,12 @@
       </c>
       <c r="B50" s="17" t="inlineStr">
         <is>
-          <t>UNC @ TCU</t>
+          <t>NCSU @ UVA</t>
         </is>
       </c>
       <c r="C50" s="17" t="inlineStr">
         <is>
-          <t>2026-08-29 16:00</t>
+          <t>2026-08-29 19:30</t>
         </is>
       </c>
       <c r="D50" s="25" t="n">
@@ -4134,34 +4136,32 @@
       </c>
       <c r="E50" s="17" t="inlineStr">
         <is>
-          <t>TOTAL</t>
+          <t>ML</t>
         </is>
       </c>
       <c r="F50" s="17" t="inlineStr">
         <is>
-          <t>Under 47.5</t>
-        </is>
-      </c>
-      <c r="G50" s="26" t="n">
-        <v>47.5</v>
-      </c>
+          <t>UVA ML</t>
+        </is>
+      </c>
+      <c r="G50" s="26" t="n"/>
       <c r="H50" s="18" t="n">
-        <v>-110</v>
+        <v>-218</v>
       </c>
       <c r="I50" s="20" t="n">
-        <v>0.4623116742984892</v>
+        <v>0.6254192861725905</v>
       </c>
       <c r="J50" s="20" t="n">
-        <v>0.5</v>
+        <v>0.6574752261956054</v>
       </c>
       <c r="K50" s="20" t="n">
-        <v>0.5238095238095238</v>
+        <v>0.6855345911949685</v>
       </c>
       <c r="L50" s="19" t="n">
-        <v>-0.06149784951103465</v>
+        <v>-0.06011530502237805</v>
       </c>
       <c r="M50" s="19" t="n">
-        <v>-0.117404985430157</v>
+        <v>-0.08769113301429471</v>
       </c>
       <c r="N50" s="20" t="n">
         <v>0</v>
@@ -5284,22 +5284,22 @@
         <v>48.5</v>
       </c>
       <c r="H68" s="18" t="n">
-        <v>-112</v>
+        <v>-115</v>
       </c>
       <c r="I68" s="20" t="n">
-        <v>0.3762461039069736</v>
+        <v>0.3794983449651635</v>
       </c>
       <c r="J68" s="20" t="n">
-        <v>0.5043297540699688</v>
+        <v>0.5108342361863488</v>
       </c>
       <c r="K68" s="20" t="n">
-        <v>0.5283018867924528</v>
+        <v>0.5348837209302325</v>
       </c>
       <c r="L68" s="19" t="n">
-        <v>-0.1520557828854793</v>
+        <v>-0.155385375965069</v>
       </c>
       <c r="M68" s="19" t="n">
-        <v>-0.2878198747475144</v>
+        <v>-0.2905030941955639</v>
       </c>
       <c r="N68" s="20" t="n">
         <v>0</v>
@@ -5418,22 +5418,22 @@
         <v>46.5</v>
       </c>
       <c r="H70" s="18" t="n">
-        <v>-110</v>
+        <v>-108</v>
       </c>
       <c r="I70" s="20" t="n">
-        <v>0.3446651319186821</v>
+        <v>0.3425002548836977</v>
       </c>
       <c r="J70" s="20" t="n">
-        <v>0.5</v>
+        <v>0.4956702459300312</v>
       </c>
       <c r="K70" s="20" t="n">
-        <v>0.5238095238095238</v>
+        <v>0.5192307692307693</v>
       </c>
       <c r="L70" s="19" t="n">
-        <v>-0.1791443918908417</v>
+        <v>-0.1767305143470715</v>
       </c>
       <c r="M70" s="19" t="n">
-        <v>-0.3420029299734251</v>
+        <v>-0.3403698794832488</v>
       </c>
       <c r="N70" s="20" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
refresh 2026-08-24 18:03 UTC
</commit_message>
<xml_diff>
--- a/NCAAF_Edge_Model.xlsx
+++ b/NCAAF_Edge_Model.xlsx
@@ -640,7 +640,7 @@
     <row r="2" ht="26" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-08-24T15:20:51+00:00 from live ESPN data. This file is a snapshot, not the model. Re-run the pipeline to refresh it.</t>
+          <t>Generated 2026-08-24T18:03:18+00:00 from live ESPN data. This file is a snapshot, not the model. Re-run the pipeline to refresh it.</t>
         </is>
       </c>
     </row>
@@ -1036,17 +1036,17 @@
       </c>
       <c r="D22" s="17" t="inlineStr">
         <is>
-          <t>Over 49.5</t>
+          <t>Over 48.5</t>
         </is>
       </c>
       <c r="E22" s="18" t="n">
-        <v>-105</v>
+        <v>-115</v>
       </c>
       <c r="F22" s="19" t="n">
-        <v>0.08339809109262664</v>
+        <v>0.08840272575750341</v>
       </c>
       <c r="G22" s="20" t="n">
-        <v>0.5955932130438462</v>
+        <v>0.6232864466877359</v>
       </c>
       <c r="H22" s="21" t="n"/>
       <c r="I22" s="17" t="inlineStr">
@@ -1313,29 +1313,29 @@
       </c>
       <c r="F6" s="17" t="inlineStr">
         <is>
-          <t>Over 49.5</t>
+          <t>Over 48.5</t>
         </is>
       </c>
       <c r="G6" s="26" t="n">
-        <v>49.5</v>
+        <v>48.5</v>
       </c>
       <c r="H6" s="18" t="n">
-        <v>-105</v>
+        <v>-115</v>
       </c>
       <c r="I6" s="20" t="n">
-        <v>0.5955932130438462</v>
+        <v>0.6232864466877359</v>
       </c>
       <c r="J6" s="20" t="n">
-        <v>0.4891657638136511</v>
+        <v>0.5108342361863488</v>
       </c>
       <c r="K6" s="20" t="n">
-        <v>0.5121951219512195</v>
+        <v>0.5348837209302325</v>
       </c>
       <c r="L6" s="19" t="n">
-        <v>0.08339809109262664</v>
+        <v>0.08840272575750341</v>
       </c>
       <c r="M6" s="19" t="n">
-        <v>0.1628248445141758</v>
+        <v>0.1652746611988105</v>
       </c>
       <c r="N6" s="20" t="n">
         <v>0</v>
@@ -1622,12 +1622,12 @@
       </c>
       <c r="B11" s="12" t="inlineStr">
         <is>
-          <t>SJSU @ USC</t>
+          <t>NMSU @ FSU</t>
         </is>
       </c>
       <c r="C11" s="12" t="inlineStr">
         <is>
-          <t>2026-08-29 19:00</t>
+          <t>2026-08-29 23:00</t>
         </is>
       </c>
       <c r="D11" s="22" t="n">
@@ -1640,29 +1640,29 @@
       </c>
       <c r="F11" s="12" t="inlineStr">
         <is>
-          <t>SJSU +38.5</t>
+          <t>NMSU +31.5</t>
         </is>
       </c>
       <c r="G11" s="23" t="n">
-        <v>-38.5</v>
+        <v>-31.5</v>
       </c>
       <c r="H11" s="13" t="n">
-        <v>-118</v>
+        <v>-115</v>
       </c>
       <c r="I11" s="15" t="n">
-        <v>0.7563609789069304</v>
+        <v>0.7484052544756881</v>
       </c>
       <c r="J11" s="15" t="n">
-        <v>0.5173641257162701</v>
+        <v>0.5108342361863488</v>
       </c>
       <c r="K11" s="15" t="n">
-        <v>0.5412844036697247</v>
+        <v>0.5348837209302325</v>
       </c>
       <c r="L11" s="14" t="n">
-        <v>0.2150765752372057</v>
+        <v>0.2135215335454556</v>
       </c>
       <c r="M11" s="14" t="n">
-        <v>0.3973448593365325</v>
+        <v>0.3991924322806341</v>
       </c>
       <c r="N11" s="15" t="n">
         <v>0</v>
@@ -1689,12 +1689,12 @@
       </c>
       <c r="B12" s="17" t="inlineStr">
         <is>
-          <t>NMSU @ FSU</t>
+          <t>SJSU @ USC</t>
         </is>
       </c>
       <c r="C12" s="17" t="inlineStr">
         <is>
-          <t>2026-08-29 23:00</t>
+          <t>2026-08-29 19:00</t>
         </is>
       </c>
       <c r="D12" s="25" t="n">
@@ -1707,29 +1707,29 @@
       </c>
       <c r="F12" s="17" t="inlineStr">
         <is>
-          <t>NMSU +31.5</t>
+          <t>SJSU +38.5</t>
         </is>
       </c>
       <c r="G12" s="26" t="n">
-        <v>-31.5</v>
+        <v>-38.5</v>
       </c>
       <c r="H12" s="18" t="n">
-        <v>-115</v>
+        <v>-120</v>
       </c>
       <c r="I12" s="20" t="n">
-        <v>0.7484052544756881</v>
+        <v>0.7585484812661867</v>
       </c>
       <c r="J12" s="20" t="n">
-        <v>0.5108342361863488</v>
+        <v>0.5217391304347826</v>
       </c>
       <c r="K12" s="20" t="n">
-        <v>0.5348837209302325</v>
+        <v>0.5454545454545454</v>
       </c>
       <c r="L12" s="19" t="n">
-        <v>0.2135215335454556</v>
+        <v>0.2130939358116413</v>
       </c>
       <c r="M12" s="19" t="n">
-        <v>0.3991924322806341</v>
+        <v>0.3906722156546757</v>
       </c>
       <c r="N12" s="20" t="n">
         <v>0</v>
@@ -2615,12 +2615,12 @@
       </c>
       <c r="B26" s="17" t="inlineStr">
         <is>
-          <t>UNC @ TCU</t>
+          <t>SAC @ EMU</t>
         </is>
       </c>
       <c r="C26" s="17" t="inlineStr">
         <is>
-          <t>2026-08-29 16:00</t>
+          <t>2026-08-29 22:30</t>
         </is>
       </c>
       <c r="D26" s="25" t="n">
@@ -2628,32 +2628,34 @@
       </c>
       <c r="E26" s="17" t="inlineStr">
         <is>
-          <t>ML</t>
+          <t>TOTAL</t>
         </is>
       </c>
       <c r="F26" s="17" t="inlineStr">
         <is>
-          <t>UNC ML</t>
-        </is>
-      </c>
-      <c r="G26" s="26" t="n"/>
+          <t>Over 52.5</t>
+        </is>
+      </c>
+      <c r="G26" s="26" t="n">
+        <v>52.5</v>
+      </c>
       <c r="H26" s="18" t="n">
-        <v>250</v>
+        <v>-108</v>
       </c>
       <c r="I26" s="20" t="n">
-        <v>0.3621290026789783</v>
+        <v>0.595359506876733</v>
       </c>
       <c r="J26" s="20" t="n">
-        <v>0.274247491638796</v>
+        <v>0.4956702459300312</v>
       </c>
       <c r="K26" s="20" t="n">
-        <v>0.2857142857142857</v>
+        <v>0.5192307692307693</v>
       </c>
       <c r="L26" s="19" t="n">
-        <v>0.0764147169646926</v>
+        <v>0.07612873764596373</v>
       </c>
       <c r="M26" s="19" t="n">
-        <v>0.267451509376424</v>
+        <v>0.1466183095403747</v>
       </c>
       <c r="N26" s="20" t="n">
         <v>0</v>
@@ -2676,12 +2678,12 @@
       </c>
       <c r="B27" s="12" t="inlineStr">
         <is>
-          <t>SAC @ EMU</t>
+          <t>AKR @ WAKE</t>
         </is>
       </c>
       <c r="C27" s="12" t="inlineStr">
         <is>
-          <t>2026-08-29 22:30</t>
+          <t>2026-09-03 23:00</t>
         </is>
       </c>
       <c r="D27" s="22" t="n">
@@ -2694,29 +2696,29 @@
       </c>
       <c r="F27" s="12" t="inlineStr">
         <is>
-          <t>Over 52.5</t>
+          <t>Over 49.5</t>
         </is>
       </c>
       <c r="G27" s="23" t="n">
-        <v>52.5</v>
+        <v>49.5</v>
       </c>
       <c r="H27" s="13" t="n">
-        <v>-108</v>
+        <v>-112</v>
       </c>
       <c r="I27" s="15" t="n">
-        <v>0.595359506876733</v>
+        <v>0.603175208172005</v>
       </c>
       <c r="J27" s="15" t="n">
-        <v>0.4956702459300312</v>
+        <v>0.5043297540699688</v>
       </c>
       <c r="K27" s="15" t="n">
-        <v>0.5192307692307693</v>
+        <v>0.5283018867924528</v>
       </c>
       <c r="L27" s="14" t="n">
-        <v>0.07612873764596373</v>
+        <v>0.07487332137955216</v>
       </c>
       <c r="M27" s="14" t="n">
-        <v>0.1466183095403747</v>
+        <v>0.1417245011827237</v>
       </c>
       <c r="N27" s="15" t="n">
         <v>0</v>
@@ -2739,12 +2741,12 @@
       </c>
       <c r="B28" s="17" t="inlineStr">
         <is>
-          <t>AKR @ WAKE</t>
+          <t>UNC @ TCU</t>
         </is>
       </c>
       <c r="C28" s="17" t="inlineStr">
         <is>
-          <t>2026-09-03 23:00</t>
+          <t>2026-08-29 16:00</t>
         </is>
       </c>
       <c r="D28" s="25" t="n">
@@ -2752,34 +2754,32 @@
       </c>
       <c r="E28" s="17" t="inlineStr">
         <is>
-          <t>TOTAL</t>
+          <t>ML</t>
         </is>
       </c>
       <c r="F28" s="17" t="inlineStr">
         <is>
-          <t>Over 49.5</t>
-        </is>
-      </c>
-      <c r="G28" s="26" t="n">
-        <v>49.5</v>
-      </c>
+          <t>UNC ML</t>
+        </is>
+      </c>
+      <c r="G28" s="26" t="n"/>
       <c r="H28" s="18" t="n">
-        <v>-112</v>
+        <v>240</v>
       </c>
       <c r="I28" s="20" t="n">
-        <v>0.603175208172005</v>
+        <v>0.3660199960886052</v>
       </c>
       <c r="J28" s="20" t="n">
-        <v>0.5043297540699688</v>
+        <v>0.2820294784580499</v>
       </c>
       <c r="K28" s="20" t="n">
-        <v>0.5283018867924528</v>
+        <v>0.2941176470588235</v>
       </c>
       <c r="L28" s="19" t="n">
-        <v>0.07487332137955216</v>
+        <v>0.07190234902978171</v>
       </c>
       <c r="M28" s="19" t="n">
-        <v>0.1417245011827237</v>
+        <v>0.2444679867012578</v>
       </c>
       <c r="N28" s="20" t="n">
         <v>0</v>
@@ -3180,12 +3180,12 @@
       </c>
       <c r="B35" s="12" t="inlineStr">
         <is>
-          <t>NCSU @ UVA</t>
+          <t>SJSU @ USC</t>
         </is>
       </c>
       <c r="C35" s="12" t="inlineStr">
         <is>
-          <t>2026-08-29 19:30</t>
+          <t>2026-08-29 19:00</t>
         </is>
       </c>
       <c r="D35" s="22" t="n">
@@ -3193,22 +3193,22 @@
       </c>
       <c r="E35" s="12" t="inlineStr">
         <is>
-          <t>ATS</t>
+          <t>TOTAL</t>
         </is>
       </c>
       <c r="F35" s="12" t="inlineStr">
         <is>
-          <t>NCSU +5.5</t>
+          <t>Under 59.5</t>
         </is>
       </c>
       <c r="G35" s="23" t="n">
-        <v>-5.5</v>
+        <v>59.5</v>
       </c>
       <c r="H35" s="13" t="n">
         <v>-108</v>
       </c>
       <c r="I35" s="15" t="n">
-        <v>0.5412896688794703</v>
+        <v>0.5413851965860426</v>
       </c>
       <c r="J35" s="15" t="n">
         <v>0.4956702459300312</v>
@@ -3217,10 +3217,10 @@
         <v>0.5192307692307693</v>
       </c>
       <c r="L35" s="14" t="n">
-        <v>0.022058899648701</v>
+        <v>0.02215442735527329</v>
       </c>
       <c r="M35" s="14" t="n">
-        <v>0.04248380673083174</v>
+        <v>0.04266778601756349</v>
       </c>
       <c r="N35" s="15" t="n">
         <v>0</v>
@@ -3243,12 +3243,12 @@
       </c>
       <c r="B36" s="17" t="inlineStr">
         <is>
-          <t>JVST @ NDSU</t>
+          <t>NCSU @ UVA</t>
         </is>
       </c>
       <c r="C36" s="17" t="inlineStr">
         <is>
-          <t>2026-08-29 21:30</t>
+          <t>2026-08-29 19:30</t>
         </is>
       </c>
       <c r="D36" s="25" t="n">
@@ -3261,32 +3261,32 @@
       </c>
       <c r="F36" s="17" t="inlineStr">
         <is>
-          <t>JVST +7</t>
+          <t>NCSU +5.5</t>
         </is>
       </c>
       <c r="G36" s="26" t="n">
-        <v>-7</v>
+        <v>-5.5</v>
       </c>
       <c r="H36" s="18" t="n">
-        <v>-110</v>
+        <v>-108</v>
       </c>
       <c r="I36" s="20" t="n">
-        <v>0.5445684137563569</v>
+        <v>0.5412896688794703</v>
       </c>
       <c r="J36" s="20" t="n">
-        <v>0.5</v>
+        <v>0.4956702459300312</v>
       </c>
       <c r="K36" s="20" t="n">
-        <v>0.5238095238095238</v>
+        <v>0.5192307692307693</v>
       </c>
       <c r="L36" s="19" t="n">
-        <v>0.02075888994683306</v>
+        <v>0.022058899648701</v>
       </c>
       <c r="M36" s="19" t="n">
-        <v>0.03762929802911508</v>
+        <v>0.04248380673083174</v>
       </c>
       <c r="N36" s="20" t="n">
-        <v>0.0505</v>
+        <v>0</v>
       </c>
       <c r="O36" s="27" t="n">
         <v>0.45</v>
@@ -3306,12 +3306,12 @@
       </c>
       <c r="B37" s="12" t="inlineStr">
         <is>
-          <t>SJSU @ USC</t>
+          <t>NCSU @ UVA</t>
         </is>
       </c>
       <c r="C37" s="12" t="inlineStr">
         <is>
-          <t>2026-08-29 19:00</t>
+          <t>2026-08-29 19:30</t>
         </is>
       </c>
       <c r="D37" s="22" t="n">
@@ -3319,34 +3319,32 @@
       </c>
       <c r="E37" s="12" t="inlineStr">
         <is>
-          <t>TOTAL</t>
+          <t>ML</t>
         </is>
       </c>
       <c r="F37" s="12" t="inlineStr">
         <is>
-          <t>Under 59.5</t>
-        </is>
-      </c>
-      <c r="G37" s="23" t="n">
-        <v>59.5</v>
-      </c>
+          <t>NCSU ML</t>
+        </is>
+      </c>
+      <c r="G37" s="23" t="n"/>
       <c r="H37" s="13" t="n">
-        <v>-110</v>
+        <v>180</v>
       </c>
       <c r="I37" s="15" t="n">
-        <v>0.543550073621027</v>
+        <v>0.3745807138274095</v>
       </c>
       <c r="J37" s="15" t="n">
-        <v>0.5</v>
+        <v>0.3425247738043947</v>
       </c>
       <c r="K37" s="15" t="n">
-        <v>0.5238095238095238</v>
+        <v>0.3571428571428572</v>
       </c>
       <c r="L37" s="14" t="n">
-        <v>0.01974054981150319</v>
+        <v>0.01743785668455239</v>
       </c>
       <c r="M37" s="14" t="n">
-        <v>0.0376865041855971</v>
+        <v>0.04882599871674664</v>
       </c>
       <c r="N37" s="15" t="n">
         <v>0</v>
@@ -3369,12 +3367,12 @@
       </c>
       <c r="B38" s="17" t="inlineStr">
         <is>
-          <t>NCSU @ UVA</t>
+          <t>MRMK @ DEL</t>
         </is>
       </c>
       <c r="C38" s="17" t="inlineStr">
         <is>
-          <t>2026-08-29 19:30</t>
+          <t>2026-09-03 23:00</t>
         </is>
       </c>
       <c r="D38" s="25" t="n">
@@ -3382,32 +3380,34 @@
       </c>
       <c r="E38" s="17" t="inlineStr">
         <is>
-          <t>ML</t>
+          <t>TOTAL</t>
         </is>
       </c>
       <c r="F38" s="17" t="inlineStr">
         <is>
-          <t>NCSU ML</t>
-        </is>
-      </c>
-      <c r="G38" s="26" t="n"/>
+          <t>Over 55.5</t>
+        </is>
+      </c>
+      <c r="G38" s="26" t="n">
+        <v>55.5</v>
+      </c>
       <c r="H38" s="18" t="n">
-        <v>180</v>
+        <v>-112</v>
       </c>
       <c r="I38" s="20" t="n">
-        <v>0.3745807138274095</v>
+        <v>0.5437650474945759</v>
       </c>
       <c r="J38" s="20" t="n">
-        <v>0.3425247738043947</v>
+        <v>0.5043297540699688</v>
       </c>
       <c r="K38" s="20" t="n">
-        <v>0.3571428571428572</v>
+        <v>0.5283018867924528</v>
       </c>
       <c r="L38" s="19" t="n">
-        <v>0.01743785668455239</v>
+        <v>0.01546316070212306</v>
       </c>
       <c r="M38" s="19" t="n">
-        <v>0.04882599871674664</v>
+        <v>0.02926955418616145</v>
       </c>
       <c r="N38" s="20" t="n">
         <v>0</v>
@@ -3420,7 +3420,11 @@
           <t>DraftKings</t>
         </is>
       </c>
-      <c r="Q38" s="17" t="n"/>
+      <c r="Q38" s="17" t="inlineStr">
+        <is>
+          <t>MRMK isn't a full FBS participant this season — model doesn't rate them reliably</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="12" t="inlineStr">
@@ -3430,12 +3434,12 @@
       </c>
       <c r="B39" s="12" t="inlineStr">
         <is>
-          <t>MRMK @ DEL</t>
+          <t>JVST @ NDSU</t>
         </is>
       </c>
       <c r="C39" s="12" t="inlineStr">
         <is>
-          <t>2026-09-03 23:00</t>
+          <t>2026-08-29 21:30</t>
         </is>
       </c>
       <c r="D39" s="22" t="n">
@@ -3443,37 +3447,37 @@
       </c>
       <c r="E39" s="12" t="inlineStr">
         <is>
-          <t>TOTAL</t>
+          <t>ATS</t>
         </is>
       </c>
       <c r="F39" s="12" t="inlineStr">
         <is>
-          <t>Over 55.5</t>
+          <t>JVST +7</t>
         </is>
       </c>
       <c r="G39" s="23" t="n">
-        <v>55.5</v>
+        <v>-7</v>
       </c>
       <c r="H39" s="13" t="n">
-        <v>-112</v>
+        <v>-115</v>
       </c>
       <c r="I39" s="15" t="n">
-        <v>0.5437650474945759</v>
+        <v>0.5499855318495314</v>
       </c>
       <c r="J39" s="15" t="n">
-        <v>0.5043297540699688</v>
+        <v>0.5108342361863488</v>
       </c>
       <c r="K39" s="15" t="n">
-        <v>0.5283018867924528</v>
+        <v>0.5348837209302325</v>
       </c>
       <c r="L39" s="14" t="n">
-        <v>0.01546316070212306</v>
+        <v>0.01510181091929885</v>
       </c>
       <c r="M39" s="14" t="n">
-        <v>0.02926955418616145</v>
+        <v>0.02680803788623665</v>
       </c>
       <c r="N39" s="15" t="n">
-        <v>0</v>
+        <v>0.0505</v>
       </c>
       <c r="O39" s="24" t="n">
         <v>0.45</v>
@@ -3483,11 +3487,7 @@
           <t>DraftKings</t>
         </is>
       </c>
-      <c r="Q39" s="12" t="inlineStr">
-        <is>
-          <t>MRMK isn't a full FBS participant this season — model doesn't rate them reliably</t>
-        </is>
-      </c>
+      <c r="Q39" s="12" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="17" t="inlineStr">
@@ -3497,12 +3497,12 @@
       </c>
       <c r="B40" s="17" t="inlineStr">
         <is>
-          <t>JVST @ NDSU</t>
+          <t>UNC @ TCU</t>
         </is>
       </c>
       <c r="C40" s="17" t="inlineStr">
         <is>
-          <t>2026-08-29 21:30</t>
+          <t>2026-08-29 16:00</t>
         </is>
       </c>
       <c r="D40" s="25" t="n">
@@ -3510,32 +3510,34 @@
       </c>
       <c r="E40" s="17" t="inlineStr">
         <is>
-          <t>ML</t>
+          <t>TOTAL</t>
         </is>
       </c>
       <c r="F40" s="17" t="inlineStr">
         <is>
-          <t>JVST ML</t>
-        </is>
-      </c>
-      <c r="G40" s="26" t="n"/>
+          <t>Over 47.5</t>
+        </is>
+      </c>
+      <c r="G40" s="26" t="n">
+        <v>47.5</v>
+      </c>
       <c r="H40" s="18" t="n">
-        <v>220</v>
+        <v>-112</v>
       </c>
       <c r="I40" s="20" t="n">
-        <v>0.3261190128306598</v>
+        <v>0.5398532027364953</v>
       </c>
       <c r="J40" s="20" t="n">
-        <v>0.299837925445705</v>
+        <v>0.5043297540699688</v>
       </c>
       <c r="K40" s="20" t="n">
-        <v>0.3125</v>
+        <v>0.5283018867924528</v>
       </c>
       <c r="L40" s="19" t="n">
-        <v>0.0136190128306598</v>
+        <v>0.01155131594404246</v>
       </c>
       <c r="M40" s="19" t="n">
-        <v>0.04358084105811144</v>
+        <v>0.02186499089408034</v>
       </c>
       <c r="N40" s="20" t="n">
         <v>0</v>
@@ -3558,12 +3560,12 @@
       </c>
       <c r="B41" s="12" t="inlineStr">
         <is>
-          <t>UNC @ TCU</t>
+          <t>JVST @ NDSU</t>
         </is>
       </c>
       <c r="C41" s="12" t="inlineStr">
         <is>
-          <t>2026-08-29 16:00</t>
+          <t>2026-08-29 21:30</t>
         </is>
       </c>
       <c r="D41" s="22" t="n">
@@ -3571,34 +3573,32 @@
       </c>
       <c r="E41" s="12" t="inlineStr">
         <is>
-          <t>TOTAL</t>
+          <t>ML</t>
         </is>
       </c>
       <c r="F41" s="12" t="inlineStr">
         <is>
-          <t>Over 47.5</t>
-        </is>
-      </c>
-      <c r="G41" s="23" t="n">
-        <v>47.5</v>
-      </c>
+          <t>JVST ML</t>
+        </is>
+      </c>
+      <c r="G41" s="23" t="n"/>
       <c r="H41" s="13" t="n">
-        <v>-112</v>
+        <v>210</v>
       </c>
       <c r="I41" s="15" t="n">
-        <v>0.5398532027364953</v>
+        <v>0.3308036085807733</v>
       </c>
       <c r="J41" s="15" t="n">
-        <v>0.5043297540699688</v>
+        <v>0.3092071169459319</v>
       </c>
       <c r="K41" s="15" t="n">
-        <v>0.5283018867924528</v>
+        <v>0.3225806451612903</v>
       </c>
       <c r="L41" s="14" t="n">
-        <v>0.01155131594404246</v>
+        <v>0.008222963419482976</v>
       </c>
       <c r="M41" s="14" t="n">
-        <v>0.02186499089408034</v>
+        <v>0.02549118660039718</v>
       </c>
       <c r="N41" s="15" t="n">
         <v>0</v>
@@ -3936,12 +3936,12 @@
       </c>
       <c r="B47" s="12" t="inlineStr">
         <is>
-          <t>NMSU @ FSU</t>
+          <t>JVST @ NDSU</t>
         </is>
       </c>
       <c r="C47" s="12" t="inlineStr">
         <is>
-          <t>2026-08-29 23:00</t>
+          <t>2026-08-29 21:30</t>
         </is>
       </c>
       <c r="D47" s="22" t="n">
@@ -3949,34 +3949,32 @@
       </c>
       <c r="E47" s="12" t="inlineStr">
         <is>
-          <t>TOTAL</t>
+          <t>ML</t>
         </is>
       </c>
       <c r="F47" s="12" t="inlineStr">
         <is>
-          <t>Under 53.5</t>
-        </is>
-      </c>
-      <c r="G47" s="23" t="n">
-        <v>53.5</v>
-      </c>
+          <t>NDSU ML</t>
+        </is>
+      </c>
+      <c r="G47" s="23" t="n"/>
       <c r="H47" s="13" t="n">
-        <v>-110</v>
+        <v>-258</v>
       </c>
       <c r="I47" s="15" t="n">
-        <v>0.4701788116717455</v>
+        <v>0.6691963914192267</v>
       </c>
       <c r="J47" s="15" t="n">
-        <v>0.5</v>
+        <v>0.6907928830540681</v>
       </c>
       <c r="K47" s="15" t="n">
-        <v>0.5238095238095238</v>
+        <v>0.7206703910614525</v>
       </c>
       <c r="L47" s="14" t="n">
-        <v>-0.05363071213777837</v>
+        <v>-0.05147399964222577</v>
       </c>
       <c r="M47" s="14" t="n">
-        <v>-0.1023859049903041</v>
+        <v>-0.07142516229425128</v>
       </c>
       <c r="N47" s="15" t="n">
         <v>0</v>
@@ -3999,12 +3997,12 @@
       </c>
       <c r="B48" s="17" t="inlineStr">
         <is>
-          <t>JVST @ NDSU</t>
+          <t>NMSU @ FSU</t>
         </is>
       </c>
       <c r="C48" s="17" t="inlineStr">
         <is>
-          <t>2026-08-29 21:30</t>
+          <t>2026-08-29 23:00</t>
         </is>
       </c>
       <c r="D48" s="25" t="n">
@@ -4012,32 +4010,34 @@
       </c>
       <c r="E48" s="17" t="inlineStr">
         <is>
-          <t>ML</t>
+          <t>TOTAL</t>
         </is>
       </c>
       <c r="F48" s="17" t="inlineStr">
         <is>
-          <t>NDSU ML</t>
-        </is>
-      </c>
-      <c r="G48" s="26" t="n"/>
+          <t>Under 53.5</t>
+        </is>
+      </c>
+      <c r="G48" s="26" t="n">
+        <v>53.5</v>
+      </c>
       <c r="H48" s="18" t="n">
-        <v>-270</v>
+        <v>-110</v>
       </c>
       <c r="I48" s="20" t="n">
-        <v>0.6738809871693402</v>
+        <v>0.4701788116717455</v>
       </c>
       <c r="J48" s="20" t="n">
-        <v>0.7001620745542949</v>
+        <v>0.5</v>
       </c>
       <c r="K48" s="20" t="n">
-        <v>0.7297297297297297</v>
+        <v>0.5238095238095238</v>
       </c>
       <c r="L48" s="19" t="n">
-        <v>-0.05584874256038952</v>
+        <v>-0.05363071213777837</v>
       </c>
       <c r="M48" s="19" t="n">
-        <v>-0.07653346202720057</v>
+        <v>-0.1023859049903041</v>
       </c>
       <c r="N48" s="20" t="n">
         <v>0</v>
@@ -4184,12 +4184,12 @@
       </c>
       <c r="B51" s="12" t="inlineStr">
         <is>
-          <t>MRMK @ DEL</t>
+          <t>JVST @ NDSU</t>
         </is>
       </c>
       <c r="C51" s="12" t="inlineStr">
         <is>
-          <t>2026-09-03 23:00</t>
+          <t>2026-08-29 21:30</t>
         </is>
       </c>
       <c r="D51" s="22" t="n">
@@ -4197,37 +4197,37 @@
       </c>
       <c r="E51" s="12" t="inlineStr">
         <is>
-          <t>TOTAL</t>
+          <t>ATS</t>
         </is>
       </c>
       <c r="F51" s="12" t="inlineStr">
         <is>
-          <t>Under 55.5</t>
+          <t>NDSU -7</t>
         </is>
       </c>
       <c r="G51" s="23" t="n">
-        <v>55.5</v>
+        <v>-7</v>
       </c>
       <c r="H51" s="13" t="n">
-        <v>-108</v>
+        <v>-105</v>
       </c>
       <c r="I51" s="15" t="n">
-        <v>0.4562349525054241</v>
+        <v>0.4500144681504686</v>
       </c>
       <c r="J51" s="15" t="n">
-        <v>0.4956702459300312</v>
+        <v>0.4891657638136511</v>
       </c>
       <c r="K51" s="15" t="n">
-        <v>0.5192307692307693</v>
+        <v>0.5121951219512195</v>
       </c>
       <c r="L51" s="14" t="n">
-        <v>-0.06299581672534516</v>
+        <v>-0.06218065380075088</v>
       </c>
       <c r="M51" s="14" t="n">
-        <v>-0.1213252766562202</v>
+        <v>-0.1152697169483107</v>
       </c>
       <c r="N51" s="15" t="n">
-        <v>0</v>
+        <v>0.0505</v>
       </c>
       <c r="O51" s="24" t="n">
         <v>0.45</v>
@@ -4237,11 +4237,7 @@
           <t>DraftKings</t>
         </is>
       </c>
-      <c r="Q51" s="12" t="inlineStr">
-        <is>
-          <t>MRMK isn't a full FBS participant this season — model doesn't rate them reliably</t>
-        </is>
-      </c>
+      <c r="Q51" s="12" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="17" t="inlineStr">
@@ -4251,12 +4247,12 @@
       </c>
       <c r="B52" s="17" t="inlineStr">
         <is>
-          <t>SJSU @ USC</t>
+          <t>MRMK @ DEL</t>
         </is>
       </c>
       <c r="C52" s="17" t="inlineStr">
         <is>
-          <t>2026-08-29 19:00</t>
+          <t>2026-09-03 23:00</t>
         </is>
       </c>
       <c r="D52" s="25" t="n">
@@ -4269,29 +4265,29 @@
       </c>
       <c r="F52" s="17" t="inlineStr">
         <is>
-          <t>Over 59.5</t>
+          <t>Under 55.5</t>
         </is>
       </c>
       <c r="G52" s="26" t="n">
-        <v>59.5</v>
+        <v>55.5</v>
       </c>
       <c r="H52" s="18" t="n">
-        <v>-110</v>
+        <v>-108</v>
       </c>
       <c r="I52" s="20" t="n">
-        <v>0.456449926378973</v>
+        <v>0.4562349525054241</v>
       </c>
       <c r="J52" s="20" t="n">
-        <v>0.5</v>
+        <v>0.4956702459300312</v>
       </c>
       <c r="K52" s="20" t="n">
-        <v>0.5238095238095238</v>
+        <v>0.5192307692307693</v>
       </c>
       <c r="L52" s="19" t="n">
-        <v>-0.06735959743055087</v>
+        <v>-0.06299581672534516</v>
       </c>
       <c r="M52" s="19" t="n">
-        <v>-0.1285955950946879</v>
+        <v>-0.1213252766562202</v>
       </c>
       <c r="N52" s="20" t="n">
         <v>0</v>
@@ -4304,7 +4300,11 @@
           <t>DraftKings</t>
         </is>
       </c>
-      <c r="Q52" s="17" t="n"/>
+      <c r="Q52" s="17" t="inlineStr">
+        <is>
+          <t>MRMK isn't a full FBS participant this season — model doesn't rate them reliably</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="12" t="inlineStr">
@@ -4314,12 +4314,12 @@
       </c>
       <c r="B53" s="12" t="inlineStr">
         <is>
-          <t>JVST @ NDSU</t>
+          <t>NCSU @ UVA</t>
         </is>
       </c>
       <c r="C53" s="12" t="inlineStr">
         <is>
-          <t>2026-08-29 21:30</t>
+          <t>2026-08-29 19:30</t>
         </is>
       </c>
       <c r="D53" s="22" t="n">
@@ -4332,32 +4332,32 @@
       </c>
       <c r="F53" s="12" t="inlineStr">
         <is>
-          <t>NDSU -7</t>
+          <t>UVA -5.5</t>
         </is>
       </c>
       <c r="G53" s="23" t="n">
-        <v>-7</v>
+        <v>-5.5</v>
       </c>
       <c r="H53" s="13" t="n">
-        <v>-110</v>
+        <v>-112</v>
       </c>
       <c r="I53" s="15" t="n">
-        <v>0.4554315862436431</v>
+        <v>0.4587103311205297</v>
       </c>
       <c r="J53" s="15" t="n">
-        <v>0.5</v>
+        <v>0.5043297540699688</v>
       </c>
       <c r="K53" s="15" t="n">
-        <v>0.5238095238095238</v>
+        <v>0.5283018867924528</v>
       </c>
       <c r="L53" s="14" t="n">
-        <v>-0.06837793756588073</v>
+        <v>-0.0695915556719231</v>
       </c>
       <c r="M53" s="14" t="n">
-        <v>-0.1239475616409477</v>
+        <v>-0.1317268732361402</v>
       </c>
       <c r="N53" s="15" t="n">
-        <v>0.0505</v>
+        <v>0</v>
       </c>
       <c r="O53" s="24" t="n">
         <v>0.45</v>
@@ -4377,12 +4377,12 @@
       </c>
       <c r="B54" s="17" t="inlineStr">
         <is>
-          <t>NCSU @ UVA</t>
+          <t>SJSU @ USC</t>
         </is>
       </c>
       <c r="C54" s="17" t="inlineStr">
         <is>
-          <t>2026-08-29 19:30</t>
+          <t>2026-08-29 19:00</t>
         </is>
       </c>
       <c r="D54" s="25" t="n">
@@ -4390,22 +4390,22 @@
       </c>
       <c r="E54" s="17" t="inlineStr">
         <is>
-          <t>ATS</t>
+          <t>TOTAL</t>
         </is>
       </c>
       <c r="F54" s="17" t="inlineStr">
         <is>
-          <t>UVA -5.5</t>
+          <t>Over 59.5</t>
         </is>
       </c>
       <c r="G54" s="26" t="n">
-        <v>-5.5</v>
+        <v>59.5</v>
       </c>
       <c r="H54" s="18" t="n">
         <v>-112</v>
       </c>
       <c r="I54" s="20" t="n">
-        <v>0.4587103311205297</v>
+        <v>0.4586148034139574</v>
       </c>
       <c r="J54" s="20" t="n">
         <v>0.5043297540699688</v>
@@ -4414,10 +4414,10 @@
         <v>0.5283018867924528</v>
       </c>
       <c r="L54" s="19" t="n">
-        <v>-0.0695915556719231</v>
+        <v>-0.06968708337849544</v>
       </c>
       <c r="M54" s="19" t="n">
-        <v>-0.1317268732361402</v>
+        <v>-0.1319076935378664</v>
       </c>
       <c r="N54" s="20" t="n">
         <v>0</v>
@@ -4841,22 +4841,22 @@
       </c>
       <c r="G61" s="23" t="n"/>
       <c r="H61" s="13" t="n">
-        <v>-310</v>
+        <v>-298</v>
       </c>
       <c r="I61" s="15" t="n">
-        <v>0.6378709973210217</v>
+        <v>0.6339800039113948</v>
       </c>
       <c r="J61" s="15" t="n">
-        <v>0.725752508361204</v>
+        <v>0.7179705215419501</v>
       </c>
       <c r="K61" s="15" t="n">
-        <v>0.7560975609756098</v>
+        <v>0.7487437185929648</v>
       </c>
       <c r="L61" s="14" t="n">
-        <v>-0.1182265636545881</v>
+        <v>-0.1147637146815701</v>
       </c>
       <c r="M61" s="14" t="n">
-        <v>-0.1563641648334875</v>
+        <v>-0.1532750283331037</v>
       </c>
       <c r="N61" s="15" t="n">
         <v>0</v>
@@ -5153,29 +5153,29 @@
       </c>
       <c r="F66" s="17" t="inlineStr">
         <is>
-          <t>Under 49.5</t>
+          <t>Under 48.5</t>
         </is>
       </c>
       <c r="G66" s="26" t="n">
-        <v>49.5</v>
+        <v>48.5</v>
       </c>
       <c r="H66" s="18" t="n">
-        <v>-115</v>
+        <v>-105</v>
       </c>
       <c r="I66" s="20" t="n">
-        <v>0.4044067869561538</v>
+        <v>0.3767135533122641</v>
       </c>
       <c r="J66" s="20" t="n">
-        <v>0.5108342361863488</v>
+        <v>0.4891657638136511</v>
       </c>
       <c r="K66" s="20" t="n">
-        <v>0.5348837209302325</v>
+        <v>0.5121951219512195</v>
       </c>
       <c r="L66" s="19" t="n">
-        <v>-0.1304769339740787</v>
+        <v>-0.1354815686389554</v>
       </c>
       <c r="M66" s="19" t="n">
-        <v>-0.2439351374297994</v>
+        <v>-0.2645116340093892</v>
       </c>
       <c r="N66" s="20" t="n">
         <v>0</v>
@@ -6051,12 +6051,12 @@
       </c>
       <c r="B80" s="17" t="inlineStr">
         <is>
-          <t>NMSU @ FSU</t>
+          <t>SJSU @ USC</t>
         </is>
       </c>
       <c r="C80" s="17" t="inlineStr">
         <is>
-          <t>2026-08-29 23:00</t>
+          <t>2026-08-29 19:00</t>
         </is>
       </c>
       <c r="D80" s="25" t="n">
@@ -6069,29 +6069,29 @@
       </c>
       <c r="F80" s="17" t="inlineStr">
         <is>
-          <t>FSU -31.5</t>
+          <t>USC -38.5</t>
         </is>
       </c>
       <c r="G80" s="26" t="n">
-        <v>-31.5</v>
+        <v>-38.5</v>
       </c>
       <c r="H80" s="18" t="n">
-        <v>-105</v>
+        <v>100</v>
       </c>
       <c r="I80" s="20" t="n">
-        <v>0.2515947455243119</v>
+        <v>0.2414515187338134</v>
       </c>
       <c r="J80" s="20" t="n">
-        <v>0.4891657638136511</v>
+        <v>0.4782608695652174</v>
       </c>
       <c r="K80" s="20" t="n">
-        <v>0.5121951219512195</v>
+        <v>0.5</v>
       </c>
       <c r="L80" s="19" t="n">
-        <v>-0.2606003764269076</v>
+        <v>-0.2585484812661866</v>
       </c>
       <c r="M80" s="19" t="n">
-        <v>-0.5087912111192006</v>
+        <v>-0.5170969625323734</v>
       </c>
       <c r="N80" s="20" t="n">
         <v>0</v>
@@ -6118,12 +6118,12 @@
       </c>
       <c r="B81" s="12" t="inlineStr">
         <is>
-          <t>SJSU @ USC</t>
+          <t>NMSU @ FSU</t>
         </is>
       </c>
       <c r="C81" s="12" t="inlineStr">
         <is>
-          <t>2026-08-29 19:00</t>
+          <t>2026-08-29 23:00</t>
         </is>
       </c>
       <c r="D81" s="22" t="n">
@@ -6136,29 +6136,29 @@
       </c>
       <c r="F81" s="12" t="inlineStr">
         <is>
-          <t>USC -38.5</t>
+          <t>FSU -31.5</t>
         </is>
       </c>
       <c r="G81" s="23" t="n">
-        <v>-38.5</v>
+        <v>-31.5</v>
       </c>
       <c r="H81" s="13" t="n">
-        <v>-102</v>
+        <v>-105</v>
       </c>
       <c r="I81" s="15" t="n">
-        <v>0.2436390210930696</v>
+        <v>0.2515947455243119</v>
       </c>
       <c r="J81" s="15" t="n">
-        <v>0.4826358742837298</v>
+        <v>0.4891657638136511</v>
       </c>
       <c r="K81" s="15" t="n">
-        <v>0.504950495049505</v>
+        <v>0.5121951219512195</v>
       </c>
       <c r="L81" s="14" t="n">
-        <v>-0.2613114739564354</v>
+        <v>-0.2606003764269076</v>
       </c>
       <c r="M81" s="14" t="n">
-        <v>-0.517499193521568</v>
+        <v>-0.5087912111192006</v>
       </c>
       <c r="N81" s="15" t="n">
         <v>0</v>
@@ -13291,10 +13291,10 @@
         <v>47.5</v>
       </c>
       <c r="K5" s="13" t="n">
-        <v>250</v>
+        <v>240</v>
       </c>
       <c r="L5" s="13" t="n">
-        <v>-310</v>
+        <v>-298</v>
       </c>
       <c r="M5" s="12" t="inlineStr">
         <is>
@@ -13434,10 +13434,10 @@
         <v>46.5</v>
       </c>
       <c r="K8" s="18" t="n">
-        <v>220</v>
+        <v>210</v>
       </c>
       <c r="L8" s="18" t="n">
-        <v>-270</v>
+        <v>-258</v>
       </c>
       <c r="M8" s="17" t="inlineStr">
         <is>
@@ -13529,7 +13529,7 @@
         <v>-5.5</v>
       </c>
       <c r="J10" s="30" t="n">
-        <v>49.5</v>
+        <v>48.5</v>
       </c>
       <c r="K10" s="18" t="n">
         <v>180</v>

</xml_diff>

<commit_message>
refresh 2026-08-24 21:57 UTC
</commit_message>
<xml_diff>
--- a/NCAAF_Edge_Model.xlsx
+++ b/NCAAF_Edge_Model.xlsx
@@ -640,7 +640,7 @@
     <row r="2" ht="26" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-08-24T18:03:18+00:00 from live ESPN data. This file is a snapshot, not the model. Re-run the pipeline to refresh it.</t>
+          <t>Generated 2026-08-24T21:57:37+00:00 from live ESPN data. This file is a snapshot, not the model. Re-run the pipeline to refresh it.</t>
         </is>
       </c>
     </row>
@@ -3079,22 +3079,22 @@
       </c>
       <c r="G33" s="23" t="n"/>
       <c r="H33" s="13" t="n">
-        <v>185</v>
+        <v>180</v>
       </c>
       <c r="I33" s="15" t="n">
-        <v>0.3799494426906008</v>
+        <v>0.383035891688529</v>
       </c>
       <c r="J33" s="15" t="n">
-        <v>0.3363518758085381</v>
+        <v>0.3425247738043947</v>
       </c>
       <c r="K33" s="15" t="n">
-        <v>0.3508771929824561</v>
+        <v>0.3571428571428572</v>
       </c>
       <c r="L33" s="14" t="n">
-        <v>0.0290722497081447</v>
+        <v>0.02589303454567188</v>
       </c>
       <c r="M33" s="14" t="n">
-        <v>0.08285591166821238</v>
+        <v>0.07250049672788117</v>
       </c>
       <c r="N33" s="15" t="n">
         <v>0</v>
@@ -4314,12 +4314,12 @@
       </c>
       <c r="B53" s="12" t="inlineStr">
         <is>
-          <t>NCSU @ UVA</t>
+          <t>MEM @ UNLV</t>
         </is>
       </c>
       <c r="C53" s="12" t="inlineStr">
         <is>
-          <t>2026-08-29 19:30</t>
+          <t>2026-08-30 02:00</t>
         </is>
       </c>
       <c r="D53" s="22" t="n">
@@ -4327,34 +4327,32 @@
       </c>
       <c r="E53" s="12" t="inlineStr">
         <is>
-          <t>ATS</t>
+          <t>ML</t>
         </is>
       </c>
       <c r="F53" s="12" t="inlineStr">
         <is>
-          <t>UVA -5.5</t>
-        </is>
-      </c>
-      <c r="G53" s="23" t="n">
-        <v>-5.5</v>
-      </c>
+          <t>UNLV ML</t>
+        </is>
+      </c>
+      <c r="G53" s="23" t="n"/>
       <c r="H53" s="13" t="n">
-        <v>-112</v>
+        <v>-218</v>
       </c>
       <c r="I53" s="15" t="n">
-        <v>0.4587103311205297</v>
+        <v>0.616964108311471</v>
       </c>
       <c r="J53" s="15" t="n">
-        <v>0.5043297540699688</v>
+        <v>0.6574752261956054</v>
       </c>
       <c r="K53" s="15" t="n">
-        <v>0.5283018867924528</v>
+        <v>0.6855345911949685</v>
       </c>
       <c r="L53" s="14" t="n">
-        <v>-0.0695915556719231</v>
+        <v>-0.06857048288349754</v>
       </c>
       <c r="M53" s="14" t="n">
-        <v>-0.1317268732361402</v>
+        <v>-0.1000248328300561</v>
       </c>
       <c r="N53" s="15" t="n">
         <v>0</v>
@@ -4377,12 +4375,12 @@
       </c>
       <c r="B54" s="17" t="inlineStr">
         <is>
-          <t>SJSU @ USC</t>
+          <t>NCSU @ UVA</t>
         </is>
       </c>
       <c r="C54" s="17" t="inlineStr">
         <is>
-          <t>2026-08-29 19:00</t>
+          <t>2026-08-29 19:30</t>
         </is>
       </c>
       <c r="D54" s="25" t="n">
@@ -4390,22 +4388,22 @@
       </c>
       <c r="E54" s="17" t="inlineStr">
         <is>
-          <t>TOTAL</t>
+          <t>ATS</t>
         </is>
       </c>
       <c r="F54" s="17" t="inlineStr">
         <is>
-          <t>Over 59.5</t>
+          <t>UVA -5.5</t>
         </is>
       </c>
       <c r="G54" s="26" t="n">
-        <v>59.5</v>
+        <v>-5.5</v>
       </c>
       <c r="H54" s="18" t="n">
         <v>-112</v>
       </c>
       <c r="I54" s="20" t="n">
-        <v>0.4586148034139574</v>
+        <v>0.4587103311205297</v>
       </c>
       <c r="J54" s="20" t="n">
         <v>0.5043297540699688</v>
@@ -4414,10 +4412,10 @@
         <v>0.5283018867924528</v>
       </c>
       <c r="L54" s="19" t="n">
-        <v>-0.06968708337849544</v>
+        <v>-0.0695915556719231</v>
       </c>
       <c r="M54" s="19" t="n">
-        <v>-0.1319076935378664</v>
+        <v>-0.1317268732361402</v>
       </c>
       <c r="N54" s="20" t="n">
         <v>0</v>
@@ -4440,12 +4438,12 @@
       </c>
       <c r="B55" s="12" t="inlineStr">
         <is>
-          <t>MEM @ UNLV</t>
+          <t>SJSU @ USC</t>
         </is>
       </c>
       <c r="C55" s="12" t="inlineStr">
         <is>
-          <t>2026-08-30 02:00</t>
+          <t>2026-08-29 19:00</t>
         </is>
       </c>
       <c r="D55" s="22" t="n">
@@ -4453,32 +4451,34 @@
       </c>
       <c r="E55" s="12" t="inlineStr">
         <is>
-          <t>ML</t>
+          <t>TOTAL</t>
         </is>
       </c>
       <c r="F55" s="12" t="inlineStr">
         <is>
-          <t>UNLV ML</t>
-        </is>
-      </c>
-      <c r="G55" s="23" t="n"/>
+          <t>Over 59.5</t>
+        </is>
+      </c>
+      <c r="G55" s="23" t="n">
+        <v>59.5</v>
+      </c>
       <c r="H55" s="13" t="n">
-        <v>-225</v>
+        <v>-112</v>
       </c>
       <c r="I55" s="15" t="n">
-        <v>0.6200505573093992</v>
+        <v>0.4586148034139574</v>
       </c>
       <c r="J55" s="15" t="n">
-        <v>0.6636481241914618</v>
+        <v>0.5043297540699688</v>
       </c>
       <c r="K55" s="15" t="n">
-        <v>0.6923076923076923</v>
+        <v>0.5283018867924528</v>
       </c>
       <c r="L55" s="14" t="n">
-        <v>-0.07225713499829312</v>
+        <v>-0.06968708337849544</v>
       </c>
       <c r="M55" s="14" t="n">
-        <v>-0.1043714172197567</v>
+        <v>-0.1319076935378664</v>
       </c>
       <c r="N55" s="15" t="n">
         <v>0</v>
@@ -13630,10 +13630,10 @@
         <v>57.5</v>
       </c>
       <c r="K12" s="18" t="n">
-        <v>185</v>
+        <v>180</v>
       </c>
       <c r="L12" s="18" t="n">
-        <v>-225</v>
+        <v>-218</v>
       </c>
       <c r="M12" s="17" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
refresh 2026-08-25 21:56 UTC
</commit_message>
<xml_diff>
--- a/NCAAF_Edge_Model.xlsx
+++ b/NCAAF_Edge_Model.xlsx
@@ -640,7 +640,7 @@
     <row r="2" ht="26" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-08-25T18:02:02+00:00 from live ESPN data. This file is a snapshot, not the model. Re-run the pipeline to refresh it.</t>
+          <t>Generated 2026-08-25T21:56:33+00:00 from live ESPN data. This file is a snapshot, not the model. Re-run the pipeline to refresh it.</t>
         </is>
       </c>
     </row>
@@ -1114,13 +1114,13 @@
         </is>
       </c>
       <c r="E24" s="18" t="n">
-        <v>-105</v>
+        <v>-102</v>
       </c>
       <c r="F24" s="19" t="n">
-        <v>0.08386062118588167</v>
+        <v>0.08784030332263559</v>
       </c>
       <c r="G24" s="20" t="n">
-        <v>0.5960557431371012</v>
+        <v>0.5927907983721405</v>
       </c>
       <c r="H24" s="21" t="n"/>
       <c r="I24" s="17" t="inlineStr">
@@ -1520,22 +1520,22 @@
         <v>-7.5</v>
       </c>
       <c r="H8" s="18" t="n">
-        <v>-105</v>
+        <v>-102</v>
       </c>
       <c r="I8" s="20" t="n">
-        <v>0.5960557431371012</v>
+        <v>0.5927907983721405</v>
       </c>
       <c r="J8" s="20" t="n">
-        <v>0.4891657638136511</v>
+        <v>0.4826358742837298</v>
       </c>
       <c r="K8" s="20" t="n">
-        <v>0.5121951219512195</v>
+        <v>0.504950495049505</v>
       </c>
       <c r="L8" s="19" t="n">
-        <v>0.08386062118588167</v>
+        <v>0.08784030332263559</v>
       </c>
       <c r="M8" s="19" t="n">
-        <v>0.1637278794581499</v>
+        <v>0.1739582477565921</v>
       </c>
       <c r="N8" s="20" t="n">
         <v>0</v>
@@ -1688,12 +1688,12 @@
       </c>
       <c r="B11" s="12" t="inlineStr">
         <is>
-          <t>BCU @ UCF</t>
+          <t>NMSU @ FSU</t>
         </is>
       </c>
       <c r="C11" s="12" t="inlineStr">
         <is>
-          <t>2026-09-03 23:00</t>
+          <t>2026-08-29 23:00</t>
         </is>
       </c>
       <c r="D11" s="22" t="n">
@@ -1706,29 +1706,29 @@
       </c>
       <c r="F11" s="12" t="inlineStr">
         <is>
-          <t>BCU +42.5</t>
+          <t>NMSU +30.5</t>
         </is>
       </c>
       <c r="G11" s="23" t="n">
-        <v>-42.5</v>
+        <v>-30.5</v>
       </c>
       <c r="H11" s="13" t="n">
-        <v>-110</v>
+        <v>-102</v>
       </c>
       <c r="I11" s="15" t="n">
-        <v>0.7495833131506973</v>
+        <v>0.7327748458688852</v>
       </c>
       <c r="J11" s="15" t="n">
-        <v>0.5</v>
+        <v>0.4826358742837298</v>
       </c>
       <c r="K11" s="15" t="n">
-        <v>0.5238095238095238</v>
+        <v>0.504950495049505</v>
       </c>
       <c r="L11" s="14" t="n">
-        <v>0.2257737893411734</v>
+        <v>0.2278243508193802</v>
       </c>
       <c r="M11" s="14" t="n">
-        <v>0.4310226887422403</v>
+        <v>0.4511815575050472</v>
       </c>
       <c r="N11" s="15" t="n">
         <v>0</v>
@@ -1743,7 +1743,7 @@
       </c>
       <c r="Q11" s="12" t="inlineStr">
         <is>
-          <t>BCU isn't a full FBS participant this season — model doesn't rate them reliably</t>
+          <t>raw model/market disagreement exceeds the safety limit</t>
         </is>
       </c>
     </row>
@@ -1755,12 +1755,12 @@
       </c>
       <c r="B12" s="17" t="inlineStr">
         <is>
-          <t>UAPB @ MIZ</t>
+          <t>BCU @ UCF</t>
         </is>
       </c>
       <c r="C12" s="17" t="inlineStr">
         <is>
-          <t>2026-09-04 00:00</t>
+          <t>2026-09-03 23:00</t>
         </is>
       </c>
       <c r="D12" s="25" t="n">
@@ -1773,29 +1773,29 @@
       </c>
       <c r="F12" s="17" t="inlineStr">
         <is>
-          <t>UAPB +54.5</t>
+          <t>BCU +42.5</t>
         </is>
       </c>
       <c r="G12" s="26" t="n">
-        <v>-54.5</v>
+        <v>-42.5</v>
       </c>
       <c r="H12" s="18" t="n">
-        <v>-112</v>
+        <v>-110</v>
       </c>
       <c r="I12" s="20" t="n">
-        <v>0.7521468293620484</v>
+        <v>0.7495833131506973</v>
       </c>
       <c r="J12" s="20" t="n">
-        <v>0.5043297540699688</v>
+        <v>0.5</v>
       </c>
       <c r="K12" s="20" t="n">
-        <v>0.5283018867924528</v>
+        <v>0.5238095238095238</v>
       </c>
       <c r="L12" s="19" t="n">
-        <v>0.2238449425695955</v>
+        <v>0.2257737893411734</v>
       </c>
       <c r="M12" s="19" t="n">
-        <v>0.4237064984353057</v>
+        <v>0.4310226887422403</v>
       </c>
       <c r="N12" s="20" t="n">
         <v>0</v>
@@ -1810,7 +1810,7 @@
       </c>
       <c r="Q12" s="17" t="inlineStr">
         <is>
-          <t>UAPB isn't a full FBS participant this season — model doesn't rate them reliably</t>
+          <t>BCU isn't a full FBS participant this season — model doesn't rate them reliably</t>
         </is>
       </c>
     </row>
@@ -1822,7 +1822,7 @@
       </c>
       <c r="B13" s="12" t="inlineStr">
         <is>
-          <t>EIU @ MINN</t>
+          <t>UAPB @ MIZ</t>
         </is>
       </c>
       <c r="C13" s="12" t="inlineStr">
@@ -1840,17 +1840,17 @@
       </c>
       <c r="F13" s="12" t="inlineStr">
         <is>
-          <t>EIU +43.5</t>
+          <t>UAPB +54.5</t>
         </is>
       </c>
       <c r="G13" s="23" t="n">
-        <v>-43.5</v>
+        <v>-54.5</v>
       </c>
       <c r="H13" s="13" t="n">
         <v>-112</v>
       </c>
       <c r="I13" s="15" t="n">
-        <v>0.7518231737767994</v>
+        <v>0.7521468293620484</v>
       </c>
       <c r="J13" s="15" t="n">
         <v>0.5043297540699688</v>
@@ -1859,10 +1859,10 @@
         <v>0.5283018867924528</v>
       </c>
       <c r="L13" s="14" t="n">
-        <v>0.2235212869843466</v>
+        <v>0.2238449425695955</v>
       </c>
       <c r="M13" s="14" t="n">
-        <v>0.4230938646489417</v>
+        <v>0.4237064984353057</v>
       </c>
       <c r="N13" s="15" t="n">
         <v>0</v>
@@ -1877,7 +1877,7 @@
       </c>
       <c r="Q13" s="12" t="inlineStr">
         <is>
-          <t>EIU isn't a full FBS participant this season — model doesn't rate them reliably</t>
+          <t>UAPB isn't a full FBS participant this season — model doesn't rate them reliably</t>
         </is>
       </c>
     </row>
@@ -1889,12 +1889,12 @@
       </c>
       <c r="B14" s="17" t="inlineStr">
         <is>
-          <t>IDHO @ UTAH</t>
+          <t>EIU @ MINN</t>
         </is>
       </c>
       <c r="C14" s="17" t="inlineStr">
         <is>
-          <t>2026-09-04 01:00</t>
+          <t>2026-09-04 00:00</t>
         </is>
       </c>
       <c r="D14" s="25" t="n">
@@ -1907,29 +1907,29 @@
       </c>
       <c r="F14" s="17" t="inlineStr">
         <is>
-          <t>IDHO +33.5</t>
+          <t>EIU +43.5</t>
         </is>
       </c>
       <c r="G14" s="26" t="n">
-        <v>-33.5</v>
+        <v>-43.5</v>
       </c>
       <c r="H14" s="18" t="n">
-        <v>-110</v>
+        <v>-112</v>
       </c>
       <c r="I14" s="20" t="n">
-        <v>0.7436440297876288</v>
+        <v>0.7518231737767994</v>
       </c>
       <c r="J14" s="20" t="n">
-        <v>0.5</v>
+        <v>0.5043297540699688</v>
       </c>
       <c r="K14" s="20" t="n">
-        <v>0.5238095238095238</v>
+        <v>0.5283018867924528</v>
       </c>
       <c r="L14" s="19" t="n">
-        <v>0.2198345059781049</v>
+        <v>0.2235212869843466</v>
       </c>
       <c r="M14" s="19" t="n">
-        <v>0.4196840568672914</v>
+        <v>0.4230938646489417</v>
       </c>
       <c r="N14" s="20" t="n">
         <v>0</v>
@@ -1944,7 +1944,7 @@
       </c>
       <c r="Q14" s="17" t="inlineStr">
         <is>
-          <t>IDHO isn't a full FBS participant this season — model doesn't rate them reliably</t>
+          <t>EIU isn't a full FBS participant this season — model doesn't rate them reliably</t>
         </is>
       </c>
     </row>
@@ -1956,12 +1956,12 @@
       </c>
       <c r="B15" s="12" t="inlineStr">
         <is>
-          <t>MRMK @ DEL</t>
+          <t>IDHO @ UTAH</t>
         </is>
       </c>
       <c r="C15" s="12" t="inlineStr">
         <is>
-          <t>2026-09-03 23:00</t>
+          <t>2026-09-04 01:00</t>
         </is>
       </c>
       <c r="D15" s="22" t="n">
@@ -1974,29 +1974,29 @@
       </c>
       <c r="F15" s="12" t="inlineStr">
         <is>
-          <t>MRMK +28.5</t>
+          <t>IDHO +33.5</t>
         </is>
       </c>
       <c r="G15" s="23" t="n">
-        <v>-28.5</v>
+        <v>-33.5</v>
       </c>
       <c r="H15" s="13" t="n">
-        <v>-108</v>
+        <v>-110</v>
       </c>
       <c r="I15" s="15" t="n">
-        <v>0.7386849373798826</v>
+        <v>0.7436440297876288</v>
       </c>
       <c r="J15" s="15" t="n">
-        <v>0.4956702459300312</v>
+        <v>0.5</v>
       </c>
       <c r="K15" s="15" t="n">
-        <v>0.5192307692307693</v>
+        <v>0.5238095238095238</v>
       </c>
       <c r="L15" s="14" t="n">
-        <v>0.2194541681491133</v>
+        <v>0.2198345059781049</v>
       </c>
       <c r="M15" s="14" t="n">
-        <v>0.4226524719908851</v>
+        <v>0.4196840568672914</v>
       </c>
       <c r="N15" s="15" t="n">
         <v>0</v>
@@ -2011,7 +2011,7 @@
       </c>
       <c r="Q15" s="12" t="inlineStr">
         <is>
-          <t>MRMK isn't a full FBS participant this season — model doesn't rate them reliably</t>
+          <t>IDHO isn't a full FBS participant this season — model doesn't rate them reliably</t>
         </is>
       </c>
     </row>
@@ -2023,12 +2023,12 @@
       </c>
       <c r="B16" s="17" t="inlineStr">
         <is>
-          <t>MASS @ RUTG</t>
+          <t>MRMK @ DEL</t>
         </is>
       </c>
       <c r="C16" s="17" t="inlineStr">
         <is>
-          <t>2026-09-03 22:00</t>
+          <t>2026-09-03 23:00</t>
         </is>
       </c>
       <c r="D16" s="25" t="n">
@@ -2041,29 +2041,29 @@
       </c>
       <c r="F16" s="17" t="inlineStr">
         <is>
-          <t>MASS +29.5</t>
+          <t>MRMK +28.5</t>
         </is>
       </c>
       <c r="G16" s="26" t="n">
-        <v>-29.5</v>
+        <v>-28.5</v>
       </c>
       <c r="H16" s="18" t="n">
-        <v>-105</v>
+        <v>-108</v>
       </c>
       <c r="I16" s="20" t="n">
-        <v>0.7307755149318647</v>
+        <v>0.7386849373798826</v>
       </c>
       <c r="J16" s="20" t="n">
-        <v>0.4891657638136511</v>
+        <v>0.4956702459300312</v>
       </c>
       <c r="K16" s="20" t="n">
-        <v>0.5121951219512195</v>
+        <v>0.5192307692307693</v>
       </c>
       <c r="L16" s="19" t="n">
-        <v>0.2185803929806451</v>
+        <v>0.2194541681491133</v>
       </c>
       <c r="M16" s="19" t="n">
-        <v>0.4267521958193548</v>
+        <v>0.4226524719908851</v>
       </c>
       <c r="N16" s="20" t="n">
         <v>0</v>
@@ -2078,7 +2078,7 @@
       </c>
       <c r="Q16" s="17" t="inlineStr">
         <is>
-          <t>raw model/market disagreement exceeds the safety limit</t>
+          <t>MRMK isn't a full FBS participant this season — model doesn't rate them reliably</t>
         </is>
       </c>
     </row>
@@ -2090,12 +2090,12 @@
       </c>
       <c r="B17" s="12" t="inlineStr">
         <is>
-          <t>SJSU @ USC</t>
+          <t>MASS @ RUTG</t>
         </is>
       </c>
       <c r="C17" s="12" t="inlineStr">
         <is>
-          <t>2026-08-29 19:00</t>
+          <t>2026-09-03 22:00</t>
         </is>
       </c>
       <c r="D17" s="22" t="n">
@@ -2108,29 +2108,29 @@
       </c>
       <c r="F17" s="12" t="inlineStr">
         <is>
-          <t>SJSU +38.5</t>
+          <t>MASS +29.5</t>
         </is>
       </c>
       <c r="G17" s="23" t="n">
-        <v>-38.5</v>
+        <v>-29.5</v>
       </c>
       <c r="H17" s="13" t="n">
-        <v>-115</v>
+        <v>-105</v>
       </c>
       <c r="I17" s="15" t="n">
-        <v>0.7530960341419698</v>
+        <v>0.7307755149318647</v>
       </c>
       <c r="J17" s="15" t="n">
-        <v>0.5108342361863488</v>
+        <v>0.4891657638136511</v>
       </c>
       <c r="K17" s="15" t="n">
-        <v>0.5348837209302325</v>
+        <v>0.5121951219512195</v>
       </c>
       <c r="L17" s="14" t="n">
-        <v>0.2182123132117373</v>
+        <v>0.2185803929806451</v>
       </c>
       <c r="M17" s="14" t="n">
-        <v>0.4079621507871608</v>
+        <v>0.4267521958193548</v>
       </c>
       <c r="N17" s="15" t="n">
         <v>0</v>
@@ -2157,12 +2157,12 @@
       </c>
       <c r="B18" s="17" t="inlineStr">
         <is>
-          <t>NCAT @ GAST</t>
+          <t>SJSU @ USC</t>
         </is>
       </c>
       <c r="C18" s="17" t="inlineStr">
         <is>
-          <t>2026-09-04 23:00</t>
+          <t>2026-08-29 19:00</t>
         </is>
       </c>
       <c r="D18" s="25" t="n">
@@ -2175,29 +2175,29 @@
       </c>
       <c r="F18" s="17" t="inlineStr">
         <is>
-          <t>NCAT +28.5</t>
+          <t>SJSU +38.5</t>
         </is>
       </c>
       <c r="G18" s="26" t="n">
-        <v>-28.5</v>
+        <v>-38.5</v>
       </c>
       <c r="H18" s="18" t="n">
-        <v>-112</v>
+        <v>-115</v>
       </c>
       <c r="I18" s="20" t="n">
-        <v>0.7452866315143292</v>
+        <v>0.7530960341419698</v>
       </c>
       <c r="J18" s="20" t="n">
-        <v>0.5043297540699688</v>
+        <v>0.5108342361863488</v>
       </c>
       <c r="K18" s="20" t="n">
-        <v>0.5283018867924528</v>
+        <v>0.5348837209302325</v>
       </c>
       <c r="L18" s="19" t="n">
-        <v>0.2169847447218763</v>
+        <v>0.2182123132117373</v>
       </c>
       <c r="M18" s="19" t="n">
-        <v>0.4107211239378373</v>
+        <v>0.4079621507871608</v>
       </c>
       <c r="N18" s="20" t="n">
         <v>0</v>
@@ -2212,7 +2212,7 @@
       </c>
       <c r="Q18" s="17" t="inlineStr">
         <is>
-          <t>NCAT isn't a full FBS participant this season — model doesn't rate them reliably</t>
+          <t>raw model/market disagreement exceeds the safety limit</t>
         </is>
       </c>
     </row>
@@ -2224,12 +2224,12 @@
       </c>
       <c r="B19" s="12" t="inlineStr">
         <is>
-          <t>NMSU @ FSU</t>
+          <t>NCAT @ GAST</t>
         </is>
       </c>
       <c r="C19" s="12" t="inlineStr">
         <is>
-          <t>2026-08-29 23:00</t>
+          <t>2026-09-04 23:00</t>
         </is>
       </c>
       <c r="D19" s="22" t="n">
@@ -2242,29 +2242,29 @@
       </c>
       <c r="F19" s="12" t="inlineStr">
         <is>
-          <t>NMSU +31.5</t>
+          <t>NCAT +28.5</t>
         </is>
       </c>
       <c r="G19" s="23" t="n">
-        <v>-31.5</v>
+        <v>-28.5</v>
       </c>
       <c r="H19" s="13" t="n">
-        <v>-115</v>
+        <v>-112</v>
       </c>
       <c r="I19" s="15" t="n">
-        <v>0.7484052544756881</v>
+        <v>0.7452866315143292</v>
       </c>
       <c r="J19" s="15" t="n">
-        <v>0.5108342361863488</v>
+        <v>0.5043297540699688</v>
       </c>
       <c r="K19" s="15" t="n">
-        <v>0.5348837209302325</v>
+        <v>0.5283018867924528</v>
       </c>
       <c r="L19" s="14" t="n">
-        <v>0.2135215335454556</v>
+        <v>0.2169847447218763</v>
       </c>
       <c r="M19" s="14" t="n">
-        <v>0.3991924322806341</v>
+        <v>0.4107211239378373</v>
       </c>
       <c r="N19" s="15" t="n">
         <v>0</v>
@@ -2279,7 +2279,7 @@
       </c>
       <c r="Q19" s="12" t="inlineStr">
         <is>
-          <t>raw model/market disagreement exceeds the safety limit</t>
+          <t>NCAT isn't a full FBS participant this season — model doesn't rate them reliably</t>
         </is>
       </c>
     </row>
@@ -3569,22 +3569,22 @@
       </c>
       <c r="G39" s="23" t="n"/>
       <c r="H39" s="13" t="n">
-        <v>245</v>
+        <v>250</v>
       </c>
       <c r="I39" s="15" t="n">
-        <v>0.3639656274205685</v>
+        <v>0.3621290026789783</v>
       </c>
       <c r="J39" s="15" t="n">
-        <v>0.2779207411219763</v>
+        <v>0.274247491638796</v>
       </c>
       <c r="K39" s="15" t="n">
-        <v>0.2898550724637681</v>
+        <v>0.2857142857142857</v>
       </c>
       <c r="L39" s="14" t="n">
-        <v>0.07411055495680036</v>
+        <v>0.0764147169646926</v>
       </c>
       <c r="M39" s="14" t="n">
-        <v>0.2556814146009613</v>
+        <v>0.267451509376424</v>
       </c>
       <c r="N39" s="15" t="n">
         <v>0</v>
@@ -4121,12 +4121,12 @@
       </c>
       <c r="B48" s="17" t="inlineStr">
         <is>
-          <t>NMSU @ FSU</t>
+          <t>NCSU @ UVA</t>
         </is>
       </c>
       <c r="C48" s="17" t="inlineStr">
         <is>
-          <t>2026-08-29 23:00</t>
+          <t>2026-08-29 19:30</t>
         </is>
       </c>
       <c r="D48" s="25" t="n">
@@ -4134,34 +4134,34 @@
       </c>
       <c r="E48" s="17" t="inlineStr">
         <is>
-          <t>TOTAL</t>
+          <t>ATS</t>
         </is>
       </c>
       <c r="F48" s="17" t="inlineStr">
         <is>
-          <t>Over 52.5</t>
+          <t>NCSU +5.5</t>
         </is>
       </c>
       <c r="G48" s="26" t="n">
-        <v>52.5</v>
+        <v>-5.5</v>
       </c>
       <c r="H48" s="18" t="n">
-        <v>-108</v>
+        <v>-105</v>
       </c>
       <c r="I48" s="20" t="n">
-        <v>0.5472084462676521</v>
+        <v>0.5380374278212803</v>
       </c>
       <c r="J48" s="20" t="n">
-        <v>0.4956702459300312</v>
+        <v>0.4891657638136511</v>
       </c>
       <c r="K48" s="20" t="n">
-        <v>0.5192307692307693</v>
+        <v>0.5121951219512195</v>
       </c>
       <c r="L48" s="19" t="n">
-        <v>0.02797767703688281</v>
+        <v>0.02584230587006076</v>
       </c>
       <c r="M48" s="19" t="n">
-        <v>0.05388293355251517</v>
+        <v>0.05045402574630908</v>
       </c>
       <c r="N48" s="20" t="n">
         <v>0</v>
@@ -4184,12 +4184,12 @@
       </c>
       <c r="B49" s="12" t="inlineStr">
         <is>
-          <t>NCSU @ UVA</t>
+          <t>COLO @ GT</t>
         </is>
       </c>
       <c r="C49" s="12" t="inlineStr">
         <is>
-          <t>2026-08-29 19:30</t>
+          <t>2026-09-04 00:00</t>
         </is>
       </c>
       <c r="D49" s="22" t="n">
@@ -4202,17 +4202,17 @@
       </c>
       <c r="F49" s="12" t="inlineStr">
         <is>
-          <t>NCSU +5.5</t>
+          <t>COLO +6.5</t>
         </is>
       </c>
       <c r="G49" s="23" t="n">
-        <v>-5.5</v>
+        <v>-6.5</v>
       </c>
       <c r="H49" s="13" t="n">
         <v>-105</v>
       </c>
       <c r="I49" s="15" t="n">
-        <v>0.5380374278212803</v>
+        <v>0.5359459352051367</v>
       </c>
       <c r="J49" s="15" t="n">
         <v>0.4891657638136511</v>
@@ -4221,10 +4221,10 @@
         <v>0.5121951219512195</v>
       </c>
       <c r="L49" s="14" t="n">
-        <v>0.02584230587006076</v>
+        <v>0.02375081325391715</v>
       </c>
       <c r="M49" s="14" t="n">
-        <v>0.05045402574630908</v>
+        <v>0.0463706354005049</v>
       </c>
       <c r="N49" s="15" t="n">
         <v>0</v>
@@ -4247,12 +4247,12 @@
       </c>
       <c r="B50" s="17" t="inlineStr">
         <is>
-          <t>COLO @ GT</t>
+          <t>NMSU @ FSU</t>
         </is>
       </c>
       <c r="C50" s="17" t="inlineStr">
         <is>
-          <t>2026-09-04 00:00</t>
+          <t>2026-08-29 23:00</t>
         </is>
       </c>
       <c r="D50" s="25" t="n">
@@ -4260,34 +4260,34 @@
       </c>
       <c r="E50" s="17" t="inlineStr">
         <is>
-          <t>ATS</t>
+          <t>TOTAL</t>
         </is>
       </c>
       <c r="F50" s="17" t="inlineStr">
         <is>
-          <t>COLO +6.5</t>
+          <t>Over 52.5</t>
         </is>
       </c>
       <c r="G50" s="26" t="n">
-        <v>-6.5</v>
+        <v>52.5</v>
       </c>
       <c r="H50" s="18" t="n">
-        <v>-105</v>
+        <v>-112</v>
       </c>
       <c r="I50" s="20" t="n">
-        <v>0.5359459352051367</v>
+        <v>0.5515382003376208</v>
       </c>
       <c r="J50" s="20" t="n">
-        <v>0.4891657638136511</v>
+        <v>0.5043297540699688</v>
       </c>
       <c r="K50" s="20" t="n">
-        <v>0.5121951219512195</v>
+        <v>0.5283018867924528</v>
       </c>
       <c r="L50" s="19" t="n">
-        <v>0.02375081325391715</v>
+        <v>0.02323631354516797</v>
       </c>
       <c r="M50" s="19" t="n">
-        <v>0.0463706354005049</v>
+        <v>0.04398302206763932</v>
       </c>
       <c r="N50" s="20" t="n">
         <v>0</v>
@@ -4686,12 +4686,12 @@
       </c>
       <c r="B57" s="12" t="inlineStr">
         <is>
-          <t>SJSU @ EMU</t>
+          <t>MEM @ UNLV</t>
         </is>
       </c>
       <c r="C57" s="12" t="inlineStr">
         <is>
-          <t>2026-09-04 22:30</t>
+          <t>2026-08-30 02:00</t>
         </is>
       </c>
       <c r="D57" s="22" t="n">
@@ -4699,34 +4699,32 @@
       </c>
       <c r="E57" s="12" t="inlineStr">
         <is>
-          <t>ATS</t>
+          <t>ML</t>
         </is>
       </c>
       <c r="F57" s="12" t="inlineStr">
         <is>
-          <t>SJSU +4.5</t>
-        </is>
-      </c>
-      <c r="G57" s="23" t="n">
-        <v>-4.5</v>
-      </c>
+          <t>MEM ML</t>
+        </is>
+      </c>
+      <c r="G57" s="23" t="n"/>
       <c r="H57" s="13" t="n">
-        <v>-105</v>
+        <v>164</v>
       </c>
       <c r="I57" s="15" t="n">
-        <v>0.5253691652874209</v>
+        <v>0.3933214139392706</v>
       </c>
       <c r="J57" s="15" t="n">
-        <v>0.4891657638136511</v>
+        <v>0.3630958183058778</v>
       </c>
       <c r="K57" s="15" t="n">
-        <v>0.5121951219512195</v>
+        <v>0.3787878787878788</v>
       </c>
       <c r="L57" s="14" t="n">
-        <v>0.01317404333620142</v>
+        <v>0.01453353515139177</v>
       </c>
       <c r="M57" s="14" t="n">
-        <v>0.02572075127544082</v>
+        <v>0.03836853279967412</v>
       </c>
       <c r="N57" s="15" t="n">
         <v>0</v>
@@ -4749,12 +4747,12 @@
       </c>
       <c r="B58" s="17" t="inlineStr">
         <is>
-          <t>MEM @ UNLV</t>
+          <t>UNC @ TCU</t>
         </is>
       </c>
       <c r="C58" s="17" t="inlineStr">
         <is>
-          <t>2026-08-30 02:00</t>
+          <t>2026-08-29 16:00</t>
         </is>
       </c>
       <c r="D58" s="25" t="n">
@@ -4762,32 +4760,34 @@
       </c>
       <c r="E58" s="17" t="inlineStr">
         <is>
-          <t>ML</t>
+          <t>TOTAL</t>
         </is>
       </c>
       <c r="F58" s="17" t="inlineStr">
         <is>
-          <t>MEM ML</t>
-        </is>
-      </c>
-      <c r="G58" s="26" t="n"/>
+          <t>Over 47.5</t>
+        </is>
+      </c>
+      <c r="G58" s="26" t="n">
+        <v>47.5</v>
+      </c>
       <c r="H58" s="18" t="n">
-        <v>160</v>
+        <v>-110</v>
       </c>
       <c r="I58" s="20" t="n">
-        <v>0.396303332895533</v>
+        <v>0.5376883257015108</v>
       </c>
       <c r="J58" s="20" t="n">
-        <v>0.3690596562184025</v>
+        <v>0.5</v>
       </c>
       <c r="K58" s="20" t="n">
-        <v>0.3846153846153846</v>
+        <v>0.5238095238095238</v>
       </c>
       <c r="L58" s="19" t="n">
-        <v>0.01168794828014835</v>
+        <v>0.01387880189198698</v>
       </c>
       <c r="M58" s="19" t="n">
-        <v>0.03038866552838582</v>
+        <v>0.02649589452106615</v>
       </c>
       <c r="N58" s="20" t="n">
         <v>0</v>
@@ -4810,12 +4810,12 @@
       </c>
       <c r="B59" s="12" t="inlineStr">
         <is>
-          <t>UNC @ TCU</t>
+          <t>SJSU @ EMU</t>
         </is>
       </c>
       <c r="C59" s="12" t="inlineStr">
         <is>
-          <t>2026-08-29 16:00</t>
+          <t>2026-09-04 22:30</t>
         </is>
       </c>
       <c r="D59" s="22" t="n">
@@ -4823,34 +4823,34 @@
       </c>
       <c r="E59" s="12" t="inlineStr">
         <is>
-          <t>TOTAL</t>
+          <t>ATS</t>
         </is>
       </c>
       <c r="F59" s="12" t="inlineStr">
         <is>
-          <t>Over 47.5</t>
+          <t>SJSU +4.5</t>
         </is>
       </c>
       <c r="G59" s="23" t="n">
-        <v>47.5</v>
+        <v>-4.5</v>
       </c>
       <c r="H59" s="13" t="n">
-        <v>-112</v>
+        <v>-105</v>
       </c>
       <c r="I59" s="15" t="n">
-        <v>0.5398532027364953</v>
+        <v>0.5253691652874209</v>
       </c>
       <c r="J59" s="15" t="n">
-        <v>0.5043297540699688</v>
+        <v>0.4891657638136511</v>
       </c>
       <c r="K59" s="15" t="n">
-        <v>0.5283018867924528</v>
+        <v>0.5121951219512195</v>
       </c>
       <c r="L59" s="14" t="n">
-        <v>0.01155131594404246</v>
+        <v>0.01317404333620142</v>
       </c>
       <c r="M59" s="14" t="n">
-        <v>0.02186499089408034</v>
+        <v>0.02572075127544082</v>
       </c>
       <c r="N59" s="15" t="n">
         <v>0</v>
@@ -5580,12 +5580,12 @@
       </c>
       <c r="B71" s="12" t="inlineStr">
         <is>
-          <t>MEM @ UNLV</t>
+          <t>JVST @ NDSU</t>
         </is>
       </c>
       <c r="C71" s="12" t="inlineStr">
         <is>
-          <t>2026-08-30 02:00</t>
+          <t>2026-08-29 21:30</t>
         </is>
       </c>
       <c r="D71" s="22" t="n">
@@ -5598,27 +5598,27 @@
       </c>
       <c r="F71" s="12" t="inlineStr">
         <is>
-          <t>UNLV ML</t>
+          <t>NDSU ML</t>
         </is>
       </c>
       <c r="G71" s="23" t="n"/>
       <c r="H71" s="13" t="n">
-        <v>-192</v>
+        <v>-265</v>
       </c>
       <c r="I71" s="15" t="n">
-        <v>0.603696667104467</v>
+        <v>0.6716849259288671</v>
       </c>
       <c r="J71" s="15" t="n">
-        <v>0.6309403437815976</v>
+        <v>0.6957699520733487</v>
       </c>
       <c r="K71" s="15" t="n">
-        <v>0.6575342465753424</v>
+        <v>0.726027397260274</v>
       </c>
       <c r="L71" s="14" t="n">
-        <v>-0.05383757947087542</v>
+        <v>-0.05434247133140691</v>
       </c>
       <c r="M71" s="14" t="n">
-        <v>-0.08187798544528968</v>
+        <v>-0.07484906428665483</v>
       </c>
       <c r="N71" s="15" t="n">
         <v>0</v>
@@ -5641,12 +5641,12 @@
       </c>
       <c r="B72" s="17" t="inlineStr">
         <is>
-          <t>JVST @ NDSU</t>
+          <t>MEM @ UNLV</t>
         </is>
       </c>
       <c r="C72" s="17" t="inlineStr">
         <is>
-          <t>2026-08-29 21:30</t>
+          <t>2026-08-30 02:00</t>
         </is>
       </c>
       <c r="D72" s="25" t="n">
@@ -5659,27 +5659,27 @@
       </c>
       <c r="F72" s="17" t="inlineStr">
         <is>
-          <t>NDSU ML</t>
+          <t>UNLV ML</t>
         </is>
       </c>
       <c r="G72" s="26" t="n"/>
       <c r="H72" s="18" t="n">
-        <v>-265</v>
+        <v>-198</v>
       </c>
       <c r="I72" s="20" t="n">
-        <v>0.6716849259288671</v>
+        <v>0.6066785860607294</v>
       </c>
       <c r="J72" s="20" t="n">
-        <v>0.6957699520733487</v>
+        <v>0.6369041816941223</v>
       </c>
       <c r="K72" s="20" t="n">
-        <v>0.726027397260274</v>
+        <v>0.6644295302013423</v>
       </c>
       <c r="L72" s="19" t="n">
-        <v>-0.05434247133140691</v>
+        <v>-0.05775094414061288</v>
       </c>
       <c r="M72" s="19" t="n">
-        <v>-0.07484906428665483</v>
+        <v>-0.08691808764597275</v>
       </c>
       <c r="N72" s="20" t="n">
         <v>0</v>
@@ -5763,12 +5763,12 @@
       </c>
       <c r="B74" s="17" t="inlineStr">
         <is>
-          <t>UNC @ TCU</t>
+          <t>SJSU @ EMU</t>
         </is>
       </c>
       <c r="C74" s="17" t="inlineStr">
         <is>
-          <t>2026-08-29 16:00</t>
+          <t>2026-09-04 22:30</t>
         </is>
       </c>
       <c r="D74" s="25" t="n">
@@ -5776,34 +5776,32 @@
       </c>
       <c r="E74" s="17" t="inlineStr">
         <is>
-          <t>TOTAL</t>
+          <t>ML</t>
         </is>
       </c>
       <c r="F74" s="17" t="inlineStr">
         <is>
-          <t>Under 47.5</t>
-        </is>
-      </c>
-      <c r="G74" s="26" t="n">
-        <v>47.5</v>
-      </c>
+          <t>EMU ML</t>
+        </is>
+      </c>
+      <c r="G74" s="26" t="n"/>
       <c r="H74" s="18" t="n">
-        <v>-108</v>
+        <v>-218</v>
       </c>
       <c r="I74" s="20" t="n">
-        <v>0.4601467972635047</v>
+        <v>0.6258400393716101</v>
       </c>
       <c r="J74" s="20" t="n">
-        <v>0.4956702459300312</v>
+        <v>0.6574752261956054</v>
       </c>
       <c r="K74" s="20" t="n">
-        <v>0.5192307692307693</v>
+        <v>0.6855345911949685</v>
       </c>
       <c r="L74" s="19" t="n">
-        <v>-0.05908397196726456</v>
+        <v>-0.05969455182335837</v>
       </c>
       <c r="M74" s="19" t="n">
-        <v>-0.1137913534184353</v>
+        <v>-0.08707737376067881</v>
       </c>
       <c r="N74" s="20" t="n">
         <v>0</v>
@@ -5826,12 +5824,12 @@
       </c>
       <c r="B75" s="12" t="inlineStr">
         <is>
-          <t>SJSU @ EMU</t>
+          <t>NCSU @ UVA</t>
         </is>
       </c>
       <c r="C75" s="12" t="inlineStr">
         <is>
-          <t>2026-09-04 22:30</t>
+          <t>2026-08-29 19:30</t>
         </is>
       </c>
       <c r="D75" s="22" t="n">
@@ -5844,7 +5842,7 @@
       </c>
       <c r="F75" s="12" t="inlineStr">
         <is>
-          <t>EMU ML</t>
+          <t>UVA ML</t>
         </is>
       </c>
       <c r="G75" s="23" t="n"/>
@@ -5852,7 +5850,7 @@
         <v>-218</v>
       </c>
       <c r="I75" s="15" t="n">
-        <v>0.6258400393716101</v>
+        <v>0.6254192861725905</v>
       </c>
       <c r="J75" s="15" t="n">
         <v>0.6574752261956054</v>
@@ -5861,10 +5859,10 @@
         <v>0.6855345911949685</v>
       </c>
       <c r="L75" s="14" t="n">
-        <v>-0.05969455182335837</v>
+        <v>-0.06011530502237805</v>
       </c>
       <c r="M75" s="14" t="n">
-        <v>-0.08707737376067881</v>
+        <v>-0.08769113301429471</v>
       </c>
       <c r="N75" s="15" t="n">
         <v>0</v>
@@ -5887,12 +5885,12 @@
       </c>
       <c r="B76" s="17" t="inlineStr">
         <is>
-          <t>NCSU @ UVA</t>
+          <t>SJSU @ EMU</t>
         </is>
       </c>
       <c r="C76" s="17" t="inlineStr">
         <is>
-          <t>2026-08-29 19:30</t>
+          <t>2026-09-04 22:30</t>
         </is>
       </c>
       <c r="D76" s="25" t="n">
@@ -5900,32 +5898,34 @@
       </c>
       <c r="E76" s="17" t="inlineStr">
         <is>
-          <t>ML</t>
+          <t>ATS</t>
         </is>
       </c>
       <c r="F76" s="17" t="inlineStr">
         <is>
-          <t>UVA ML</t>
-        </is>
-      </c>
-      <c r="G76" s="26" t="n"/>
+          <t>EMU -4.5</t>
+        </is>
+      </c>
+      <c r="G76" s="26" t="n">
+        <v>-4.5</v>
+      </c>
       <c r="H76" s="18" t="n">
-        <v>-218</v>
+        <v>-115</v>
       </c>
       <c r="I76" s="20" t="n">
-        <v>0.6254192861725905</v>
+        <v>0.4746308347125791</v>
       </c>
       <c r="J76" s="20" t="n">
-        <v>0.6574752261956054</v>
+        <v>0.5108342361863488</v>
       </c>
       <c r="K76" s="20" t="n">
-        <v>0.6855345911949685</v>
+        <v>0.5348837209302325</v>
       </c>
       <c r="L76" s="19" t="n">
-        <v>-0.06011530502237805</v>
+        <v>-0.06025288621765346</v>
       </c>
       <c r="M76" s="19" t="n">
-        <v>-0.08769113301429471</v>
+        <v>-0.112646700319961</v>
       </c>
       <c r="N76" s="20" t="n">
         <v>0</v>
@@ -5948,12 +5948,12 @@
       </c>
       <c r="B77" s="12" t="inlineStr">
         <is>
-          <t>SJSU @ EMU</t>
+          <t>UNC @ TCU</t>
         </is>
       </c>
       <c r="C77" s="12" t="inlineStr">
         <is>
-          <t>2026-09-04 22:30</t>
+          <t>2026-08-29 16:00</t>
         </is>
       </c>
       <c r="D77" s="22" t="n">
@@ -5961,34 +5961,34 @@
       </c>
       <c r="E77" s="12" t="inlineStr">
         <is>
-          <t>ATS</t>
+          <t>TOTAL</t>
         </is>
       </c>
       <c r="F77" s="12" t="inlineStr">
         <is>
-          <t>EMU -4.5</t>
+          <t>Under 47.5</t>
         </is>
       </c>
       <c r="G77" s="23" t="n">
-        <v>-4.5</v>
+        <v>47.5</v>
       </c>
       <c r="H77" s="13" t="n">
-        <v>-115</v>
+        <v>-110</v>
       </c>
       <c r="I77" s="15" t="n">
-        <v>0.4746308347125791</v>
+        <v>0.4623116742984892</v>
       </c>
       <c r="J77" s="15" t="n">
-        <v>0.5108342361863488</v>
+        <v>0.5</v>
       </c>
       <c r="K77" s="15" t="n">
-        <v>0.5348837209302325</v>
+        <v>0.5238095238095238</v>
       </c>
       <c r="L77" s="14" t="n">
-        <v>-0.06025288621765346</v>
+        <v>-0.06149784951103465</v>
       </c>
       <c r="M77" s="14" t="n">
-        <v>-0.112646700319961</v>
+        <v>-0.117404985430157</v>
       </c>
       <c r="N77" s="15" t="n">
         <v>0</v>
@@ -6204,12 +6204,12 @@
       </c>
       <c r="B81" s="12" t="inlineStr">
         <is>
-          <t>COLO @ GT</t>
+          <t>NMSU @ FSU</t>
         </is>
       </c>
       <c r="C81" s="12" t="inlineStr">
         <is>
-          <t>2026-09-04 00:00</t>
+          <t>2026-08-29 23:00</t>
         </is>
       </c>
       <c r="D81" s="22" t="n">
@@ -6217,34 +6217,34 @@
       </c>
       <c r="E81" s="12" t="inlineStr">
         <is>
-          <t>ATS</t>
+          <t>TOTAL</t>
         </is>
       </c>
       <c r="F81" s="12" t="inlineStr">
         <is>
-          <t>GT -6.5</t>
+          <t>Under 52.5</t>
         </is>
       </c>
       <c r="G81" s="23" t="n">
-        <v>-6.5</v>
+        <v>52.5</v>
       </c>
       <c r="H81" s="13" t="n">
-        <v>-115</v>
+        <v>-108</v>
       </c>
       <c r="I81" s="15" t="n">
-        <v>0.4640540647948633</v>
+        <v>0.4484617996623792</v>
       </c>
       <c r="J81" s="15" t="n">
-        <v>0.5108342361863488</v>
+        <v>0.4956702459300312</v>
       </c>
       <c r="K81" s="15" t="n">
-        <v>0.5348837209302325</v>
+        <v>0.5192307692307693</v>
       </c>
       <c r="L81" s="14" t="n">
-        <v>-0.07082965613536918</v>
+        <v>-0.07076896956839007</v>
       </c>
       <c r="M81" s="14" t="n">
-        <v>-0.132420661470473</v>
+        <v>-0.1362957932428252</v>
       </c>
       <c r="N81" s="15" t="n">
         <v>0</v>
@@ -6267,12 +6267,12 @@
       </c>
       <c r="B82" s="17" t="inlineStr">
         <is>
-          <t>NCSU @ UVA</t>
+          <t>COLO @ GT</t>
         </is>
       </c>
       <c r="C82" s="17" t="inlineStr">
         <is>
-          <t>2026-08-29 19:30</t>
+          <t>2026-09-04 00:00</t>
         </is>
       </c>
       <c r="D82" s="25" t="n">
@@ -6285,17 +6285,17 @@
       </c>
       <c r="F82" s="17" t="inlineStr">
         <is>
-          <t>UVA -5.5</t>
+          <t>GT -6.5</t>
         </is>
       </c>
       <c r="G82" s="26" t="n">
-        <v>-5.5</v>
+        <v>-6.5</v>
       </c>
       <c r="H82" s="18" t="n">
         <v>-115</v>
       </c>
       <c r="I82" s="20" t="n">
-        <v>0.4619625721787197</v>
+        <v>0.4640540647948633</v>
       </c>
       <c r="J82" s="20" t="n">
         <v>0.5108342361863488</v>
@@ -6304,10 +6304,10 @@
         <v>0.5348837209302325</v>
       </c>
       <c r="L82" s="19" t="n">
-        <v>-0.07292114875151279</v>
+        <v>-0.07082965613536918</v>
       </c>
       <c r="M82" s="19" t="n">
-        <v>-0.1363308433180458</v>
+        <v>-0.132420661470473</v>
       </c>
       <c r="N82" s="20" t="n">
         <v>0</v>
@@ -6330,12 +6330,12 @@
       </c>
       <c r="B83" s="12" t="inlineStr">
         <is>
-          <t>NMSU @ FSU</t>
+          <t>NCSU @ UVA</t>
         </is>
       </c>
       <c r="C83" s="12" t="inlineStr">
         <is>
-          <t>2026-08-29 23:00</t>
+          <t>2026-08-29 19:30</t>
         </is>
       </c>
       <c r="D83" s="22" t="n">
@@ -6343,34 +6343,34 @@
       </c>
       <c r="E83" s="12" t="inlineStr">
         <is>
-          <t>TOTAL</t>
+          <t>ATS</t>
         </is>
       </c>
       <c r="F83" s="12" t="inlineStr">
         <is>
-          <t>Under 52.5</t>
+          <t>UVA -5.5</t>
         </is>
       </c>
       <c r="G83" s="23" t="n">
-        <v>52.5</v>
+        <v>-5.5</v>
       </c>
       <c r="H83" s="13" t="n">
-        <v>-112</v>
+        <v>-115</v>
       </c>
       <c r="I83" s="15" t="n">
-        <v>0.4527915537323479</v>
+        <v>0.4619625721787197</v>
       </c>
       <c r="J83" s="15" t="n">
-        <v>0.5043297540699688</v>
+        <v>0.5108342361863488</v>
       </c>
       <c r="K83" s="15" t="n">
-        <v>0.5283018867924528</v>
+        <v>0.5348837209302325</v>
       </c>
       <c r="L83" s="14" t="n">
-        <v>-0.07551033306010491</v>
+        <v>-0.07292114875151279</v>
       </c>
       <c r="M83" s="14" t="n">
-        <v>-0.1429302732923415</v>
+        <v>-0.1363308433180458</v>
       </c>
       <c r="N83" s="15" t="n">
         <v>0</v>
@@ -6863,22 +6863,22 @@
       </c>
       <c r="G91" s="23" t="n"/>
       <c r="H91" s="13" t="n">
-        <v>-305</v>
+        <v>-310</v>
       </c>
       <c r="I91" s="15" t="n">
-        <v>0.6360343725794315</v>
+        <v>0.6378709973210217</v>
       </c>
       <c r="J91" s="15" t="n">
-        <v>0.7220792588780237</v>
+        <v>0.725752508361204</v>
       </c>
       <c r="K91" s="15" t="n">
-        <v>0.7530864197530864</v>
+        <v>0.7560975609756098</v>
       </c>
       <c r="L91" s="14" t="n">
-        <v>-0.1170520471736549</v>
+        <v>-0.1182265636545881</v>
       </c>
       <c r="M91" s="14" t="n">
-        <v>-0.1554297675584598</v>
+        <v>-0.1563641648334875</v>
       </c>
       <c r="N91" s="15" t="n">
         <v>0</v>
@@ -7161,12 +7161,12 @@
       </c>
       <c r="B96" s="17" t="inlineStr">
         <is>
-          <t>UNC @ TCU</t>
+          <t>NCAT @ GAST</t>
         </is>
       </c>
       <c r="C96" s="17" t="inlineStr">
         <is>
-          <t>2026-08-29 16:00</t>
+          <t>2026-09-04 23:00</t>
         </is>
       </c>
       <c r="D96" s="25" t="n">
@@ -7174,34 +7174,34 @@
       </c>
       <c r="E96" s="17" t="inlineStr">
         <is>
-          <t>ATS</t>
+          <t>TOTAL</t>
         </is>
       </c>
       <c r="F96" s="17" t="inlineStr">
         <is>
-          <t>TCU -7.5</t>
+          <t>Over 63.5</t>
         </is>
       </c>
       <c r="G96" s="26" t="n">
-        <v>-7.5</v>
+        <v>63.5</v>
       </c>
       <c r="H96" s="18" t="n">
-        <v>-115</v>
+        <v>-110</v>
       </c>
       <c r="I96" s="20" t="n">
-        <v>0.4039442568628988</v>
+        <v>0.3904378805908039</v>
       </c>
       <c r="J96" s="20" t="n">
-        <v>0.5108342361863488</v>
+        <v>0.5</v>
       </c>
       <c r="K96" s="20" t="n">
-        <v>0.5348837209302325</v>
+        <v>0.5238095238095238</v>
       </c>
       <c r="L96" s="19" t="n">
-        <v>-0.1309394640673337</v>
+        <v>-0.13337164321872</v>
       </c>
       <c r="M96" s="19" t="n">
-        <v>-0.2447998676041457</v>
+        <v>-0.2546185915993744</v>
       </c>
       <c r="N96" s="20" t="n">
         <v>0</v>
@@ -7214,7 +7214,11 @@
           <t>DraftKings</t>
         </is>
       </c>
-      <c r="Q96" s="17" t="n"/>
+      <c r="Q96" s="17" t="inlineStr">
+        <is>
+          <t>NCAT isn't a full FBS participant this season — model doesn't rate them reliably</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="12" t="inlineStr">
@@ -7224,12 +7228,12 @@
       </c>
       <c r="B97" s="12" t="inlineStr">
         <is>
-          <t>NCAT @ GAST</t>
+          <t>UNC @ TCU</t>
         </is>
       </c>
       <c r="C97" s="12" t="inlineStr">
         <is>
-          <t>2026-09-04 23:00</t>
+          <t>2026-08-29 16:00</t>
         </is>
       </c>
       <c r="D97" s="22" t="n">
@@ -7237,34 +7241,34 @@
       </c>
       <c r="E97" s="12" t="inlineStr">
         <is>
-          <t>TOTAL</t>
+          <t>ATS</t>
         </is>
       </c>
       <c r="F97" s="12" t="inlineStr">
         <is>
-          <t>Over 63.5</t>
+          <t>TCU -7.5</t>
         </is>
       </c>
       <c r="G97" s="23" t="n">
-        <v>63.5</v>
+        <v>-7.5</v>
       </c>
       <c r="H97" s="13" t="n">
-        <v>-110</v>
+        <v>-118</v>
       </c>
       <c r="I97" s="15" t="n">
-        <v>0.3904378805908039</v>
+        <v>0.4072092016278595</v>
       </c>
       <c r="J97" s="15" t="n">
-        <v>0.5</v>
+        <v>0.5173641257162701</v>
       </c>
       <c r="K97" s="15" t="n">
-        <v>0.5238095238095238</v>
+        <v>0.5412844036697247</v>
       </c>
       <c r="L97" s="14" t="n">
-        <v>-0.13337164321872</v>
+        <v>-0.1340752020418653</v>
       </c>
       <c r="M97" s="14" t="n">
-        <v>-0.2546185915993744</v>
+        <v>-0.2476982546197173</v>
       </c>
       <c r="N97" s="15" t="n">
         <v>0</v>
@@ -7277,11 +7281,7 @@
           <t>DraftKings</t>
         </is>
       </c>
-      <c r="Q97" s="12" t="inlineStr">
-        <is>
-          <t>NCAT isn't a full FBS participant this season — model doesn't rate them reliably</t>
-        </is>
-      </c>
+      <c r="Q97" s="12" t="n"/>
     </row>
     <row r="98">
       <c r="A98" s="17" t="inlineStr">
@@ -8532,12 +8532,12 @@
       </c>
       <c r="B117" s="12" t="inlineStr">
         <is>
-          <t>NMSU @ FSU</t>
+          <t>NCAT @ GAST</t>
         </is>
       </c>
       <c r="C117" s="12" t="inlineStr">
         <is>
-          <t>2026-08-29 23:00</t>
+          <t>2026-09-04 23:00</t>
         </is>
       </c>
       <c r="D117" s="22" t="n">
@@ -8550,29 +8550,29 @@
       </c>
       <c r="F117" s="12" t="inlineStr">
         <is>
-          <t>FSU -31.5</t>
+          <t>GAST -28.5</t>
         </is>
       </c>
       <c r="G117" s="23" t="n">
-        <v>-31.5</v>
+        <v>-28.5</v>
       </c>
       <c r="H117" s="13" t="n">
-        <v>-105</v>
+        <v>-108</v>
       </c>
       <c r="I117" s="15" t="n">
-        <v>0.2515947455243119</v>
+        <v>0.2547133684856709</v>
       </c>
       <c r="J117" s="15" t="n">
-        <v>0.4891657638136511</v>
+        <v>0.4956702459300312</v>
       </c>
       <c r="K117" s="15" t="n">
-        <v>0.5121951219512195</v>
+        <v>0.5192307692307693</v>
       </c>
       <c r="L117" s="14" t="n">
-        <v>-0.2606003764269076</v>
+        <v>-0.2645174007450984</v>
       </c>
       <c r="M117" s="14" t="n">
-        <v>-0.5087912111192006</v>
+        <v>-0.5094409199535228</v>
       </c>
       <c r="N117" s="15" t="n">
         <v>0</v>
@@ -8587,7 +8587,7 @@
       </c>
       <c r="Q117" s="12" t="inlineStr">
         <is>
-          <t>raw model/market disagreement exceeds the safety limit</t>
+          <t>NCAT isn't a full FBS participant this season — model doesn't rate them reliably</t>
         </is>
       </c>
     </row>
@@ -8599,12 +8599,12 @@
       </c>
       <c r="B118" s="17" t="inlineStr">
         <is>
-          <t>NCAT @ GAST</t>
+          <t>SJSU @ USC</t>
         </is>
       </c>
       <c r="C118" s="17" t="inlineStr">
         <is>
-          <t>2026-09-04 23:00</t>
+          <t>2026-08-29 19:00</t>
         </is>
       </c>
       <c r="D118" s="25" t="n">
@@ -8617,29 +8617,29 @@
       </c>
       <c r="F118" s="17" t="inlineStr">
         <is>
-          <t>GAST -28.5</t>
+          <t>USC -38.5</t>
         </is>
       </c>
       <c r="G118" s="26" t="n">
-        <v>-28.5</v>
+        <v>-38.5</v>
       </c>
       <c r="H118" s="18" t="n">
-        <v>-108</v>
+        <v>-105</v>
       </c>
       <c r="I118" s="20" t="n">
-        <v>0.2547133684856709</v>
+        <v>0.2469039658580302</v>
       </c>
       <c r="J118" s="20" t="n">
-        <v>0.4956702459300312</v>
+        <v>0.4891657638136511</v>
       </c>
       <c r="K118" s="20" t="n">
-        <v>0.5192307692307693</v>
+        <v>0.5121951219512195</v>
       </c>
       <c r="L118" s="19" t="n">
-        <v>-0.2645174007450984</v>
+        <v>-0.2652911560931893</v>
       </c>
       <c r="M118" s="19" t="n">
-        <v>-0.5094409199535228</v>
+        <v>-0.5179493999914648</v>
       </c>
       <c r="N118" s="20" t="n">
         <v>0</v>
@@ -8654,7 +8654,7 @@
       </c>
       <c r="Q118" s="17" t="inlineStr">
         <is>
-          <t>NCAT isn't a full FBS participant this season — model doesn't rate them reliably</t>
+          <t>raw model/market disagreement exceeds the safety limit</t>
         </is>
       </c>
     </row>
@@ -8666,12 +8666,12 @@
       </c>
       <c r="B119" s="12" t="inlineStr">
         <is>
-          <t>SJSU @ USC</t>
+          <t>MASS @ RUTG</t>
         </is>
       </c>
       <c r="C119" s="12" t="inlineStr">
         <is>
-          <t>2026-08-29 19:00</t>
+          <t>2026-09-03 22:00</t>
         </is>
       </c>
       <c r="D119" s="22" t="n">
@@ -8684,29 +8684,29 @@
       </c>
       <c r="F119" s="12" t="inlineStr">
         <is>
-          <t>USC -38.5</t>
+          <t>RUTG -29.5</t>
         </is>
       </c>
       <c r="G119" s="23" t="n">
-        <v>-38.5</v>
+        <v>-29.5</v>
       </c>
       <c r="H119" s="13" t="n">
-        <v>-105</v>
+        <v>-115</v>
       </c>
       <c r="I119" s="15" t="n">
-        <v>0.2469039658580302</v>
+        <v>0.2692244850681354</v>
       </c>
       <c r="J119" s="15" t="n">
-        <v>0.4891657638136511</v>
+        <v>0.5108342361863488</v>
       </c>
       <c r="K119" s="15" t="n">
-        <v>0.5121951219512195</v>
+        <v>0.5348837209302325</v>
       </c>
       <c r="L119" s="14" t="n">
-        <v>-0.2652911560931893</v>
+        <v>-0.2656592358620971</v>
       </c>
       <c r="M119" s="14" t="n">
-        <v>-0.5179493999914648</v>
+        <v>-0.4966672670465295</v>
       </c>
       <c r="N119" s="15" t="n">
         <v>0</v>
@@ -8733,12 +8733,12 @@
       </c>
       <c r="B120" s="17" t="inlineStr">
         <is>
-          <t>MASS @ RUTG</t>
+          <t>MRMK @ DEL</t>
         </is>
       </c>
       <c r="C120" s="17" t="inlineStr">
         <is>
-          <t>2026-09-03 22:00</t>
+          <t>2026-09-03 23:00</t>
         </is>
       </c>
       <c r="D120" s="25" t="n">
@@ -8751,29 +8751,29 @@
       </c>
       <c r="F120" s="17" t="inlineStr">
         <is>
-          <t>RUTG -29.5</t>
+          <t>DEL -28.5</t>
         </is>
       </c>
       <c r="G120" s="26" t="n">
-        <v>-29.5</v>
+        <v>-28.5</v>
       </c>
       <c r="H120" s="18" t="n">
-        <v>-115</v>
+        <v>-112</v>
       </c>
       <c r="I120" s="20" t="n">
-        <v>0.2692244850681354</v>
+        <v>0.2613150626201174</v>
       </c>
       <c r="J120" s="20" t="n">
-        <v>0.5108342361863488</v>
+        <v>0.5043297540699688</v>
       </c>
       <c r="K120" s="20" t="n">
-        <v>0.5348837209302325</v>
+        <v>0.5283018867924528</v>
       </c>
       <c r="L120" s="19" t="n">
-        <v>-0.2656592358620971</v>
+        <v>-0.2669868241723354</v>
       </c>
       <c r="M120" s="19" t="n">
-        <v>-0.4966672670465295</v>
+        <v>-0.5053679171833493</v>
       </c>
       <c r="N120" s="20" t="n">
         <v>0</v>
@@ -8788,7 +8788,7 @@
       </c>
       <c r="Q120" s="17" t="inlineStr">
         <is>
-          <t>raw model/market disagreement exceeds the safety limit</t>
+          <t>MRMK isn't a full FBS participant this season — model doesn't rate them reliably</t>
         </is>
       </c>
     </row>
@@ -8800,12 +8800,12 @@
       </c>
       <c r="B121" s="12" t="inlineStr">
         <is>
-          <t>MRMK @ DEL</t>
+          <t>IDHO @ UTAH</t>
         </is>
       </c>
       <c r="C121" s="12" t="inlineStr">
         <is>
-          <t>2026-09-03 23:00</t>
+          <t>2026-09-04 01:00</t>
         </is>
       </c>
       <c r="D121" s="22" t="n">
@@ -8818,29 +8818,29 @@
       </c>
       <c r="F121" s="12" t="inlineStr">
         <is>
-          <t>DEL -28.5</t>
+          <t>UTAH -33.5</t>
         </is>
       </c>
       <c r="G121" s="23" t="n">
-        <v>-28.5</v>
+        <v>-33.5</v>
       </c>
       <c r="H121" s="13" t="n">
-        <v>-112</v>
+        <v>-110</v>
       </c>
       <c r="I121" s="15" t="n">
-        <v>0.2613150626201174</v>
+        <v>0.2563559702123712</v>
       </c>
       <c r="J121" s="15" t="n">
-        <v>0.5043297540699688</v>
+        <v>0.5</v>
       </c>
       <c r="K121" s="15" t="n">
-        <v>0.5283018867924528</v>
+        <v>0.5238095238095238</v>
       </c>
       <c r="L121" s="14" t="n">
-        <v>-0.2669868241723354</v>
+        <v>-0.2674535535971527</v>
       </c>
       <c r="M121" s="14" t="n">
-        <v>-0.5053679171833493</v>
+        <v>-0.5105931477763822</v>
       </c>
       <c r="N121" s="15" t="n">
         <v>0</v>
@@ -8855,7 +8855,7 @@
       </c>
       <c r="Q121" s="12" t="inlineStr">
         <is>
-          <t>MRMK isn't a full FBS participant this season — model doesn't rate them reliably</t>
+          <t>IDHO isn't a full FBS participant this season — model doesn't rate them reliably</t>
         </is>
       </c>
     </row>
@@ -8867,12 +8867,12 @@
       </c>
       <c r="B122" s="17" t="inlineStr">
         <is>
-          <t>IDHO @ UTAH</t>
+          <t>INST @ PUR</t>
         </is>
       </c>
       <c r="C122" s="17" t="inlineStr">
         <is>
-          <t>2026-09-04 01:00</t>
+          <t>2026-09-04 23:00</t>
         </is>
       </c>
       <c r="D122" s="25" t="n">
@@ -8885,29 +8885,29 @@
       </c>
       <c r="F122" s="17" t="inlineStr">
         <is>
-          <t>UTAH -33.5</t>
+          <t>PUR -35.5</t>
         </is>
       </c>
       <c r="G122" s="26" t="n">
-        <v>-33.5</v>
+        <v>-35.5</v>
       </c>
       <c r="H122" s="18" t="n">
         <v>-110</v>
       </c>
       <c r="I122" s="20" t="n">
-        <v>0.2563559702123712</v>
+        <v>0.2528934298318226</v>
       </c>
       <c r="J122" s="20" t="n">
-        <v>0.5</v>
+        <v>0.5021949078138718</v>
       </c>
       <c r="K122" s="20" t="n">
         <v>0.5238095238095238</v>
       </c>
       <c r="L122" s="19" t="n">
-        <v>-0.2674535535971527</v>
+        <v>-0.2709160939777012</v>
       </c>
       <c r="M122" s="19" t="n">
-        <v>-0.5105931477763822</v>
+        <v>-0.5172034521392477</v>
       </c>
       <c r="N122" s="20" t="n">
         <v>0</v>
@@ -8922,7 +8922,7 @@
       </c>
       <c r="Q122" s="17" t="inlineStr">
         <is>
-          <t>IDHO isn't a full FBS participant this season — model doesn't rate them reliably</t>
+          <t>INST isn't a full FBS participant this season — model doesn't rate them reliably</t>
         </is>
       </c>
     </row>
@@ -8934,12 +8934,12 @@
       </c>
       <c r="B123" s="12" t="inlineStr">
         <is>
-          <t>INST @ PUR</t>
+          <t>EIU @ MINN</t>
         </is>
       </c>
       <c r="C123" s="12" t="inlineStr">
         <is>
-          <t>2026-09-04 23:00</t>
+          <t>2026-09-04 00:00</t>
         </is>
       </c>
       <c r="D123" s="22" t="n">
@@ -8952,29 +8952,29 @@
       </c>
       <c r="F123" s="12" t="inlineStr">
         <is>
-          <t>PUR -35.5</t>
+          <t>MINN -43.5</t>
         </is>
       </c>
       <c r="G123" s="23" t="n">
-        <v>-35.5</v>
+        <v>-43.5</v>
       </c>
       <c r="H123" s="13" t="n">
-        <v>-110</v>
+        <v>-108</v>
       </c>
       <c r="I123" s="15" t="n">
-        <v>0.2528934298318226</v>
+        <v>0.2481768262232006</v>
       </c>
       <c r="J123" s="15" t="n">
-        <v>0.5021949078138718</v>
+        <v>0.4956702459300312</v>
       </c>
       <c r="K123" s="15" t="n">
-        <v>0.5238095238095238</v>
+        <v>0.5192307692307693</v>
       </c>
       <c r="L123" s="14" t="n">
-        <v>-0.2709160939777012</v>
+        <v>-0.2710539430075687</v>
       </c>
       <c r="M123" s="14" t="n">
-        <v>-0.5172034521392477</v>
+        <v>-0.5220298161627247</v>
       </c>
       <c r="N123" s="15" t="n">
         <v>0</v>
@@ -8989,7 +8989,7 @@
       </c>
       <c r="Q123" s="12" t="inlineStr">
         <is>
-          <t>INST isn't a full FBS participant this season — model doesn't rate them reliably</t>
+          <t>EIU isn't a full FBS participant this season — model doesn't rate them reliably</t>
         </is>
       </c>
     </row>
@@ -9001,7 +9001,7 @@
       </c>
       <c r="B124" s="17" t="inlineStr">
         <is>
-          <t>EIU @ MINN</t>
+          <t>UAPB @ MIZ</t>
         </is>
       </c>
       <c r="C124" s="17" t="inlineStr">
@@ -9019,17 +9019,17 @@
       </c>
       <c r="F124" s="17" t="inlineStr">
         <is>
-          <t>MINN -43.5</t>
+          <t>MIZ -54.5</t>
         </is>
       </c>
       <c r="G124" s="26" t="n">
-        <v>-43.5</v>
+        <v>-54.5</v>
       </c>
       <c r="H124" s="18" t="n">
         <v>-108</v>
       </c>
       <c r="I124" s="20" t="n">
-        <v>0.2481768262232006</v>
+        <v>0.2478531706379516</v>
       </c>
       <c r="J124" s="20" t="n">
         <v>0.4956702459300312</v>
@@ -9038,10 +9038,10 @@
         <v>0.5192307692307693</v>
       </c>
       <c r="L124" s="19" t="n">
-        <v>-0.2710539430075687</v>
+        <v>-0.2713775985928176</v>
       </c>
       <c r="M124" s="19" t="n">
-        <v>-0.5220298161627247</v>
+        <v>-0.5226531528454265</v>
       </c>
       <c r="N124" s="20" t="n">
         <v>0</v>
@@ -9056,7 +9056,7 @@
       </c>
       <c r="Q124" s="17" t="inlineStr">
         <is>
-          <t>EIU isn't a full FBS participant this season — model doesn't rate them reliably</t>
+          <t>UAPB isn't a full FBS participant this season — model doesn't rate them reliably</t>
         </is>
       </c>
     </row>
@@ -9068,12 +9068,12 @@
       </c>
       <c r="B125" s="12" t="inlineStr">
         <is>
-          <t>UAPB @ MIZ</t>
+          <t>BCU @ UCF</t>
         </is>
       </c>
       <c r="C125" s="12" t="inlineStr">
         <is>
-          <t>2026-09-04 00:00</t>
+          <t>2026-09-03 23:00</t>
         </is>
       </c>
       <c r="D125" s="22" t="n">
@@ -9086,29 +9086,29 @@
       </c>
       <c r="F125" s="12" t="inlineStr">
         <is>
-          <t>MIZ -54.5</t>
+          <t>UCF -42.5</t>
         </is>
       </c>
       <c r="G125" s="23" t="n">
-        <v>-54.5</v>
+        <v>-42.5</v>
       </c>
       <c r="H125" s="13" t="n">
-        <v>-108</v>
+        <v>-110</v>
       </c>
       <c r="I125" s="15" t="n">
-        <v>0.2478531706379516</v>
+        <v>0.2504166868493028</v>
       </c>
       <c r="J125" s="15" t="n">
-        <v>0.4956702459300312</v>
+        <v>0.5</v>
       </c>
       <c r="K125" s="15" t="n">
-        <v>0.5192307692307693</v>
+        <v>0.5238095238095238</v>
       </c>
       <c r="L125" s="14" t="n">
-        <v>-0.2713775985928176</v>
+        <v>-0.273392836960221</v>
       </c>
       <c r="M125" s="14" t="n">
-        <v>-0.5226531528454265</v>
+        <v>-0.5219317796513311</v>
       </c>
       <c r="N125" s="15" t="n">
         <v>0</v>
@@ -9123,7 +9123,7 @@
       </c>
       <c r="Q125" s="12" t="inlineStr">
         <is>
-          <t>UAPB isn't a full FBS participant this season — model doesn't rate them reliably</t>
+          <t>BCU isn't a full FBS participant this season — model doesn't rate them reliably</t>
         </is>
       </c>
     </row>
@@ -9135,12 +9135,12 @@
       </c>
       <c r="B126" s="17" t="inlineStr">
         <is>
-          <t>BCU @ UCF</t>
+          <t>NMSU @ FSU</t>
         </is>
       </c>
       <c r="C126" s="17" t="inlineStr">
         <is>
-          <t>2026-09-03 23:00</t>
+          <t>2026-08-29 23:00</t>
         </is>
       </c>
       <c r="D126" s="25" t="n">
@@ -9153,29 +9153,29 @@
       </c>
       <c r="F126" s="17" t="inlineStr">
         <is>
-          <t>UCF -42.5</t>
+          <t>FSU -30.5</t>
         </is>
       </c>
       <c r="G126" s="26" t="n">
-        <v>-42.5</v>
+        <v>-30.5</v>
       </c>
       <c r="H126" s="18" t="n">
-        <v>-110</v>
+        <v>-118</v>
       </c>
       <c r="I126" s="20" t="n">
-        <v>0.2504166868493028</v>
+        <v>0.2672251541311149</v>
       </c>
       <c r="J126" s="20" t="n">
-        <v>0.5</v>
+        <v>0.5173641257162701</v>
       </c>
       <c r="K126" s="20" t="n">
-        <v>0.5238095238095238</v>
+        <v>0.5412844036697247</v>
       </c>
       <c r="L126" s="19" t="n">
-        <v>-0.273392836960221</v>
+        <v>-0.2740592495386099</v>
       </c>
       <c r="M126" s="19" t="n">
-        <v>-0.5219317796513311</v>
+        <v>-0.5063128508425166</v>
       </c>
       <c r="N126" s="20" t="n">
         <v>0</v>
@@ -9190,7 +9190,7 @@
       </c>
       <c r="Q126" s="17" t="inlineStr">
         <is>
-          <t>BCU isn't a full FBS participant this season — model doesn't rate them reliably</t>
+          <t>raw model/market disagreement exceeds the safety limit</t>
         </is>
       </c>
     </row>
@@ -16227,10 +16227,10 @@
         <v>47.5</v>
       </c>
       <c r="K5" s="13" t="n">
-        <v>245</v>
+        <v>250</v>
       </c>
       <c r="L5" s="13" t="n">
-        <v>-305</v>
+        <v>-310</v>
       </c>
       <c r="M5" s="12" t="inlineStr">
         <is>
@@ -16511,7 +16511,7 @@
       </c>
       <c r="H11" s="12" t="inlineStr"/>
       <c r="I11" s="23" t="n">
-        <v>-31.5</v>
+        <v>-30.5</v>
       </c>
       <c r="J11" s="29" t="n">
         <v>52.5</v>
@@ -16566,10 +16566,10 @@
         <v>56.5</v>
       </c>
       <c r="K12" s="18" t="n">
-        <v>160</v>
+        <v>164</v>
       </c>
       <c r="L12" s="18" t="n">
-        <v>-192</v>
+        <v>-198</v>
       </c>
       <c r="M12" s="17" t="inlineStr">
         <is>
@@ -17424,10 +17424,10 @@
         <v>48.5</v>
       </c>
       <c r="K30" s="18" t="n">
-        <v>-3200</v>
+        <v>-2800</v>
       </c>
       <c r="L30" s="18" t="n">
-        <v>1400</v>
+        <v>1300</v>
       </c>
       <c r="M30" s="17" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
refresh 2026-09-06 15:28 UTC
</commit_message>
<xml_diff>
--- a/NCAAF_Edge_Model.xlsx
+++ b/NCAAF_Edge_Model.xlsx
@@ -642,7 +642,7 @@
     <row r="2" ht="26" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-09-06T13:07:39+00:00 from live ESPN data. This file is a snapshot, not the model. Re-run the pipeline to refresh it.</t>
+          <t>Generated 2026-09-06T15:28:37+00:00 from live ESPN data. This file is a snapshot, not the model. Re-run the pipeline to refresh it.</t>
         </is>
       </c>
     </row>
@@ -1155,13 +1155,13 @@
         </is>
       </c>
       <c r="E25" s="13" t="n">
-        <v>170</v>
+        <v>180</v>
       </c>
       <c r="F25" s="14" t="n">
-        <v>0.1100965613025194</v>
+        <v>0.1169510508323464</v>
       </c>
       <c r="G25" s="15" t="n">
-        <v>0.4804669316728897</v>
+        <v>0.4740939079752036</v>
       </c>
       <c r="H25" s="16" t="n"/>
       <c r="I25" s="12" t="inlineStr">
@@ -1807,22 +1807,22 @@
       </c>
       <c r="G9" s="23" t="n"/>
       <c r="H9" s="13" t="n">
-        <v>170</v>
+        <v>180</v>
       </c>
       <c r="I9" s="15" t="n">
-        <v>0.4804669316728897</v>
+        <v>0.4740939079752036</v>
       </c>
       <c r="J9" s="15" t="n">
-        <v>0.3552708211997671</v>
+        <v>0.3425247738043947</v>
       </c>
       <c r="K9" s="15" t="n">
-        <v>0.3703703703703703</v>
+        <v>0.3571428571428572</v>
       </c>
       <c r="L9" s="14" t="n">
-        <v>0.1100965613025194</v>
+        <v>0.1169510508323464</v>
       </c>
       <c r="M9" s="14" t="n">
-        <v>0.2972607155168024</v>
+        <v>0.3274629423305699</v>
       </c>
       <c r="N9" s="15" t="n">
         <v>0</v>
@@ -2812,16 +2812,16 @@
       </c>
       <c r="B25" s="12" t="inlineStr">
         <is>
-          <t>UL @ USC</t>
+          <t>WIS @ ND</t>
         </is>
       </c>
       <c r="C25" s="12" t="inlineStr">
         <is>
-          <t>2026-09-13 03:00</t>
+          <t>2026-09-06 23:30</t>
         </is>
       </c>
       <c r="D25" s="22" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E25" s="12" t="inlineStr">
         <is>
@@ -2830,35 +2830,35 @@
       </c>
       <c r="F25" s="12" t="inlineStr">
         <is>
-          <t>UL +28.5</t>
+          <t>WIS +21</t>
         </is>
       </c>
       <c r="G25" s="23" t="n">
-        <v>-28.5</v>
+        <v>-21</v>
       </c>
       <c r="H25" s="13" t="n">
-        <v>-110</v>
+        <v>-105</v>
       </c>
       <c r="I25" s="15" t="n">
-        <v>0.7341224033276599</v>
+        <v>0.7243553267010203</v>
       </c>
       <c r="J25" s="15" t="n">
-        <v>0.5</v>
+        <v>0.4891657638136511</v>
       </c>
       <c r="K25" s="15" t="n">
-        <v>0.5238095238095238</v>
+        <v>0.5121951219512195</v>
       </c>
       <c r="L25" s="14" t="n">
-        <v>0.210312879518136</v>
+        <v>0.2121602047498008</v>
       </c>
       <c r="M25" s="14" t="n">
-        <v>0.4015064063528053</v>
+        <v>0.4102869840085517</v>
       </c>
       <c r="N25" s="15" t="n">
-        <v>0</v>
+        <v>0.0095</v>
       </c>
       <c r="O25" s="24" t="n">
-        <v>0.725</v>
+        <v>0.4</v>
       </c>
       <c r="P25" s="12" t="inlineStr">
         <is>
@@ -2879,16 +2879,16 @@
       </c>
       <c r="B26" s="17" t="inlineStr">
         <is>
-          <t>WIS @ ND</t>
+          <t>UL @ USC</t>
         </is>
       </c>
       <c r="C26" s="17" t="inlineStr">
         <is>
-          <t>2026-09-06 23:30</t>
+          <t>2026-09-13 03:00</t>
         </is>
       </c>
       <c r="D26" s="25" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E26" s="17" t="inlineStr">
         <is>
@@ -2897,35 +2897,35 @@
       </c>
       <c r="F26" s="17" t="inlineStr">
         <is>
-          <t>WIS +20.5</t>
+          <t>UL +28.5</t>
         </is>
       </c>
       <c r="G26" s="26" t="n">
-        <v>-20.5</v>
+        <v>-28.5</v>
       </c>
       <c r="H26" s="18" t="n">
-        <v>-105</v>
+        <v>-110</v>
       </c>
       <c r="I26" s="20" t="n">
-        <v>0.7198027099861445</v>
+        <v>0.7341224033276599</v>
       </c>
       <c r="J26" s="20" t="n">
-        <v>0.4891657638136511</v>
+        <v>0.5</v>
       </c>
       <c r="K26" s="20" t="n">
-        <v>0.5121951219512195</v>
+        <v>0.5238095238095238</v>
       </c>
       <c r="L26" s="19" t="n">
-        <v>0.207607588034925</v>
+        <v>0.210312879518136</v>
       </c>
       <c r="M26" s="19" t="n">
-        <v>0.4053291004491392</v>
+        <v>0.4015064063528053</v>
       </c>
       <c r="N26" s="20" t="n">
         <v>0</v>
       </c>
       <c r="O26" s="27" t="n">
-        <v>0.4</v>
+        <v>0.725</v>
       </c>
       <c r="P26" s="17" t="inlineStr">
         <is>
@@ -5084,17 +5084,17 @@
       </c>
       <c r="F59" s="12" t="inlineStr">
         <is>
-          <t>MICH +4.5</t>
+          <t>MICH +5.5</t>
         </is>
       </c>
       <c r="G59" s="23" t="n">
-        <v>4.5</v>
+        <v>5.5</v>
       </c>
       <c r="H59" s="13" t="n">
         <v>-105</v>
       </c>
       <c r="I59" s="15" t="n">
-        <v>0.6171353381292989</v>
+        <v>0.6270122766739621</v>
       </c>
       <c r="J59" s="15" t="n">
         <v>0.4891657638136511</v>
@@ -5103,10 +5103,10 @@
         <v>0.5121951219512195</v>
       </c>
       <c r="L59" s="14" t="n">
-        <v>0.1049402161780794</v>
+        <v>0.1148171547227426</v>
       </c>
       <c r="M59" s="14" t="n">
-        <v>0.2048832792048216</v>
+        <v>0.2241668258872593</v>
       </c>
       <c r="N59" s="15" t="n">
         <v>0</v>
@@ -5588,58 +5588,64 @@
       </c>
       <c r="B67" s="12" t="inlineStr">
         <is>
-          <t>LOU @ MISS</t>
+          <t>APP @ ECU</t>
         </is>
       </c>
       <c r="C67" s="12" t="inlineStr">
         <is>
-          <t>2026-09-06 23:30</t>
+          <t>2026-09-12 16:00</t>
         </is>
       </c>
       <c r="D67" s="22" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E67" s="12" t="inlineStr">
         <is>
-          <t>ML</t>
+          <t>ATS</t>
         </is>
       </c>
       <c r="F67" s="12" t="inlineStr">
         <is>
-          <t>LOU ML</t>
-        </is>
-      </c>
-      <c r="G67" s="23" t="n"/>
+          <t>APP +10</t>
+        </is>
+      </c>
+      <c r="G67" s="23" t="n">
+        <v>-10</v>
+      </c>
       <c r="H67" s="13" t="n">
-        <v>210</v>
+        <v>-110</v>
       </c>
       <c r="I67" s="15" t="n">
-        <v>0.4046035584729659</v>
+        <v>0.6048256402521389</v>
       </c>
       <c r="J67" s="15" t="n">
-        <v>0.3092071169459319</v>
+        <v>0.5</v>
       </c>
       <c r="K67" s="15" t="n">
-        <v>0.3225806451612903</v>
+        <v>0.5238095238095238</v>
       </c>
       <c r="L67" s="14" t="n">
-        <v>0.0820229133116756</v>
+        <v>0.08101611644261508</v>
       </c>
       <c r="M67" s="14" t="n">
-        <v>0.2542710312661944</v>
+        <v>0.1489872529042741</v>
       </c>
       <c r="N67" s="15" t="n">
-        <v>0</v>
+        <v>0.0367</v>
       </c>
       <c r="O67" s="24" t="n">
-        <v>0.4</v>
+        <v>0.725</v>
       </c>
       <c r="P67" s="12" t="inlineStr">
         <is>
           <t>DraftKings</t>
         </is>
       </c>
-      <c r="Q67" s="12" t="n"/>
+      <c r="Q67" s="12" t="inlineStr">
+        <is>
+          <t>outside the top 10 plays for this week</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="17" t="inlineStr">
@@ -5649,12 +5655,12 @@
       </c>
       <c r="B68" s="17" t="inlineStr">
         <is>
-          <t>APP @ ECU</t>
+          <t>ARK @ UTAH</t>
         </is>
       </c>
       <c r="C68" s="17" t="inlineStr">
         <is>
-          <t>2026-09-12 16:00</t>
+          <t>2026-09-13 02:15</t>
         </is>
       </c>
       <c r="D68" s="25" t="n">
@@ -5667,32 +5673,32 @@
       </c>
       <c r="F68" s="17" t="inlineStr">
         <is>
-          <t>APP +10</t>
+          <t>ARK +11.5</t>
         </is>
       </c>
       <c r="G68" s="26" t="n">
-        <v>-10</v>
+        <v>-11.5</v>
       </c>
       <c r="H68" s="18" t="n">
-        <v>-110</v>
+        <v>-108</v>
       </c>
       <c r="I68" s="20" t="n">
-        <v>0.6048256402521389</v>
+        <v>0.5996411451304783</v>
       </c>
       <c r="J68" s="20" t="n">
-        <v>0.5</v>
+        <v>0.4956702459300312</v>
       </c>
       <c r="K68" s="20" t="n">
-        <v>0.5238095238095238</v>
+        <v>0.5192307692307693</v>
       </c>
       <c r="L68" s="19" t="n">
-        <v>0.08101611644261508</v>
+        <v>0.08041037589970901</v>
       </c>
       <c r="M68" s="19" t="n">
-        <v>0.1489872529042741</v>
+        <v>0.154864427658699</v>
       </c>
       <c r="N68" s="20" t="n">
-        <v>0.0367</v>
+        <v>0</v>
       </c>
       <c r="O68" s="27" t="n">
         <v>0.725</v>
@@ -5716,64 +5722,58 @@
       </c>
       <c r="B69" s="12" t="inlineStr">
         <is>
-          <t>ARK @ UTAH</t>
+          <t>LOU @ MISS</t>
         </is>
       </c>
       <c r="C69" s="12" t="inlineStr">
         <is>
-          <t>2026-09-13 02:15</t>
+          <t>2026-09-06 23:30</t>
         </is>
       </c>
       <c r="D69" s="22" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E69" s="12" t="inlineStr">
         <is>
-          <t>ATS</t>
+          <t>ML</t>
         </is>
       </c>
       <c r="F69" s="12" t="inlineStr">
         <is>
-          <t>ARK +11.5</t>
-        </is>
-      </c>
-      <c r="G69" s="23" t="n">
-        <v>-11.5</v>
-      </c>
+          <t>LOU ML</t>
+        </is>
+      </c>
+      <c r="G69" s="23" t="n"/>
       <c r="H69" s="13" t="n">
-        <v>-108</v>
+        <v>205</v>
       </c>
       <c r="I69" s="15" t="n">
-        <v>0.5996411451304783</v>
+        <v>0.4073033707865168</v>
       </c>
       <c r="J69" s="15" t="n">
-        <v>0.4956702459300312</v>
+        <v>0.3146067415730336</v>
       </c>
       <c r="K69" s="15" t="n">
-        <v>0.5192307692307693</v>
+        <v>0.3278688524590164</v>
       </c>
       <c r="L69" s="14" t="n">
-        <v>0.08041037589970901</v>
+        <v>0.07943451832750043</v>
       </c>
       <c r="M69" s="14" t="n">
-        <v>0.154864427658699</v>
+        <v>0.2422752808988762</v>
       </c>
       <c r="N69" s="15" t="n">
         <v>0</v>
       </c>
       <c r="O69" s="24" t="n">
-        <v>0.725</v>
+        <v>0.4</v>
       </c>
       <c r="P69" s="12" t="inlineStr">
         <is>
           <t>DraftKings</t>
         </is>
       </c>
-      <c r="Q69" s="12" t="inlineStr">
-        <is>
-          <t>outside the top 10 plays for this week</t>
-        </is>
-      </c>
+      <c r="Q69" s="12" t="n"/>
     </row>
     <row r="70">
       <c r="A70" s="17" t="inlineStr">
@@ -5980,60 +5980,64 @@
       </c>
       <c r="B73" s="12" t="inlineStr">
         <is>
-          <t>WIS @ ND</t>
+          <t>USA @ TULN</t>
         </is>
       </c>
       <c r="C73" s="12" t="inlineStr">
         <is>
-          <t>2026-09-06 23:30</t>
+          <t>2026-09-12 23:00</t>
         </is>
       </c>
       <c r="D73" s="22" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E73" s="12" t="inlineStr">
         <is>
-          <t>TOTAL</t>
+          <t>ATS</t>
         </is>
       </c>
       <c r="F73" s="12" t="inlineStr">
         <is>
-          <t>Over 46.5</t>
+          <t>USA +10</t>
         </is>
       </c>
       <c r="G73" s="23" t="n">
-        <v>46.5</v>
+        <v>-10</v>
       </c>
       <c r="H73" s="13" t="n">
-        <v>-105</v>
+        <v>-112</v>
       </c>
       <c r="I73" s="15" t="n">
-        <v>0.5832382897791041</v>
+        <v>0.5969393227641155</v>
       </c>
       <c r="J73" s="15" t="n">
-        <v>0.4891657638136511</v>
+        <v>0.5043297540699688</v>
       </c>
       <c r="K73" s="15" t="n">
-        <v>0.5121951219512195</v>
+        <v>0.5283018867924528</v>
       </c>
       <c r="L73" s="14" t="n">
-        <v>0.07104316782788456</v>
+        <v>0.06863743597166272</v>
       </c>
       <c r="M73" s="14" t="n">
-        <v>0.1387033276639651</v>
+        <v>0.1250239810832942</v>
       </c>
       <c r="N73" s="15" t="n">
-        <v>0</v>
+        <v>0.0377</v>
       </c>
       <c r="O73" s="24" t="n">
-        <v>0.4</v>
+        <v>0.725</v>
       </c>
       <c r="P73" s="12" t="inlineStr">
         <is>
           <t>DraftKings</t>
         </is>
       </c>
-      <c r="Q73" s="12" t="n"/>
+      <c r="Q73" s="12" t="inlineStr">
+        <is>
+          <t>outside the top 10 plays for this week</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="17" t="inlineStr">
@@ -6043,12 +6047,12 @@
       </c>
       <c r="B74" s="17" t="inlineStr">
         <is>
-          <t>OU @ MICH</t>
+          <t>OSU @ TEX</t>
         </is>
       </c>
       <c r="C74" s="17" t="inlineStr">
         <is>
-          <t>2026-09-12 16:00</t>
+          <t>2026-09-12 23:30</t>
         </is>
       </c>
       <c r="D74" s="25" t="n">
@@ -6061,29 +6065,29 @@
       </c>
       <c r="F74" s="17" t="inlineStr">
         <is>
-          <t>Over 44.5</t>
+          <t>Over 47.5</t>
         </is>
       </c>
       <c r="G74" s="26" t="n">
-        <v>44.5</v>
+        <v>47.5</v>
       </c>
       <c r="H74" s="18" t="n">
-        <v>-118</v>
+        <v>-110</v>
       </c>
       <c r="I74" s="20" t="n">
-        <v>0.6114217086662477</v>
+        <v>0.5922287555912803</v>
       </c>
       <c r="J74" s="20" t="n">
-        <v>0.5173641257162701</v>
+        <v>0.5</v>
       </c>
       <c r="K74" s="20" t="n">
-        <v>0.5412844036697247</v>
+        <v>0.5238095238095238</v>
       </c>
       <c r="L74" s="19" t="n">
-        <v>0.07013730499652293</v>
+        <v>0.06841923178175646</v>
       </c>
       <c r="M74" s="19" t="n">
-        <v>0.1295756990613728</v>
+        <v>0.1306185334015352</v>
       </c>
       <c r="N74" s="20" t="n">
         <v>0</v>
@@ -6098,7 +6102,7 @@
       </c>
       <c r="Q74" s="17" t="inlineStr">
         <is>
-          <t>correlated with a stronger play on the same game</t>
+          <t>outside the top 10 plays for this week</t>
         </is>
       </c>
     </row>
@@ -6110,64 +6114,60 @@
       </c>
       <c r="B75" s="12" t="inlineStr">
         <is>
-          <t>USA @ TULN</t>
+          <t>WIS @ ND</t>
         </is>
       </c>
       <c r="C75" s="12" t="inlineStr">
         <is>
-          <t>2026-09-12 23:00</t>
+          <t>2026-09-06 23:30</t>
         </is>
       </c>
       <c r="D75" s="22" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E75" s="12" t="inlineStr">
         <is>
-          <t>ATS</t>
+          <t>TOTAL</t>
         </is>
       </c>
       <c r="F75" s="12" t="inlineStr">
         <is>
-          <t>USA +10</t>
+          <t>Over 46.5</t>
         </is>
       </c>
       <c r="G75" s="23" t="n">
-        <v>-10</v>
+        <v>46.5</v>
       </c>
       <c r="H75" s="13" t="n">
-        <v>-112</v>
+        <v>-108</v>
       </c>
       <c r="I75" s="15" t="n">
-        <v>0.5969393227641155</v>
+        <v>0.5864905308372941</v>
       </c>
       <c r="J75" s="15" t="n">
-        <v>0.5043297540699688</v>
+        <v>0.4956702459300312</v>
       </c>
       <c r="K75" s="15" t="n">
-        <v>0.5283018867924528</v>
+        <v>0.5192307692307693</v>
       </c>
       <c r="L75" s="14" t="n">
-        <v>0.06863743597166272</v>
+        <v>0.0672597616065248</v>
       </c>
       <c r="M75" s="14" t="n">
-        <v>0.1250239810832942</v>
+        <v>0.1295373186496035</v>
       </c>
       <c r="N75" s="15" t="n">
-        <v>0.0377</v>
+        <v>0</v>
       </c>
       <c r="O75" s="24" t="n">
-        <v>0.725</v>
+        <v>0.4</v>
       </c>
       <c r="P75" s="12" t="inlineStr">
         <is>
           <t>DraftKings</t>
         </is>
       </c>
-      <c r="Q75" s="12" t="inlineStr">
-        <is>
-          <t>outside the top 10 plays for this week</t>
-        </is>
-      </c>
+      <c r="Q75" s="12" t="n"/>
     </row>
     <row r="76">
       <c r="A76" s="17" t="inlineStr">
@@ -6177,12 +6177,12 @@
       </c>
       <c r="B76" s="17" t="inlineStr">
         <is>
-          <t>OSU @ TEX</t>
+          <t>SDSU @ UCLA</t>
         </is>
       </c>
       <c r="C76" s="17" t="inlineStr">
         <is>
-          <t>2026-09-12 23:30</t>
+          <t>2026-09-12 23:15</t>
         </is>
       </c>
       <c r="D76" s="25" t="n">
@@ -6195,17 +6195,17 @@
       </c>
       <c r="F76" s="17" t="inlineStr">
         <is>
-          <t>Over 47.5</t>
+          <t>Over 48.5</t>
         </is>
       </c>
       <c r="G76" s="26" t="n">
-        <v>47.5</v>
+        <v>48.5</v>
       </c>
       <c r="H76" s="18" t="n">
         <v>-110</v>
       </c>
       <c r="I76" s="20" t="n">
-        <v>0.5922287555912803</v>
+        <v>0.5904462655465561</v>
       </c>
       <c r="J76" s="20" t="n">
         <v>0.5</v>
@@ -6214,10 +6214,10 @@
         <v>0.5238095238095238</v>
       </c>
       <c r="L76" s="19" t="n">
-        <v>0.06841923178175646</v>
+        <v>0.06663674173703227</v>
       </c>
       <c r="M76" s="19" t="n">
-        <v>0.1306185334015352</v>
+        <v>0.1272155978616072</v>
       </c>
       <c r="N76" s="20" t="n">
         <v>0</v>
@@ -6244,12 +6244,12 @@
       </c>
       <c r="B77" s="12" t="inlineStr">
         <is>
-          <t>SDSU @ UCLA</t>
+          <t>MSST @ MINN</t>
         </is>
       </c>
       <c r="C77" s="12" t="inlineStr">
         <is>
-          <t>2026-09-12 23:15</t>
+          <t>2026-09-12 19:30</t>
         </is>
       </c>
       <c r="D77" s="22" t="n">
@@ -6257,34 +6257,34 @@
       </c>
       <c r="E77" s="12" t="inlineStr">
         <is>
-          <t>TOTAL</t>
+          <t>ATS</t>
         </is>
       </c>
       <c r="F77" s="12" t="inlineStr">
         <is>
-          <t>Over 48.5</t>
+          <t>MINN +1.5</t>
         </is>
       </c>
       <c r="G77" s="23" t="n">
-        <v>48.5</v>
+        <v>1.5</v>
       </c>
       <c r="H77" s="13" t="n">
-        <v>-110</v>
+        <v>-112</v>
       </c>
       <c r="I77" s="15" t="n">
-        <v>0.5904462655465561</v>
+        <v>0.5943465059010947</v>
       </c>
       <c r="J77" s="15" t="n">
-        <v>0.5</v>
+        <v>0.5043297540699688</v>
       </c>
       <c r="K77" s="15" t="n">
-        <v>0.5238095238095238</v>
+        <v>0.5283018867924528</v>
       </c>
       <c r="L77" s="14" t="n">
-        <v>0.06663674173703227</v>
+        <v>0.0660446191086419</v>
       </c>
       <c r="M77" s="14" t="n">
-        <v>0.1272155978616072</v>
+        <v>0.1250130290270721</v>
       </c>
       <c r="N77" s="15" t="n">
         <v>0</v>
@@ -6299,7 +6299,7 @@
       </c>
       <c r="Q77" s="12" t="inlineStr">
         <is>
-          <t>outside the top 10 plays for this week</t>
+          <t>correlated with a stronger play on the same game</t>
         </is>
       </c>
     </row>
@@ -6311,12 +6311,12 @@
       </c>
       <c r="B78" s="17" t="inlineStr">
         <is>
-          <t>MSST @ MINN</t>
+          <t>OU @ MICH</t>
         </is>
       </c>
       <c r="C78" s="17" t="inlineStr">
         <is>
-          <t>2026-09-12 19:30</t>
+          <t>2026-09-12 16:00</t>
         </is>
       </c>
       <c r="D78" s="25" t="n">
@@ -6324,34 +6324,34 @@
       </c>
       <c r="E78" s="17" t="inlineStr">
         <is>
-          <t>ATS</t>
+          <t>TOTAL</t>
         </is>
       </c>
       <c r="F78" s="17" t="inlineStr">
         <is>
-          <t>MINN +1.5</t>
+          <t>Over 45.5</t>
         </is>
       </c>
       <c r="G78" s="26" t="n">
-        <v>1.5</v>
+        <v>45.5</v>
       </c>
       <c r="H78" s="18" t="n">
-        <v>-112</v>
+        <v>-108</v>
       </c>
       <c r="I78" s="20" t="n">
-        <v>0.5943465059010947</v>
+        <v>0.5828841461753553</v>
       </c>
       <c r="J78" s="20" t="n">
-        <v>0.5043297540699688</v>
+        <v>0.4956702459300312</v>
       </c>
       <c r="K78" s="20" t="n">
-        <v>0.5283018867924528</v>
+        <v>0.5192307692307693</v>
       </c>
       <c r="L78" s="19" t="n">
-        <v>0.0660446191086419</v>
+        <v>0.06365337694458606</v>
       </c>
       <c r="M78" s="19" t="n">
-        <v>0.1250130290270721</v>
+        <v>0.122591688930314</v>
       </c>
       <c r="N78" s="20" t="n">
         <v>0</v>
@@ -9268,16 +9268,16 @@
       </c>
       <c r="B125" s="12" t="inlineStr">
         <is>
-          <t>WSU @ WASH</t>
+          <t>PSU @ TEM</t>
         </is>
       </c>
       <c r="C125" s="12" t="inlineStr">
         <is>
-          <t>2026-09-06 20:00</t>
+          <t>2026-09-12 16:00</t>
         </is>
       </c>
       <c r="D125" s="22" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E125" s="12" t="inlineStr">
         <is>
@@ -9296,7 +9296,7 @@
         <v>-105</v>
       </c>
       <c r="I125" s="15" t="n">
-        <v>0.5085402935366987</v>
+        <v>0.5045564584546383</v>
       </c>
       <c r="J125" s="15" t="n">
         <v>0.4891657638136511</v>
@@ -9305,16 +9305,16 @@
         <v>0.5121951219512195</v>
       </c>
       <c r="L125" s="14" t="n">
-        <v>-0.003654828414520805</v>
+        <v>-0.007638663496581266</v>
       </c>
       <c r="M125" s="14" t="n">
-        <v>-0.007135617380731096</v>
+        <v>-0.01491358111237295</v>
       </c>
       <c r="N125" s="15" t="n">
         <v>0</v>
       </c>
       <c r="O125" s="24" t="n">
-        <v>0.4</v>
+        <v>0.725</v>
       </c>
       <c r="P125" s="12" t="inlineStr">
         <is>
@@ -9331,7 +9331,7 @@
       </c>
       <c r="B126" s="17" t="inlineStr">
         <is>
-          <t>PSU @ TEM</t>
+          <t>USF @ ARMY</t>
         </is>
       </c>
       <c r="C126" s="17" t="inlineStr">
@@ -9349,29 +9349,29 @@
       </c>
       <c r="F126" s="17" t="inlineStr">
         <is>
-          <t>Over 51.5</t>
+          <t>Under 52.5</t>
         </is>
       </c>
       <c r="G126" s="26" t="n">
-        <v>51.5</v>
+        <v>52.5</v>
       </c>
       <c r="H126" s="18" t="n">
-        <v>-105</v>
+        <v>-112</v>
       </c>
       <c r="I126" s="20" t="n">
-        <v>0.5045564584546383</v>
+        <v>0.520100508114556</v>
       </c>
       <c r="J126" s="20" t="n">
-        <v>0.4891657638136511</v>
+        <v>0.5043297540699688</v>
       </c>
       <c r="K126" s="20" t="n">
-        <v>0.5121951219512195</v>
+        <v>0.5283018867924528</v>
       </c>
       <c r="L126" s="19" t="n">
-        <v>-0.007638663496581266</v>
+        <v>-0.008201378677896831</v>
       </c>
       <c r="M126" s="19" t="n">
-        <v>-0.01491358111237295</v>
+        <v>-0.01552403821173332</v>
       </c>
       <c r="N126" s="20" t="n">
         <v>0</v>
@@ -9394,12 +9394,12 @@
       </c>
       <c r="B127" s="12" t="inlineStr">
         <is>
-          <t>USF @ ARMY</t>
+          <t>ARIZ @ BYU</t>
         </is>
       </c>
       <c r="C127" s="12" t="inlineStr">
         <is>
-          <t>2026-09-12 16:00</t>
+          <t>2026-09-12 19:30</t>
         </is>
       </c>
       <c r="D127" s="22" t="n">
@@ -9412,29 +9412,29 @@
       </c>
       <c r="F127" s="12" t="inlineStr">
         <is>
-          <t>Under 52.5</t>
+          <t>Over 51.5</t>
         </is>
       </c>
       <c r="G127" s="23" t="n">
-        <v>52.5</v>
+        <v>51.5</v>
       </c>
       <c r="H127" s="13" t="n">
-        <v>-112</v>
+        <v>-108</v>
       </c>
       <c r="I127" s="15" t="n">
-        <v>0.520100508114556</v>
+        <v>0.5078086995128284</v>
       </c>
       <c r="J127" s="15" t="n">
-        <v>0.5043297540699688</v>
+        <v>0.4956702459300312</v>
       </c>
       <c r="K127" s="15" t="n">
-        <v>0.5283018867924528</v>
+        <v>0.5192307692307693</v>
       </c>
       <c r="L127" s="14" t="n">
-        <v>-0.008201378677896831</v>
+        <v>-0.01142206971794091</v>
       </c>
       <c r="M127" s="14" t="n">
-        <v>-0.01552403821173332</v>
+        <v>-0.02199806019751566</v>
       </c>
       <c r="N127" s="15" t="n">
         <v>0</v>
@@ -9457,12 +9457,12 @@
       </c>
       <c r="B128" s="17" t="inlineStr">
         <is>
-          <t>ARIZ @ BYU</t>
+          <t>ODU @ VT</t>
         </is>
       </c>
       <c r="C128" s="17" t="inlineStr">
         <is>
-          <t>2026-09-12 19:30</t>
+          <t>2026-09-12 16:00</t>
         </is>
       </c>
       <c r="D128" s="25" t="n">
@@ -9482,22 +9482,22 @@
         <v>51.5</v>
       </c>
       <c r="H128" s="18" t="n">
-        <v>-108</v>
+        <v>-115</v>
       </c>
       <c r="I128" s="20" t="n">
-        <v>0.5078086995128284</v>
+        <v>0.5233527870201667</v>
       </c>
       <c r="J128" s="20" t="n">
-        <v>0.4956702459300312</v>
+        <v>0.5108342361863488</v>
       </c>
       <c r="K128" s="20" t="n">
-        <v>0.5192307692307693</v>
+        <v>0.5348837209302325</v>
       </c>
       <c r="L128" s="19" t="n">
-        <v>-0.01142206971794091</v>
+        <v>-0.01153093391006577</v>
       </c>
       <c r="M128" s="19" t="n">
-        <v>-0.02199806019751566</v>
+        <v>-0.02155783296229702</v>
       </c>
       <c r="N128" s="20" t="n">
         <v>0</v>
@@ -9520,16 +9520,16 @@
       </c>
       <c r="B129" s="12" t="inlineStr">
         <is>
-          <t>ODU @ VT</t>
+          <t>WSU @ WASH</t>
         </is>
       </c>
       <c r="C129" s="12" t="inlineStr">
         <is>
-          <t>2026-09-12 16:00</t>
+          <t>2026-09-06 20:00</t>
         </is>
       </c>
       <c r="D129" s="22" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E129" s="12" t="inlineStr">
         <is>
@@ -9545,28 +9545,28 @@
         <v>51.5</v>
       </c>
       <c r="H129" s="13" t="n">
-        <v>-115</v>
+        <v>-112</v>
       </c>
       <c r="I129" s="15" t="n">
-        <v>0.5233527870201667</v>
+        <v>0.5161222886648575</v>
       </c>
       <c r="J129" s="15" t="n">
-        <v>0.5108342361863488</v>
+        <v>0.5043297540699688</v>
       </c>
       <c r="K129" s="15" t="n">
-        <v>0.5348837209302325</v>
+        <v>0.5283018867924528</v>
       </c>
       <c r="L129" s="14" t="n">
-        <v>-0.01153093391006577</v>
+        <v>-0.01217959812759528</v>
       </c>
       <c r="M129" s="14" t="n">
-        <v>-0.02155783296229702</v>
+        <v>-0.02305423931294825</v>
       </c>
       <c r="N129" s="15" t="n">
         <v>0</v>
       </c>
       <c r="O129" s="24" t="n">
-        <v>0.725</v>
+        <v>0.4</v>
       </c>
       <c r="P129" s="12" t="inlineStr">
         <is>
@@ -10591,16 +10591,16 @@
       </c>
       <c r="B146" s="17" t="inlineStr">
         <is>
-          <t>ODU @ VT</t>
+          <t>WSU @ WASH</t>
         </is>
       </c>
       <c r="C146" s="17" t="inlineStr">
         <is>
-          <t>2026-09-12 16:00</t>
+          <t>2026-09-06 20:00</t>
         </is>
       </c>
       <c r="D146" s="25" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E146" s="17" t="inlineStr">
         <is>
@@ -10616,28 +10616,28 @@
         <v>51.5</v>
       </c>
       <c r="H146" s="18" t="n">
-        <v>-105</v>
+        <v>-108</v>
       </c>
       <c r="I146" s="20" t="n">
-        <v>0.4766472129798333</v>
+        <v>0.4838777113351425</v>
       </c>
       <c r="J146" s="20" t="n">
-        <v>0.4891657638136511</v>
+        <v>0.4956702459300312</v>
       </c>
       <c r="K146" s="20" t="n">
-        <v>0.5121951219512195</v>
+        <v>0.5192307692307693</v>
       </c>
       <c r="L146" s="19" t="n">
-        <v>-0.03554790897138627</v>
+        <v>-0.03535305789562682</v>
       </c>
       <c r="M146" s="19" t="n">
-        <v>-0.06940306037270655</v>
+        <v>-0.06808737076194782</v>
       </c>
       <c r="N146" s="20" t="n">
         <v>0</v>
       </c>
       <c r="O146" s="27" t="n">
-        <v>0.725</v>
+        <v>0.4</v>
       </c>
       <c r="P146" s="17" t="inlineStr">
         <is>
@@ -10654,12 +10654,12 @@
       </c>
       <c r="B147" s="12" t="inlineStr">
         <is>
-          <t>ARIZ @ BYU</t>
+          <t>ODU @ VT</t>
         </is>
       </c>
       <c r="C147" s="12" t="inlineStr">
         <is>
-          <t>2026-09-12 19:30</t>
+          <t>2026-09-12 16:00</t>
         </is>
       </c>
       <c r="D147" s="22" t="n">
@@ -10679,22 +10679,22 @@
         <v>51.5</v>
       </c>
       <c r="H147" s="13" t="n">
-        <v>-112</v>
+        <v>-105</v>
       </c>
       <c r="I147" s="15" t="n">
-        <v>0.4921913004871716</v>
+        <v>0.4766472129798333</v>
       </c>
       <c r="J147" s="15" t="n">
-        <v>0.5043297540699688</v>
+        <v>0.4891657638136511</v>
       </c>
       <c r="K147" s="15" t="n">
-        <v>0.5283018867924528</v>
+        <v>0.5121951219512195</v>
       </c>
       <c r="L147" s="14" t="n">
-        <v>-0.03611058630528119</v>
+        <v>-0.03554790897138627</v>
       </c>
       <c r="M147" s="14" t="n">
-        <v>-0.06835218122071085</v>
+        <v>-0.06940306037270655</v>
       </c>
       <c r="N147" s="15" t="n">
         <v>0</v>
@@ -10717,12 +10717,12 @@
       </c>
       <c r="B148" s="17" t="inlineStr">
         <is>
-          <t>USF @ ARMY</t>
+          <t>ARIZ @ BYU</t>
         </is>
       </c>
       <c r="C148" s="17" t="inlineStr">
         <is>
-          <t>2026-09-12 16:00</t>
+          <t>2026-09-12 19:30</t>
         </is>
       </c>
       <c r="D148" s="25" t="n">
@@ -10735,29 +10735,29 @@
       </c>
       <c r="F148" s="17" t="inlineStr">
         <is>
-          <t>Over 52.5</t>
+          <t>Under 51.5</t>
         </is>
       </c>
       <c r="G148" s="26" t="n">
-        <v>52.5</v>
+        <v>51.5</v>
       </c>
       <c r="H148" s="18" t="n">
-        <v>-108</v>
+        <v>-112</v>
       </c>
       <c r="I148" s="20" t="n">
-        <v>0.479899491885444</v>
+        <v>0.4921913004871716</v>
       </c>
       <c r="J148" s="20" t="n">
-        <v>0.4956702459300312</v>
+        <v>0.5043297540699688</v>
       </c>
       <c r="K148" s="20" t="n">
-        <v>0.5192307692307693</v>
+        <v>0.5283018867924528</v>
       </c>
       <c r="L148" s="19" t="n">
-        <v>-0.03933127734532527</v>
+        <v>-0.03611058630528119</v>
       </c>
       <c r="M148" s="19" t="n">
-        <v>-0.0757491267391448</v>
+        <v>-0.06835218122071085</v>
       </c>
       <c r="N148" s="20" t="n">
         <v>0</v>
@@ -10780,7 +10780,7 @@
       </c>
       <c r="B149" s="12" t="inlineStr">
         <is>
-          <t>PSU @ TEM</t>
+          <t>USF @ ARMY</t>
         </is>
       </c>
       <c r="C149" s="12" t="inlineStr">
@@ -10798,29 +10798,29 @@
       </c>
       <c r="F149" s="12" t="inlineStr">
         <is>
-          <t>Under 51.5</t>
+          <t>Over 52.5</t>
         </is>
       </c>
       <c r="G149" s="23" t="n">
-        <v>51.5</v>
+        <v>52.5</v>
       </c>
       <c r="H149" s="13" t="n">
-        <v>-115</v>
+        <v>-108</v>
       </c>
       <c r="I149" s="15" t="n">
-        <v>0.4954435415453617</v>
+        <v>0.479899491885444</v>
       </c>
       <c r="J149" s="15" t="n">
-        <v>0.5108342361863488</v>
+        <v>0.4956702459300312</v>
       </c>
       <c r="K149" s="15" t="n">
-        <v>0.5348837209302325</v>
+        <v>0.5192307692307693</v>
       </c>
       <c r="L149" s="14" t="n">
-        <v>-0.03944017938487077</v>
+        <v>-0.03933127734532527</v>
       </c>
       <c r="M149" s="14" t="n">
-        <v>-0.0737359875456281</v>
+        <v>-0.0757491267391448</v>
       </c>
       <c r="N149" s="15" t="n">
         <v>0</v>
@@ -10843,16 +10843,16 @@
       </c>
       <c r="B150" s="17" t="inlineStr">
         <is>
-          <t>WSU @ WASH</t>
+          <t>PSU @ TEM</t>
         </is>
       </c>
       <c r="C150" s="17" t="inlineStr">
         <is>
-          <t>2026-09-06 20:00</t>
+          <t>2026-09-12 16:00</t>
         </is>
       </c>
       <c r="D150" s="25" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E150" s="17" t="inlineStr">
         <is>
@@ -10871,7 +10871,7 @@
         <v>-115</v>
       </c>
       <c r="I150" s="20" t="n">
-        <v>0.4914597064633013</v>
+        <v>0.4954435415453617</v>
       </c>
       <c r="J150" s="20" t="n">
         <v>0.5108342361863488</v>
@@ -10880,16 +10880,16 @@
         <v>0.5348837209302325</v>
       </c>
       <c r="L150" s="19" t="n">
-        <v>-0.04342401446693123</v>
+        <v>-0.03944017938487077</v>
       </c>
       <c r="M150" s="19" t="n">
-        <v>-0.08118402704687161</v>
+        <v>-0.0737359875456281</v>
       </c>
       <c r="N150" s="20" t="n">
         <v>0</v>
       </c>
       <c r="O150" s="27" t="n">
-        <v>0.4</v>
+        <v>0.725</v>
       </c>
       <c r="P150" s="17" t="inlineStr">
         <is>
@@ -13780,12 +13780,12 @@
       </c>
       <c r="B197" s="12" t="inlineStr">
         <is>
-          <t>MSST @ MINN</t>
+          <t>OU @ MICH</t>
         </is>
       </c>
       <c r="C197" s="12" t="inlineStr">
         <is>
-          <t>2026-09-12 19:30</t>
+          <t>2026-09-12 16:00</t>
         </is>
       </c>
       <c r="D197" s="22" t="n">
@@ -13793,34 +13793,34 @@
       </c>
       <c r="E197" s="12" t="inlineStr">
         <is>
-          <t>ATS</t>
+          <t>TOTAL</t>
         </is>
       </c>
       <c r="F197" s="12" t="inlineStr">
         <is>
-          <t>MSST -1.5</t>
+          <t>Under 45.5</t>
         </is>
       </c>
       <c r="G197" s="23" t="n">
-        <v>1.5</v>
+        <v>45.5</v>
       </c>
       <c r="H197" s="13" t="n">
-        <v>-108</v>
+        <v>-112</v>
       </c>
       <c r="I197" s="15" t="n">
-        <v>0.4056534940989053</v>
+        <v>0.4171158538246447</v>
       </c>
       <c r="J197" s="15" t="n">
-        <v>0.4956702459300312</v>
+        <v>0.5043297540699688</v>
       </c>
       <c r="K197" s="15" t="n">
-        <v>0.5192307692307693</v>
+        <v>0.5283018867924528</v>
       </c>
       <c r="L197" s="14" t="n">
-        <v>-0.113577275131864</v>
+        <v>-0.1111860329678082</v>
       </c>
       <c r="M197" s="14" t="n">
-        <v>-0.2187414187724787</v>
+        <v>-0.2104592766890655</v>
       </c>
       <c r="N197" s="15" t="n">
         <v>0</v>
@@ -13843,12 +13843,12 @@
       </c>
       <c r="B198" s="17" t="inlineStr">
         <is>
-          <t>SDSU @ UCLA</t>
+          <t>MSST @ MINN</t>
         </is>
       </c>
       <c r="C198" s="17" t="inlineStr">
         <is>
-          <t>2026-09-12 23:15</t>
+          <t>2026-09-12 19:30</t>
         </is>
       </c>
       <c r="D198" s="25" t="n">
@@ -13856,34 +13856,34 @@
       </c>
       <c r="E198" s="17" t="inlineStr">
         <is>
-          <t>TOTAL</t>
+          <t>ATS</t>
         </is>
       </c>
       <c r="F198" s="17" t="inlineStr">
         <is>
-          <t>Under 48.5</t>
+          <t>MSST -1.5</t>
         </is>
       </c>
       <c r="G198" s="26" t="n">
-        <v>48.5</v>
+        <v>1.5</v>
       </c>
       <c r="H198" s="18" t="n">
-        <v>-110</v>
+        <v>-108</v>
       </c>
       <c r="I198" s="20" t="n">
-        <v>0.4095537344534439</v>
+        <v>0.4056534940989053</v>
       </c>
       <c r="J198" s="20" t="n">
-        <v>0.5</v>
+        <v>0.4956702459300312</v>
       </c>
       <c r="K198" s="20" t="n">
-        <v>0.5238095238095238</v>
+        <v>0.5192307692307693</v>
       </c>
       <c r="L198" s="19" t="n">
-        <v>-0.1142557893560799</v>
+        <v>-0.113577275131864</v>
       </c>
       <c r="M198" s="19" t="n">
-        <v>-0.218124688770698</v>
+        <v>-0.2187414187724787</v>
       </c>
       <c r="N198" s="20" t="n">
         <v>0</v>
@@ -13906,12 +13906,12 @@
       </c>
       <c r="B199" s="12" t="inlineStr">
         <is>
-          <t>MSST @ MINN</t>
+          <t>SDSU @ UCLA</t>
         </is>
       </c>
       <c r="C199" s="12" t="inlineStr">
         <is>
-          <t>2026-09-12 19:30</t>
+          <t>2026-09-12 23:15</t>
         </is>
       </c>
       <c r="D199" s="22" t="n">
@@ -13919,32 +13919,34 @@
       </c>
       <c r="E199" s="12" t="inlineStr">
         <is>
-          <t>ML</t>
+          <t>TOTAL</t>
         </is>
       </c>
       <c r="F199" s="12" t="inlineStr">
         <is>
-          <t>MSST ML</t>
-        </is>
-      </c>
-      <c r="G199" s="23" t="n"/>
+          <t>Under 48.5</t>
+        </is>
+      </c>
+      <c r="G199" s="23" t="n">
+        <v>48.5</v>
+      </c>
       <c r="H199" s="13" t="n">
-        <v>-125</v>
+        <v>-110</v>
       </c>
       <c r="I199" s="15" t="n">
-        <v>0.4406866615660716</v>
+        <v>0.4095537344534439</v>
       </c>
       <c r="J199" s="15" t="n">
-        <v>0.5324675324675325</v>
+        <v>0.5</v>
       </c>
       <c r="K199" s="15" t="n">
-        <v>0.5555555555555556</v>
+        <v>0.5238095238095238</v>
       </c>
       <c r="L199" s="14" t="n">
-        <v>-0.114868893989484</v>
+        <v>-0.1142557893560799</v>
       </c>
       <c r="M199" s="14" t="n">
-        <v>-0.2067640091810711</v>
+        <v>-0.218124688770698</v>
       </c>
       <c r="N199" s="15" t="n">
         <v>0</v>
@@ -13967,16 +13969,16 @@
       </c>
       <c r="B200" s="17" t="inlineStr">
         <is>
-          <t>OSU @ TEX</t>
+          <t>WIS @ ND</t>
         </is>
       </c>
       <c r="C200" s="17" t="inlineStr">
         <is>
-          <t>2026-09-12 23:30</t>
+          <t>2026-09-06 23:30</t>
         </is>
       </c>
       <c r="D200" s="25" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E200" s="17" t="inlineStr">
         <is>
@@ -13985,35 +13987,35 @@
       </c>
       <c r="F200" s="17" t="inlineStr">
         <is>
-          <t>Under 47.5</t>
+          <t>Under 46.5</t>
         </is>
       </c>
       <c r="G200" s="26" t="n">
-        <v>47.5</v>
+        <v>46.5</v>
       </c>
       <c r="H200" s="18" t="n">
-        <v>-110</v>
+        <v>-112</v>
       </c>
       <c r="I200" s="20" t="n">
-        <v>0.4077712444087197</v>
+        <v>0.4135094691627059</v>
       </c>
       <c r="J200" s="20" t="n">
-        <v>0.5</v>
+        <v>0.5043297540699688</v>
       </c>
       <c r="K200" s="20" t="n">
-        <v>0.5238095238095238</v>
+        <v>0.5283018867924528</v>
       </c>
       <c r="L200" s="19" t="n">
-        <v>-0.1160382794008041</v>
+        <v>-0.1147924176297469</v>
       </c>
       <c r="M200" s="19" t="n">
-        <v>-0.221527624310626</v>
+        <v>-0.2172856476563066</v>
       </c>
       <c r="N200" s="20" t="n">
         <v>0</v>
       </c>
       <c r="O200" s="27" t="n">
-        <v>0.725</v>
+        <v>0.4</v>
       </c>
       <c r="P200" s="17" t="inlineStr">
         <is>
@@ -14030,12 +14032,12 @@
       </c>
       <c r="B201" s="12" t="inlineStr">
         <is>
-          <t>USA @ TULN</t>
+          <t>MSST @ MINN</t>
         </is>
       </c>
       <c r="C201" s="12" t="inlineStr">
         <is>
-          <t>2026-09-12 23:00</t>
+          <t>2026-09-12 19:30</t>
         </is>
       </c>
       <c r="D201" s="22" t="n">
@@ -14043,37 +14045,35 @@
       </c>
       <c r="E201" s="12" t="inlineStr">
         <is>
-          <t>ATS</t>
+          <t>ML</t>
         </is>
       </c>
       <c r="F201" s="12" t="inlineStr">
         <is>
-          <t>TULN -10</t>
-        </is>
-      </c>
-      <c r="G201" s="23" t="n">
-        <v>-10</v>
-      </c>
+          <t>MSST ML</t>
+        </is>
+      </c>
+      <c r="G201" s="23" t="n"/>
       <c r="H201" s="13" t="n">
-        <v>-108</v>
+        <v>-125</v>
       </c>
       <c r="I201" s="15" t="n">
-        <v>0.4030606772358844</v>
+        <v>0.4406866615660716</v>
       </c>
       <c r="J201" s="15" t="n">
-        <v>0.4956702459300312</v>
+        <v>0.5324675324675325</v>
       </c>
       <c r="K201" s="15" t="n">
-        <v>0.5192307692307693</v>
+        <v>0.5555555555555556</v>
       </c>
       <c r="L201" s="14" t="n">
-        <v>-0.1161700919948849</v>
+        <v>-0.114868893989484</v>
       </c>
       <c r="M201" s="14" t="n">
-        <v>-0.2153021401066282</v>
+        <v>-0.2067640091810711</v>
       </c>
       <c r="N201" s="15" t="n">
-        <v>0.0377</v>
+        <v>0</v>
       </c>
       <c r="O201" s="24" t="n">
         <v>0.725</v>
@@ -14093,12 +14093,12 @@
       </c>
       <c r="B202" s="17" t="inlineStr">
         <is>
-          <t>OU @ MICH</t>
+          <t>OSU @ TEX</t>
         </is>
       </c>
       <c r="C202" s="17" t="inlineStr">
         <is>
-          <t>2026-09-12 16:00</t>
+          <t>2026-09-12 23:30</t>
         </is>
       </c>
       <c r="D202" s="25" t="n">
@@ -14111,29 +14111,29 @@
       </c>
       <c r="F202" s="17" t="inlineStr">
         <is>
-          <t>Under 44.5</t>
+          <t>Under 47.5</t>
         </is>
       </c>
       <c r="G202" s="26" t="n">
-        <v>44.5</v>
+        <v>47.5</v>
       </c>
       <c r="H202" s="18" t="n">
-        <v>-102</v>
+        <v>-110</v>
       </c>
       <c r="I202" s="20" t="n">
-        <v>0.3885782913337523</v>
+        <v>0.4077712444087197</v>
       </c>
       <c r="J202" s="20" t="n">
-        <v>0.4826358742837298</v>
+        <v>0.5</v>
       </c>
       <c r="K202" s="20" t="n">
-        <v>0.504950495049505</v>
+        <v>0.5238095238095238</v>
       </c>
       <c r="L202" s="19" t="n">
-        <v>-0.1163722037157526</v>
+        <v>-0.1160382794008041</v>
       </c>
       <c r="M202" s="19" t="n">
-        <v>-0.2304625995155101</v>
+        <v>-0.221527624310626</v>
       </c>
       <c r="N202" s="20" t="n">
         <v>0</v>
@@ -14156,53 +14156,53 @@
       </c>
       <c r="B203" s="12" t="inlineStr">
         <is>
-          <t>WIS @ ND</t>
+          <t>USA @ TULN</t>
         </is>
       </c>
       <c r="C203" s="12" t="inlineStr">
         <is>
-          <t>2026-09-06 23:30</t>
+          <t>2026-09-12 23:00</t>
         </is>
       </c>
       <c r="D203" s="22" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E203" s="12" t="inlineStr">
         <is>
-          <t>TOTAL</t>
+          <t>ATS</t>
         </is>
       </c>
       <c r="F203" s="12" t="inlineStr">
         <is>
-          <t>Under 46.5</t>
+          <t>TULN -10</t>
         </is>
       </c>
       <c r="G203" s="23" t="n">
-        <v>46.5</v>
+        <v>-10</v>
       </c>
       <c r="H203" s="13" t="n">
-        <v>-115</v>
+        <v>-108</v>
       </c>
       <c r="I203" s="15" t="n">
-        <v>0.4167617102208959</v>
+        <v>0.4030606772358844</v>
       </c>
       <c r="J203" s="15" t="n">
-        <v>0.5108342361863488</v>
+        <v>0.4956702459300312</v>
       </c>
       <c r="K203" s="15" t="n">
-        <v>0.5348837209302325</v>
+        <v>0.5192307692307693</v>
       </c>
       <c r="L203" s="14" t="n">
-        <v>-0.1181220107093366</v>
+        <v>-0.1161700919948849</v>
       </c>
       <c r="M203" s="14" t="n">
-        <v>-0.220836802630499</v>
+        <v>-0.2153021401066282</v>
       </c>
       <c r="N203" s="15" t="n">
-        <v>0</v>
+        <v>0.0377</v>
       </c>
       <c r="O203" s="24" t="n">
-        <v>0.4</v>
+        <v>0.725</v>
       </c>
       <c r="P203" s="12" t="inlineStr">
         <is>
@@ -14280,16 +14280,16 @@
       </c>
       <c r="B205" s="12" t="inlineStr">
         <is>
-          <t>ASU @ TA&amp;M</t>
+          <t>LOU @ MISS</t>
         </is>
       </c>
       <c r="C205" s="12" t="inlineStr">
         <is>
-          <t>2026-09-12 16:00</t>
+          <t>2026-09-06 23:30</t>
         </is>
       </c>
       <c r="D205" s="22" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E205" s="12" t="inlineStr">
         <is>
@@ -14298,44 +14298,40 @@
       </c>
       <c r="F205" s="12" t="inlineStr">
         <is>
-          <t>TA&amp;M ML</t>
+          <t>MISS ML</t>
         </is>
       </c>
       <c r="G205" s="23" t="n"/>
       <c r="H205" s="13" t="n">
-        <v>-650</v>
+        <v>-250</v>
       </c>
       <c r="I205" s="15" t="n">
-        <v>0.7419084049890994</v>
+        <v>0.5926966292134832</v>
       </c>
       <c r="J205" s="15" t="n">
-        <v>0.8316498316498315</v>
+        <v>0.6853932584269663</v>
       </c>
       <c r="K205" s="15" t="n">
-        <v>0.8666666666666667</v>
+        <v>0.7142857142857143</v>
       </c>
       <c r="L205" s="14" t="n">
-        <v>-0.1247582616775673</v>
+        <v>-0.1215890850722311</v>
       </c>
       <c r="M205" s="14" t="n">
-        <v>-0.1439518403971931</v>
+        <v>-0.1702247191011236</v>
       </c>
       <c r="N205" s="15" t="n">
         <v>0</v>
       </c>
       <c r="O205" s="24" t="n">
-        <v>0.725</v>
+        <v>0.4</v>
       </c>
       <c r="P205" s="12" t="inlineStr">
         <is>
           <t>DraftKings</t>
         </is>
       </c>
-      <c r="Q205" s="12" t="inlineStr">
-        <is>
-          <t>price outside allowed range</t>
-        </is>
-      </c>
+      <c r="Q205" s="12" t="n"/>
     </row>
     <row r="206">
       <c r="A206" s="17" t="inlineStr">
@@ -14345,12 +14341,12 @@
       </c>
       <c r="B206" s="17" t="inlineStr">
         <is>
-          <t>MTSU @ MRSH</t>
+          <t>ASU @ TA&amp;M</t>
         </is>
       </c>
       <c r="C206" s="17" t="inlineStr">
         <is>
-          <t>2026-09-12 23:00</t>
+          <t>2026-09-12 16:00</t>
         </is>
       </c>
       <c r="D206" s="25" t="n">
@@ -14358,34 +14354,32 @@
       </c>
       <c r="E206" s="17" t="inlineStr">
         <is>
-          <t>TOTAL</t>
+          <t>ML</t>
         </is>
       </c>
       <c r="F206" s="17" t="inlineStr">
         <is>
-          <t>Over 57.5</t>
-        </is>
-      </c>
-      <c r="G206" s="26" t="n">
-        <v>57.5</v>
-      </c>
+          <t>TA&amp;M ML</t>
+        </is>
+      </c>
+      <c r="G206" s="26" t="n"/>
       <c r="H206" s="18" t="n">
-        <v>-115</v>
+        <v>-650</v>
       </c>
       <c r="I206" s="20" t="n">
-        <v>0.4096491933569829</v>
+        <v>0.7419084049890994</v>
       </c>
       <c r="J206" s="20" t="n">
-        <v>0.5108342361863488</v>
+        <v>0.8316498316498315</v>
       </c>
       <c r="K206" s="20" t="n">
-        <v>0.5348837209302325</v>
+        <v>0.8666666666666667</v>
       </c>
       <c r="L206" s="19" t="n">
-        <v>-0.1252345275732496</v>
+        <v>-0.1247582616775673</v>
       </c>
       <c r="M206" s="19" t="n">
-        <v>-0.2341341167673798</v>
+        <v>-0.1439518403971931</v>
       </c>
       <c r="N206" s="20" t="n">
         <v>0</v>
@@ -14398,7 +14392,11 @@
           <t>DraftKings</t>
         </is>
       </c>
-      <c r="Q206" s="17" t="n"/>
+      <c r="Q206" s="17" t="inlineStr">
+        <is>
+          <t>price outside allowed range</t>
+        </is>
+      </c>
     </row>
     <row r="207">
       <c r="A207" s="12" t="inlineStr">
@@ -14408,51 +14406,53 @@
       </c>
       <c r="B207" s="12" t="inlineStr">
         <is>
-          <t>LOU @ MISS</t>
+          <t>MTSU @ MRSH</t>
         </is>
       </c>
       <c r="C207" s="12" t="inlineStr">
         <is>
-          <t>2026-09-06 23:30</t>
+          <t>2026-09-12 23:00</t>
         </is>
       </c>
       <c r="D207" s="22" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E207" s="12" t="inlineStr">
         <is>
-          <t>ML</t>
+          <t>TOTAL</t>
         </is>
       </c>
       <c r="F207" s="12" t="inlineStr">
         <is>
-          <t>MISS ML</t>
-        </is>
-      </c>
-      <c r="G207" s="23" t="n"/>
+          <t>Over 57.5</t>
+        </is>
+      </c>
+      <c r="G207" s="23" t="n">
+        <v>57.5</v>
+      </c>
       <c r="H207" s="13" t="n">
-        <v>-258</v>
+        <v>-115</v>
       </c>
       <c r="I207" s="15" t="n">
-        <v>0.5953964415270341</v>
+        <v>0.4096491933569829</v>
       </c>
       <c r="J207" s="15" t="n">
-        <v>0.6907928830540681</v>
+        <v>0.5108342361863488</v>
       </c>
       <c r="K207" s="15" t="n">
-        <v>0.7206703910614525</v>
+        <v>0.5348837209302325</v>
       </c>
       <c r="L207" s="14" t="n">
-        <v>-0.1252739495344184</v>
+        <v>-0.1252345275732496</v>
       </c>
       <c r="M207" s="14" t="n">
-        <v>-0.1738297439276039</v>
+        <v>-0.2341341167673798</v>
       </c>
       <c r="N207" s="15" t="n">
         <v>0</v>
       </c>
       <c r="O207" s="24" t="n">
-        <v>0.4</v>
+        <v>0.725</v>
       </c>
       <c r="P207" s="12" t="inlineStr">
         <is>
@@ -15353,12 +15353,12 @@
       </c>
       <c r="B222" s="17" t="inlineStr">
         <is>
-          <t>OU @ MICH</t>
+          <t>USU @ WASH</t>
         </is>
       </c>
       <c r="C222" s="17" t="inlineStr">
         <is>
-          <t>2026-09-12 16:00</t>
+          <t>2026-09-12 19:30</t>
         </is>
       </c>
       <c r="D222" s="25" t="n">
@@ -15366,47 +15366,49 @@
       </c>
       <c r="E222" s="17" t="inlineStr">
         <is>
-          <t>ATS</t>
+          <t>ML</t>
         </is>
       </c>
       <c r="F222" s="17" t="inlineStr">
         <is>
-          <t>OU -4.5</t>
-        </is>
-      </c>
-      <c r="G222" s="26" t="n">
-        <v>4.5</v>
-      </c>
+          <t>WASH ML</t>
+        </is>
+      </c>
+      <c r="G222" s="26" t="n"/>
       <c r="H222" s="18" t="n">
-        <v>-115</v>
+        <v>-2400</v>
       </c>
       <c r="I222" s="20" t="n">
-        <v>0.3828646618707011</v>
+        <v>0.8035054206790249</v>
       </c>
       <c r="J222" s="20" t="n">
-        <v>0.5108342361863488</v>
+        <v>0.9258160237388724</v>
       </c>
       <c r="K222" s="20" t="n">
-        <v>0.5348837209302325</v>
+        <v>0.96</v>
       </c>
       <c r="L222" s="19" t="n">
-        <v>-0.1520190590595314</v>
+        <v>-0.1564945793209751</v>
       </c>
       <c r="M222" s="19" t="n">
-        <v>-0.2842095451982545</v>
+        <v>-0.1630151867926824</v>
       </c>
       <c r="N222" s="20" t="n">
         <v>0</v>
       </c>
       <c r="O222" s="27" t="n">
-        <v>0.725</v>
+        <v>0.4</v>
       </c>
       <c r="P222" s="17" t="inlineStr">
         <is>
           <t>DraftKings</t>
         </is>
       </c>
-      <c r="Q222" s="17" t="n"/>
+      <c r="Q222" s="17" t="inlineStr">
+        <is>
+          <t>price outside allowed range</t>
+        </is>
+      </c>
     </row>
     <row r="223">
       <c r="A223" s="12" t="inlineStr">
@@ -15439,22 +15441,22 @@
       </c>
       <c r="G223" s="23" t="n"/>
       <c r="H223" s="13" t="n">
-        <v>-205</v>
+        <v>-218</v>
       </c>
       <c r="I223" s="15" t="n">
-        <v>0.5195330683271102</v>
+        <v>0.5259060920247964</v>
       </c>
       <c r="J223" s="15" t="n">
-        <v>0.6447291788002329</v>
+        <v>0.6574752261956054</v>
       </c>
       <c r="K223" s="15" t="n">
-        <v>0.6721311475409836</v>
+        <v>0.6855345911949685</v>
       </c>
       <c r="L223" s="14" t="n">
-        <v>-0.1525980792138734</v>
+        <v>-0.1596284991701721</v>
       </c>
       <c r="M223" s="14" t="n">
-        <v>-0.227036166635275</v>
+        <v>-0.2328525813583245</v>
       </c>
       <c r="N223" s="15" t="n">
         <v>0</v>
@@ -15477,12 +15479,12 @@
       </c>
       <c r="B224" s="17" t="inlineStr">
         <is>
-          <t>USU @ WASH</t>
+          <t>MTSU @ MRSH</t>
         </is>
       </c>
       <c r="C224" s="17" t="inlineStr">
         <is>
-          <t>2026-09-12 19:30</t>
+          <t>2026-09-12 23:00</t>
         </is>
       </c>
       <c r="D224" s="25" t="n">
@@ -15495,33 +15497,33 @@
       </c>
       <c r="F224" s="17" t="inlineStr">
         <is>
-          <t>WASH ML</t>
+          <t>MRSH ML</t>
         </is>
       </c>
       <c r="G224" s="26" t="n"/>
       <c r="H224" s="18" t="n">
-        <v>-2400</v>
+        <v>-1000</v>
       </c>
       <c r="I224" s="20" t="n">
-        <v>0.8035054206790249</v>
+        <v>0.7492447435969138</v>
       </c>
       <c r="J224" s="20" t="n">
-        <v>0.9258160237388724</v>
+        <v>0.8720930232558138</v>
       </c>
       <c r="K224" s="20" t="n">
-        <v>0.96</v>
+        <v>0.9090909090909091</v>
       </c>
       <c r="L224" s="19" t="n">
-        <v>-0.1564945793209751</v>
+        <v>-0.1598461654939952</v>
       </c>
       <c r="M224" s="19" t="n">
-        <v>-0.1630151867926824</v>
+        <v>-0.1758307820433947</v>
       </c>
       <c r="N224" s="20" t="n">
         <v>0</v>
       </c>
       <c r="O224" s="27" t="n">
-        <v>0.4</v>
+        <v>0.725</v>
       </c>
       <c r="P224" s="17" t="inlineStr">
         <is>
@@ -15542,12 +15544,12 @@
       </c>
       <c r="B225" s="12" t="inlineStr">
         <is>
-          <t>MTSU @ MRSH</t>
+          <t>NMSU @ HAW</t>
         </is>
       </c>
       <c r="C225" s="12" t="inlineStr">
         <is>
-          <t>2026-09-12 23:00</t>
+          <t>2026-09-13 03:59</t>
         </is>
       </c>
       <c r="D225" s="22" t="n">
@@ -15555,49 +15557,47 @@
       </c>
       <c r="E225" s="12" t="inlineStr">
         <is>
-          <t>ML</t>
+          <t>ATS</t>
         </is>
       </c>
       <c r="F225" s="12" t="inlineStr">
         <is>
-          <t>MRSH ML</t>
-        </is>
-      </c>
-      <c r="G225" s="23" t="n"/>
+          <t>HAW -11.5</t>
+        </is>
+      </c>
+      <c r="G225" s="23" t="n">
+        <v>-11.5</v>
+      </c>
       <c r="H225" s="13" t="n">
-        <v>-1000</v>
+        <v>-112</v>
       </c>
       <c r="I225" s="15" t="n">
-        <v>0.7492447435969138</v>
+        <v>0.366946682340708</v>
       </c>
       <c r="J225" s="15" t="n">
-        <v>0.8720930232558138</v>
+        <v>0.5043297540699688</v>
       </c>
       <c r="K225" s="15" t="n">
-        <v>0.9090909090909091</v>
+        <v>0.5283018867924528</v>
       </c>
       <c r="L225" s="14" t="n">
-        <v>-0.1598461654939952</v>
+        <v>-0.1613552044517448</v>
       </c>
       <c r="M225" s="14" t="n">
-        <v>-0.1758307820433947</v>
+        <v>-0.3054223512836598</v>
       </c>
       <c r="N225" s="15" t="n">
         <v>0</v>
       </c>
       <c r="O225" s="24" t="n">
-        <v>0.725</v>
+        <v>0.839</v>
       </c>
       <c r="P225" s="12" t="inlineStr">
         <is>
           <t>DraftKings</t>
         </is>
       </c>
-      <c r="Q225" s="12" t="inlineStr">
-        <is>
-          <t>price outside allowed range</t>
-        </is>
-      </c>
+      <c r="Q225" s="12" t="n"/>
     </row>
     <row r="226">
       <c r="A226" s="17" t="inlineStr">
@@ -15607,12 +15607,12 @@
       </c>
       <c r="B226" s="17" t="inlineStr">
         <is>
-          <t>NMSU @ HAW</t>
+          <t>OU @ MICH</t>
         </is>
       </c>
       <c r="C226" s="17" t="inlineStr">
         <is>
-          <t>2026-09-13 03:59</t>
+          <t>2026-09-12 16:00</t>
         </is>
       </c>
       <c r="D226" s="25" t="n">
@@ -15625,35 +15625,35 @@
       </c>
       <c r="F226" s="17" t="inlineStr">
         <is>
-          <t>HAW -11.5</t>
+          <t>OU -5.5</t>
         </is>
       </c>
       <c r="G226" s="26" t="n">
-        <v>-11.5</v>
+        <v>5.5</v>
       </c>
       <c r="H226" s="18" t="n">
-        <v>-112</v>
+        <v>-115</v>
       </c>
       <c r="I226" s="20" t="n">
-        <v>0.366946682340708</v>
+        <v>0.3729877233260379</v>
       </c>
       <c r="J226" s="20" t="n">
-        <v>0.5043297540699688</v>
+        <v>0.5108342361863488</v>
       </c>
       <c r="K226" s="20" t="n">
-        <v>0.5283018867924528</v>
+        <v>0.5348837209302325</v>
       </c>
       <c r="L226" s="19" t="n">
-        <v>-0.1613552044517448</v>
+        <v>-0.1618959976041946</v>
       </c>
       <c r="M226" s="19" t="n">
-        <v>-0.3054223512836598</v>
+        <v>-0.3026751259556683</v>
       </c>
       <c r="N226" s="20" t="n">
         <v>0</v>
       </c>
       <c r="O226" s="27" t="n">
-        <v>0.839</v>
+        <v>0.725</v>
       </c>
       <c r="P226" s="17" t="inlineStr">
         <is>
@@ -17847,53 +17847,51 @@
       </c>
       <c r="B260" s="17" t="inlineStr">
         <is>
-          <t>WIS @ ND</t>
+          <t>TLSA @ SHSU</t>
         </is>
       </c>
       <c r="C260" s="17" t="inlineStr">
         <is>
-          <t>2026-09-06 23:30</t>
+          <t>2026-09-12 23:00</t>
         </is>
       </c>
       <c r="D260" s="25" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E260" s="17" t="inlineStr">
         <is>
-          <t>ATS</t>
+          <t>ML</t>
         </is>
       </c>
       <c r="F260" s="17" t="inlineStr">
         <is>
-          <t>ND -20.5</t>
-        </is>
-      </c>
-      <c r="G260" s="26" t="n">
-        <v>-20.5</v>
-      </c>
+          <t>TLSA ML</t>
+        </is>
+      </c>
+      <c r="G260" s="26" t="n"/>
       <c r="H260" s="18" t="n">
-        <v>-115</v>
+        <v>-425</v>
       </c>
       <c r="I260" s="20" t="n">
-        <v>0.2801972900138555</v>
+        <v>0.5543580019223056</v>
       </c>
       <c r="J260" s="20" t="n">
-        <v>0.5108342361863488</v>
+        <v>0.7768331562167907</v>
       </c>
       <c r="K260" s="20" t="n">
-        <v>0.5348837209302325</v>
+        <v>0.8095238095238095</v>
       </c>
       <c r="L260" s="19" t="n">
-        <v>-0.254686430916377</v>
+        <v>-0.255165807601504</v>
       </c>
       <c r="M260" s="19" t="n">
-        <v>-0.4761528925827919</v>
+        <v>-0.315204821154799</v>
       </c>
       <c r="N260" s="20" t="n">
         <v>0</v>
       </c>
       <c r="O260" s="27" t="n">
-        <v>0.4</v>
+        <v>0.725</v>
       </c>
       <c r="P260" s="17" t="inlineStr">
         <is>
@@ -17902,7 +17900,7 @@
       </c>
       <c r="Q260" s="17" t="inlineStr">
         <is>
-          <t>raw model/market disagreement exceeds the safety limit</t>
+          <t>price outside allowed range</t>
         </is>
       </c>
     </row>
@@ -17914,12 +17912,12 @@
       </c>
       <c r="B261" s="12" t="inlineStr">
         <is>
-          <t>TLSA @ SHSU</t>
+          <t>UL @ USC</t>
         </is>
       </c>
       <c r="C261" s="12" t="inlineStr">
         <is>
-          <t>2026-09-12 23:00</t>
+          <t>2026-09-13 03:00</t>
         </is>
       </c>
       <c r="D261" s="22" t="n">
@@ -17927,32 +17925,34 @@
       </c>
       <c r="E261" s="12" t="inlineStr">
         <is>
-          <t>ML</t>
+          <t>ATS</t>
         </is>
       </c>
       <c r="F261" s="12" t="inlineStr">
         <is>
-          <t>TLSA ML</t>
-        </is>
-      </c>
-      <c r="G261" s="23" t="n"/>
+          <t>USC -28.5</t>
+        </is>
+      </c>
+      <c r="G261" s="23" t="n">
+        <v>-28.5</v>
+      </c>
       <c r="H261" s="13" t="n">
-        <v>-425</v>
+        <v>-110</v>
       </c>
       <c r="I261" s="15" t="n">
-        <v>0.5543580019223056</v>
+        <v>0.2658775966723402</v>
       </c>
       <c r="J261" s="15" t="n">
-        <v>0.7768331562167907</v>
+        <v>0.5</v>
       </c>
       <c r="K261" s="15" t="n">
-        <v>0.8095238095238095</v>
+        <v>0.5238095238095238</v>
       </c>
       <c r="L261" s="14" t="n">
-        <v>-0.255165807601504</v>
+        <v>-0.2579319271371837</v>
       </c>
       <c r="M261" s="14" t="n">
-        <v>-0.315204821154799</v>
+        <v>-0.492415497261896</v>
       </c>
       <c r="N261" s="15" t="n">
         <v>0</v>
@@ -17967,7 +17967,7 @@
       </c>
       <c r="Q261" s="12" t="inlineStr">
         <is>
-          <t>price outside allowed range</t>
+          <t>raw model/market disagreement exceeds the safety limit</t>
         </is>
       </c>
     </row>
@@ -17979,16 +17979,16 @@
       </c>
       <c r="B262" s="17" t="inlineStr">
         <is>
-          <t>UL @ USC</t>
+          <t>WIS @ ND</t>
         </is>
       </c>
       <c r="C262" s="17" t="inlineStr">
         <is>
-          <t>2026-09-13 03:00</t>
+          <t>2026-09-06 23:30</t>
         </is>
       </c>
       <c r="D262" s="25" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E262" s="17" t="inlineStr">
         <is>
@@ -17997,35 +17997,35 @@
       </c>
       <c r="F262" s="17" t="inlineStr">
         <is>
-          <t>USC -28.5</t>
+          <t>ND -21</t>
         </is>
       </c>
       <c r="G262" s="26" t="n">
-        <v>-28.5</v>
+        <v>-21</v>
       </c>
       <c r="H262" s="18" t="n">
-        <v>-110</v>
+        <v>-115</v>
       </c>
       <c r="I262" s="20" t="n">
-        <v>0.2658775966723402</v>
+        <v>0.2756446732989797</v>
       </c>
       <c r="J262" s="20" t="n">
-        <v>0.5</v>
+        <v>0.5108342361863488</v>
       </c>
       <c r="K262" s="20" t="n">
-        <v>0.5238095238095238</v>
+        <v>0.5348837209302325</v>
       </c>
       <c r="L262" s="19" t="n">
-        <v>-0.2579319271371837</v>
+        <v>-0.2592390476312528</v>
       </c>
       <c r="M262" s="19" t="n">
-        <v>-0.492415497261896</v>
+        <v>-0.4800652702801479</v>
       </c>
       <c r="N262" s="20" t="n">
-        <v>0</v>
+        <v>0.0095</v>
       </c>
       <c r="O262" s="27" t="n">
-        <v>0.725</v>
+        <v>0.4</v>
       </c>
       <c r="P262" s="17" t="inlineStr">
         <is>
@@ -19428,24 +19428,24 @@
       </c>
       <c r="B18" s="12" t="inlineStr">
         <is>
-          <t>EMU @ MSU</t>
+          <t>CAL @ SYR</t>
         </is>
       </c>
       <c r="C18" s="12" t="inlineStr">
         <is>
-          <t>ML</t>
+          <t>ATS</t>
         </is>
       </c>
       <c r="D18" s="12" t="inlineStr">
         <is>
-          <t>EMU ML</t>
+          <t>SYR +1.5</t>
         </is>
       </c>
       <c r="E18" s="13" t="n">
-        <v>550</v>
+        <v>-108</v>
       </c>
       <c r="F18" s="16" t="n">
-        <v>16.5</v>
+        <v>23</v>
       </c>
       <c r="G18" s="12" t="inlineStr">
         <is>
@@ -19466,17 +19466,17 @@
       </c>
       <c r="K18" s="12" t="inlineStr">
         <is>
-          <t>LEAN</t>
+          <t>GOOD</t>
         </is>
       </c>
       <c r="L18" s="14" t="n">
-        <v>0.1106</v>
+        <v>0.0987</v>
       </c>
       <c r="M18" s="14" t="n"/>
       <c r="N18" s="12" t="n"/>
       <c r="O18" s="12" t="inlineStr">
         <is>
-          <t>Draft Kings</t>
+          <t>DraftKings</t>
         </is>
       </c>
     </row>
@@ -19488,24 +19488,24 @@
       </c>
       <c r="B19" s="17" t="inlineStr">
         <is>
-          <t>CAL @ SYR</t>
+          <t>EMU @ MSU</t>
         </is>
       </c>
       <c r="C19" s="17" t="inlineStr">
         <is>
-          <t>ATS</t>
+          <t>ML</t>
         </is>
       </c>
       <c r="D19" s="17" t="inlineStr">
         <is>
-          <t>SYR +1.5</t>
+          <t>EMU ML</t>
         </is>
       </c>
       <c r="E19" s="18" t="n">
-        <v>-108</v>
+        <v>550</v>
       </c>
       <c r="F19" s="21" t="n">
-        <v>23</v>
+        <v>16.5</v>
       </c>
       <c r="G19" s="17" t="inlineStr">
         <is>
@@ -19526,17 +19526,17 @@
       </c>
       <c r="K19" s="17" t="inlineStr">
         <is>
-          <t>GOOD</t>
+          <t>LEAN</t>
         </is>
       </c>
       <c r="L19" s="19" t="n">
-        <v>0.0987</v>
+        <v>0.1106</v>
       </c>
       <c r="M19" s="19" t="n"/>
       <c r="N19" s="17" t="n"/>
       <c r="O19" s="17" t="inlineStr">
         <is>
-          <t>DraftKings</t>
+          <t>Draft Kings</t>
         </is>
       </c>
     </row>
@@ -19553,19 +19553,19 @@
       </c>
       <c r="C20" s="12" t="inlineStr">
         <is>
-          <t>TOTAL</t>
+          <t>ML</t>
         </is>
       </c>
       <c r="D20" s="12" t="inlineStr">
         <is>
-          <t>Over 46.5</t>
+          <t>MICH ML</t>
         </is>
       </c>
       <c r="E20" s="13" t="n">
-        <v>-105</v>
+        <v>170</v>
       </c>
       <c r="F20" s="16" t="n">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="G20" s="12" t="inlineStr">
         <is>
@@ -19586,17 +19586,17 @@
       </c>
       <c r="K20" s="12" t="inlineStr">
         <is>
-          <t>LEAN</t>
+          <t>GOOD</t>
         </is>
       </c>
       <c r="L20" s="14" t="n">
-        <v>0.0851</v>
+        <v>0.1101</v>
       </c>
       <c r="M20" s="14" t="n"/>
       <c r="N20" s="12" t="n"/>
       <c r="O20" s="12" t="inlineStr">
         <is>
-          <t>Draft Kings</t>
+          <t>DraftKings</t>
         </is>
       </c>
     </row>
@@ -19608,24 +19608,24 @@
       </c>
       <c r="B21" s="17" t="inlineStr">
         <is>
-          <t>ASU @ TA&amp;M</t>
+          <t>OU @ MICH</t>
         </is>
       </c>
       <c r="C21" s="17" t="inlineStr">
         <is>
-          <t>ATS</t>
+          <t>TOTAL</t>
         </is>
       </c>
       <c r="D21" s="17" t="inlineStr">
         <is>
-          <t>ASU +14.5</t>
+          <t>Over 46.5</t>
         </is>
       </c>
       <c r="E21" s="18" t="n">
-        <v>-110</v>
+        <v>-105</v>
       </c>
       <c r="F21" s="21" t="n">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="G21" s="17" t="inlineStr">
         <is>
@@ -19650,7 +19650,7 @@
         </is>
       </c>
       <c r="L21" s="19" t="n">
-        <v>0.1221</v>
+        <v>0.0851</v>
       </c>
       <c r="M21" s="19" t="n"/>
       <c r="N21" s="17" t="n"/>
@@ -19673,19 +19673,19 @@
       </c>
       <c r="C22" s="12" t="inlineStr">
         <is>
-          <t>ML</t>
+          <t>ATS</t>
         </is>
       </c>
       <c r="D22" s="12" t="inlineStr">
         <is>
-          <t>ASU ML</t>
+          <t>ASU +14.5</t>
         </is>
       </c>
       <c r="E22" s="13" t="n">
-        <v>410</v>
+        <v>-110</v>
       </c>
       <c r="F22" s="16" t="n">
-        <v>16.5</v>
+        <v>26</v>
       </c>
       <c r="G22" s="12" t="inlineStr">
         <is>
@@ -19710,13 +19710,13 @@
         </is>
       </c>
       <c r="L22" s="14" t="n">
-        <v>0.1061</v>
+        <v>0.1221</v>
       </c>
       <c r="M22" s="14" t="n"/>
       <c r="N22" s="12" t="n"/>
       <c r="O22" s="12" t="inlineStr">
         <is>
-          <t>DraftKings</t>
+          <t>Draft Kings</t>
         </is>
       </c>
     </row>
@@ -19733,19 +19733,19 @@
       </c>
       <c r="C23" s="17" t="inlineStr">
         <is>
-          <t>TOTAL</t>
+          <t>ML</t>
         </is>
       </c>
       <c r="D23" s="17" t="inlineStr">
         <is>
-          <t>Over 50.5</t>
+          <t>ASU ML</t>
         </is>
       </c>
       <c r="E23" s="18" t="n">
-        <v>-112</v>
+        <v>410</v>
       </c>
       <c r="F23" s="21" t="n">
-        <v>25</v>
+        <v>16.5</v>
       </c>
       <c r="G23" s="17" t="inlineStr">
         <is>
@@ -19770,13 +19770,13 @@
         </is>
       </c>
       <c r="L23" s="19" t="n">
-        <v>0.09660000000000001</v>
+        <v>0.1061</v>
       </c>
       <c r="M23" s="19" t="n"/>
       <c r="N23" s="17" t="n"/>
       <c r="O23" s="17" t="inlineStr">
         <is>
-          <t>Draft Kings</t>
+          <t>DraftKings</t>
         </is>
       </c>
     </row>
@@ -19788,7 +19788,7 @@
       </c>
       <c r="B24" s="12" t="inlineStr">
         <is>
-          <t>ORE @ OKST</t>
+          <t>ASU @ TA&amp;M</t>
         </is>
       </c>
       <c r="C24" s="12" t="inlineStr">
@@ -19798,14 +19798,14 @@
       </c>
       <c r="D24" s="12" t="inlineStr">
         <is>
-          <t>Under 60.5</t>
+          <t>Over 50.5</t>
         </is>
       </c>
       <c r="E24" s="13" t="n">
         <v>-112</v>
       </c>
       <c r="F24" s="16" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="G24" s="12" t="inlineStr">
         <is>
@@ -19830,7 +19830,7 @@
         </is>
       </c>
       <c r="L24" s="14" t="n">
-        <v>0.1106</v>
+        <v>0.09660000000000001</v>
       </c>
       <c r="M24" s="14" t="n"/>
       <c r="N24" s="12" t="n"/>
@@ -19848,24 +19848,24 @@
       </c>
       <c r="B25" s="17" t="inlineStr">
         <is>
-          <t>ODU @ VT</t>
+          <t>ORE @ OKST</t>
         </is>
       </c>
       <c r="C25" s="17" t="inlineStr">
         <is>
-          <t>ML</t>
+          <t>TOTAL</t>
         </is>
       </c>
       <c r="D25" s="17" t="inlineStr">
         <is>
-          <t>ODU ML</t>
+          <t>Under 60.5</t>
         </is>
       </c>
       <c r="E25" s="18" t="n">
-        <v>455</v>
+        <v>-112</v>
       </c>
       <c r="F25" s="21" t="n">
-        <v>15.5</v>
+        <v>26</v>
       </c>
       <c r="G25" s="17" t="inlineStr">
         <is>
@@ -19890,7 +19890,7 @@
         </is>
       </c>
       <c r="L25" s="19" t="n">
-        <v>0.1006</v>
+        <v>0.1106</v>
       </c>
       <c r="M25" s="19" t="n"/>
       <c r="N25" s="17" t="n"/>
@@ -19908,24 +19908,24 @@
       </c>
       <c r="B26" s="12" t="inlineStr">
         <is>
-          <t>WAKE @ PUR</t>
+          <t>ODU @ VT</t>
         </is>
       </c>
       <c r="C26" s="12" t="inlineStr">
         <is>
-          <t>ATS</t>
+          <t>ML</t>
         </is>
       </c>
       <c r="D26" s="12" t="inlineStr">
         <is>
-          <t>PUR +3.5</t>
+          <t>ODU ML</t>
         </is>
       </c>
       <c r="E26" s="13" t="n">
-        <v>-115</v>
+        <v>455</v>
       </c>
       <c r="F26" s="16" t="n">
-        <v>26</v>
+        <v>15.5</v>
       </c>
       <c r="G26" s="12" t="inlineStr">
         <is>
@@ -19946,11 +19946,11 @@
       </c>
       <c r="K26" s="12" t="inlineStr">
         <is>
-          <t>GOOD</t>
+          <t>LEAN</t>
         </is>
       </c>
       <c r="L26" s="14" t="n">
-        <v>0.0922</v>
+        <v>0.1006</v>
       </c>
       <c r="M26" s="14" t="n"/>
       <c r="N26" s="12" t="n"/>
@@ -19973,19 +19973,19 @@
       </c>
       <c r="C27" s="17" t="inlineStr">
         <is>
-          <t>TOTAL</t>
+          <t>ATS</t>
         </is>
       </c>
       <c r="D27" s="17" t="inlineStr">
         <is>
-          <t>Over 49.5</t>
+          <t>PUR +3.5</t>
         </is>
       </c>
       <c r="E27" s="18" t="n">
-        <v>-110</v>
+        <v>-115</v>
       </c>
       <c r="F27" s="21" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="G27" s="17" t="inlineStr">
         <is>
@@ -20006,11 +20006,11 @@
       </c>
       <c r="K27" s="17" t="inlineStr">
         <is>
-          <t>LEAN</t>
+          <t>GOOD</t>
         </is>
       </c>
       <c r="L27" s="19" t="n">
-        <v>0.1129</v>
+        <v>0.0922</v>
       </c>
       <c r="M27" s="19" t="n"/>
       <c r="N27" s="17" t="n"/>
@@ -20028,7 +20028,7 @@
       </c>
       <c r="B28" s="12" t="inlineStr">
         <is>
-          <t>PSU @ TEM</t>
+          <t>WAKE @ PUR</t>
         </is>
       </c>
       <c r="C28" s="12" t="inlineStr">
@@ -20038,11 +20038,11 @@
       </c>
       <c r="D28" s="12" t="inlineStr">
         <is>
-          <t>Over 51.5</t>
+          <t>Over 49.5</t>
         </is>
       </c>
       <c r="E28" s="13" t="n">
-        <v>-105</v>
+        <v>-110</v>
       </c>
       <c r="F28" s="16" t="n">
         <v>25</v>
@@ -20070,13 +20070,13 @@
         </is>
       </c>
       <c r="L28" s="14" t="n">
-        <v>0.09859999999999999</v>
+        <v>0.1129</v>
       </c>
       <c r="M28" s="14" t="n"/>
       <c r="N28" s="12" t="n"/>
       <c r="O28" s="12" t="inlineStr">
         <is>
-          <t>DraftKings</t>
+          <t>Draft Kings</t>
         </is>
       </c>
     </row>
@@ -20088,24 +20088,24 @@
       </c>
       <c r="B29" s="17" t="inlineStr">
         <is>
-          <t>APP @ ECU</t>
+          <t>PSU @ TEM</t>
         </is>
       </c>
       <c r="C29" s="17" t="inlineStr">
         <is>
-          <t>ATS</t>
+          <t>TOTAL</t>
         </is>
       </c>
       <c r="D29" s="17" t="inlineStr">
         <is>
-          <t>APP +10</t>
+          <t>Over 51.5</t>
         </is>
       </c>
       <c r="E29" s="18" t="n">
-        <v>-110</v>
+        <v>-105</v>
       </c>
       <c r="F29" s="21" t="n">
-        <v>22.5</v>
+        <v>25</v>
       </c>
       <c r="G29" s="17" t="inlineStr">
         <is>
@@ -20126,17 +20126,17 @@
       </c>
       <c r="K29" s="17" t="inlineStr">
         <is>
-          <t>GOOD</t>
+          <t>LEAN</t>
         </is>
       </c>
       <c r="L29" s="19" t="n">
-        <v>0.0818</v>
+        <v>0.09859999999999999</v>
       </c>
       <c r="M29" s="19" t="n"/>
       <c r="N29" s="17" t="n"/>
       <c r="O29" s="17" t="inlineStr">
         <is>
-          <t>Draft Kings</t>
+          <t>DraftKings</t>
         </is>
       </c>
     </row>
@@ -20148,24 +20148,24 @@
       </c>
       <c r="B30" s="12" t="inlineStr">
         <is>
-          <t>OU @ MICH</t>
+          <t>APP @ ECU</t>
         </is>
       </c>
       <c r="C30" s="12" t="inlineStr">
         <is>
-          <t>ML</t>
+          <t>ATS</t>
         </is>
       </c>
       <c r="D30" s="12" t="inlineStr">
         <is>
-          <t>MICH ML</t>
+          <t>APP +10</t>
         </is>
       </c>
       <c r="E30" s="13" t="n">
-        <v>170</v>
+        <v>-110</v>
       </c>
       <c r="F30" s="16" t="n">
-        <v>20</v>
+        <v>22.5</v>
       </c>
       <c r="G30" s="12" t="inlineStr">
         <is>
@@ -20190,13 +20190,13 @@
         </is>
       </c>
       <c r="L30" s="14" t="n">
-        <v>0.1101</v>
+        <v>0.0818</v>
       </c>
       <c r="M30" s="14" t="n"/>
       <c r="N30" s="12" t="n"/>
       <c r="O30" s="12" t="inlineStr">
         <is>
-          <t>DraftKings</t>
+          <t>Draft Kings</t>
         </is>
       </c>
     </row>
@@ -31664,10 +31664,10 @@
         <v>54.5</v>
       </c>
       <c r="K101" s="13" t="n">
-        <v>210</v>
+        <v>205</v>
       </c>
       <c r="L101" s="13" t="n">
-        <v>-258</v>
+        <v>-250</v>
       </c>
       <c r="M101" s="12" t="inlineStr">
         <is>
@@ -31711,7 +31711,7 @@
         </is>
       </c>
       <c r="I102" s="26" t="n">
-        <v>-20.5</v>
+        <v>-21</v>
       </c>
       <c r="J102" s="30" t="n">
         <v>46.5</v>
@@ -32055,16 +32055,16 @@
       </c>
       <c r="H110" s="17" t="inlineStr"/>
       <c r="I110" s="26" t="n">
-        <v>4.5</v>
+        <v>5.5</v>
       </c>
       <c r="J110" s="30" t="n">
-        <v>44.5</v>
+        <v>45.5</v>
       </c>
       <c r="K110" s="18" t="n">
-        <v>-205</v>
+        <v>-218</v>
       </c>
       <c r="L110" s="18" t="n">
-        <v>170</v>
+        <v>180</v>
       </c>
       <c r="M110" s="17" t="inlineStr">
         <is>

</xml_diff>